<commit_message>
Fix OLTP blank loan duration display and document verification
</commit_message>
<xml_diff>
--- a/Documents/AppSheet_Data_Dictionary.xlsx
+++ b/Documents/AppSheet_Data_Dictionary.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Re3bfc4ac406b431e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="R87e03c4747354fc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="Re1527714b54946bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R75b6566451fb4126"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="R86bb6bdffefe40c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R0545f66847c64d8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Rd3af4178374c4d7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="Re2ead377192147da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="Reb92849621844765"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R576eae966e1345c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R978a4ba07c8c4260"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="R75d6a21b95274030"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R2a868ad445134b0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R4613ddcc51d648f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="R67417f7e53dd4691"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="Rda1957a88dc94402"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Re70cec8acec54064"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R8d3d6b9820814c70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="Re7acea659d5e4ccb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="Ra17567394299421b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2349,7 +2349,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93b4f3212ec24d5b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70f9e137722642ce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2768,7 +2768,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c975c93679348ac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65e1100419c94299"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8507,30 +8507,31 @@
         <x:v>[Close Date]</x:v>
       </x:c>
     </x:row>
-    <x:row r="215" ht="15" customHeight="1">
-      <x:c r="A215" s="57" t="str">
+    <x:row r="215" ht="100" customHeight="1">
+      <x:c r="A215" s="82" t="str">
         <x:v>Loans</x:v>
       </x:c>
-      <x:c r="B215" s="57" t="n">
+      <x:c r="B215" s="82" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="C215" s="59" t="str">
+      <x:c r="C215" s="82" t="str">
         <x:v>Loan Duration</x:v>
       </x:c>
-      <x:c r="D215" s="59" t="str">
+      <x:c r="D215" s="82" t="str">
         <x:v>VC / Number</x:v>
       </x:c>
-      <x:c r="E215" s="57" t="str">
+      <x:c r="E215" s="82" t="str">
         <x:v>OLTP + OLAP</x:v>
       </x:c>
-      <x:c r="F215" s="57" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G215" s="59" t="str">
-        <x:v>Closed-loan duration in calendar days, based on Close Date and inclusive of the Loan Date.</x:v>
-      </x:c>
-      <x:c r="H215" s="59" t="str">
-        <x:v>IF( ISNOTBLANK([Close Date]), FLOOR(TOTALHOURS([Close Date] - [Loan Date]) / 24) + 1, "")</x:v>
+      <x:c r="F215" s="82" t="str">
+        <x:v>OLTP Show_If: ISNOTBLANK([Close Date]); OLAP unchanged</x:v>
+      </x:c>
+      <x:c r="G215" s="82" t="str">
+        <x:v>Closed-loan inclusive days. OLTP hides this field when Close Date is blank. Verified OLTP 3.000045; client acceptance pending.</x:v>
+      </x:c>
+      <x:c r="H215" s="82" t="str">
+        <x:v>OLTP: IF(ISNOTBLANK([Close Date]), FLOOR(TOTALHOURS([Close Date] - [Loan Date]) / 24) + 1, NUMBER(""))
+OLAP (unchanged documented formula): IF(ISNOTBLANK([Close Date]), FLOOR(TOTALHOURS([Close Date] - [Loan Date]) / 24) + 1, "")</x:v>
       </x:c>
     </x:row>
     <x:row r="216" ht="15" customHeight="1">
@@ -13268,7 +13269,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82452079846c4a65"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57edb54b226b48d5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13697,7 +13698,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7deb2b9fc0f942a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cb140f7855042e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14151,7 +14152,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R582be9882b104751"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d246e28a5a84a47"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20313,7 +20314,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1ff55aa7b3f41ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23a67f253c664d9d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24812,7 +24813,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re21d7c6b7f49410b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7369905d8e254a36"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25011,7 +25012,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5da0cbd605924f34"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10f1088617064b22"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26664,7 +26665,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc58431f867aa40d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e59f3d312674445"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record isolated OLTP performance lab and initial UI experiments
</commit_message>
<xml_diff>
--- a/Documents/AppSheet_Data_Dictionary.xlsx
+++ b/Documents/AppSheet_Data_Dictionary.xlsx
@@ -2,16 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R978a4ba07c8c4260"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="R75d6a21b95274030"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R2a868ad445134b0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R4613ddcc51d648f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="R67417f7e53dd4691"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="Rda1957a88dc94402"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Re70cec8acec54064"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R8d3d6b9820814c70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="Re7acea659d5e4ccb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="Ra17567394299421b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R32a5d246172544f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="Rf0ca5ad63efa4310"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R07da4098017e4194"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R1bece01d84ae4db8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="Rd690d0d1f5a94f0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R73343225c5e44584"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Rcb916faa39ac4fb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="Rda7e58d67ee840a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="Raabae55c90ae4d55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R4273b0fd2e364e70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="R5a7d7385f1494ed0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,7 +26,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="11">
+  <x:fonts count="13">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -85,8 +86,18 @@
       <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -121,6 +132,26 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -258,7 +289,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="89">
+  <x:cellXfs count="98">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -442,6 +473,27 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2349,8 +2401,493 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70f9e137722642ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra191bf39f8514c51"/>
   </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="38" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="55" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="100" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="97" t="str">
+        <x:v>Experiment</x:v>
+      </x:c>
+      <x:c r="B1" s="97" t="str">
+        <x:v>App version</x:v>
+      </x:c>
+      <x:c r="C1" s="97" t="str">
+        <x:v>Table</x:v>
+      </x:c>
+      <x:c r="D1" s="97" t="str">
+        <x:v>Column / setting</x:v>
+      </x:c>
+      <x:c r="E1" s="97" t="str">
+        <x:v>Type</x:v>
+      </x:c>
+      <x:c r="F1" s="97" t="str">
+        <x:v>Scope / status</x:v>
+      </x:c>
+      <x:c r="G1" s="97" t="str">
+        <x:v>Purpose / dependencies</x:v>
+      </x:c>
+      <x:c r="H1" s="97" t="str">
+        <x:v>Exact definition</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="150" customHeight="1">
+      <x:c r="A2" s="93" t="str">
+        <x:v>P02a</x:v>
+      </x:c>
+      <x:c r="B2" s="93" t="str">
+        <x:v>1.000012</x:v>
+      </x:c>
+      <x:c r="C2" s="93" t="str">
+        <x:v>Payments</x:v>
+      </x:c>
+      <x:c r="D2" s="93" t="str">
+        <x:v>Posted Amount</x:v>
+      </x:c>
+      <x:c r="E2" s="93" t="str">
+        <x:v>VC / Price</x:v>
+      </x:c>
+      <x:c r="F2" s="93" t="str">
+        <x:v>Isolated test in progress; no production change.</x:v>
+      </x:c>
+      <x:c r="G2" s="93" t="str">
+        <x:v>Use existing Related Repayments Ref list instead of full-table SELECT. Posting Difference depends on this value. Existing financial reconciliation action predicates unchanged.</x:v>
+      </x:c>
+      <x:c r="H2" s="93" t="str">
+        <x:v>SUM([Related Repayments][Amount Received])</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="150" customHeight="1">
+      <x:c r="A3" s="93" t="str">
+        <x:v>P03a</x:v>
+      </x:c>
+      <x:c r="B3" s="93" t="str">
+        <x:v>1.000006</x:v>
+      </x:c>
+      <x:c r="C3" s="93" t="str">
+        <x:v>Statistics</x:v>
+      </x:c>
+      <x:c r="D3" s="93" t="str">
+        <x:v>Security filter</x:v>
+      </x:c>
+      <x:c r="E3" s="93" t="str">
+        <x:v>Table filter</x:v>
+      </x:c>
+      <x:c r="F3" s="93" t="str">
+        <x:v>Clone-only diagnostic. Restored 1.000007.</x:v>
+      </x:c>
+      <x:c r="G3" s="93" t="str">
+        <x:v>FALSE excludes Statistics rows. Does not fully remove reporting definitions or all historical dependencies. No receipt-latency improvement demonstrated.</x:v>
+      </x:c>
+      <x:c r="H3" s="93" t="str">
+        <x:v>FALSE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="150" customHeight="1">
+      <x:c r="A4" s="93" t="str">
+        <x:v>P03a rollback</x:v>
+      </x:c>
+      <x:c r="B4" s="93" t="str">
+        <x:v>1.000007</x:v>
+      </x:c>
+      <x:c r="C4" s="93" t="str">
+        <x:v>Statistics</x:v>
+      </x:c>
+      <x:c r="D4" s="93" t="str">
+        <x:v>Security filter</x:v>
+      </x:c>
+      <x:c r="E4" s="93" t="str">
+        <x:v>Table filter</x:v>
+      </x:c>
+      <x:c r="F4" s="93" t="str">
+        <x:v>Original empty filter restored and verified.</x:v>
+      </x:c>
+      <x:c r="G4" s="93" t="str">
+        <x:v>Restores original row population. No data rows deleted.</x:v>
+      </x:c>
+      <x:c r="H4" s="93" t="str"/>
+    </x:row>
+    <x:row r="5" ht="150" customHeight="1">
+      <x:c r="A5" s="93" t="str">
+        <x:v>P01a</x:v>
+      </x:c>
+      <x:c r="B5" s="93" t="str">
+        <x:v>1.000004</x:v>
+      </x:c>
+      <x:c r="C5" s="93" t="str">
+        <x:v>Payments</x:v>
+      </x:c>
+      <x:c r="D5" s="93" t="str">
+        <x:v>Eligible Charges</x:v>
+      </x:c>
+      <x:c r="E5" s="93" t="str">
+        <x:v>VC / List Ref Charges</x:v>
+      </x:c>
+      <x:c r="F5" s="93" t="str">
+        <x:v>Test clone only. Restored at 1.000005.</x:v>
+      </x:c>
+      <x:c r="G5" s="93" t="str">
+        <x:v>Skip scans for Posted rows. Processing and Error eligibility unchanged. Eligible Outstanding consequently becomes zero on Posted rows. Freeze, Post and Reconcile checks retained.</x:v>
+      </x:c>
+      <x:c r="H5" s="93" t="str">
+        <x:v>IF([Status] = "Posted", LIST(), SELECT(Charges[Row ID], AND([Ref Loans].[Ref Borrowers] = [_THISROW].[Ref Borrower], [Amount Remaining] &gt; 0, IFS(IN([_THISROW].[Allocation Method], LIST("Single Full", "Single Partial", "First-day Auto")), [Row ID] = [_THISROW].[Ref Target Charge], [_THISROW].[Allocation Method] = "Loan Close", [Ref Loans] = [_THISROW].[Ref Target Charge].[Ref Loans], IN([_THISROW].[Allocation Method], LIST("Receive All", "Lump Sum")), [Charge Date] &lt;= [_THISROW].[Payment Date], TRUE, FALSE))))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="150" customHeight="1">
+      <x:c r="A6" s="93" t="str">
+        <x:v>P01a rollback</x:v>
+      </x:c>
+      <x:c r="B6" s="93" t="str">
+        <x:v>1.000005</x:v>
+      </x:c>
+      <x:c r="C6" s="93" t="str">
+        <x:v>Payments</x:v>
+      </x:c>
+      <x:c r="D6" s="93" t="str">
+        <x:v>Eligible Charges</x:v>
+      </x:c>
+      <x:c r="E6" s="93" t="str">
+        <x:v>VC / List Ref Charges</x:v>
+      </x:c>
+      <x:c r="F6" s="93" t="str">
+        <x:v>Test clone current baseline. Production definition unchanged.</x:v>
+      </x:c>
+      <x:c r="G6" s="93" t="str">
+        <x:v>Original full eligibility expression restored for reversal controls.</x:v>
+      </x:c>
+      <x:c r="H6" s="93" t="str">
+        <x:v>SELECT(Charges[Row ID], AND([Ref Loans].[Ref Borrowers] = [_THISROW].[Ref Borrower], [Amount Remaining] &gt; 0, IFS(IN([_THISROW].[Allocation Method], LIST("Single Full", "Single Partial", "First-day Auto")), [Row ID] = [_THISROW].[Ref Target Charge], [_THISROW].[Allocation Method] = "Loan Close", [Ref Loans] = [_THISROW].[Ref Target Charge].[Ref Loans], IN([_THISROW].[Allocation Method], LIST("Receive All", "Lump Sum")), [Charge Date] &lt;= [_THISROW].[Payment Date], TRUE, FALSE)))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="150" customHeight="1">
+      <x:c r="A7" s="93" t="str">
+        <x:v>P01b</x:v>
+      </x:c>
+      <x:c r="B7" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C7" s="93" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D7" s="93" t="str">
+        <x:v>Calculated Order</x:v>
+      </x:c>
+      <x:c r="E7" s="93" t="str">
+        <x:v>VC / Number</x:v>
+      </x:c>
+      <x:c r="F7" s="93" t="str">
+        <x:v>Rejected after failed receipt. Restored 1.000009.</x:v>
+      </x:c>
+      <x:c r="G7" s="93" t="str">
+        <x:v>Attempted frozen-value reuse. Allocation Order became 1 while stored components remained zero. Receipt Error, no repayment. Not an improvement despite faster Add response.</x:v>
+      </x:c>
+      <x:c r="H7" s="93" t="str">
+        <x:v>IF([Allocation Order] &gt; 0, [Allocation Order], 1 + COUNT(SELECT(Payment Allocations[Row ID], AND([Ref Payment] = [_THISROW].[Ref Payment], OR([Charge Date Snapshot] &gt; [_THISROW].[Charge Date Snapshot], AND([Charge Date Snapshot] = [_THISROW].[Charge Date Snapshot], [Charge Row Number Snapshot] &gt; [_THISROW].[Charge Row Number Snapshot]))))))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="150" customHeight="1">
+      <x:c r="A8" s="93" t="str">
+        <x:v>P01b</x:v>
+      </x:c>
+      <x:c r="B8" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C8" s="93" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D8" s="93" t="str">
+        <x:v>Calculated Amount</x:v>
+      </x:c>
+      <x:c r="E8" s="93" t="str">
+        <x:v>VC / Price</x:v>
+      </x:c>
+      <x:c r="F8" s="93" t="str">
+        <x:v>Rejected after failed receipt. Restored 1.000009.</x:v>
+      </x:c>
+      <x:c r="G8" s="93" t="str">
+        <x:v>Attempted frozen-value reuse. Allocation Order became 1 while stored components remained zero. Receipt Error, no repayment. Not an improvement despite faster Add response.</x:v>
+      </x:c>
+      <x:c r="H8" s="93" t="str">
+        <x:v>IF([Allocation Order] &gt; 0, [Allocated Amount], MAX(LIST(DECIMAL(0), MIN(LIST(DECIMAL([Amount Remaining Snapshot]), DECIMAL([Ref Payment].[Amount Received]) - DECIMAL(SUM(SELECT(Payment Allocations[Amount Remaining Snapshot], AND([Ref Payment] = [_THISROW].[Ref Payment], [Calculated Order] &lt; [_THISROW].[Calculated Order])))))))))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="150" customHeight="1">
+      <x:c r="A9" s="93" t="str">
+        <x:v>P01b</x:v>
+      </x:c>
+      <x:c r="B9" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C9" s="93" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D9" s="93" t="str">
+        <x:v>Calculated Interest</x:v>
+      </x:c>
+      <x:c r="E9" s="93" t="str">
+        <x:v>VC / Price</x:v>
+      </x:c>
+      <x:c r="F9" s="93" t="str">
+        <x:v>Rejected after failed receipt. Restored 1.000009.</x:v>
+      </x:c>
+      <x:c r="G9" s="93" t="str">
+        <x:v>Attempted frozen-value reuse. Allocation Order became 1 while stored components remained zero. Receipt Error, no repayment. Not an improvement despite faster Add response.</x:v>
+      </x:c>
+      <x:c r="H9" s="93" t="str">
+        <x:v>IF([Allocation Order] &gt; 0, [Allocated Interest], MIN(LIST(MAX(LIST(DECIMAL(0), DECIMAL([Interest Remaining Snapshot]))), DECIMAL([Calculated Amount]))))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="150" customHeight="1">
+      <x:c r="A10" s="93" t="str">
+        <x:v>P01b</x:v>
+      </x:c>
+      <x:c r="B10" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C10" s="93" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D10" s="93" t="str">
+        <x:v>Calculated Principal</x:v>
+      </x:c>
+      <x:c r="E10" s="93" t="str">
+        <x:v>VC / Price</x:v>
+      </x:c>
+      <x:c r="F10" s="93" t="str">
+        <x:v>Rejected after failed receipt. Restored 1.000009.</x:v>
+      </x:c>
+      <x:c r="G10" s="93" t="str">
+        <x:v>Attempted frozen-value reuse. Allocation Order became 1 while stored components remained zero. Receipt Error, no repayment. Not an improvement despite faster Add response.</x:v>
+      </x:c>
+      <x:c r="H10" s="93" t="str">
+        <x:v>IF([Allocation Order] &gt; 0, [Allocated Principal], MIN(LIST(MAX(LIST(DECIMAL(0), DECIMAL([Principal Remaining Snapshot]))), DECIMAL([Calculated Amount]) - DECIMAL([Calculated Interest]))))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="150" customHeight="1">
+      <x:c r="A11" s="93" t="str">
+        <x:v>P01b rollback</x:v>
+      </x:c>
+      <x:c r="B11" s="93" t="str">
+        <x:v>1.000009</x:v>
+      </x:c>
+      <x:c r="C11" s="93" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D11" s="93" t="str">
+        <x:v>Calculated Order</x:v>
+      </x:c>
+      <x:c r="E11" s="93" t="str">
+        <x:v>VC / Number</x:v>
+      </x:c>
+      <x:c r="F11" s="93" t="str">
+        <x:v>Original formulas restored and version verified.</x:v>
+      </x:c>
+      <x:c r="G11" s="93" t="str">
+        <x:v>Recovery uses original calculation and existing Retry after resetting only the unposted synthetic allocation's order from 1 to 0.</x:v>
+      </x:c>
+      <x:c r="H11" s="93" t="str">
+        <x:v>1 + COUNT(SELECT(Payment Allocations[Row ID], AND([Ref Payment] = [_THISROW].[Ref Payment], OR([Charge Date Snapshot] &gt; [_THISROW].[Charge Date Snapshot], AND([Charge Date Snapshot] = [_THISROW].[Charge Date Snapshot], [Charge Row Number Snapshot] &gt; [_THISROW].[Charge Row Number Snapshot])))))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="150" customHeight="1">
+      <x:c r="A12" s="93" t="str">
+        <x:v>P01b rollback</x:v>
+      </x:c>
+      <x:c r="B12" s="93" t="str">
+        <x:v>1.000009</x:v>
+      </x:c>
+      <x:c r="C12" s="93" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D12" s="93" t="str">
+        <x:v>Calculated Amount</x:v>
+      </x:c>
+      <x:c r="E12" s="93" t="str">
+        <x:v>VC / Price</x:v>
+      </x:c>
+      <x:c r="F12" s="93" t="str">
+        <x:v>Original formulas restored and version verified.</x:v>
+      </x:c>
+      <x:c r="G12" s="93" t="str">
+        <x:v>Recovery uses original calculation and existing Retry after resetting only the unposted synthetic allocation's order from 1 to 0.</x:v>
+      </x:c>
+      <x:c r="H12" s="93" t="str">
+        <x:v>MAX(LIST(DECIMAL(0), MIN(LIST(DECIMAL([Amount Remaining Snapshot]), DECIMAL([Ref Payment].[Amount Received]) - DECIMAL(SUM(SELECT(Payment Allocations[Amount Remaining Snapshot], AND([Ref Payment] = [_THISROW].[Ref Payment], [Calculated Order] &lt; [_THISROW].[Calculated Order]))))))))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="150" customHeight="1">
+      <x:c r="A13" s="93" t="str">
+        <x:v>P01b rollback</x:v>
+      </x:c>
+      <x:c r="B13" s="93" t="str">
+        <x:v>1.000009</x:v>
+      </x:c>
+      <x:c r="C13" s="93" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D13" s="93" t="str">
+        <x:v>Calculated Interest</x:v>
+      </x:c>
+      <x:c r="E13" s="93" t="str">
+        <x:v>VC / Price</x:v>
+      </x:c>
+      <x:c r="F13" s="93" t="str">
+        <x:v>Original formulas restored and version verified.</x:v>
+      </x:c>
+      <x:c r="G13" s="93" t="str">
+        <x:v>Recovery uses original calculation and existing Retry after resetting only the unposted synthetic allocation's order from 1 to 0.</x:v>
+      </x:c>
+      <x:c r="H13" s="93" t="str">
+        <x:v>MIN(LIST(MAX(LIST(DECIMAL(0), DECIMAL([Interest Remaining Snapshot]))), DECIMAL([Calculated Amount])))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="150" customHeight="1">
+      <x:c r="A14" s="93" t="str">
+        <x:v>P01b rollback</x:v>
+      </x:c>
+      <x:c r="B14" s="93" t="str">
+        <x:v>1.000009</x:v>
+      </x:c>
+      <x:c r="C14" s="93" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D14" s="93" t="str">
+        <x:v>Calculated Principal</x:v>
+      </x:c>
+      <x:c r="E14" s="93" t="str">
+        <x:v>VC / Price</x:v>
+      </x:c>
+      <x:c r="F14" s="93" t="str">
+        <x:v>Original formulas restored and version verified.</x:v>
+      </x:c>
+      <x:c r="G14" s="93" t="str">
+        <x:v>Recovery uses original calculation and existing Retry after resetting only the unposted synthetic allocation's order from 1 to 0.</x:v>
+      </x:c>
+      <x:c r="H14" s="93" t="str">
+        <x:v>MIN(LIST(MAX(LIST(DECIMAL(0), DECIMAL([Principal Remaining Snapshot]))), DECIMAL([Calculated Amount]) - DECIMAL([Calculated Interest])))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="150" customHeight="1">
+      <x:c r="A15" s="93" t="str">
+        <x:v>P01c</x:v>
+      </x:c>
+      <x:c r="B15" s="93" t="str">
+        <x:v>1.000010</x:v>
+      </x:c>
+      <x:c r="C15" s="93" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D15" s="93" t="str">
+        <x:v>Calculated Order</x:v>
+      </x:c>
+      <x:c r="E15" s="93" t="str">
+        <x:v>VC / Number</x:v>
+      </x:c>
+      <x:c r="F15" s="93" t="str">
+        <x:v>Three Posted samples. Restored 1.000011; not accepted for production.</x:v>
+      </x:c>
+      <x:c r="G15" s="93" t="str">
+        <x:v>Reuse stored helper values only after parent receipt is Posted. All Processing and Error calculations retain original expressions to avoid the P01b freeze-order failure.</x:v>
+      </x:c>
+      <x:c r="H15" s="93" t="str">
+        <x:v>IF([Ref Payment].[Status] = "Posted", [Allocation Order], 1 + COUNT(SELECT(Payment Allocations[Row ID], AND([Ref Payment] = [_THISROW].[Ref Payment], OR([Charge Date Snapshot] &gt; [_THISROW].[Charge Date Snapshot], AND([Charge Date Snapshot] = [_THISROW].[Charge Date Snapshot], [Charge Row Number Snapshot] &gt; [_THISROW].[Charge Row Number Snapshot]))))))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="150" customHeight="1">
+      <x:c r="A16" s="93" t="str">
+        <x:v>P01c</x:v>
+      </x:c>
+      <x:c r="B16" s="93" t="str">
+        <x:v>1.000010</x:v>
+      </x:c>
+      <x:c r="C16" s="93" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D16" s="93" t="str">
+        <x:v>Calculated Amount</x:v>
+      </x:c>
+      <x:c r="E16" s="93" t="str">
+        <x:v>VC / Price</x:v>
+      </x:c>
+      <x:c r="F16" s="93" t="str">
+        <x:v>Three Posted samples. Restored 1.000011; not accepted for production.</x:v>
+      </x:c>
+      <x:c r="G16" s="93" t="str">
+        <x:v>Reuse stored helper values only after parent receipt is Posted. All Processing and Error calculations retain original expressions to avoid the P01b freeze-order failure.</x:v>
+      </x:c>
+      <x:c r="H16" s="93" t="str">
+        <x:v>IF([Ref Payment].[Status] = "Posted", [Allocated Amount], MAX(LIST(DECIMAL(0), MIN(LIST(DECIMAL([Amount Remaining Snapshot]), DECIMAL([Ref Payment].[Amount Received]) - DECIMAL(SUM(SELECT(Payment Allocations[Amount Remaining Snapshot], AND([Ref Payment] = [_THISROW].[Ref Payment], [Calculated Order] &lt; [_THISROW].[Calculated Order])))))))))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="150" customHeight="1">
+      <x:c r="A17" s="93" t="str">
+        <x:v>P01c</x:v>
+      </x:c>
+      <x:c r="B17" s="93" t="str">
+        <x:v>1.000010</x:v>
+      </x:c>
+      <x:c r="C17" s="93" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D17" s="93" t="str">
+        <x:v>Calculated Interest</x:v>
+      </x:c>
+      <x:c r="E17" s="93" t="str">
+        <x:v>VC / Price</x:v>
+      </x:c>
+      <x:c r="F17" s="93" t="str">
+        <x:v>Three Posted samples. Restored 1.000011; not accepted for production.</x:v>
+      </x:c>
+      <x:c r="G17" s="93" t="str">
+        <x:v>Reuse stored helper values only after parent receipt is Posted. All Processing and Error calculations retain original expressions to avoid the P01b freeze-order failure.</x:v>
+      </x:c>
+      <x:c r="H17" s="93" t="str">
+        <x:v>IF([Ref Payment].[Status] = "Posted", [Allocated Interest], MIN(LIST(MAX(LIST(DECIMAL(0), DECIMAL([Interest Remaining Snapshot]))), DECIMAL([Calculated Amount]))))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="150" customHeight="1">
+      <x:c r="A18" s="93" t="str">
+        <x:v>P01c</x:v>
+      </x:c>
+      <x:c r="B18" s="93" t="str">
+        <x:v>1.000010</x:v>
+      </x:c>
+      <x:c r="C18" s="93" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D18" s="93" t="str">
+        <x:v>Calculated Principal</x:v>
+      </x:c>
+      <x:c r="E18" s="93" t="str">
+        <x:v>VC / Price</x:v>
+      </x:c>
+      <x:c r="F18" s="93" t="str">
+        <x:v>Three Posted samples. Restored 1.000011; not accepted for production.</x:v>
+      </x:c>
+      <x:c r="G18" s="93" t="str">
+        <x:v>Reuse stored helper values only after parent receipt is Posted. All Processing and Error calculations retain original expressions to avoid the P01b freeze-order failure.</x:v>
+      </x:c>
+      <x:c r="H18" s="93" t="str">
+        <x:v>IF([Ref Payment].[Status] = "Posted", [Allocated Principal], MIN(LIST(MAX(LIST(DECIMAL(0), DECIMAL([Principal Remaining Snapshot]))), DECIMAL([Calculated Amount]) - DECIMAL([Calculated Interest]))))</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
@@ -2768,7 +3305,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65e1100419c94299"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61a0a56b90bf4c19"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13269,7 +13806,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57edb54b226b48d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd21574397ba4b6a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13698,7 +14235,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cb140f7855042e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raddd74db07aa40d1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14152,7 +14689,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d246e28a5a84a47"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46dfcd6435b74222"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20314,7 +20851,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23a67f253c664d9d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a3aae16d3f842a7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24813,7 +25350,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7369905d8e254a36"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e01aa2a35344fc7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25012,7 +25549,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10f1088617064b22"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0520f58cb3e4219"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26665,7 +27202,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e59f3d312674445"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83875edb16244620"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record tuning comparisons and new-GUI-only cache test checkpoint
</commit_message>
<xml_diff>
--- a/Documents/AppSheet_Data_Dictionary.xlsx
+++ b/Documents/AppSheet_Data_Dictionary.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R32a5d246172544f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="Rf0ca5ad63efa4310"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R07da4098017e4194"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R1bece01d84ae4db8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="Rd690d0d1f5a94f0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R73343225c5e44584"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Rcb916faa39ac4fb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="Rda7e58d67ee840a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="Raabae55c90ae4d55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R4273b0fd2e364e70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="R5a7d7385f1494ed0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R59e42d0eb5594056"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="R6ac6453d12c6483d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="Rda90031e5a174c14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="Ra837a5ea449e4b9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="R658a96a33d3b49ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="Rc280eb80e53445b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="R8daaa05516ce442b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R48ce2de77c5745d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="R8403af4920f14a58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R60ad872993b94151"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="Refffd5c193504f4d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -97,7 +97,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="13">
+  <x:fills count="19">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -132,6 +132,36 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -289,7 +319,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="98">
+  <x:cellXfs count="104">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -494,6 +524,24 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="12" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2401,7 +2449,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra191bf39f8514c51"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ea27d42e7534a37"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2421,28 +2469,28 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="97" t="str">
+      <x:c r="A1" s="103" t="str">
         <x:v>Experiment</x:v>
       </x:c>
-      <x:c r="B1" s="97" t="str">
+      <x:c r="B1" s="103" t="str">
         <x:v>App version</x:v>
       </x:c>
-      <x:c r="C1" s="97" t="str">
+      <x:c r="C1" s="103" t="str">
         <x:v>Table</x:v>
       </x:c>
-      <x:c r="D1" s="97" t="str">
+      <x:c r="D1" s="103" t="str">
         <x:v>Column / setting</x:v>
       </x:c>
-      <x:c r="E1" s="97" t="str">
+      <x:c r="E1" s="103" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="F1" s="97" t="str">
+      <x:c r="F1" s="103" t="str">
         <x:v>Scope / status</x:v>
       </x:c>
-      <x:c r="G1" s="97" t="str">
+      <x:c r="G1" s="103" t="str">
         <x:v>Purpose / dependencies</x:v>
       </x:c>
-      <x:c r="H1" s="97" t="str">
+      <x:c r="H1" s="103" t="str">
         <x:v>Exact definition</x:v>
       </x:c>
     </x:row>
@@ -2463,7 +2511,7 @@
         <x:v>VC / Price</x:v>
       </x:c>
       <x:c r="F2" s="93" t="str">
-        <x:v>Isolated test in progress; no production change.</x:v>
+        <x:v>Three Posted samples; restored and verified 1.000013. No production change.</x:v>
       </x:c>
       <x:c r="G2" s="93" t="str">
         <x:v>Use existing Related Repayments Ref list instead of full-table SELECT. Posting Difference depends on this value. Existing financial reconciliation action predicates unchanged.</x:v>
@@ -2884,6 +2932,422 @@
       </x:c>
       <x:c r="H18" s="93" t="str">
         <x:v>IF([Ref Payment].[Status] = "Posted", [Allocated Principal], MIN(LIST(MAX(LIST(DECIMAL(0), DECIMAL([Principal Remaining Snapshot]))), DECIMAL([Calculated Amount]) - DECIMAL([Calculated Interest]))))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="150" customHeight="1">
+      <x:c r="A19" s="93" t="str">
+        <x:v>P02a rollback</x:v>
+      </x:c>
+      <x:c r="B19" s="93" t="str">
+        <x:v>1.000013</x:v>
+      </x:c>
+      <x:c r="C19" s="93" t="str">
+        <x:v>Payments</x:v>
+      </x:c>
+      <x:c r="D19" s="93" t="str">
+        <x:v>Posted Amount</x:v>
+      </x:c>
+      <x:c r="E19" s="93" t="str">
+        <x:v>VC / Price</x:v>
+      </x:c>
+      <x:c r="F19" s="93" t="str">
+        <x:v>Original formula restored and verified.</x:v>
+      </x:c>
+      <x:c r="G19" s="93" t="str">
+        <x:v>Restores baseline full-table SELECT; Posting Difference dependency unchanged.</x:v>
+      </x:c>
+      <x:c r="H19" s="93" t="str">
+        <x:v>SUM(SELECT(Repayments[Amount Received], [Ref Payment] = [_THISROW].[Row ID]))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="150" customHeight="1">
+      <x:c r="A20" s="93" t="str">
+        <x:v>P04a</x:v>
+      </x:c>
+      <x:c r="B20" s="93" t="str">
+        <x:v>1.000014</x:v>
+      </x:c>
+      <x:c r="C20" s="93" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D20" s="93" t="str">
+        <x:v>Calculated Amount</x:v>
+      </x:c>
+      <x:c r="E20" s="93" t="str">
+        <x:v>VC / Price</x:v>
+      </x:c>
+      <x:c r="F20" s="93" t="str">
+        <x:v>Three Posted samples; original restored and verified at 1.000018.</x:v>
+      </x:c>
+      <x:c r="G20" s="93" t="str">
+        <x:v>Compare immutable snapshot date/row number directly instead of nested Calculated Order evaluation. Preserves newest-first and tie ordering, full allocation coverage, zero rows and posting guards.</x:v>
+      </x:c>
+      <x:c r="H20" s="93" t="str">
+        <x:v>MAX(LIST(DECIMAL(0), MIN(LIST(DECIMAL([Amount Remaining Snapshot]), DECIMAL([Ref Payment].[Amount Received]) - DECIMAL(SUM(SELECT(Payment Allocations[Amount Remaining Snapshot], AND([Ref Payment] = [_THISROW].[Ref Payment], OR([Charge Date Snapshot] &gt; [_THISROW].[Charge Date Snapshot], AND([Charge Date Snapshot] = [_THISROW].[Charge Date Snapshot], [Charge Row Number Snapshot] &gt; [_THISROW].[Charge Row Number Snapshot]))))))))))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="150" customHeight="1">
+      <x:c r="A21" s="93" t="str">
+        <x:v>P06-cache</x:v>
+      </x:c>
+      <x:c r="B21" s="93" t="str">
+        <x:v>1.000015</x:v>
+      </x:c>
+      <x:c r="C21" s="93" t="str">
+        <x:v>App settings</x:v>
+      </x:c>
+      <x:c r="D21" s="93" t="str">
+        <x:v>Server caching</x:v>
+      </x:c>
+      <x:c r="E21" s="93" t="str">
+        <x:v>Setting</x:v>
+      </x:c>
+      <x:c r="F21" s="93" t="str">
+        <x:v>Verified ON in clone; API remains OFF.</x:v>
+      </x:c>
+      <x:c r="G21" s="93" t="str">
+        <x:v>Only caching changed; P04a retained. Delta OFF, Quick ON; warm explicit sync samples exclude initialization and editor preview.</x:v>
+      </x:c>
+      <x:c r="H21" s="93" t="str">
+        <x:v>ON (prior OFF)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="150" customHeight="1">
+      <x:c r="A22" s="93" t="str">
+        <x:v>P06-delta</x:v>
+      </x:c>
+      <x:c r="B22" s="93" t="str">
+        <x:v>1.000016</x:v>
+      </x:c>
+      <x:c r="C22" s="93" t="str">
+        <x:v>App settings</x:v>
+      </x:c>
+      <x:c r="D22" s="93" t="str">
+        <x:v>Delta sync</x:v>
+      </x:c>
+      <x:c r="E22" s="93" t="str">
+        <x:v>Setting</x:v>
+      </x:c>
+      <x:c r="F22" s="93" t="str">
+        <x:v>Five idle syncs; direct note freshness and restoration passed. Restored OFF at 1.000017.</x:v>
+      </x:c>
+      <x:c r="G22" s="93" t="str">
+        <x:v>Cache ON and Quick ON retained; compare with 1.000015. Date-driven VC rollover and cross-table freshness not certified.</x:v>
+      </x:c>
+      <x:c r="H22" s="93" t="str">
+        <x:v>ON (prior OFF)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="150" customHeight="1">
+      <x:c r="A23" s="93" t="str">
+        <x:v>P06-quick</x:v>
+      </x:c>
+      <x:c r="B23" s="93" t="str">
+        <x:v>1.000017</x:v>
+      </x:c>
+      <x:c r="C23" s="93" t="str">
+        <x:v>App settings</x:v>
+      </x:c>
+      <x:c r="D23" s="93" t="str">
+        <x:v>Quick sync</x:v>
+      </x:c>
+      <x:c r="E23" s="93" t="str">
+        <x:v>Setting</x:v>
+      </x:c>
+      <x:c r="F23" s="93" t="str">
+        <x:v>Five idle syncs; median 1.312s. Restored ON at 1.000018.</x:v>
+      </x:c>
+      <x:c r="G23" s="93" t="str">
+        <x:v>Delta restored OFF and cache remains ON. Compare to 1.000015, differing only in Quick sync.</x:v>
+      </x:c>
+      <x:c r="H23" s="93" t="str">
+        <x:v>OFF (prior ON)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="150" customHeight="1">
+      <x:c r="A24" s="93" t="str">
+        <x:v>P04a rollback</x:v>
+      </x:c>
+      <x:c r="B24" s="93" t="str">
+        <x:v>1.000018</x:v>
+      </x:c>
+      <x:c r="C24" s="93" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D24" s="93" t="str">
+        <x:v>Calculated Amount</x:v>
+      </x:c>
+      <x:c r="E24" s="93" t="str">
+        <x:v>VC / Price</x:v>
+      </x:c>
+      <x:c r="F24" s="93" t="str">
+        <x:v>Original verified in saved appdoc.</x:v>
+      </x:c>
+      <x:c r="G24" s="93" t="str">
+        <x:v>Baseline formula restored; all earlier formula variants restored.</x:v>
+      </x:c>
+      <x:c r="H24" s="93" t="str">
+        <x:v>MAX(LIST(DECIMAL(0), MIN(LIST(DECIMAL([Amount Remaining Snapshot]), DECIMAL([Ref Payment].[Amount Received]) - DECIMAL(SUM(SELECT(Payment Allocations[Amount Remaining Snapshot], AND([Ref Payment] = [_THISROW].[Ref Payment], [Calculated Order] &lt; [_THISROW].[Calculated Order]))))))))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="150" customHeight="1">
+      <x:c r="A25" s="93" t="str">
+        <x:v>P06 rollback</x:v>
+      </x:c>
+      <x:c r="B25" s="93" t="str">
+        <x:v>1.000018</x:v>
+      </x:c>
+      <x:c r="C25" s="93" t="str">
+        <x:v>App settings</x:v>
+      </x:c>
+      <x:c r="D25" s="93" t="str">
+        <x:v>Sync settings</x:v>
+      </x:c>
+      <x:c r="E25" s="93" t="str">
+        <x:v>Settings</x:v>
+      </x:c>
+      <x:c r="F25" s="93" t="str">
+        <x:v>Isolation baseline restored.</x:v>
+      </x:c>
+      <x:c r="G25" s="93" t="str">
+        <x:v>Server cache OFF; delta OFF; quick ON. Start sync, delayed sync and automatic updates retained ON.</x:v>
+      </x:c>
+      <x:c r="H25" s="93" t="str">
+        <x:v>Cache OFF; Delta OFF; Quick ON</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="150" customHeight="1">
+      <x:c r="A26" s="93" t="str">
+        <x:v>P03b intermediate</x:v>
+      </x:c>
+      <x:c r="B26" s="93" t="str">
+        <x:v>1.000019</x:v>
+      </x:c>
+      <x:c r="C26" s="93" t="str">
+        <x:v>Statistics</x:v>
+      </x:c>
+      <x:c r="D26" s="93" t="str">
+        <x:v>App table availability</x:v>
+      </x:c>
+      <x:c r="E26" s="93" t="str">
+        <x:v>Table / 26 columns, 23 VC</x:v>
+      </x:c>
+      <x:c r="F26" s="93" t="str">
+        <x:v>Removed from test app; non-runnable until dependent views repaired.</x:v>
+      </x:c>
+      <x:c r="G26" s="93" t="str">
+        <x:v>Database table retained. Missing KPIs and Reporting App Shortcut caused load errors. No receipts submitted in this invalid version.</x:v>
+      </x:c>
+      <x:c r="H26" s="93" t="str">
+        <x:v>ABSENT from clone app; physical database unchanged</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="150" customHeight="1">
+      <x:c r="A27" s="93" t="str">
+        <x:v>P03b</x:v>
+      </x:c>
+      <x:c r="B27" s="93" t="str">
+        <x:v>1.000020</x:v>
+      </x:c>
+      <x:c r="C27" s="93" t="str">
+        <x:v>Statistics</x:v>
+      </x:c>
+      <x:c r="D27" s="93" t="str">
+        <x:v>App table availability</x:v>
+      </x:c>
+      <x:c r="E27" s="93" t="str">
+        <x:v>Table / 26 columns, 23 VC</x:v>
+      </x:c>
+      <x:c r="F27" s="93" t="str">
+        <x:v>Three Posted six-charge samples. Restored complete definition at verified 1.000022.</x:v>
+      </x:c>
+      <x:c r="G27" s="93" t="str">
+        <x:v>Diagnostic only. Associated format rules removed by editor; manual generation and reporting actions need review before any real migration. Full rollback 1.000018.</x:v>
+      </x:c>
+      <x:c r="H27" s="93" t="str">
+        <x:v>ABSENT from clone app; physical database unchanged</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="150" customHeight="1">
+      <x:c r="A28" s="93" t="str">
+        <x:v>P03b rollback</x:v>
+      </x:c>
+      <x:c r="B28" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C28" s="93" t="str">
+        <x:v>Statistics</x:v>
+      </x:c>
+      <x:c r="D28" s="93" t="str">
+        <x:v>App table availability</x:v>
+      </x:c>
+      <x:c r="E28" s="93" t="str">
+        <x:v>Table / 26 columns, 23 VC</x:v>
+      </x:c>
+      <x:c r="F28" s="93" t="str">
+        <x:v>Restored complete 1.000018 using native version history.</x:v>
+      </x:c>
+      <x:c r="G28" s="93" t="str">
+        <x:v>Statistics, KPIs, Reporting App Shortcut verified present; configuration baseline restored before materialization.</x:v>
+      </x:c>
+      <x:c r="H28" s="93" t="str">
+        <x:v>PRESENT; original definitions restored</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="150" customHeight="1">
+      <x:c r="A29" s="93" t="str">
+        <x:v>P09 schema</x:v>
+      </x:c>
+      <x:c r="B29" s="93" t="str">
+        <x:v>1.000025</x:v>
+      </x:c>
+      <x:c r="C29" s="93" t="str">
+        <x:v>Charges</x:v>
+      </x:c>
+      <x:c r="D29" s="93" t="str">
+        <x:v>Perf Cached Principal Paid</x:v>
+      </x:c>
+      <x:c r="E29" s="93" t="str">
+        <x:v>Physical / Price</x:v>
+      </x:c>
+      <x:c r="F29" s="93" t="str">
+        <x:v>Test-only; hidden and nonsearchable; writable by refresh action.</x:v>
+      </x:c>
+      <x:c r="G29" s="93" t="str">
+        <x:v>Regenerated at 1.000023; all original 25 column key/type/label/formula/qualifier definitions verified unchanged. Initially hidden and readonly at 1.000024, then writable at 1.000025 for data-action assignment. No cache-reader changes yet.</x:v>
+      </x:c>
+      <x:c r="H29" s="93" t="str">
+        <x:v>No app formula; ledger-derived value populated by explicit refresh</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="150" customHeight="1">
+      <x:c r="A30" s="93" t="str">
+        <x:v>P09 schema</x:v>
+      </x:c>
+      <x:c r="B30" s="93" t="str">
+        <x:v>1.000025</x:v>
+      </x:c>
+      <x:c r="C30" s="93" t="str">
+        <x:v>Charges</x:v>
+      </x:c>
+      <x:c r="D30" s="93" t="str">
+        <x:v>Perf Cached Interest Paid</x:v>
+      </x:c>
+      <x:c r="E30" s="93" t="str">
+        <x:v>Physical / Price</x:v>
+      </x:c>
+      <x:c r="F30" s="93" t="str">
+        <x:v>Test-only; hidden and nonsearchable; writable by refresh action.</x:v>
+      </x:c>
+      <x:c r="G30" s="93" t="str">
+        <x:v>Regenerated at 1.000023; all original 25 column key/type/label/formula/qualifier definitions verified unchanged. Initially hidden and readonly at 1.000024, then writable at 1.000025 for data-action assignment. No cache-reader changes yet.</x:v>
+      </x:c>
+      <x:c r="H30" s="93" t="str">
+        <x:v>No app formula; ledger-derived value populated by explicit refresh</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="150" customHeight="1">
+      <x:c r="A31" s="93" t="str">
+        <x:v>P09 refresh</x:v>
+      </x:c>
+      <x:c r="B31" s="93" t="str">
+        <x:v>1.000025</x:v>
+      </x:c>
+      <x:c r="C31" s="93" t="str">
+        <x:v>Charges</x:v>
+      </x:c>
+      <x:c r="D31" s="93" t="str">
+        <x:v>Perf - Refresh Charge Paid Cache</x:v>
+      </x:c>
+      <x:c r="E31" s="93" t="str">
+        <x:v>Action / SET_COLUMN_VALUE</x:v>
+      </x:c>
+      <x:c r="F31" s="93" t="str">
+        <x:v>Verified hidden; only two cache assignments.</x:v>
+      </x:c>
+      <x:c r="G31" s="93" t="str">
+        <x:v>Recomputes both components from authoritative related repayment rows; idempotent.</x:v>
+      </x:c>
+      <x:c r="H31" s="93" t="str">
+        <x:v>Perf Cached Principal Paid = SUM([Related Repayments][Principal Paid]); Perf Cached Interest Paid = SUM([Related Repayments][Interest Paid])</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="150" customHeight="1">
+      <x:c r="A32" s="93" t="str">
+        <x:v>P09 backfill</x:v>
+      </x:c>
+      <x:c r="B32" s="93" t="str">
+        <x:v>1.000026</x:v>
+      </x:c>
+      <x:c r="C32" s="93" t="str">
+        <x:v>Statistics</x:v>
+      </x:c>
+      <x:c r="D32" s="93" t="str">
+        <x:v>Perf - Backfill All Charge Caches</x:v>
+      </x:c>
+      <x:c r="E32" s="93" t="str">
+        <x:v>Action / REF_ACTION</x:v>
+      </x:c>
+      <x:c r="F32" s="93" t="str">
+        <x:v>Verified target before execution; no cache reads changed.</x:v>
+      </x:c>
+      <x:c r="G32" s="93" t="str">
+        <x:v>One-time initialization over copied database only.</x:v>
+      </x:c>
+      <x:c r="H32" s="93" t="str">
+        <x:v>ReferencedTable Charges; ReferencedRows Charges[Row ID]; ReferencedAction Perf - Refresh Charge Paid Cache</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="150" customHeight="1">
+      <x:c r="A33" s="93" t="str">
+        <x:v>P09 bounded initialization</x:v>
+      </x:c>
+      <x:c r="B33" s="93" t="str">
+        <x:v>1.000027</x:v>
+      </x:c>
+      <x:c r="C33" s="93" t="str">
+        <x:v>Statistics / Charges</x:v>
+      </x:c>
+      <x:c r="D33" s="93" t="str">
+        <x:v>Perf - Initialize Charge Caches</x:v>
+      </x:c>
+      <x:c r="E33" s="93" t="str">
+        <x:v>Bot / REF_ACTION</x:v>
+      </x:c>
+      <x:c r="F33" s="93" t="str">
+        <x:v>UI Test execution in progress; no cache readers changed.</x:v>
+      </x:c>
+      <x:c r="G33" s="93" t="str">
+        <x:v>Replaces failed all-row client backfill. No notification task.</x:v>
+      </x:c>
+      <x:c r="H33" s="93" t="str">
+        <x:v>TOP(SELECT(Charges[Row ID], OR(ISBLANK([Perf Cached Principal Paid]), ISBLANK([Perf Cached Interest Paid]))), 100); action Perf - Refresh Charge Paid Cache</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="150" customHeight="1">
+      <x:c r="A34" s="93" t="str">
+        <x:v>P09 new GUI trigger</x:v>
+      </x:c>
+      <x:c r="B34" s="93" t="str">
+        <x:v>1.000028</x:v>
+      </x:c>
+      <x:c r="C34" s="93" t="str">
+        <x:v>Statistics</x:v>
+      </x:c>
+      <x:c r="D34" s="93" t="str">
+        <x:v>Perf - Initialize Next Cache Batch</x:v>
+      </x:c>
+      <x:c r="E34" s="93" t="str">
+        <x:v>Action / SET_COLUMN_VALUE</x:v>
+      </x:c>
+      <x:c r="F34" s="93" t="str">
+        <x:v>Replaces all-row client wrapper. First click outcome pending.</x:v>
+      </x:c>
+      <x:c r="G34" s="93" t="str">
+        <x:v>Non-key Statistics ID only; original MAIN must be restored. No references found in baseline inventory. New GUI only from this point.</x:v>
+      </x:c>
+      <x:c r="H34" s="93" t="str">
+        <x:v>Statistics ID = CONCATENATE("PERF-CACHE-INIT-", UNIQUEID())</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3305,7 +3769,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61a0a56b90bf4c19"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11e2bb00962f43d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13806,7 +14270,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd21574397ba4b6a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R480a90986b924ce4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14235,7 +14699,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raddd74db07aa40d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1bfb898f9754e54"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14689,7 +15153,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46dfcd6435b74222"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re282524943c848e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20851,7 +21315,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a3aae16d3f842a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc9aaed3b11b450c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25350,7 +25814,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e01aa2a35344fc7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1093c69855d474b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25549,7 +26013,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0520f58cb3e4219"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd24fffd2968c41c5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27202,7 +27666,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83875edb16244620"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49b6a59df6ba4693"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Report new-GUI OLTP benchmarks and restore test calculation path
</commit_message>
<xml_diff>
--- a/Documents/AppSheet_Data_Dictionary.xlsx
+++ b/Documents/AppSheet_Data_Dictionary.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R59e42d0eb5594056"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="R6ac6453d12c6483d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="Rda90031e5a174c14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="Ra837a5ea449e4b9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="R658a96a33d3b49ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="Rc280eb80e53445b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="R8daaa05516ce442b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R48ce2de77c5745d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="R8403af4920f14a58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R60ad872993b94151"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="Refffd5c193504f4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R79a7c6c8c0da487a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="R5c9112ad24ec482d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="Rc34619690220467b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R1462e69c86444983"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="Re0b2c4e28ca34940"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R76948fb212d745ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Rfa94536683874f06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R7adcb098727f467d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="R36bc897ce824407c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="Rcaada003fd364f52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="R0e18422c473a4c10"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -97,7 +97,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="19">
+  <x:fills count="23">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -132,6 +132,26 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -319,7 +339,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="104">
+  <x:cellXfs count="108">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -542,6 +562,18 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="12" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2449,7 +2481,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ea27d42e7534a37"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb70980dd8bbe4447"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2469,28 +2501,28 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="103" t="str">
+      <x:c r="A1" s="107" t="str">
         <x:v>Experiment</x:v>
       </x:c>
-      <x:c r="B1" s="103" t="str">
+      <x:c r="B1" s="107" t="str">
         <x:v>App version</x:v>
       </x:c>
-      <x:c r="C1" s="103" t="str">
+      <x:c r="C1" s="107" t="str">
         <x:v>Table</x:v>
       </x:c>
-      <x:c r="D1" s="103" t="str">
+      <x:c r="D1" s="107" t="str">
         <x:v>Column / setting</x:v>
       </x:c>
-      <x:c r="E1" s="103" t="str">
+      <x:c r="E1" s="107" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="F1" s="103" t="str">
+      <x:c r="F1" s="107" t="str">
         <x:v>Scope / status</x:v>
       </x:c>
-      <x:c r="G1" s="103" t="str">
+      <x:c r="G1" s="107" t="str">
         <x:v>Purpose / dependencies</x:v>
       </x:c>
-      <x:c r="H1" s="103" t="str">
+      <x:c r="H1" s="107" t="str">
         <x:v>Exact definition</x:v>
       </x:c>
     </x:row>
@@ -3289,7 +3321,7 @@
         <x:v>Action / REF_ACTION</x:v>
       </x:c>
       <x:c r="F32" s="93" t="str">
-        <x:v>Verified target before execution; no cache reads changed.</x:v>
+        <x:v>Client all-row attempt crashed; wrapper replaced. Do not replay.</x:v>
       </x:c>
       <x:c r="G32" s="93" t="str">
         <x:v>One-time initialization over copied database only.</x:v>
@@ -3315,7 +3347,7 @@
         <x:v>Bot / REF_ACTION</x:v>
       </x:c>
       <x:c r="F33" s="93" t="str">
-        <x:v>UI Test execution in progress; no cache readers changed.</x:v>
+        <x:v>Initialization completed; bot disabled at 1.000031. Legacy Test-page use discontinued.</x:v>
       </x:c>
       <x:c r="G33" s="93" t="str">
         <x:v>Replaces failed all-row client backfill. No notification task.</x:v>
@@ -3341,13 +3373,299 @@
         <x:v>Action / SET_COLUMN_VALUE</x:v>
       </x:c>
       <x:c r="F34" s="93" t="str">
-        <x:v>Replaces all-row client wrapper. First click outcome pending.</x:v>
+        <x:v>New-GUI trigger executed; Statistics ID restored MAIN; trigger hidden 1.000038.</x:v>
       </x:c>
       <x:c r="G34" s="93" t="str">
         <x:v>Non-key Statistics ID only; original MAIN must be restored. No references found in baseline inventory. New GUI only from this point.</x:v>
       </x:c>
       <x:c r="H34" s="93" t="str">
         <x:v>Statistics ID = CONCATENATE("PERF-CACHE-INIT-", UNIQUEID())</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="150" customHeight="1">
+      <x:c r="A35" s="93" t="str">
+        <x:v>P09 reconciliation</x:v>
+      </x:c>
+      <x:c r="B35" s="93" t="str">
+        <x:v>1.000030</x:v>
+      </x:c>
+      <x:c r="C35" s="93" t="str">
+        <x:v>Statistics / Charges</x:v>
+      </x:c>
+      <x:c r="D35" s="93" t="str">
+        <x:v>Perf - Initialize Next Cache Batch display name</x:v>
+      </x:c>
+      <x:c r="E35" s="93" t="str">
+        <x:v>Action display expression</x:v>
+      </x:c>
+      <x:c r="F35" s="93" t="str">
+        <x:v>New editor preview: missing 0; mismatched 0.</x:v>
+      </x:c>
+      <x:c r="G35" s="93" t="str">
+        <x:v>Compares cache fields with original paid VCs before changing readers. Synthetic components 0 and 3100 also verified.</x:v>
+      </x:c>
+      <x:c r="H35" s="93" t="str">
+        <x:v>CONCATENATE("Perf initialize | missing ", COUNT(SELECT(Charges[Row ID], OR(ISBLANK([Perf Cached Principal Paid]), ISBLANK([Perf Cached Interest Paid])))), " | mismatched ", COUNT(SELECT(Charges[Row ID], OR([Perf Cached Principal Paid] &lt;&gt; [Principal Paid], [Perf Cached Interest Paid] &lt;&gt; [Interest Paid]))))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="150" customHeight="1">
+      <x:c r="A36" s="93" t="str">
+        <x:v>P09 maintenance</x:v>
+      </x:c>
+      <x:c r="B36" s="93" t="str">
+        <x:v>1.000032</x:v>
+      </x:c>
+      <x:c r="C36" s="93" t="str">
+        <x:v>Payments</x:v>
+      </x:c>
+      <x:c r="D36" s="93" t="str">
+        <x:v>Perf - Refresh Borrower Charge Caches</x:v>
+      </x:c>
+      <x:c r="E36" s="93" t="str">
+        <x:v>Action / REF_ACTION</x:v>
+      </x:c>
+      <x:c r="F36" s="93" t="str">
+        <x:v>Hidden; now unused after receipt rollback.</x:v>
+      </x:c>
+      <x:c r="G36" s="93" t="str">
+        <x:v>Refreshes both components for all charges of the receipt borrower. Ledger recomputation is idempotent.</x:v>
+      </x:c>
+      <x:c r="H36" s="93" t="str">
+        <x:v>ReferencedTable Charges; ReferencedRows SELECT(Charges[Row ID], [Ref Loans].[Ref Borrowers] = [_THISROW].[Ref Borrower]); ReferencedAction Perf - Refresh Charge Paid Cache</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="150" customHeight="1">
+      <x:c r="A37" s="93" t="str">
+        <x:v>P09 receipt sequence</x:v>
+      </x:c>
+      <x:c r="B37" s="93" t="str">
+        <x:v>1.000033</x:v>
+      </x:c>
+      <x:c r="C37" s="93" t="str">
+        <x:v>Payments</x:v>
+      </x:c>
+      <x:c r="D37" s="93" t="str">
+        <x:v>Payment - Process Receipt</x:v>
+      </x:c>
+      <x:c r="E37" s="93" t="str">
+        <x:v>Action / COMPOSITE</x:v>
+      </x:c>
+      <x:c r="F37" s="93" t="str">
+        <x:v>Historical seven-step test sequence; original five steps restored 1.000037.</x:v>
+      </x:c>
+      <x:c r="G37" s="93" t="str">
+        <x:v>Includes refresh cost before snapshots and after posting. Original posting/reconciliation actions and predicates unchanged.</x:v>
+      </x:c>
+      <x:c r="H37" s="93" t="str">
+        <x:v>Perf - Refresh Borrower Charge Caches; Payment - Create Snapshots; Payment - Freeze Plan; Payment - Post Plan; Perf - Refresh Borrower Charge Caches; Payment - Reconcile; Payment - Close Paid Loans</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="150" customHeight="1">
+      <x:c r="A38" s="93" t="str">
+        <x:v>P09 cached reader</x:v>
+      </x:c>
+      <x:c r="B38" s="93" t="str">
+        <x:v>1.000034</x:v>
+      </x:c>
+      <x:c r="C38" s="93" t="str">
+        <x:v>Charges</x:v>
+      </x:c>
+      <x:c r="D38" s="93" t="str">
+        <x:v>Principal Paid</x:v>
+      </x:c>
+      <x:c r="E38" s="93" t="str">
+        <x:v>VC / Price</x:v>
+      </x:c>
+      <x:c r="F38" s="93" t="str">
+        <x:v>Rejected P09a cache lag; originals restored 1.000037. No production change.</x:v>
+      </x:c>
+      <x:c r="G38" s="93" t="str">
+        <x:v>Blank fallback retains original sum. Original formula SUM([Related Repayments][Principal Paid]); baseline rollback 1.000032.</x:v>
+      </x:c>
+      <x:c r="H38" s="93" t="str">
+        <x:v>IF(ISNOTBLANK([Perf Cached Principal Paid]), [Perf Cached Principal Paid], SUM([Related Repayments][Principal Paid]))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="150" customHeight="1">
+      <x:c r="A39" s="93" t="str">
+        <x:v>P09 cached reader</x:v>
+      </x:c>
+      <x:c r="B39" s="93" t="str">
+        <x:v>1.000034</x:v>
+      </x:c>
+      <x:c r="C39" s="93" t="str">
+        <x:v>Charges</x:v>
+      </x:c>
+      <x:c r="D39" s="93" t="str">
+        <x:v>Interest Paid</x:v>
+      </x:c>
+      <x:c r="E39" s="93" t="str">
+        <x:v>VC / Price</x:v>
+      </x:c>
+      <x:c r="F39" s="93" t="str">
+        <x:v>Rejected P09a cache lag; originals restored 1.000037. No production change.</x:v>
+      </x:c>
+      <x:c r="G39" s="93" t="str">
+        <x:v>Blank fallback retains original sum. Original formula SUM([Related Repayments][Interest Paid]); baseline rollback 1.000032.</x:v>
+      </x:c>
+      <x:c r="H39" s="93" t="str">
+        <x:v>IF(ISNOTBLANK([Perf Cached Interest Paid]), [Perf Cached Interest Paid], SUM([Related Repayments][Interest Paid]))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="150" customHeight="1">
+      <x:c r="A40" s="93" t="str">
+        <x:v>P09 independent reconciliation</x:v>
+      </x:c>
+      <x:c r="B40" s="93" t="str">
+        <x:v>1.000034</x:v>
+      </x:c>
+      <x:c r="C40" s="93" t="str">
+        <x:v>Statistics / Charges</x:v>
+      </x:c>
+      <x:c r="D40" s="93" t="str">
+        <x:v>Perf - Initialize Next Cache Batch display name</x:v>
+      </x:c>
+      <x:c r="E40" s="93" t="str">
+        <x:v>Action display expression</x:v>
+      </x:c>
+      <x:c r="F40" s="93" t="str">
+        <x:v>Independent ledger comparison verified; action hidden in final 1.000038.</x:v>
+      </x:c>
+      <x:c r="G40" s="93" t="str">
+        <x:v>Must not compare cached fields with cached-reader VCs; doing so would be tautological. Initialization bot disabled at 1.000031; Statistics ID restored MAIN.</x:v>
+      </x:c>
+      <x:c r="H40" s="93" t="str">
+        <x:v>CONCATENATE("Perf initialize | missing ", COUNT(SELECT(Charges[Row ID], OR(ISBLANK([Perf Cached Principal Paid]), ISBLANK([Perf Cached Interest Paid])))), " | mismatched ", COUNT(SELECT(Charges[Row ID], OR([Perf Cached Principal Paid] &lt;&gt; SUM([Related Repayments][Principal Paid]), [Perf Cached Interest Paid] &lt;&gt; SUM([Related Repayments][Interest Paid])))))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="150" customHeight="1">
+      <x:c r="A41" s="93" t="str">
+        <x:v>P09b direct refresh</x:v>
+      </x:c>
+      <x:c r="B41" s="93" t="str">
+        <x:v>1.000035</x:v>
+      </x:c>
+      <x:c r="C41" s="93" t="str">
+        <x:v>Charges</x:v>
+      </x:c>
+      <x:c r="D41" s="93" t="str">
+        <x:v>Perf - Refresh Charge Paid Cache</x:v>
+      </x:c>
+      <x:c r="E41" s="93" t="str">
+        <x:v>Action / SET_COLUMN_VALUE</x:v>
+      </x:c>
+      <x:c r="F41" s="93" t="str">
+        <x:v>Tested path reconciled; 14.06%/20.87% slower than before/after controls. Hidden and unused at 1.000038.</x:v>
+      </x:c>
+      <x:c r="G41" s="93" t="str">
+        <x:v>Direct table sum corrects observed same-sequence related-list lag. No concurrent or external-writer certification.</x:v>
+      </x:c>
+      <x:c r="H41" s="93" t="str">
+        <x:v>Perf Cached Principal Paid = SUM(SELECT(Repayments[Principal Paid], [Ref Charges] = [_THISROW].[Row ID])); Perf Cached Interest Paid = SUM(SELECT(Repayments[Interest Paid], [Ref Charges] = [_THISROW].[Row ID]))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="150" customHeight="1">
+      <x:c r="A42" s="93" t="str">
+        <x:v>P09 final rollback</x:v>
+      </x:c>
+      <x:c r="B42" s="93" t="str">
+        <x:v>1.000037</x:v>
+      </x:c>
+      <x:c r="C42" s="93" t="str">
+        <x:v>Charges</x:v>
+      </x:c>
+      <x:c r="D42" s="93" t="str">
+        <x:v>Principal Paid</x:v>
+      </x:c>
+      <x:c r="E42" s="93" t="str">
+        <x:v>VC / Price</x:v>
+      </x:c>
+      <x:c r="F42" s="93" t="str">
+        <x:v>Original ledger reader restored and verified.</x:v>
+      </x:c>
+      <x:c r="G42" s="93" t="str">
+        <x:v>Cache column remains unused historical evidence.</x:v>
+      </x:c>
+      <x:c r="H42" s="93" t="str">
+        <x:v>SUM([Related Repayments][Principal Paid])</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="150" customHeight="1">
+      <x:c r="A43" s="93" t="str">
+        <x:v>P09 final rollback</x:v>
+      </x:c>
+      <x:c r="B43" s="93" t="str">
+        <x:v>1.000037</x:v>
+      </x:c>
+      <x:c r="C43" s="93" t="str">
+        <x:v>Charges</x:v>
+      </x:c>
+      <x:c r="D43" s="93" t="str">
+        <x:v>Interest Paid</x:v>
+      </x:c>
+      <x:c r="E43" s="93" t="str">
+        <x:v>VC / Price</x:v>
+      </x:c>
+      <x:c r="F43" s="93" t="str">
+        <x:v>Original ledger reader restored and verified.</x:v>
+      </x:c>
+      <x:c r="G43" s="93" t="str">
+        <x:v>Intermediate 1.000036 was incomplete; no receipts submitted there.</x:v>
+      </x:c>
+      <x:c r="H43" s="93" t="str">
+        <x:v>SUM([Related Repayments][Interest Paid])</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="150" customHeight="1">
+      <x:c r="A44" s="93" t="str">
+        <x:v>P09 final rollback</x:v>
+      </x:c>
+      <x:c r="B44" s="93" t="str">
+        <x:v>1.000037</x:v>
+      </x:c>
+      <x:c r="C44" s="93" t="str">
+        <x:v>Payments</x:v>
+      </x:c>
+      <x:c r="D44" s="93" t="str">
+        <x:v>Payment - Process Receipt</x:v>
+      </x:c>
+      <x:c r="E44" s="93" t="str">
+        <x:v>Action / COMPOSITE</x:v>
+      </x:c>
+      <x:c r="F44" s="93" t="str">
+        <x:v>Original five-step flow restored; three reversal controls Posted.</x:v>
+      </x:c>
+      <x:c r="G44" s="93" t="str">
+        <x:v>No cache maintenance remains in receipt path.</x:v>
+      </x:c>
+      <x:c r="H44" s="93" t="str">
+        <x:v>Payment - Create Snapshots; Payment - Freeze Plan; Payment - Post Plan; Payment - Reconcile; Payment - Close Paid Loans</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="150" customHeight="1">
+      <x:c r="A45" s="93" t="str">
+        <x:v>Final lab cleanup</x:v>
+      </x:c>
+      <x:c r="B45" s="93" t="str">
+        <x:v>1.000038</x:v>
+      </x:c>
+      <x:c r="C45" s="93" t="str">
+        <x:v>Statistics</x:v>
+      </x:c>
+      <x:c r="D45" s="93" t="str">
+        <x:v>Perf - Initialize Next Cache Batch</x:v>
+      </x:c>
+      <x:c r="E45" s="93" t="str">
+        <x:v>Action visibility</x:v>
+      </x:c>
+      <x:c r="F45" s="93" t="str">
+        <x:v>Hidden; initializer bot disabled; Statistics ID MAIN restored.</x:v>
+      </x:c>
+      <x:c r="G45" s="93" t="str">
+        <x:v>Retained for lab recovery only. Do not treat historical cache values as current balances.</x:v>
+      </x:c>
+      <x:c r="H45" s="93" t="str">
+        <x:v>Prominence Do_Not_Display</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3769,7 +4087,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11e2bb00962f43d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8620a662bba43e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14270,7 +14588,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R480a90986b924ce4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6e837d5874345c9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14699,7 +15017,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1bfb898f9754e54"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7ba59e715e6475a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15153,7 +15471,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re282524943c848e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc09f573333634c04"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21315,7 +21633,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc9aaed3b11b450c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c185013b6e14191"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25814,7 +26132,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1093c69855d474b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3de0ff88828946af"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26013,7 +26331,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd24fffd2968c41c5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R529ecd47cea74163"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27666,7 +27984,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49b6a59df6ba4693"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53ac300938f14aeb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document combined P01a P04a clone benchmarks and correctness validation
</commit_message>
<xml_diff>
--- a/Documents/AppSheet_Data_Dictionary.xlsx
+++ b/Documents/AppSheet_Data_Dictionary.xlsx
@@ -2,17 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R79a7c6c8c0da487a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="R5c9112ad24ec482d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="Rc34619690220467b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R1462e69c86444983"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="Re0b2c4e28ca34940"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R76948fb212d745ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Rfa94536683874f06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R7adcb098727f467d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="R36bc897ce824407c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="Rcaada003fd364f52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="R0e18422c473a4c10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R40d968f488b94b9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="Rbe56627832684152"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R743c9184c04c4c69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R579f951143204693"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="Rbecdea6db3e74270"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R6ddbb7d808c34d6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Rddd8a4cc54c94382"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R46b5baab65624f37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="R62a32becd5c84be0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R97eeea045c2348ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="Rdbcc72a35e1b4de4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="Rb3cb830aff454437"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -97,7 +98,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="23">
+  <x:fills count="24">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -132,6 +133,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -339,7 +345,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="108">
+  <x:cellXfs count="111">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -574,6 +580,11 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="12" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2481,7 +2492,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb70980dd8bbe4447"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcc21160190041a8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3666,6 +3677,207 @@
       </x:c>
       <x:c r="H45" s="93" t="str">
         <x:v>Prominence Do_Not_Display</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="38" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="55" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="100" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="110" t="str">
+        <x:v>Experiment</x:v>
+      </x:c>
+      <x:c r="B1" s="110" t="str">
+        <x:v>App version</x:v>
+      </x:c>
+      <x:c r="C1" s="110" t="str">
+        <x:v>Table</x:v>
+      </x:c>
+      <x:c r="D1" s="110" t="str">
+        <x:v>Column / setting</x:v>
+      </x:c>
+      <x:c r="E1" s="110" t="str">
+        <x:v>Type</x:v>
+      </x:c>
+      <x:c r="F1" s="110" t="str">
+        <x:v>Scope / status</x:v>
+      </x:c>
+      <x:c r="G1" s="110" t="str">
+        <x:v>Purpose / dependencies</x:v>
+      </x:c>
+      <x:c r="H1" s="110" t="str">
+        <x:v>Exact definition</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="150" customHeight="1">
+      <x:c r="A2" s="93" t="str">
+        <x:v>P01a</x:v>
+      </x:c>
+      <x:c r="B2" s="93" t="str">
+        <x:v>1.000044</x:v>
+      </x:c>
+      <x:c r="C2" s="93" t="str">
+        <x:v>Payments</x:v>
+      </x:c>
+      <x:c r="D2" s="93" t="str">
+        <x:v>Eligible Charges</x:v>
+      </x:c>
+      <x:c r="E2" s="93" t="str">
+        <x:v>List / Ref Charges</x:v>
+      </x:c>
+      <x:c r="F2" s="93" t="str">
+        <x:v>Combined candidate retained in test clone</x:v>
+      </x:c>
+      <x:c r="G2" s="93" t="str">
+        <x:v>Posted returns empty; other statuses retain original selection. Eligible Outstanding and Amount Received description become zero on Posted.</x:v>
+      </x:c>
+      <x:c r="H2" s="93" t="str">
+        <x:v>IF([Status] = "Posted", LIST(), SELECT(Charges[Row ID], AND([Ref Loans].[Ref Borrowers] = [_THISROW].[Ref Borrower], [Amount Remaining] &gt; 0, IFS(IN([_THISROW].[Allocation Method], LIST("Single Full", "Single Partial", "First-day Auto")), [Row ID] = [_THISROW].[Ref Target Charge], [_THISROW].[Allocation Method] = "Loan Close", [Ref Loans] = [_THISROW].[Ref Target Charge].[Ref Loans], IN([_THISROW].[Allocation Method], LIST("Receive All", "Lump Sum")), [Charge Date] &lt;= [_THISROW].[Payment Date], TRUE, FALSE))))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="150" customHeight="1">
+      <x:c r="A3" s="93" t="str">
+        <x:v>P04a</x:v>
+      </x:c>
+      <x:c r="B3" s="93" t="str">
+        <x:v>1.000044</x:v>
+      </x:c>
+      <x:c r="C3" s="93" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D3" s="93" t="str">
+        <x:v>Calculated Amount</x:v>
+      </x:c>
+      <x:c r="E3" s="93" t="str">
+        <x:v>Price</x:v>
+      </x:c>
+      <x:c r="F3" s="93" t="str">
+        <x:v>Combined candidate retained in test clone</x:v>
+      </x:c>
+      <x:c r="G3" s="93" t="str">
+        <x:v>Direct date-descending / row-descending predecessor; snapshots, guards and posting sequence unchanged.</x:v>
+      </x:c>
+      <x:c r="H3" s="93" t="str">
+        <x:v>MAX(LIST(DECIMAL(0), MIN(LIST(DECIMAL([Amount Remaining Snapshot]), DECIMAL([Ref Payment].[Amount Received]) - DECIMAL(SUM(SELECT(Payment Allocations[Amount Remaining Snapshot], AND([Ref Payment] = [_THISROW].[Ref Payment], OR([Charge Date Snapshot] &gt; [_THISROW].[Charge Date Snapshot], AND([Charge Date Snapshot] = [_THISROW].[Charge Date Snapshot], [Charge Row Number Snapshot] &gt; [_THISROW].[Charge Row Number Snapshot]))))))))))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="150" customHeight="1">
+      <x:c r="A4" s="93" t="str">
+        <x:v>Rollback</x:v>
+      </x:c>
+      <x:c r="B4" s="93" t="str">
+        <x:v>1.000038</x:v>
+      </x:c>
+      <x:c r="C4" s="93" t="str">
+        <x:v>Payments</x:v>
+      </x:c>
+      <x:c r="D4" s="93" t="str">
+        <x:v>Eligible Charges</x:v>
+      </x:c>
+      <x:c r="E4" s="93" t="str">
+        <x:v>List / Ref Charges</x:v>
+      </x:c>
+      <x:c r="F4" s="93" t="str">
+        <x:v>Original definition</x:v>
+      </x:c>
+      <x:c r="G4" s="93" t="str">
+        <x:v>Restore this expression to remove P01a.</x:v>
+      </x:c>
+      <x:c r="H4" s="93" t="str">
+        <x:v>SELECT(Charges[Row ID], AND([Ref Loans].[Ref Borrowers] = [_THISROW].[Ref Borrower], [Amount Remaining] &gt; 0, IFS(IN([_THISROW].[Allocation Method], LIST("Single Full", "Single Partial", "First-day Auto")), [Row ID] = [_THISROW].[Ref Target Charge], [_THISROW].[Allocation Method] = "Loan Close", [Ref Loans] = [_THISROW].[Ref Target Charge].[Ref Loans], IN([_THISROW].[Allocation Method], LIST("Receive All", "Lump Sum")), [Charge Date] &lt;= [_THISROW].[Payment Date], TRUE, FALSE)))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="150" customHeight="1">
+      <x:c r="A5" s="93" t="str">
+        <x:v>Rollback</x:v>
+      </x:c>
+      <x:c r="B5" s="93" t="str">
+        <x:v>1.000038</x:v>
+      </x:c>
+      <x:c r="C5" s="93" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D5" s="93" t="str">
+        <x:v>Calculated Amount</x:v>
+      </x:c>
+      <x:c r="E5" s="93" t="str">
+        <x:v>Price</x:v>
+      </x:c>
+      <x:c r="F5" s="93" t="str">
+        <x:v>Original definition</x:v>
+      </x:c>
+      <x:c r="G5" s="93" t="str">
+        <x:v>Restore this expression to remove P04a.</x:v>
+      </x:c>
+      <x:c r="H5" s="93" t="str">
+        <x:v>MAX(LIST(DECIMAL(0), MIN(LIST(DECIMAL([Amount Remaining Snapshot]), DECIMAL([Ref Payment].[Amount Received]) - DECIMAL(SUM(SELECT(Payment Allocations[Amount Remaining Snapshot], AND([Ref Payment] = [_THISROW].[Ref Payment], [Calculated Order] &lt; [_THISROW].[Calculated Order]))))))))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="150" customHeight="1">
+      <x:c r="A6" s="93" t="str">
+        <x:v>Diagnostic</x:v>
+      </x:c>
+      <x:c r="B6" s="93" t="str">
+        <x:v>1.000042 → 1.000044</x:v>
+      </x:c>
+      <x:c r="C6" s="93" t="str">
+        <x:v>Payments</x:v>
+      </x:c>
+      <x:c r="D6" s="93" t="str">
+        <x:v>Visible Allocations</x:v>
+      </x:c>
+      <x:c r="E6" s="93" t="str">
+        <x:v>List / Ref Payment Allocations</x:v>
+      </x:c>
+      <x:c r="F6" s="93" t="str">
+        <x:v>Temporary all-row display restored; outside timing runs</x:v>
+      </x:c>
+      <x:c r="G6" s="93" t="str">
+        <x:v>All plan rows including zero allocations inspected, then positive-only original restored.</x:v>
+      </x:c>
+      <x:c r="H6" s="93" t="str">
+        <x:v>SELECT(Payment Allocations[Row ID], AND([Ref Payment] = [_THISROW].[Row ID], [Allocated Amount] &gt; 0))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="150" customHeight="1">
+      <x:c r="A7" s="93" t="str">
+        <x:v>Diagnostic</x:v>
+      </x:c>
+      <x:c r="B7" s="93" t="str">
+        <x:v>1.000043 → 1.000044</x:v>
+      </x:c>
+      <x:c r="C7" s="93" t="str">
+        <x:v>Borrowers</x:v>
+      </x:c>
+      <x:c r="D7" s="93" t="str">
+        <x:v>Receive All Charges</x:v>
+      </x:c>
+      <x:c r="E7" s="93" t="str">
+        <x:v>Action position</x:v>
+      </x:c>
+      <x:c r="F7" s="93" t="str">
+        <x:v>Temporary Prominent restored to Inline; outside timing runs</x:v>
+      </x:c>
+      <x:c r="G7" s="93" t="str">
+        <x:v>Normal receipt logic unchanged; new desktop UI exercised.</x:v>
+      </x:c>
+      <x:c r="H7" s="93" t="str">
+        <x:v>Inline</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4087,7 +4299,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8620a662bba43e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2371162a0c8e4a85"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14588,7 +14800,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6e837d5874345c9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58556346a9974dfe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15017,7 +15229,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7ba59e715e6475a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R093ff56894c845fe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15471,7 +15683,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc09f573333634c04"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf54ba8223f7e4bef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21633,7 +21845,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c185013b6e14191"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6bd4ce0df6064818"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26132,7 +26344,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3de0ff88828946af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26ef912329af41c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26331,7 +26543,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R529ecd47cea74163"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb02371891eba49a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27984,7 +28196,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53ac300938f14aeb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4bc6996d5bb44c0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document production partner controls and borrower location setup
</commit_message>
<xml_diff>
--- a/Documents/AppSheet_Data_Dictionary.xlsx
+++ b/Documents/AppSheet_Data_Dictionary.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R40d968f488b94b9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="Rbe56627832684152"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R743c9184c04c4c69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R579f951143204693"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="Rbecdea6db3e74270"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R6ddbb7d808c34d6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Rddd8a4cc54c94382"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R46b5baab65624f37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="R62a32becd5c84be0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R97eeea045c2348ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="Rdbcc72a35e1b4de4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="Rb3cb830aff454437"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rd893d693986c4194"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="R9008d850b3294414"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R4f0d0bb4bf454887"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="Rfc1bf38aaf9445f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="Rb950f955cc40458d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R31f9e8394d0d444a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="R0bf2af24bdc74f3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R842a9edd6fe64612"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="R921fa5e8f16f4a65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R3a4b5860a0404a46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="Rfa88407996944400"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="R9eb1450f87104df8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -722,8 +722,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="DataModelColumns" displayName="DataModelColumns" ref="A4:H392" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:H392"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="DataModelColumns" displayName="DataModelColumns" ref="A4:H398" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:H398"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Table"/>
     <x:tableColumn id="2" name="Inventory order"/>
@@ -769,7 +769,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="DataModelSliceColumns" displayName="DataModelSliceColumns" ref="A4:D440" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="DataModelSliceColumns" displayName="DataModelSliceColumns" ref="A4:D448" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="App"/>
     <x:tableColumn id="2" name="Slice"/>
@@ -781,8 +781,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="DataModelAppVariances" displayName="DataModelAppVariances" ref="A4:F227" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:F227"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="DataModelAppVariances" displayName="DataModelAppVariances" ref="A4:F232" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:F232"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Object Type"/>
     <x:tableColumn id="2" name="Table"/>
@@ -1079,7 +1079,7 @@
         <x:v>Reconciliation status</x:v>
       </x:c>
       <x:c r="B5" s="85" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok). Collection settings reconciled in production Operations app; standalone forms/default/setup-review verified. OLAP standalone app opened successfully; its new-column loading is pending reconciliation. Other inventory retains dated scope.</x:v>
+        <x:v>OLTP 3.000050; 13 September 2026. Partner controls, borrower locations and affected slice memberships verified. New OLAP field loading remains pending. Earlier unrelated inventory retains dated scope.</x:v>
       </x:c>
       <x:c r="C5" s="73"/>
       <x:c r="D5" s="73"/>
@@ -1091,7 +1091,7 @@
         <x:v>Live baselines</x:v>
       </x:c>
       <x:c r="B6" s="85" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); rollback OLTP 3.000014. Native backup Money Collection Backup 20260908 (12 tables, rows copied); local runner/docs rollback retained. OLAP last documented 1.100016; no OLAP configuration changed.</x:v>
+        <x:v>Setup rollback OLTP 3.000045; final 3.000050. App restore does not restore database schema/data. Private cell before-image retained outside Git. No OLAP configuration changed.</x:v>
       </x:c>
       <x:c r="C6" s="73"/>
       <x:c r="D6" s="73"/>
@@ -2492,7 +2492,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcc21160190041a8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a30166ee3ba430b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3907,7 +3907,7 @@
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>14 native tables. OLTP loads10: Borrowers has14 physical +28 VCs; new bank table7+3 and singleton settings4+0. OLAP loading of new fields not reconciled; prior counts retained.</x:v>
+        <x:v>13 September 2026: OLTP Borrowers 16 physical +29 VCs; Partners 8 physical +0 VCs. Counts include source ordinal. Other tables and OLAP counts retain prior verification scope.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
@@ -3958,16 +3958,16 @@
         <x:v>OLTP + OLAP</x:v>
       </x:c>
       <x:c r="D5" s="56" t="n">
-        <x:v>14</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E5" s="56" t="n">
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F5" s="56" t="n">
         <x:v>65</x:v>
       </x:c>
       <x:c r="G5" s="58" t="str">
-        <x:v>Borrower master; Row ID remains immutable key. Seven new collection fields and two OLTP helpers. OLAP65 VC count is prior baseline; loading of seven new physical fields not reconciled.</x:v>
+        <x:v>OLTP: 45 columns, including source ordinal/key; City and Working Location added. OLAP loading of new fields pending; prior OLAP VCs retained.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" customHeight="1">
@@ -4118,8 +4118,8 @@
       <x:c r="C12" s="57" t="str">
         <x:v>OLTP + OLAP</x:v>
       </x:c>
-      <x:c r="D12" s="57" t="str">
-        <x:v>5</x:v>
+      <x:c r="D12" s="57" t="n">
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E12" s="57" t="str">
         <x:v>0</x:v>
@@ -4128,7 +4128,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G12" s="59" t="str">
-        <x:v>Partner master records used for capital participation and settlement reporting.</x:v>
+        <x:v>Partner identity, email, language and integration opt-in; OLTP 8 stored columns including ordinal/key. New OLAP field loading pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="65" customHeight="1">
@@ -4299,7 +4299,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2371162a0c8e4a85"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41a7575e92db4f9c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4332,7 +4332,7 @@
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>8 September 2026: Auto Charge Enabled added to Loans in both apps. Eleven existing model expressions reconciled. Manual workflow acceptance remains pending.</x:v>
+        <x:v>13 September 2026: five stored partner/location fields added in OLTP 3.000050. No messaging activation. Earlier unrelated inventory retains dated verification scope.</x:v>
       </x:c>
       <x:c r="B2"/>
       <x:c r="C2"/>
@@ -4493,7 +4493,7 @@
         <x:v>Description</x:v>
       </x:c>
       <x:c r="D9" s="59" t="str">
-        <x:v>Physical / LongText</x:v>
+        <x:v>Physical / Text (OLTP); LongText (OLAP prior)</x:v>
       </x:c>
       <x:c r="E9" s="57" t="str">
         <x:v>OLTP + OLAP</x:v>
@@ -4502,7 +4502,7 @@
         <x:v>-</x:v>
       </x:c>
       <x:c r="G9" s="59" t="str">
-        <x:v>Stores the authoritative source value for Description.</x:v>
+        <x:v>OLTP Text confirmed during location setup; earlier OLAP LongText inventory retained pending reconciliation.</x:v>
       </x:c>
       <x:c r="H9" s="59" t="str">
         <x:v>Stored source column</x:v>
@@ -14289,7 +14289,7 @@
         <x:v>Editable</x:v>
       </x:c>
       <x:c r="G374" s="87" t="str">
-        <x:v>Opt-in for the existing AI collection workflow; position 12.</x:v>
+        <x:v>Existing borrower opt-in; also required alongside Collection dashboard eligibility for the proposed partner daily briefing. Existing flag values unchanged.</x:v>
       </x:c>
       <x:c r="H374" s="87" t="str">
         <x:v>Stored; initial value FALSE</x:v>
@@ -14787,6 +14787,136 @@
       </x:c>
       <x:c r="H393" s="73" t="str">
         <x:v>Initial value: TRUE. No app formula. Native key h7VnJR1ERY4o6UUaiANzwe. Restore nominal rates without re-enabling generation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="394" ht="42" customHeight="1">
+      <x:c r="A394" s="73" t="str">
+        <x:v>Partners</x:v>
+      </x:c>
+      <x:c r="B394" s="73" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C394" s="73" t="str">
+        <x:v>Instagram Username</x:v>
+      </x:c>
+      <x:c r="D394" s="73" t="str">
+        <x:v>Physical / Text</x:v>
+      </x:c>
+      <x:c r="E394" s="73" t="str">
+        <x:v>OLTP; OLAP pending</x:v>
+      </x:c>
+      <x:c r="F394" s="73" t="str">
+        <x:v>Shown, editable, optional, searchable</x:v>
+      </x:c>
+      <x:c r="G394" s="73" t="str">
+        <x:v>Partner Instagram handle. App position 6. No separate partner list.</x:v>
+      </x:c>
+      <x:c r="H394" s="73" t="str">
+        <x:v>Stored; no formula, default, key or label. Verification binding belongs to later agent implementation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="395" ht="42" customHeight="1">
+      <x:c r="A395" s="73" t="str">
+        <x:v>Partners</x:v>
+      </x:c>
+      <x:c r="B395" s="73" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="C395" s="73" t="str">
+        <x:v>Language Preference</x:v>
+      </x:c>
+      <x:c r="D395" s="73" t="str">
+        <x:v>Physical / Text</x:v>
+      </x:c>
+      <x:c r="E395" s="73" t="str">
+        <x:v>OLTP; OLAP pending</x:v>
+      </x:c>
+      <x:c r="F395" s="73" t="str">
+        <x:v>Shown, editable, optional, searchable</x:v>
+      </x:c>
+      <x:c r="G395" s="73" t="str">
+        <x:v>Language for partner notices, replies and email. App position 7.</x:v>
+      </x:c>
+      <x:c r="H395" s="73" t="str">
+        <x:v>Stored; blank initial value. Preferences not inferred or populated. Borrower drafts retain approved Thai.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="396" ht="42" customHeight="1">
+      <x:c r="A396" s="73" t="str">
+        <x:v>Partners</x:v>
+      </x:c>
+      <x:c r="B396" s="73" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C396" s="73" t="str">
+        <x:v>IG Integration Enabled</x:v>
+      </x:c>
+      <x:c r="D396" s="73" t="str">
+        <x:v>Physical / Yes/No</x:v>
+      </x:c>
+      <x:c r="E396" s="73" t="str">
+        <x:v>OLTP; OLAP pending</x:v>
+      </x:c>
+      <x:c r="F396" s="73" t="str">
+        <x:v>Shown, editable, optional, searchable</x:v>
+      </x:c>
+      <x:c r="G396" s="73" t="str">
+        <x:v>Master opt-in for partner Instagram and email fallback. App position 8.</x:v>
+      </x:c>
+      <x:c r="H396" s="73" t="str">
+        <x:v>Initial value FALSE; no app formula. Existing partners unchecked. Only TRUE permits future agent communication.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="397" ht="42" customHeight="1">
+      <x:c r="A397" s="73" t="str">
+        <x:v>Borrowers</x:v>
+      </x:c>
+      <x:c r="B397" s="73" t="n">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="C397" s="73" t="str">
+        <x:v>City</x:v>
+      </x:c>
+      <x:c r="D397" s="73" t="str">
+        <x:v>Physical / Text</x:v>
+      </x:c>
+      <x:c r="E397" s="73" t="str">
+        <x:v>OLTP; OLAP pending</x:v>
+      </x:c>
+      <x:c r="F397" s="73" t="str">
+        <x:v>Shown, editable, optional, searchable</x:v>
+      </x:c>
+      <x:c r="G397" s="73" t="str">
+        <x:v>Borrower city from the owner location sheet. App position 15.</x:v>
+      </x:c>
+      <x:c r="H397" s="73" t="str">
+        <x:v>Stored; blank initial value; display name: "เมือง / City". Source blanks preserved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="398" ht="42" customHeight="1">
+      <x:c r="A398" s="73" t="str">
+        <x:v>Borrowers</x:v>
+      </x:c>
+      <x:c r="B398" s="73" t="n">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="C398" s="73" t="str">
+        <x:v>Working Location</x:v>
+      </x:c>
+      <x:c r="D398" s="73" t="str">
+        <x:v>Physical / Text</x:v>
+      </x:c>
+      <x:c r="E398" s="73" t="str">
+        <x:v>OLTP; OLAP pending</x:v>
+      </x:c>
+      <x:c r="F398" s="73" t="str">
+        <x:v>Shown, editable, optional, searchable</x:v>
+      </x:c>
+      <x:c r="G398" s="73" t="str">
+        <x:v>Workplace/locality from the owner location sheet. App position 16.</x:v>
+      </x:c>
+      <x:c r="H398" s="73" t="str">
+        <x:v>Stored; blank initial value; display name: "สถานที่ทำงาน / Working Location". Uncertainty preserved.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14800,7 +14930,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58556346a9974dfe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82c1edae5ecb4b6f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15229,7 +15359,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R093ff56894c845fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6373227e1eb1402d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15325,13 +15455,13 @@
         <x:v>Read-only</x:v>
       </x:c>
       <x:c r="F5" s="83" t="n">
-        <x:v>19</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="G5" s="83" t="str">
-        <x:v>Existing collection-board filter retained; seven physical collection settings appended during regeneration.</x:v>
+        <x:v>Existing daily collection population. Future agent additionally requires due/overdue and AI Collection Enabled; dashboard filter unchanged.</x:v>
       </x:c>
       <x:c r="H5" s="83" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); base-row details provide effective bank and setup issues.</x:v>
+        <x:v>OLTP 3.000050; location columns included after regeneration. Existing row filter and update mode retained.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="55" customHeight="1">
@@ -15351,13 +15481,13 @@
         <x:v>Adds, Updates, Deletes</x:v>
       </x:c>
       <x:c r="F6" s="83" t="n">
-        <x:v>42</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="G6" s="83" t="str">
-        <x:v>Existing borrower-list filter retained; nine collection fields appended.</x:v>
+        <x:v>Primary borrower list; City and Working Location exposed in existing form/detail views.</x:v>
       </x:c>
       <x:c r="H6" s="83" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); borrower edit/detail views expose the new fields.</x:v>
+        <x:v>OLTP 3.000050; location columns included after regeneration. Existing row filter and update mode retained.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" customHeight="1">
@@ -15667,13 +15797,13 @@
         <x:v>Updates only</x:v>
       </x:c>
       <x:c r="F19" s="87" t="n">
-        <x:v>42</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="G19" s="87" t="str">
         <x:v>Enabled borrowers needing name, Instagram or receiving-bank setup.</x:v>
       </x:c>
       <x:c r="H19" s="87" t="str">
-        <x:v>Auto-assigned actions; menu table view; disabled borrowers excluded intentionally.</x:v>
+        <x:v>OLTP 3.000050; location columns included after regeneration. Existing row filter and update mode retained.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -15683,7 +15813,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf54ba8223f7e4bef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8379e6cd54e749fd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21838,6 +21968,118 @@
         <x:v>Collection Setup Issues</x:v>
       </x:c>
     </x:row>
+    <x:row r="441">
+      <x:c r="A441" t="str">
+        <x:v>OLTP</x:v>
+      </x:c>
+      <x:c r="B441" t="str">
+        <x:v>Collection Setup Review</x:v>
+      </x:c>
+      <x:c r="C441" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="D441" t="str">
+        <x:v>Collection Account Number</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="442">
+      <x:c r="A442" t="str">
+        <x:v>OLTP</x:v>
+      </x:c>
+      <x:c r="B442" t="str">
+        <x:v>Collection Setup Review</x:v>
+      </x:c>
+      <x:c r="C442" t="n">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="D442" t="str">
+        <x:v>City</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="443">
+      <x:c r="A443" t="str">
+        <x:v>OLTP</x:v>
+      </x:c>
+      <x:c r="B443" t="str">
+        <x:v>Collection Setup Review</x:v>
+      </x:c>
+      <x:c r="C443" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="D443" t="str">
+        <x:v>Working Location</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="444">
+      <x:c r="A444" t="str">
+        <x:v>OLTP</x:v>
+      </x:c>
+      <x:c r="B444" t="str">
+        <x:v>Todays Collection Board</x:v>
+      </x:c>
+      <x:c r="C444" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="D444" t="str">
+        <x:v>City</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="445">
+      <x:c r="A445" t="str">
+        <x:v>OLTP</x:v>
+      </x:c>
+      <x:c r="B445" t="str">
+        <x:v>Todays Collection Board</x:v>
+      </x:c>
+      <x:c r="C445" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D445" t="str">
+        <x:v>Working Location</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="446">
+      <x:c r="A446" t="str">
+        <x:v>OLTP</x:v>
+      </x:c>
+      <x:c r="B446" t="str">
+        <x:v>Visible Borrowers</x:v>
+      </x:c>
+      <x:c r="C446" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="D446" t="str">
+        <x:v>Collection Account Number</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="447">
+      <x:c r="A447" t="str">
+        <x:v>OLTP</x:v>
+      </x:c>
+      <x:c r="B447" t="str">
+        <x:v>Visible Borrowers</x:v>
+      </x:c>
+      <x:c r="C447" t="n">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="D447" t="str">
+        <x:v>City</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="448">
+      <x:c r="A448" t="str">
+        <x:v>OLTP</x:v>
+      </x:c>
+      <x:c r="B448" t="str">
+        <x:v>Visible Borrowers</x:v>
+      </x:c>
+      <x:c r="C448" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="D448" t="str">
+        <x:v>Working Location</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>
@@ -21845,7 +22087,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6bd4ce0df6064818"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd662c409624492a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26331,7 +26573,107 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="F227" s="87" t="str">
-        <x:v>Enabled borrowers with nonempty setup issues;42 columns; update only.</x:v>
+        <x:v>Enabled borrowers with setup issues; 45 columns at OLTP 3.000050; update only.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="228">
+      <x:c r="A228" t="str">
+        <x:v>Column</x:v>
+      </x:c>
+      <x:c r="B228" t="str">
+        <x:v>Partners</x:v>
+      </x:c>
+      <x:c r="C228" t="str">
+        <x:v>Instagram Username</x:v>
+      </x:c>
+      <x:c r="D228" t="str">
+        <x:v>Yes — 3.000050</x:v>
+      </x:c>
+      <x:c r="E228" t="str">
+        <x:v>Pending reconciliation</x:v>
+      </x:c>
+      <x:c r="F228" t="str">
+        <x:v>Stored in shared database; OLTP configured. OLAP app not regenerated by this task.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="229">
+      <x:c r="A229" t="str">
+        <x:v>Column</x:v>
+      </x:c>
+      <x:c r="B229" t="str">
+        <x:v>Partners</x:v>
+      </x:c>
+      <x:c r="C229" t="str">
+        <x:v>Language Preference</x:v>
+      </x:c>
+      <x:c r="D229" t="str">
+        <x:v>Yes — 3.000050</x:v>
+      </x:c>
+      <x:c r="E229" t="str">
+        <x:v>Pending reconciliation</x:v>
+      </x:c>
+      <x:c r="F229" t="str">
+        <x:v>Stored in shared database; OLTP configured. OLAP app not regenerated by this task.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="230">
+      <x:c r="A230" t="str">
+        <x:v>Column</x:v>
+      </x:c>
+      <x:c r="B230" t="str">
+        <x:v>Partners</x:v>
+      </x:c>
+      <x:c r="C230" t="str">
+        <x:v>IG Integration Enabled</x:v>
+      </x:c>
+      <x:c r="D230" t="str">
+        <x:v>Yes — 3.000050</x:v>
+      </x:c>
+      <x:c r="E230" t="str">
+        <x:v>Pending reconciliation</x:v>
+      </x:c>
+      <x:c r="F230" t="str">
+        <x:v>Stored in shared database; OLTP configured. OLAP app not regenerated by this task.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="231">
+      <x:c r="A231" t="str">
+        <x:v>Column</x:v>
+      </x:c>
+      <x:c r="B231" t="str">
+        <x:v>Borrowers</x:v>
+      </x:c>
+      <x:c r="C231" t="str">
+        <x:v>City</x:v>
+      </x:c>
+      <x:c r="D231" t="str">
+        <x:v>Yes — 3.000050</x:v>
+      </x:c>
+      <x:c r="E231" t="str">
+        <x:v>Pending reconciliation</x:v>
+      </x:c>
+      <x:c r="F231" t="str">
+        <x:v>Stored in shared database; OLTP configured. OLAP app not regenerated by this task.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="232">
+      <x:c r="A232" t="str">
+        <x:v>Column</x:v>
+      </x:c>
+      <x:c r="B232" t="str">
+        <x:v>Borrowers</x:v>
+      </x:c>
+      <x:c r="C232" t="str">
+        <x:v>Working Location</x:v>
+      </x:c>
+      <x:c r="D232" t="str">
+        <x:v>Yes — 3.000050</x:v>
+      </x:c>
+      <x:c r="E232" t="str">
+        <x:v>Pending reconciliation</x:v>
+      </x:c>
+      <x:c r="F232" t="str">
+        <x:v>Stored in shared database; OLTP configured. OLAP app not regenerated by this task.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -26344,7 +26686,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26ef912329af41c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfe8af29d8ae41ed"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26543,7 +26885,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb02371891eba49a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e5f7a3347484eb0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28196,7 +28538,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4bc6996d5bb44c0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf15aefded0a44967"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Reconcile OLAP partner management and shared borrower schema
</commit_message>
<xml_diff>
--- a/Documents/AppSheet_Data_Dictionary.xlsx
+++ b/Documents/AppSheet_Data_Dictionary.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rd893d693986c4194"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="R9008d850b3294414"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R4f0d0bb4bf454887"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="Rfc1bf38aaf9445f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="Rb950f955cc40458d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R31f9e8394d0d444a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="R0bf2af24bdc74f3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R842a9edd6fe64612"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="R921fa5e8f16f4a65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R3a4b5860a0404a46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="Rfa88407996944400"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="R9eb1450f87104df8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R04429f714ad54310"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="R6eb4a437eb894a35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R62093d1a3d63442f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R37c42161bd4d4552"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="Rbbe168736fc445fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="Rc7efbb7a1e174594"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="R5f2f79c51fcb4170"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="Rc452e6abf5684e0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="R45c8270d30ce4000"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="Rdd80efcc0a714ace"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="R4d73f202be074a83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="Rccf1c12d05d14804"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -769,7 +769,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="DataModelSliceColumns" displayName="DataModelSliceColumns" ref="A4:D448" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="DataModelSliceColumns" displayName="DataModelSliceColumns" ref="A4:D492" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="App"/>
     <x:tableColumn id="2" name="Slice"/>
@@ -1079,7 +1079,7 @@
         <x:v>Reconciliation status</x:v>
       </x:c>
       <x:c r="B5" s="85" t="str">
-        <x:v>OLTP 3.000050; 13 September 2026. Partner controls, borrower locations and affected slice memberships verified. New OLAP field loading remains pending. Earlier unrelated inventory retains dated scope.</x:v>
+        <x:v>13 September 2026: OLTP 3.000050 and OLAP 1.100031 partner/location fields and affected slices reconciled. OLAP partner forms and borrower read-only detail checked. No agent activation.</x:v>
       </x:c>
       <x:c r="C5" s="73"/>
       <x:c r="D5" s="73"/>
@@ -1091,7 +1091,7 @@
         <x:v>Live baselines</x:v>
       </x:c>
       <x:c r="B6" s="85" t="str">
-        <x:v>Setup rollback OLTP 3.000045; final 3.000050. App restore does not restore database schema/data. Private cell before-image retained outside Git. No OLAP configuration changed.</x:v>
+        <x:v>Rollback: OLTP 3.000045; OLAP 1.100028. App restore does not restore shared database data/schema. Private location before-image remains outside Git. Owner acceptance pending.</x:v>
       </x:c>
       <x:c r="C6" s="73"/>
       <x:c r="D6" s="73"/>
@@ -2492,7 +2492,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a30166ee3ba430b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfdcff336c8174e33"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3907,7 +3907,7 @@
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>13 September 2026: OLTP Borrowers 16 physical +29 VCs; Partners 8 physical +0 VCs. Counts include source ordinal. Other tables and OLAP counts retain prior verification scope.</x:v>
+        <x:v>13 September 2026: shared partner/location fields reconciled in both apps. OLTP 3.000050; OLAP 1.100031. Other tables retain dated verification scope.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
@@ -3967,7 +3967,7 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="G5" s="58" t="str">
-        <x:v>OLTP: 45 columns, including source ordinal/key; City and Working Location added. OLAP loading of new fields pending; prior OLAP VCs retained.</x:v>
+        <x:v>OLTP 45 =16 stored +29 VCs; OLAP 81 =16 stored +65 VCs. OLAP read-only, new location fields loaded. Counts include ordinal/key.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" customHeight="1">
@@ -4128,7 +4128,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G12" s="59" t="str">
-        <x:v>Partner identity, email, language and integration opt-in; OLTP 8 stored columns including ordinal/key. New OLAP field loading pending.</x:v>
+        <x:v>OLTP 8 stored; OLAP 20 =8 stored +12 VCs. OLAP owns partner management, with existing add/update/delete mode preserved.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="65" customHeight="1">
@@ -4299,7 +4299,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41a7575e92db4f9c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R285d3bc61d2041ae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4332,7 +4332,7 @@
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>13 September 2026: five stored partner/location fields added in OLTP 3.000050. No messaging activation. Earlier unrelated inventory retains dated verification scope.</x:v>
+        <x:v>13 September 2026: OLTP 3.000050 and OLAP 1.100031 partner/location setup reconciled. Existing OLAP Borrowers remains read-only; no messaging activation. Other inventory retains dated scope.</x:v>
       </x:c>
       <x:c r="B2"/>
       <x:c r="C2"/>
@@ -4493,7 +4493,7 @@
         <x:v>Description</x:v>
       </x:c>
       <x:c r="D9" s="59" t="str">
-        <x:v>Physical / Text (OLTP); LongText (OLAP prior)</x:v>
+        <x:v>Physical / Text</x:v>
       </x:c>
       <x:c r="E9" s="57" t="str">
         <x:v>OLTP + OLAP</x:v>
@@ -4502,7 +4502,7 @@
         <x:v>-</x:v>
       </x:c>
       <x:c r="G9" s="59" t="str">
-        <x:v>OLTP Text confirmed during location setup; earlier OLAP LongText inventory retained pending reconciliation.</x:v>
+        <x:v>Text confirmed in both apps during partner/location setup reconciliation.</x:v>
       </x:c>
       <x:c r="H9" s="59" t="str">
         <x:v>Stored source column</x:v>
@@ -10458,7 +10458,7 @@
         <x:v>OLTP + OLAP</x:v>
       </x:c>
       <x:c r="F230" s="57" t="str">
-        <x:v>OLTP: PII; OLAP: Required</x:v>
+        <x:v>OLTP: PII; OLAP: Required, PII</x:v>
       </x:c>
       <x:c r="G230" s="59" t="str">
         <x:v>Stores the authoritative source value for Email.</x:v>
@@ -14165,7 +14165,7 @@
 OLAP v1.100016: List. Same REF_ROWS expression. Initial value blank. No operational payment actions or processing formulas imported.</x:v>
       </x:c>
     </x:row>
-    <x:row r="370" ht="15" customHeight="1">
+    <x:row r="370" ht="78" customHeight="1">
       <x:c r="A370" s="87" t="str">
         <x:v>Borrowers</x:v>
       </x:c>
@@ -14179,19 +14179,19 @@
         <x:v>Physical / Text</x:v>
       </x:c>
       <x:c r="E370" s="87" t="str">
-        <x:v>OLTP; OLAP pending</x:v>
+        <x:v>OLTP + OLAP</x:v>
       </x:c>
       <x:c r="F370" s="87" t="str">
-        <x:v>Editable</x:v>
+        <x:v>OLTP editable; OLAP table read-only; shown, optional, searchable</x:v>
       </x:c>
       <x:c r="G370" s="87" t="str">
         <x:v>Explicit message address; no suffix stripping. App physical position 8.</x:v>
       </x:c>
       <x:c r="H370" s="87" t="str">
-        <x:v>Stored; blank initial value; display name: "ชื่อที่ใช้เรียก / Communication Name"</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="371" ht="15" customHeight="1">
+        <x:v>Stored; blank initial value. OLTP display name "ชื่อที่ใช้เรียก / Communication Name"; OLAP default field name.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="371" ht="78" customHeight="1">
       <x:c r="A371" s="87" t="str">
         <x:v>Borrowers</x:v>
       </x:c>
@@ -14205,10 +14205,10 @@
         <x:v>Physical / Text</x:v>
       </x:c>
       <x:c r="E371" s="87" t="str">
-        <x:v>OLTP; OLAP pending</x:v>
+        <x:v>OLTP + OLAP</x:v>
       </x:c>
       <x:c r="F371" s="87" t="str">
-        <x:v>Editable</x:v>
+        <x:v>OLTP editable; OLAP table read-only; shown, optional, searchable</x:v>
       </x:c>
       <x:c r="G371" s="87" t="str">
         <x:v>Borrower Instagram handle without @; app physical position 9.</x:v>
@@ -14217,7 +14217,7 @@
         <x:v>Stored; blank initial value</x:v>
       </x:c>
     </x:row>
-    <x:row r="372" ht="15" customHeight="1">
+    <x:row r="372" ht="78" customHeight="1">
       <x:c r="A372" s="87" t="str">
         <x:v>Borrowers</x:v>
       </x:c>
@@ -14228,22 +14228,22 @@
         <x:v>Instagram Conversation URL</x:v>
       </x:c>
       <x:c r="D372" s="87" t="str">
-        <x:v>Physical / Url</x:v>
+        <x:v>Physical / Url (OLTP); Text (OLAP)</x:v>
       </x:c>
       <x:c r="E372" s="87" t="str">
-        <x:v>OLTP; OLAP pending</x:v>
+        <x:v>OLTP + OLAP</x:v>
       </x:c>
       <x:c r="F372" s="87" t="str">
-        <x:v>Editable</x:v>
+        <x:v>OLTP editable; OLAP table read-only; shown, optional, searchable</x:v>
       </x:c>
       <x:c r="G372" s="87" t="str">
         <x:v>Verified conversation link; native Text, app Url; position 10.</x:v>
       </x:c>
       <x:c r="H372" s="87" t="str">
-        <x:v>Stored; blank initial value</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="373" ht="15" customHeight="1">
+        <x:v>Stored native Text; OLTP Url, OLAP Text. Both initial values blank; existing app type variance preserved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="373" ht="78" customHeight="1">
       <x:c r="A373" s="87" t="str">
         <x:v>Borrowers</x:v>
       </x:c>
@@ -14257,19 +14257,19 @@
         <x:v>Physical / DateTime</x:v>
       </x:c>
       <x:c r="E373" s="87" t="str">
-        <x:v>OLTP; OLAP pending</x:v>
+        <x:v>OLTP + OLAP</x:v>
       </x:c>
       <x:c r="F373" s="87" t="str">
-        <x:v>Editable</x:v>
+        <x:v>OLTP editable; OLAP table read-only; shown, optional, searchable</x:v>
       </x:c>
       <x:c r="G373" s="87" t="str">
         <x:v>Time mapping was actually checked; position 11.</x:v>
       </x:c>
       <x:c r="H373" s="87" t="str">
-        <x:v>Stored; blank initial value (removed inferred NOW())</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="374" ht="15" customHeight="1">
+        <x:v>Stored; blank initial value in both apps. OLAP inherited NOW() removed during 13 September reconciliation. Existing values unchanged.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="374" ht="78" customHeight="1">
       <x:c r="A374" s="87" t="str">
         <x:v>Borrowers</x:v>
       </x:c>
@@ -14283,19 +14283,19 @@
         <x:v>Physical / Yes/No</x:v>
       </x:c>
       <x:c r="E374" s="87" t="str">
-        <x:v>OLTP; OLAP pending</x:v>
+        <x:v>OLTP + OLAP</x:v>
       </x:c>
       <x:c r="F374" s="87" t="str">
-        <x:v>Editable</x:v>
+        <x:v>OLTP editable; OLAP table read-only; shown, optional, searchable</x:v>
       </x:c>
       <x:c r="G374" s="87" t="str">
         <x:v>Existing borrower opt-in; also required alongside Collection dashboard eligibility for the proposed partner daily briefing. Existing flag values unchanged.</x:v>
       </x:c>
       <x:c r="H374" s="87" t="str">
-        <x:v>Stored; initial value FALSE</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="375" ht="15" customHeight="1">
+        <x:v>Stored; initial FALSE in both apps. OLAP table remains read-only; existing values unchanged.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="375" ht="78" customHeight="1">
       <x:c r="A375" s="87" t="str">
         <x:v>Borrowers</x:v>
       </x:c>
@@ -14309,19 +14309,19 @@
         <x:v>Physical / Yes/No</x:v>
       </x:c>
       <x:c r="E375" s="87" t="str">
-        <x:v>OLTP; OLAP pending</x:v>
+        <x:v>OLTP + OLAP</x:v>
       </x:c>
       <x:c r="F375" s="87" t="str">
-        <x:v>Editable</x:v>
+        <x:v>OLTP editable; OLAP table read-only; shown, optional, searchable</x:v>
       </x:c>
       <x:c r="G375" s="87" t="str">
         <x:v>Independent penalty eligibility; position 13. Existing fees never reversed by this flag.</x:v>
       </x:c>
       <x:c r="H375" s="87" t="str">
-        <x:v>Stored; initial value FALSE; daily eligibility held in runner SQLite</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="376" ht="15" customHeight="1">
+        <x:v>Stored; initial FALSE in both apps. Existing values and collection runtime unchanged.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="376" ht="78" customHeight="1">
       <x:c r="A376" s="87" t="str">
         <x:v>Borrowers</x:v>
       </x:c>
@@ -14335,10 +14335,10 @@
         <x:v>Physical / Ref</x:v>
       </x:c>
       <x:c r="E376" s="87" t="str">
-        <x:v>OLTP; OLAP pending</x:v>
+        <x:v>OLTP + OLAP</x:v>
       </x:c>
       <x:c r="F376" s="87" t="str">
-        <x:v>Editable, Optional</x:v>
+        <x:v>OLTP editable; OLAP table read-only; shown, optional, searchable</x:v>
       </x:c>
       <x:c r="G376" s="87" t="str">
         <x:v>Borrower-specific receiving bank; position 14.</x:v>
@@ -14789,7 +14789,7 @@
         <x:v>Initial value: TRUE. No app formula. Native key h7VnJR1ERY4o6UUaiANzwe. Restore nominal rates without re-enabling generation.</x:v>
       </x:c>
     </x:row>
-    <x:row r="394" ht="42" customHeight="1">
+    <x:row r="394" ht="78" customHeight="1">
       <x:c r="A394" s="73" t="str">
         <x:v>Partners</x:v>
       </x:c>
@@ -14803,19 +14803,19 @@
         <x:v>Physical / Text</x:v>
       </x:c>
       <x:c r="E394" s="73" t="str">
-        <x:v>OLTP; OLAP pending</x:v>
+        <x:v>OLTP + OLAP</x:v>
       </x:c>
       <x:c r="F394" s="73" t="str">
         <x:v>Shown, editable, optional, searchable</x:v>
       </x:c>
       <x:c r="G394" s="73" t="str">
-        <x:v>Partner Instagram handle. App position 6. No separate partner list.</x:v>
+        <x:v>Partner Instagram handle. Stored position 6 in both apps; managed through OLAP Partners_Form.</x:v>
       </x:c>
       <x:c r="H394" s="73" t="str">
         <x:v>Stored; no formula, default, key or label. Verification binding belongs to later agent implementation.</x:v>
       </x:c>
     </x:row>
-    <x:row r="395" ht="42" customHeight="1">
+    <x:row r="395" ht="78" customHeight="1">
       <x:c r="A395" s="73" t="str">
         <x:v>Partners</x:v>
       </x:c>
@@ -14829,19 +14829,19 @@
         <x:v>Physical / Text</x:v>
       </x:c>
       <x:c r="E395" s="73" t="str">
-        <x:v>OLTP; OLAP pending</x:v>
+        <x:v>OLTP + OLAP</x:v>
       </x:c>
       <x:c r="F395" s="73" t="str">
         <x:v>Shown, editable, optional, searchable</x:v>
       </x:c>
       <x:c r="G395" s="73" t="str">
-        <x:v>Language for partner notices, replies and email. App position 7.</x:v>
+        <x:v>Partner notices/replies/email language; stored position 7 in both apps. OLAP owns partner management.</x:v>
       </x:c>
       <x:c r="H395" s="73" t="str">
         <x:v>Stored; blank initial value. Preferences not inferred or populated. Borrower drafts retain approved Thai.</x:v>
       </x:c>
     </x:row>
-    <x:row r="396" ht="42" customHeight="1">
+    <x:row r="396" ht="78" customHeight="1">
       <x:c r="A396" s="73" t="str">
         <x:v>Partners</x:v>
       </x:c>
@@ -14855,19 +14855,19 @@
         <x:v>Physical / Yes/No</x:v>
       </x:c>
       <x:c r="E396" s="73" t="str">
-        <x:v>OLTP; OLAP pending</x:v>
+        <x:v>OLTP + OLAP</x:v>
       </x:c>
       <x:c r="F396" s="73" t="str">
         <x:v>Shown, editable, optional, searchable</x:v>
       </x:c>
       <x:c r="G396" s="73" t="str">
-        <x:v>Master opt-in for partner Instagram and email fallback. App position 8.</x:v>
+        <x:v>Master opt-in for partner Instagram and email fallback; stored position 8 in both apps. Defaults FALSE; future agent only.</x:v>
       </x:c>
       <x:c r="H396" s="73" t="str">
         <x:v>Initial value FALSE; no app formula. Existing partners unchecked. Only TRUE permits future agent communication.</x:v>
       </x:c>
     </x:row>
-    <x:row r="397" ht="42" customHeight="1">
+    <x:row r="397" ht="78" customHeight="1">
       <x:c r="A397" s="73" t="str">
         <x:v>Borrowers</x:v>
       </x:c>
@@ -14881,10 +14881,10 @@
         <x:v>Physical / Text</x:v>
       </x:c>
       <x:c r="E397" s="73" t="str">
-        <x:v>OLTP; OLAP pending</x:v>
+        <x:v>OLTP + OLAP</x:v>
       </x:c>
       <x:c r="F397" s="73" t="str">
-        <x:v>Shown, editable, optional, searchable</x:v>
+        <x:v>OLTP editable; OLAP table read-only; shown, optional, searchable</x:v>
       </x:c>
       <x:c r="G397" s="73" t="str">
         <x:v>Borrower city from the owner location sheet. App position 15.</x:v>
@@ -14893,7 +14893,7 @@
         <x:v>Stored; blank initial value; display name: "เมือง / City". Source blanks preserved.</x:v>
       </x:c>
     </x:row>
-    <x:row r="398" ht="42" customHeight="1">
+    <x:row r="398" ht="78" customHeight="1">
       <x:c r="A398" s="73" t="str">
         <x:v>Borrowers</x:v>
       </x:c>
@@ -14907,10 +14907,10 @@
         <x:v>Physical / Text</x:v>
       </x:c>
       <x:c r="E398" s="73" t="str">
-        <x:v>OLTP; OLAP pending</x:v>
+        <x:v>OLTP + OLAP</x:v>
       </x:c>
       <x:c r="F398" s="73" t="str">
-        <x:v>Shown, editable, optional, searchable</x:v>
+        <x:v>OLTP editable; OLAP table read-only; shown, optional, searchable</x:v>
       </x:c>
       <x:c r="G398" s="73" t="str">
         <x:v>Workplace/locality from the owner location sheet. App position 16.</x:v>
@@ -14930,7 +14930,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82c1edae5ecb4b6f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R008277dddce642bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15359,7 +15359,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6373227e1eb1402d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra680af7fa9eb4228"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15490,7 +15490,7 @@
         <x:v>OLTP 3.000050; location columns included after regeneration. Existing row filter and update mode retained.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="15" customHeight="1">
+    <x:row r="7" ht="96" customHeight="1">
       <x:c r="A7" s="57" t="str">
         <x:v>OLAP</x:v>
       </x:c>
@@ -15507,14 +15507,16 @@
         <x:v>Read-only</x:v>
       </x:c>
       <x:c r="F7" s="57" t="n">
-        <x:v>56</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="G7" s="59" t="str">
         <x:v>Read-only OLAP subset of borrowers whose outstanding principal is greater than zero.</x:v>
       </x:c>
-      <x:c r="H7" s="59"/>
-    </x:row>
-    <x:row r="8" ht="15" customHeight="1">
+      <x:c r="H7" s="59" t="str">
+        <x:v>OLAP 1.100031: exact membership reconciled; City and Working Location appended. Existing filter, actions and read-only mode retained. Earlier membership gaps corrected in inventory.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="96" customHeight="1">
       <x:c r="A8" s="57" t="str">
         <x:v>OLAP</x:v>
       </x:c>
@@ -15531,14 +15533,16 @@
         <x:v>Read-only</x:v>
       </x:c>
       <x:c r="F8" s="57" t="n">
-        <x:v>56</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="G8" s="59" t="str">
         <x:v>Read-only OLAP subset of borrowers contributing positive interest profit in the last 30 days.</x:v>
       </x:c>
-      <x:c r="H8" s="59"/>
-    </x:row>
-    <x:row r="9" ht="15" customHeight="1">
+      <x:c r="H8" s="59" t="str">
+        <x:v>OLAP 1.100031: exact membership reconciled; City and Working Location appended. Existing filter, actions and read-only mode retained. Earlier membership gaps corrected in inventory.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="96" customHeight="1">
       <x:c r="A9" s="57" t="str">
         <x:v>OLAP</x:v>
       </x:c>
@@ -15549,18 +15553,20 @@
         <x:v>Borrowers</x:v>
       </x:c>
       <x:c r="D9" s="59" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>(blank — no row filter)</x:v>
       </x:c>
       <x:c r="E9" s="57" t="str">
         <x:v>Read-only</x:v>
       </x:c>
       <x:c r="F9" s="57" t="n">
-        <x:v>51</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="G9" s="59" t="str">
         <x:v>Curated, read-only borrower feed for downstream reporting and dashboard reconciliation, including the borrower value/stability matrix fields.</x:v>
       </x:c>
-      <x:c r="H9" s="59"/>
+      <x:c r="H9" s="59" t="str">
+        <x:v>OLAP 1.100031: exact membership reconciled; City and Working Location appended. Existing filter, actions and read-only mode retained. Earlier membership gaps corrected in inventory.</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="15" customHeight="1">
       <x:c r="A10" s="57" t="str">
@@ -15754,7 +15760,7 @@
       </x:c>
       <x:c r="H17" s="59"/>
     </x:row>
-    <x:row r="18">
+    <x:row r="18" ht="96" customHeight="1">
       <x:c r="A18" s="72" t="str">
         <x:v>OLAP</x:v>
       </x:c>
@@ -15771,13 +15777,13 @@
         <x:v>Read-only</x:v>
       </x:c>
       <x:c r="F18" s="72" t="n">
-        <x:v>11</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G18" s="72" t="str">
         <x:v>Read-only daily collection export and message-review slice using OLAP-native current-status, amount, charge-list, hidden-flag, and overdue fields.</x:v>
       </x:c>
       <x:c r="H18" s="72" t="str">
-        <x:v>OLAP read-only mirror of the OLTP Todays Collection Board for daily collection export and message-drafting review. The exact column set is adapted to available OLAP fields.</x:v>
+        <x:v>OLAP 1.100031: exact membership reconciled; City and Working Location appended. Existing filter, actions and read-only mode retained. Earlier membership gaps corrected in inventory.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" customHeight="1">
@@ -15813,7 +15819,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8379e6cd54e749fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a23d02162ae4d84"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20856,7 +20862,7 @@
         <x:v>Reporting Borrowers</x:v>
       </x:c>
       <x:c r="C361" t="n">
-        <x:v>41</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="D361" t="str">
         <x:v>Matrix Active Borrower Count</x:v>
@@ -20870,7 +20876,7 @@
         <x:v>Reporting Borrowers</x:v>
       </x:c>
       <x:c r="C362" t="n">
-        <x:v>42</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="D362" t="str">
         <x:v>Matrix Equal Share Benchmark</x:v>
@@ -20884,7 +20890,7 @@
         <x:v>Reporting Borrowers</x:v>
       </x:c>
       <x:c r="C363" t="n">
-        <x:v>43</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="D363" t="str">
         <x:v>Matrix Economic Contribution</x:v>
@@ -20898,7 +20904,7 @@
         <x:v>Reporting Borrowers</x:v>
       </x:c>
       <x:c r="C364" t="n">
-        <x:v>44</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="D364" t="str">
         <x:v>Matrix Recent Reliability Score</x:v>
@@ -20954,7 +20960,7 @@
         <x:v>Reporting Borrowers</x:v>
       </x:c>
       <x:c r="C368" t="n">
-        <x:v>48</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="D368" t="str">
         <x:v>Matrix History Sufficient</x:v>
@@ -20968,7 +20974,7 @@
         <x:v>Reporting Borrowers</x:v>
       </x:c>
       <x:c r="C369" t="n">
-        <x:v>49</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="D369" t="str">
         <x:v>Matrix Stability Score</x:v>
@@ -20982,7 +20988,7 @@
         <x:v>Reporting Borrowers</x:v>
       </x:c>
       <x:c r="C370" t="n">
-        <x:v>50</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D370" t="str">
         <x:v>Matrix Quadrant</x:v>
@@ -20996,7 +21002,7 @@
         <x:v>Reporting Borrowers</x:v>
       </x:c>
       <x:c r="C371" t="n">
-        <x:v>51</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="D371" t="str">
         <x:v>Matrix Bubble Label</x:v>
@@ -22077,6 +22083,622 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="D448" t="str">
+        <x:v>Working Location</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="449">
+      <x:c r="A449" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B449" t="str">
+        <x:v>Reporting Borrowers</x:v>
+      </x:c>
+      <x:c r="C449" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="D449" t="str">
+        <x:v>Hidden Flag</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="450">
+      <x:c r="A450" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B450" t="str">
+        <x:v>Reporting Borrowers</x:v>
+      </x:c>
+      <x:c r="C450" t="n">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="D450" t="str">
+        <x:v>Matrix Scaled Economic Contribution</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="451">
+      <x:c r="A451" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B451" t="str">
+        <x:v>Reporting Borrowers</x:v>
+      </x:c>
+      <x:c r="C451" t="n">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="D451" t="str">
+        <x:v>Related Payments</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="452">
+      <x:c r="A452" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B452" t="str">
+        <x:v>Reporting Borrowers</x:v>
+      </x:c>
+      <x:c r="C452" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="D452" t="str">
+        <x:v>City</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="453">
+      <x:c r="A453" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B453" t="str">
+        <x:v>Reporting Borrowers</x:v>
+      </x:c>
+      <x:c r="C453" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="D453" t="str">
+        <x:v>Working Location</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="454">
+      <x:c r="A454" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B454" t="str">
+        <x:v>Borrowers with Outstanding Loans</x:v>
+      </x:c>
+      <x:c r="C454" t="n">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="D454" t="str">
+        <x:v>Hidden Flag</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="455">
+      <x:c r="A455" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B455" t="str">
+        <x:v>Borrowers with Outstanding Loans</x:v>
+      </x:c>
+      <x:c r="C455" t="n">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="D455" t="str">
+        <x:v>Projected Monthly Profit Contribution</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="456">
+      <x:c r="A456" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B456" t="str">
+        <x:v>Borrowers with Outstanding Loans</x:v>
+      </x:c>
+      <x:c r="C456" t="n">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="D456" t="str">
+        <x:v>Matrix Active Borrower Count</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="457">
+      <x:c r="A457" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B457" t="str">
+        <x:v>Borrowers with Outstanding Loans</x:v>
+      </x:c>
+      <x:c r="C457" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="D457" t="str">
+        <x:v>Matrix Equal Share Benchmark</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="458">
+      <x:c r="A458" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B458" t="str">
+        <x:v>Borrowers with Outstanding Loans</x:v>
+      </x:c>
+      <x:c r="C458" t="n">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="D458" t="str">
+        <x:v>Matrix Economic Contribution</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="459">
+      <x:c r="A459" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B459" t="str">
+        <x:v>Borrowers with Outstanding Loans</x:v>
+      </x:c>
+      <x:c r="C459" t="n">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="D459" t="str">
+        <x:v>Matrix Recent Reliability Score</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="460">
+      <x:c r="A460" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B460" t="str">
+        <x:v>Borrowers with Outstanding Loans</x:v>
+      </x:c>
+      <x:c r="C460" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="D460" t="str">
+        <x:v>Matrix Historical Reliability Score</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="461">
+      <x:c r="A461" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B461" t="str">
+        <x:v>Borrowers with Outstanding Loans</x:v>
+      </x:c>
+      <x:c r="C461" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D461" t="str">
+        <x:v>Matrix Delay Severity Score</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="462">
+      <x:c r="A462" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B462" t="str">
+        <x:v>Borrowers with Outstanding Loans</x:v>
+      </x:c>
+      <x:c r="C462" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="D462" t="str">
+        <x:v>Matrix Current Condition Score</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="463">
+      <x:c r="A463" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B463" t="str">
+        <x:v>Borrowers with Outstanding Loans</x:v>
+      </x:c>
+      <x:c r="C463" t="n">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="D463" t="str">
+        <x:v>Matrix History Sufficient</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="464">
+      <x:c r="A464" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B464" t="str">
+        <x:v>Borrowers with Outstanding Loans</x:v>
+      </x:c>
+      <x:c r="C464" t="n">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="D464" t="str">
+        <x:v>Matrix Stability Score</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="465">
+      <x:c r="A465" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B465" t="str">
+        <x:v>Borrowers with Outstanding Loans</x:v>
+      </x:c>
+      <x:c r="C465" t="n">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="D465" t="str">
+        <x:v>Matrix Quadrant</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="466">
+      <x:c r="A466" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B466" t="str">
+        <x:v>Borrowers with Outstanding Loans</x:v>
+      </x:c>
+      <x:c r="C466" t="n">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="D466" t="str">
+        <x:v>Matrix Bubble Label</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="467">
+      <x:c r="A467" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B467" t="str">
+        <x:v>Borrowers with Outstanding Loans</x:v>
+      </x:c>
+      <x:c r="C467" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="D467" t="str">
+        <x:v>Profit Last 10 Days</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="468">
+      <x:c r="A468" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B468" t="str">
+        <x:v>Borrowers with Outstanding Loans</x:v>
+      </x:c>
+      <x:c r="C468" t="n">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="D468" t="str">
+        <x:v>Matrix Scaled Economic Contribution</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="469">
+      <x:c r="A469" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B469" t="str">
+        <x:v>Borrowers with Outstanding Loans</x:v>
+      </x:c>
+      <x:c r="C469" t="n">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="D469" t="str">
+        <x:v>Related Payments</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="470">
+      <x:c r="A470" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B470" t="str">
+        <x:v>Borrowers with Outstanding Loans</x:v>
+      </x:c>
+      <x:c r="C470" t="n">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="D470" t="str">
+        <x:v>City</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="471">
+      <x:c r="A471" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B471" t="str">
+        <x:v>Borrowers with Outstanding Loans</x:v>
+      </x:c>
+      <x:c r="C471" t="n">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="D471" t="str">
+        <x:v>Working Location</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="472">
+      <x:c r="A472" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B472" t="str">
+        <x:v>Profit Contribution 30D</x:v>
+      </x:c>
+      <x:c r="C472" t="n">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="D472" t="str">
+        <x:v>Hidden Flag</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="473">
+      <x:c r="A473" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B473" t="str">
+        <x:v>Profit Contribution 30D</x:v>
+      </x:c>
+      <x:c r="C473" t="n">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="D473" t="str">
+        <x:v>Projected Monthly Profit Contribution</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="474">
+      <x:c r="A474" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B474" t="str">
+        <x:v>Profit Contribution 30D</x:v>
+      </x:c>
+      <x:c r="C474" t="n">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="D474" t="str">
+        <x:v>Matrix Active Borrower Count</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="475">
+      <x:c r="A475" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B475" t="str">
+        <x:v>Profit Contribution 30D</x:v>
+      </x:c>
+      <x:c r="C475" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="D475" t="str">
+        <x:v>Matrix Equal Share Benchmark</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="476">
+      <x:c r="A476" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B476" t="str">
+        <x:v>Profit Contribution 30D</x:v>
+      </x:c>
+      <x:c r="C476" t="n">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="D476" t="str">
+        <x:v>Matrix Economic Contribution</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="477">
+      <x:c r="A477" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B477" t="str">
+        <x:v>Profit Contribution 30D</x:v>
+      </x:c>
+      <x:c r="C477" t="n">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="D477" t="str">
+        <x:v>Matrix Recent Reliability Score</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="478">
+      <x:c r="A478" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B478" t="str">
+        <x:v>Profit Contribution 30D</x:v>
+      </x:c>
+      <x:c r="C478" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="D478" t="str">
+        <x:v>Matrix Historical Reliability Score</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="479">
+      <x:c r="A479" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B479" t="str">
+        <x:v>Profit Contribution 30D</x:v>
+      </x:c>
+      <x:c r="C479" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D479" t="str">
+        <x:v>Matrix Delay Severity Score</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="480">
+      <x:c r="A480" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B480" t="str">
+        <x:v>Profit Contribution 30D</x:v>
+      </x:c>
+      <x:c r="C480" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="D480" t="str">
+        <x:v>Matrix Current Condition Score</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="481">
+      <x:c r="A481" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B481" t="str">
+        <x:v>Profit Contribution 30D</x:v>
+      </x:c>
+      <x:c r="C481" t="n">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="D481" t="str">
+        <x:v>Matrix History Sufficient</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="482">
+      <x:c r="A482" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B482" t="str">
+        <x:v>Profit Contribution 30D</x:v>
+      </x:c>
+      <x:c r="C482" t="n">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="D482" t="str">
+        <x:v>Matrix Stability Score</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="483">
+      <x:c r="A483" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B483" t="str">
+        <x:v>Profit Contribution 30D</x:v>
+      </x:c>
+      <x:c r="C483" t="n">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="D483" t="str">
+        <x:v>Matrix Quadrant</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="484">
+      <x:c r="A484" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B484" t="str">
+        <x:v>Profit Contribution 30D</x:v>
+      </x:c>
+      <x:c r="C484" t="n">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="D484" t="str">
+        <x:v>Matrix Bubble Label</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="485">
+      <x:c r="A485" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B485" t="str">
+        <x:v>Profit Contribution 30D</x:v>
+      </x:c>
+      <x:c r="C485" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="D485" t="str">
+        <x:v>Profit Last 10 Days</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="486">
+      <x:c r="A486" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B486" t="str">
+        <x:v>Profit Contribution 30D</x:v>
+      </x:c>
+      <x:c r="C486" t="n">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="D486" t="str">
+        <x:v>Matrix Scaled Economic Contribution</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="487">
+      <x:c r="A487" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B487" t="str">
+        <x:v>Profit Contribution 30D</x:v>
+      </x:c>
+      <x:c r="C487" t="n">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="D487" t="str">
+        <x:v>Related Payments</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="488">
+      <x:c r="A488" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B488" t="str">
+        <x:v>Profit Contribution 30D</x:v>
+      </x:c>
+      <x:c r="C488" t="n">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="D488" t="str">
+        <x:v>City</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="489">
+      <x:c r="A489" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B489" t="str">
+        <x:v>Profit Contribution 30D</x:v>
+      </x:c>
+      <x:c r="C489" t="n">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="D489" t="str">
+        <x:v>Working Location</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="490">
+      <x:c r="A490" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B490" t="str">
+        <x:v>Todays Collection Board</x:v>
+      </x:c>
+      <x:c r="C490" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D490" t="str">
+        <x:v>Related Payments</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="491">
+      <x:c r="A491" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B491" t="str">
+        <x:v>Todays Collection Board</x:v>
+      </x:c>
+      <x:c r="C491" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D491" t="str">
+        <x:v>City</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="492">
+      <x:c r="A492" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B492" t="str">
+        <x:v>Todays Collection Board</x:v>
+      </x:c>
+      <x:c r="C492" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="D492" t="str">
         <x:v>Working Location</x:v>
       </x:c>
     </x:row>
@@ -22087,7 +22709,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd662c409624492a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfff62d5c127344a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26110,10 +26732,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E204" s="87" t="str">
-        <x:v>Pending reconciliation</x:v>
+        <x:v>Yes — 1.100031</x:v>
       </x:c>
       <x:c r="F204" s="87" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); collection settings owned by OLTP.</x:v>
+        <x:v>Verified loaded in OLAP. Partner fields managed in OLAP; borrower table remains read-only. Existing financial formulas and row flags unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="205" ht="15" customHeight="1">
@@ -26130,10 +26752,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E205" s="87" t="str">
-        <x:v>Pending reconciliation</x:v>
+        <x:v>Yes — 1.100031</x:v>
       </x:c>
       <x:c r="F205" s="87" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); collection settings owned by OLTP.</x:v>
+        <x:v>Verified loaded in OLAP. Partner fields managed in OLAP; borrower table remains read-only. Existing financial formulas and row flags unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="206" ht="15" customHeight="1">
@@ -26150,10 +26772,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E206" s="87" t="str">
-        <x:v>Pending reconciliation</x:v>
+        <x:v>Yes — 1.100031</x:v>
       </x:c>
       <x:c r="F206" s="87" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); collection settings owned by OLTP.</x:v>
+        <x:v>OLTP Url; OLAP Text; native Text. Existing type variance preserved. Both initial values blank.</x:v>
       </x:c>
     </x:row>
     <x:row r="207" ht="15" customHeight="1">
@@ -26170,10 +26792,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E207" s="87" t="str">
-        <x:v>Pending reconciliation</x:v>
+        <x:v>Yes — 1.100031</x:v>
       </x:c>
       <x:c r="F207" s="87" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); collection settings owned by OLTP.</x:v>
+        <x:v>Verified loaded in OLAP. Partner fields managed in OLAP; borrower table remains read-only. Existing financial formulas and row flags unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="208" ht="15" customHeight="1">
@@ -26190,10 +26812,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E208" s="87" t="str">
-        <x:v>Pending reconciliation</x:v>
+        <x:v>Yes — 1.100031</x:v>
       </x:c>
       <x:c r="F208" s="87" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); collection settings owned by OLTP.</x:v>
+        <x:v>Verified loaded in OLAP. Partner fields managed in OLAP; borrower table remains read-only. Existing financial formulas and row flags unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="209" ht="15" customHeight="1">
@@ -26210,10 +26832,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E209" s="87" t="str">
-        <x:v>Pending reconciliation</x:v>
+        <x:v>Yes — 1.100031</x:v>
       </x:c>
       <x:c r="F209" s="87" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); collection settings owned by OLTP.</x:v>
+        <x:v>Verified loaded in OLAP. Partner fields managed in OLAP; borrower table remains read-only. Existing financial formulas and row flags unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="210" ht="15" customHeight="1">
@@ -26230,10 +26852,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E210" s="87" t="str">
-        <x:v>Pending reconciliation</x:v>
+        <x:v>Yes — 1.100031</x:v>
       </x:c>
       <x:c r="F210" s="87" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); collection settings owned by OLTP.</x:v>
+        <x:v>Verified loaded in OLAP. Partner fields managed in OLAP; borrower table remains read-only. Existing financial formulas and row flags unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="211" ht="15" customHeight="1">
@@ -26590,10 +27212,10 @@
         <x:v>Yes — 3.000050</x:v>
       </x:c>
       <x:c r="E228" t="str">
-        <x:v>Pending reconciliation</x:v>
+        <x:v>Yes — 1.100031</x:v>
       </x:c>
       <x:c r="F228" t="str">
-        <x:v>Stored in shared database; OLTP configured. OLAP app not regenerated by this task.</x:v>
+        <x:v>Verified loaded in OLAP. Partner fields managed in OLAP; borrower table remains read-only. Existing financial formulas and row flags unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="229">
@@ -26610,10 +27232,10 @@
         <x:v>Yes — 3.000050</x:v>
       </x:c>
       <x:c r="E229" t="str">
-        <x:v>Pending reconciliation</x:v>
+        <x:v>Yes — 1.100031</x:v>
       </x:c>
       <x:c r="F229" t="str">
-        <x:v>Stored in shared database; OLTP configured. OLAP app not regenerated by this task.</x:v>
+        <x:v>Verified loaded in OLAP. Partner fields managed in OLAP; borrower table remains read-only. Existing financial formulas and row flags unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="230">
@@ -26630,10 +27252,10 @@
         <x:v>Yes — 3.000050</x:v>
       </x:c>
       <x:c r="E230" t="str">
-        <x:v>Pending reconciliation</x:v>
+        <x:v>Yes — 1.100031</x:v>
       </x:c>
       <x:c r="F230" t="str">
-        <x:v>Stored in shared database; OLTP configured. OLAP app not regenerated by this task.</x:v>
+        <x:v>Verified loaded in OLAP. Partner fields managed in OLAP; borrower table remains read-only. Existing financial formulas and row flags unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="231">
@@ -26650,10 +27272,10 @@
         <x:v>Yes — 3.000050</x:v>
       </x:c>
       <x:c r="E231" t="str">
-        <x:v>Pending reconciliation</x:v>
+        <x:v>Yes — 1.100031</x:v>
       </x:c>
       <x:c r="F231" t="str">
-        <x:v>Stored in shared database; OLTP configured. OLAP app not regenerated by this task.</x:v>
+        <x:v>Verified loaded in OLAP. Partner fields managed in OLAP; borrower table remains read-only. Existing financial formulas and row flags unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="232">
@@ -26670,10 +27292,10 @@
         <x:v>Yes — 3.000050</x:v>
       </x:c>
       <x:c r="E232" t="str">
-        <x:v>Pending reconciliation</x:v>
+        <x:v>Yes — 1.100031</x:v>
       </x:c>
       <x:c r="F232" t="str">
-        <x:v>Stored in shared database; OLTP configured. OLAP app not regenerated by this task.</x:v>
+        <x:v>Verified loaded in OLAP. Partner fields managed in OLAP; borrower table remains read-only. Existing financial formulas and row flags unchanged.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -26686,7 +27308,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfe8af29d8ae41ed"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ac7d86e7b3745a2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26885,7 +27507,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e5f7a3347484eb0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1174ee0ff2f24e7f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28538,7 +29160,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf15aefded0a44967"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R116bec59645c48da"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Restrict partner language to English and Thai in both apps
</commit_message>
<xml_diff>
--- a/Documents/AppSheet_Data_Dictionary.xlsx
+++ b/Documents/AppSheet_Data_Dictionary.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R04429f714ad54310"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="R6eb4a437eb894a35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R62093d1a3d63442f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R37c42161bd4d4552"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="Rbbe168736fc445fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="Rc7efbb7a1e174594"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="R5f2f79c51fcb4170"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="Rc452e6abf5684e0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="R45c8270d30ce4000"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="Rdd80efcc0a714ace"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="R4d73f202be074a83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="Rccf1c12d05d14804"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rc06f07df53d747a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="Rd8b57970c9d04d2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R23d84db091ef4245"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R3e9179c3f0944505"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="Rf7af349bb1fb4388"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="Rf15c677865284f33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="R9b2a36d805394c51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R2f2d077a8018482f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="Rf4f07b18f7ec4605"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R231bb5271c2440fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="R159a540e4ddd4f34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="R88a15560b3a74227"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1079,7 +1079,7 @@
         <x:v>Reconciliation status</x:v>
       </x:c>
       <x:c r="B5" s="85" t="str">
-        <x:v>13 September 2026: OLTP 3.000050 and OLAP 1.100031 partner/location fields and affected slices reconciled. OLAP partner forms and borrower read-only detail checked. No agent activation.</x:v>
+        <x:v>13 September 2026: language enum verified in OLTP 3.000052 and OLAP 1.100033. OLAP current partner form shows English and ไทย. Earlier partner/location fields and slices retain recorded reconciliation scope.</x:v>
       </x:c>
       <x:c r="C5" s="73"/>
       <x:c r="D5" s="73"/>
@@ -1091,7 +1091,7 @@
         <x:v>Live baselines</x:v>
       </x:c>
       <x:c r="B6" s="85" t="str">
-        <x:v>Rollback: OLTP 3.000045; OLAP 1.100028. App restore does not restore shared database data/schema. Private location before-image remains outside Git. Owner acceptance pending.</x:v>
+        <x:v>Language enum rollback: OLTP 3.000050; OLAP 1.100031. Earlier setup rollback: OLTP 3.000045; OLAP 1.100028. App restoration does not restore database data/schema. Owner acceptance pending.</x:v>
       </x:c>
       <x:c r="C6" s="73"/>
       <x:c r="D6" s="73"/>
@@ -2492,7 +2492,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfdcff336c8174e33"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb86f79d7430741b4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3907,7 +3907,7 @@
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>13 September 2026: shared partner/location fields reconciled in both apps. OLTP 3.000050; OLAP 1.100031. Other tables retain dated verification scope.</x:v>
+        <x:v>13 September 2026: language enum updated in OLTP 3.000052 and OLAP 1.100033; table counts unchanged. Other tables retain dated verification scope.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
@@ -4299,7 +4299,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R285d3bc61d2041ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fecfe5482854df6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4332,7 +4332,7 @@
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>13 September 2026: OLTP 3.000050 and OLAP 1.100031 partner/location setup reconciled. Existing OLAP Borrowers remains read-only; no messaging activation. Other inventory retains dated scope.</x:v>
+        <x:v>13 September 2026: language enum verified in OLTP 3.000052 and OLAP 1.100033. Earlier partner/location and slice reconciliation retains its recorded scope. No messaging activation.</x:v>
       </x:c>
       <x:c r="B2"/>
       <x:c r="C2"/>
@@ -14815,7 +14815,7 @@
         <x:v>Stored; no formula, default, key or label. Verification binding belongs to later agent implementation.</x:v>
       </x:c>
     </x:row>
-    <x:row r="395" ht="78" customHeight="1">
+    <x:row r="395" ht="110" customHeight="1">
       <x:c r="A395" s="73" t="str">
         <x:v>Partners</x:v>
       </x:c>
@@ -14826,7 +14826,7 @@
         <x:v>Language Preference</x:v>
       </x:c>
       <x:c r="D395" s="73" t="str">
-        <x:v>Physical / Text</x:v>
+        <x:v>Physical / Enum (base Text)</x:v>
       </x:c>
       <x:c r="E395" s="73" t="str">
         <x:v>OLTP + OLAP</x:v>
@@ -14838,7 +14838,7 @@
         <x:v>Partner notices/replies/email language; stored position 7 in both apps. OLAP owns partner management.</x:v>
       </x:c>
       <x:c r="H395" s="73" t="str">
-        <x:v>Stored; blank initial value. Preferences not inferred or populated. Borrower drafts retain approved Thai.</x:v>
+        <x:v>Native database Text; app Enum in both apps. Dropdown: English, ไทย. Other values and other-value autocomplete disabled. Optional; blank initial value. Partner data unchanged. Borrower drafts retain approved Thai.</x:v>
       </x:c>
     </x:row>
     <x:row r="396" ht="78" customHeight="1">
@@ -14930,7 +14930,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R008277dddce642bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b384d860a054e21"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15359,7 +15359,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra680af7fa9eb4228"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5756f82d70bf4226"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15819,7 +15819,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a23d02162ae4d84"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70c120d9e6da4213"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22709,7 +22709,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfff62d5c127344a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4bbb7c6dfe74f47"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27229,13 +27229,13 @@
         <x:v>Language Preference</x:v>
       </x:c>
       <x:c r="D229" t="str">
-        <x:v>Yes — 3.000050</x:v>
+        <x:v>Yes — 3.000052</x:v>
       </x:c>
       <x:c r="E229" t="str">
-        <x:v>Yes — 1.100031</x:v>
+        <x:v>Yes — 1.100033</x:v>
       </x:c>
       <x:c r="F229" t="str">
-        <x:v>Verified loaded in OLAP. Partner fields managed in OLAP; borrower table remains read-only. Existing financial formulas and row flags unchanged.</x:v>
+        <x:v>Both apps: Enum, base Text, Dropdown, exactly English and ไทย; custom values disabled. Partner management remains in OLAP.</x:v>
       </x:c>
     </x:row>
     <x:row r="230">
@@ -27308,7 +27308,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ac7d86e7b3745a2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R663a3c3fbdf44d48"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27507,7 +27507,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1174ee0ff2f24e7f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bcb49d128a34f23"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29160,7 +29160,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R116bec59645c48da"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb12fc9a145a54bcc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document partial borrower cleanup and browser recovery checkpoint
</commit_message>
<xml_diff>
--- a/Documents/AppSheet_Data_Dictionary.xlsx
+++ b/Documents/AppSheet_Data_Dictionary.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rc06f07df53d747a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="Rd8b57970c9d04d2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R23d84db091ef4245"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R3e9179c3f0944505"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="Rf7af349bb1fb4388"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="Rf15c677865284f33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="R9b2a36d805394c51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R2f2d077a8018482f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="Rf4f07b18f7ec4605"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R231bb5271c2440fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="R159a540e4ddd4f34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="R88a15560b3a74227"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R9651d12c89b948fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="Rbf63829385f54798"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="Rabbefa11283742cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R766e019bb4a74dd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="R725af707c5154085"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R6bff1397ce6e46a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Raeaba5653582496c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R5628ca0a872f4855"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="Rdf6bc609c39d470a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R8f2e8b19e06740e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="Re2fc66bc4b9045ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="Rbc75ea26b2d241d9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1079,7 +1079,7 @@
         <x:v>Reconciliation status</x:v>
       </x:c>
       <x:c r="B5" s="85" t="str">
-        <x:v>13 September 2026: language enum verified in OLTP 3.000052 and OLAP 1.100033. OLAP current partner form shows English and ไทย. Earlier partner/location fields and slices retain recorded reconciliation scope.</x:v>
+        <x:v>Borrower cleanup PARTIAL: five OLTP settings saved; Chrome control failed before final version/readback. OLAP remains prior configuration. See authoritative borrower cleanup change log.</x:v>
       </x:c>
       <x:c r="C5" s="73"/>
       <x:c r="D5" s="73"/>
@@ -2492,7 +2492,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb86f79d7430741b4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf31271142f442b5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4299,7 +4299,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fecfe5482854df6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5dd9cb54c937408e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4332,7 +4332,7 @@
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>13 September 2026: language enum verified in OLTP 3.000052 and OLAP 1.100033. Earlier partner/location and slice reconciliation retains its recorded scope. No messaging activation.</x:v>
+        <x:v>13 September 2026: borrower cleanup PARTIAL. Five OLTP settings saved; post-save readback and OLAP reconciliation pending. All other inventory retains prior verification scope.</x:v>
       </x:c>
       <x:c r="B2"/>
       <x:c r="C2"/>
@@ -4430,7 +4430,7 @@
         <x:v>Stored source column; initial value: UNIQUEID("PackedUUID")</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="15" customHeight="1">
+    <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="57" t="str">
         <x:v>Borrowers</x:v>
       </x:c>
@@ -4452,8 +4452,8 @@
       <x:c r="G7" s="59" t="str">
         <x:v>Stores the authoritative source value for Borrower Name.</x:v>
       </x:c>
-      <x:c r="H7" s="59" t="str">
-        <x:v>Stored source column</x:v>
+      <x:c r="H7" s="82" t="str">
+        <x:v>Internal name preserved. OLTP display changed to Borrower Name - Thai. OLAP display reconciliation pending. Final readback/tests pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" customHeight="1">
@@ -4482,7 +4482,7 @@
         <x:v>Stored source column</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="15" customHeight="1">
+    <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="57" t="str">
         <x:v>Borrowers</x:v>
       </x:c>
@@ -4504,8 +4504,8 @@
       <x:c r="G9" s="59" t="str">
         <x:v>Text confirmed in both apps during partner/location setup reconciliation.</x:v>
       </x:c>
-      <x:c r="H9" s="59" t="str">
-        <x:v>Stored source column</x:v>
+      <x:c r="H9" s="82" t="str">
+        <x:v>Internal Description preserved. OLTP display changed to English Name. OLAP and Partner Operations GUI label reconciliation pending. Final readback/tests pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" customHeight="1">
@@ -14182,13 +14182,13 @@
         <x:v>OLTP + OLAP</x:v>
       </x:c>
       <x:c r="F370" s="87" t="str">
-        <x:v>OLTP editable; OLAP table read-only; shown, optional, searchable</x:v>
+        <x:v>OLTP required; OLAP prior optional, table read-only. Pending final reconciliation.</x:v>
       </x:c>
       <x:c r="G370" s="87" t="str">
         <x:v>Explicit message address; no suffix stripping. App physical position 8.</x:v>
       </x:c>
-      <x:c r="H370" s="87" t="str">
-        <x:v>Stored; blank initial value. OLTP display name "ชื่อที่ใช้เรียก / Communication Name"; OLAP default field name.</x:v>
+      <x:c r="H370" s="88" t="str">
+        <x:v>OLTP Require enabled. OLAP reconciliation pending. Blank initial value retained. Final readback/tests pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="371" ht="78" customHeight="1">
@@ -14291,8 +14291,8 @@
       <x:c r="G374" s="87" t="str">
         <x:v>Existing borrower opt-in; also required alongside Collection dashboard eligibility for the proposed partner daily briefing. Existing flag values unchanged.</x:v>
       </x:c>
-      <x:c r="H374" s="87" t="str">
-        <x:v>Stored; initial FALSE in both apps. OLAP table remains read-only; existing values unchanged.</x:v>
+      <x:c r="H374" s="88" t="str">
+        <x:v>OLTP initial changed to TRUE for new rows. Existing row values untouched. OLAP reconciliation pending. Final readback/tests pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="375" ht="78" customHeight="1">
@@ -14884,13 +14884,13 @@
         <x:v>OLTP + OLAP</x:v>
       </x:c>
       <x:c r="F397" s="73" t="str">
-        <x:v>OLTP editable; OLAP table read-only; shown, optional, searchable</x:v>
+        <x:v>OLTP required; OLAP prior optional, table read-only. Pending final reconciliation.</x:v>
       </x:c>
       <x:c r="G397" s="73" t="str">
         <x:v>Borrower city from the owner location sheet. App position 15.</x:v>
       </x:c>
       <x:c r="H397" s="73" t="str">
-        <x:v>Stored; blank initial value; display name: "เมือง / City". Source blanks preserved.</x:v>
+        <x:v>OLTP Require enabled; display เมือง / City and blank initial retained. OLAP reconciliation pending. Final readback/tests pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="398" ht="78" customHeight="1">
@@ -14930,7 +14930,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b384d860a054e21"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbefa88207b7e4147"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15359,7 +15359,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5756f82d70bf4226"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71c01aec0b6d4a7a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15819,7 +15819,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70c120d9e6da4213"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R742f04d9bb684197"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22709,7 +22709,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4bbb7c6dfe74f47"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb899178b9b345b0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27308,7 +27308,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R663a3c3fbdf44d48"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bf1c2fe6a734552"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27507,7 +27507,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bcb49d128a34f23"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbec54b2403354202"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29160,7 +29160,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb12fc9a145a54bcc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a2caa9c6b2f4583"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Complete shared borrower cleanup and address reconciliation
</commit_message>
<xml_diff>
--- a/Documents/AppSheet_Data_Dictionary.xlsx
+++ b/Documents/AppSheet_Data_Dictionary.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R9651d12c89b948fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="Rbf63829385f54798"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="Rabbefa11283742cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R766e019bb4a74dd2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="R725af707c5154085"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R6bff1397ce6e46a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Raeaba5653582496c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R5628ca0a872f4855"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="Rdf6bc609c39d470a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R8f2e8b19e06740e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="Re2fc66bc4b9045ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="Rbc75ea26b2d241d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rb9853f0907c541e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="Rc818e69beb2a4e35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R5e6079b1c2934bbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R4bebfdc085464e4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="Rfc856e925703480f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R7c83090d20924339"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="R114839d9779d4251"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R98ba3e208b9a45e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="R84a3dc1cfc4b409b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R54931ad81cbb4447"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="Rf9ef1b83482c4b54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="Rd158215a355f46b5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -722,8 +722,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="DataModelColumns" displayName="DataModelColumns" ref="A4:H398" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:H398"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="DataModelColumns" displayName="DataModelColumns" ref="A4:H399" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:H399"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Table"/>
     <x:tableColumn id="2" name="Inventory order"/>
@@ -769,7 +769,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="DataModelSliceColumns" displayName="DataModelSliceColumns" ref="A4:D492" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="DataModelSliceColumns" displayName="DataModelSliceColumns" ref="A4:D498" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="App"/>
     <x:tableColumn id="2" name="Slice"/>
@@ -781,8 +781,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="DataModelAppVariances" displayName="DataModelAppVariances" ref="A4:F232" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:F232"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="DataModelAppVariances" displayName="DataModelAppVariances" ref="A4:F233" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:F233"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Object Type"/>
     <x:tableColumn id="2" name="Table"/>
@@ -1079,7 +1079,7 @@
         <x:v>Reconciliation status</x:v>
       </x:c>
       <x:c r="B5" s="85" t="str">
-        <x:v>Borrower cleanup PARTIAL: five OLTP settings saved; Chrome control failed before final version/readback. OLAP remains prior configuration. See authoritative borrower cleanup change log.</x:v>
+        <x:v>Borrower cleanup verified: OLTP 3.000064; OLAP 1.100041. New-GUI form/detail checks passed; owner acceptance pending. Retired inventory is explicitly labeled.</x:v>
       </x:c>
       <x:c r="C5" s="73"/>
       <x:c r="D5" s="73"/>
@@ -1091,7 +1091,7 @@
         <x:v>Live baselines</x:v>
       </x:c>
       <x:c r="B6" s="85" t="str">
-        <x:v>Language enum rollback: OLTP 3.000050; OLAP 1.100031. Earlier setup rollback: OLTP 3.000045; OLAP 1.100028. App restoration does not restore database data/schema. Owner acceptance pending.</x:v>
+        <x:v>Cleanup rollback OLTP 3.000052 / OLAP 1.100033; native database copy Money BACKUP Borrower Cleanup 20260913. Restore schema/data separately and preserve intervening edits.</x:v>
       </x:c>
       <x:c r="C6" s="73"/>
       <x:c r="D6" s="73"/>
@@ -2492,7 +2492,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf31271142f442b5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79a4e735b1af4cdc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3907,7 +3907,7 @@
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>13 September 2026: language enum updated in OLTP 3.000052 and OLAP 1.100033; table counts unchanged. Other tables retain dated verification scope.</x:v>
+        <x:v>13 September 2026: Borrowers cleanup complete in both apps; stored counts include ordinal/key. Two collection tables retired.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
@@ -3958,16 +3958,16 @@
         <x:v>OLTP + OLAP</x:v>
       </x:c>
       <x:c r="D5" s="56" t="n">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E5" s="56" t="n">
-        <x:v>29</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="F5" s="56" t="n">
         <x:v>65</x:v>
       </x:c>
       <x:c r="G5" s="58" t="str">
-        <x:v>OLTP 45 =16 stored +29 VCs; OLAP 81 =16 stored +65 VCs. OLAP read-only, new location fields loaded. Counts include ordinal/key.</x:v>
+        <x:v>OLTP 38 =12 stored +26 VCs; OLAP 77 =12 stored +65 VCs. Address loaded; obsolete fields removed. OLAP read-only.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" customHeight="1">
@@ -4254,19 +4254,19 @@
         <x:v>Money database</x:v>
       </x:c>
       <x:c r="C18" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired — neither app</x:v>
       </x:c>
       <x:c r="D18" s="87" t="n">
-        <x:v>7</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E18" s="87" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="F18" s="87" t="str">
-        <x:v>Not configured by this build</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F18" s="87" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G18" s="87" t="str">
-        <x:v>Receiving-account master; add/update only in OLTP. Deactivate used accounts. Two user-authorized records; no details in this dictionary.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" customHeight="1">
@@ -4277,19 +4277,19 @@
         <x:v>Money database</x:v>
       </x:c>
       <x:c r="C19" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired — neither app</x:v>
       </x:c>
       <x:c r="D19" s="87" t="n">
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E19" s="87" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F19" s="87" t="str">
-        <x:v>Not configured by this build</x:v>
+      <x:c r="F19" s="87" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G19" s="87" t="str">
-        <x:v>One shared default receiving-account selection. Update only; no adds/deletes in OLTP.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4299,7 +4299,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5dd9cb54c937408e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40613c357604443c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4332,7 +4332,7 @@
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>13 September 2026: borrower cleanup PARTIAL. Five OLTP settings saved; post-save readback and OLAP reconciliation pending. All other inventory retains prior verification scope.</x:v>
+        <x:v>13 September 2026: borrower cleanup reconciled in OLTP 3.000064 and OLAP 1.100041. Retired rows are historical, not active schema.</x:v>
       </x:c>
       <x:c r="B2"/>
       <x:c r="C2"/>
@@ -4453,7 +4453,7 @@
         <x:v>Stores the authoritative source value for Borrower Name.</x:v>
       </x:c>
       <x:c r="H7" s="82" t="str">
-        <x:v>Internal name preserved. OLTP display changed to Borrower Name - Thai. OLAP display reconciliation pending. Final readback/tests pending.</x:v>
+        <x:v>Internal Borrower Name retained; display Borrower Name - Thai in both apps.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" customHeight="1">
@@ -4470,16 +4470,16 @@
         <x:v>Physical / Phone</x:v>
       </x:c>
       <x:c r="E8" s="57" t="str">
-        <x:v>OLTP + OLAP</x:v>
+        <x:v>Retired — neither app</x:v>
       </x:c>
       <x:c r="F8" s="57" t="str">
-        <x:v>PII</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="G8" s="59" t="str">
-        <x:v>Stores the authoritative source value for Telephone.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
       <x:c r="H8" s="59" t="str">
-        <x:v>Stored source column</x:v>
+        <x:v>Historical definition retired; see cleanup change log for rollback.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
@@ -4505,7 +4505,7 @@
         <x:v>Text confirmed in both apps during partner/location setup reconciliation.</x:v>
       </x:c>
       <x:c r="H9" s="82" t="str">
-        <x:v>Internal Description preserved. OLTP display changed to English Name. OLAP and Partner Operations GUI label reconciliation pending. Final readback/tests pending.</x:v>
+        <x:v>Internal Description retained; display English Name in both apps. Existing formulas/API keys preserved.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" customHeight="1">
@@ -14182,13 +14182,13 @@
         <x:v>OLTP + OLAP</x:v>
       </x:c>
       <x:c r="F370" s="87" t="str">
-        <x:v>OLTP required; OLAP prior optional, table read-only. Pending final reconciliation.</x:v>
+        <x:v>Required; OLTP editable, OLAP table read-only</x:v>
       </x:c>
       <x:c r="G370" s="87" t="str">
-        <x:v>Explicit message address; no suffix stripping. App physical position 8.</x:v>
+        <x:v>Explicit communication name; required. Stored position 7 in both apps.</x:v>
       </x:c>
       <x:c r="H370" s="88" t="str">
-        <x:v>OLTP Require enabled. OLAP reconciliation pending. Blank initial value retained. Final readback/tests pending.</x:v>
+        <x:v>Required in both apps. OLTP editable; OLAP table remains read-only. Blank initial value.</x:v>
       </x:c>
     </x:row>
     <x:row r="371" ht="78" customHeight="1">
@@ -14231,16 +14231,16 @@
         <x:v>Physical / Url (OLTP); Text (OLAP)</x:v>
       </x:c>
       <x:c r="E372" s="87" t="str">
-        <x:v>OLTP + OLAP</x:v>
+        <x:v>Retired — neither app</x:v>
       </x:c>
       <x:c r="F372" s="87" t="str">
-        <x:v>OLTP editable; OLAP table read-only; shown, optional, searchable</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="G372" s="87" t="str">
-        <x:v>Verified conversation link; native Text, app Url; position 10.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
       <x:c r="H372" s="87" t="str">
-        <x:v>Stored native Text; OLTP Url, OLAP Text. Both initial values blank; existing app type variance preserved.</x:v>
+        <x:v>Historical definition retired; see cleanup change log for rollback.</x:v>
       </x:c>
     </x:row>
     <x:row r="373" ht="78" customHeight="1">
@@ -14257,16 +14257,16 @@
         <x:v>Physical / DateTime</x:v>
       </x:c>
       <x:c r="E373" s="87" t="str">
-        <x:v>OLTP + OLAP</x:v>
+        <x:v>Retired — neither app</x:v>
       </x:c>
       <x:c r="F373" s="87" t="str">
-        <x:v>OLTP editable; OLAP table read-only; shown, optional, searchable</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="G373" s="87" t="str">
-        <x:v>Time mapping was actually checked; position 11.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
       <x:c r="H373" s="87" t="str">
-        <x:v>Stored; blank initial value in both apps. OLAP inherited NOW() removed during 13 September reconciliation. Existing values unchanged.</x:v>
+        <x:v>Historical definition retired; see cleanup change log for rollback.</x:v>
       </x:c>
     </x:row>
     <x:row r="374" ht="78" customHeight="1">
@@ -14292,7 +14292,7 @@
         <x:v>Existing borrower opt-in; also required alongside Collection dashboard eligibility for the proposed partner daily briefing. Existing flag values unchanged.</x:v>
       </x:c>
       <x:c r="H374" s="88" t="str">
-        <x:v>OLTP initial changed to TRUE for new rows. Existing row values untouched. OLAP reconciliation pending. Final readback/tests pending.</x:v>
+        <x:v>Initial TRUE in both apps for new rows only. Existing row values not edited by cleanup.</x:v>
       </x:c>
     </x:row>
     <x:row r="375" ht="78" customHeight="1">
@@ -14309,16 +14309,16 @@
         <x:v>Physical / Yes/No</x:v>
       </x:c>
       <x:c r="E375" s="87" t="str">
-        <x:v>OLTP + OLAP</x:v>
+        <x:v>Retired — neither app</x:v>
       </x:c>
       <x:c r="F375" s="87" t="str">
-        <x:v>OLTP editable; OLAP table read-only; shown, optional, searchable</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="G375" s="87" t="str">
-        <x:v>Independent penalty eligibility; position 13. Existing fees never reversed by this flag.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
       <x:c r="H375" s="87" t="str">
-        <x:v>Stored; initial FALSE in both apps. Existing values and collection runtime unchanged.</x:v>
+        <x:v>Historical definition retired; see cleanup change log for rollback.</x:v>
       </x:c>
     </x:row>
     <x:row r="376" ht="78" customHeight="1">
@@ -14335,16 +14335,16 @@
         <x:v>Physical / Ref</x:v>
       </x:c>
       <x:c r="E376" s="87" t="str">
-        <x:v>OLTP + OLAP</x:v>
+        <x:v>Retired — neither app</x:v>
       </x:c>
       <x:c r="F376" s="87" t="str">
-        <x:v>OLTP editable; OLAP table read-only; shown, optional, searchable</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="G376" s="87" t="str">
-        <x:v>Borrower-specific receiving bank; position 14.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
       <x:c r="H376" s="87" t="str">
-        <x:v>Stored native Reference and app Ref -&gt; Collection Bank Accounts; independent lifecycle</x:v>
+        <x:v>Historical definition retired; see cleanup change log for rollback.</x:v>
       </x:c>
     </x:row>
     <x:row r="377" ht="15" customHeight="1">
@@ -14361,16 +14361,16 @@
         <x:v>Virtual / Ref</x:v>
       </x:c>
       <x:c r="E377" s="87" t="str">
-        <x:v>OLTP only</x:v>
+        <x:v>Retired — neither app</x:v>
       </x:c>
       <x:c r="F377" s="87" t="str">
-        <x:v>Read-only</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="G377" s="87" t="str">
-        <x:v>Borrower override, otherwise singleton default; Ref -&gt; Collection Bank Accounts.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
       <x:c r="H377" s="87" t="str">
-        <x:v>IF(ISNOTBLANK([Receiving Bank Account]), [Receiving Bank Account], IF(COUNT(Collection Settings[Row ID]) = 1, ANY(Collection Settings[Default Receiving Bank Account]), ""))</x:v>
+        <x:v>Historical definition retired; see cleanup change log for rollback.</x:v>
       </x:c>
     </x:row>
     <x:row r="378" ht="15" customHeight="1">
@@ -14387,16 +14387,16 @@
         <x:v>Virtual / Text</x:v>
       </x:c>
       <x:c r="E378" s="87" t="str">
-        <x:v>OLTP only</x:v>
+        <x:v>Retired — neither app</x:v>
       </x:c>
       <x:c r="F378" s="87" t="str">
-        <x:v>Read-only</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="G378" s="87" t="str">
-        <x:v>Enabled borrower name, Instagram mapping/duplicate and effective-bank checks.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
       <x:c r="H378" s="87" t="str">
-        <x:v>IF([AI Collection Enabled], CONCATENATE(IF(ISBLANK(TRIM([Communication Name])), "Enter communication name. ", ""), IF(ISBLANK([Instagram Username]), "Enter Instagram username. ", IF(OR(CONTAINS([Instagram Username], "@"), CONTAINS([Instagram Username], " "), CONTAINS([Instagram Username], "/")), "Use username only, without @, spaces or URL. ", "")), IF(AND(ISNOTBLANK([Instagram Username]), COUNT(SELECT(Borrowers[Row ID], AND(LOWER([Instagram Username]) = LOWER([_THISROW].[Instagram Username]), [Row ID] &lt;&gt; [_THISROW].[Row ID]))) &gt; 0), "Instagram username is mapped to another borrower. ", ""), IF(NOT(STARTSWITH([Instagram Conversation URL], "https://www.instagram.com/direct/t/")), "Enter verified Instagram conversation URL. ", ""), IF(ISBLANK([Instagram Verified At]), "Verify Instagram mapping. ", ""), IF(ISBLANK([Effective Receiving Bank Account]), "Select borrower bank or one shared default. ", IF(NOT([Effective Receiving Bank Account].[Active]), "Receiving bank account is inactive. ", IF(OR(ISBLANK([Effective Receiving Bank Account].[Bank Name]), ISBLANK([Effective Receiving Bank Account].[Account Number]), ISBLANK([Effective Receiving Bank Account].[Account Holder Name])), "Complete receiving bank details. ", "")))), "")</x:v>
+        <x:v>Historical definition retired; see cleanup change log for rollback.</x:v>
       </x:c>
     </x:row>
     <x:row r="379" ht="15" customHeight="1">
@@ -14413,16 +14413,16 @@
         <x:v>Physical / Number</x:v>
       </x:c>
       <x:c r="E379" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired — neither app</x:v>
       </x:c>
       <x:c r="F379" s="87" t="str">
-        <x:v>Hidden</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="G379" s="87" t="str">
-        <x:v>Source ordinal, never identity.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
       <x:c r="H379" s="87" t="str">
-        <x:v>Stored system column</x:v>
+        <x:v>Historical definition retired; see cleanup change log for rollback.</x:v>
       </x:c>
     </x:row>
     <x:row r="380" ht="15" customHeight="1">
@@ -14439,16 +14439,16 @@
         <x:v>Physical / Text</x:v>
       </x:c>
       <x:c r="E380" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired — neither app</x:v>
       </x:c>
       <x:c r="F380" s="87" t="str">
-        <x:v>Key, Required, Hidden</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="G380" s="87" t="str">
-        <x:v>Immutable native key.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
       <x:c r="H380" s="87" t="str">
-        <x:v>Stored; initial value UNIQUEID("PackedUUID")</x:v>
+        <x:v>Historical definition retired; see cleanup change log for rollback.</x:v>
       </x:c>
     </x:row>
     <x:row r="381" ht="15" customHeight="1">
@@ -14465,16 +14465,16 @@
         <x:v>Physical / Text</x:v>
       </x:c>
       <x:c r="E381" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired — neither app</x:v>
       </x:c>
       <x:c r="F381" s="87" t="str">
-        <x:v>Label, Required, Editable</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="G381" s="87" t="str">
-        <x:v>Recognizable receiving-account label.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
       <x:c r="H381" s="87" t="str">
-        <x:v>Stored</x:v>
+        <x:v>Historical definition retired; see cleanup change log for rollback.</x:v>
       </x:c>
     </x:row>
     <x:row r="382" ht="15" customHeight="1">
@@ -14491,16 +14491,16 @@
         <x:v>Physical / Text</x:v>
       </x:c>
       <x:c r="E382" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired — neither app</x:v>
       </x:c>
       <x:c r="F382" s="87" t="str">
-        <x:v>Required, Editable</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="G382" s="87" t="str">
-        <x:v>Bank shown in messages.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
       <x:c r="H382" s="87" t="str">
-        <x:v>Stored</x:v>
+        <x:v>Historical definition retired; see cleanup change log for rollback.</x:v>
       </x:c>
     </x:row>
     <x:row r="383" ht="15" customHeight="1">
@@ -14517,16 +14517,16 @@
         <x:v>Physical / Text</x:v>
       </x:c>
       <x:c r="E383" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired — neither app</x:v>
       </x:c>
       <x:c r="F383" s="87" t="str">
-        <x:v>Required, Editable</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="G383" s="87" t="str">
-        <x:v>Preserve leading zeros and supplied separators.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
       <x:c r="H383" s="87" t="str">
-        <x:v>Stored</x:v>
+        <x:v>Historical definition retired; see cleanup change log for rollback.</x:v>
       </x:c>
     </x:row>
     <x:row r="384" ht="15" customHeight="1">
@@ -14543,16 +14543,16 @@
         <x:v>Physical / Text</x:v>
       </x:c>
       <x:c r="E384" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired — neither app</x:v>
       </x:c>
       <x:c r="F384" s="87" t="str">
-        <x:v>Required, Editable</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="G384" s="87" t="str">
-        <x:v>Receiving account holder.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
       <x:c r="H384" s="87" t="str">
-        <x:v>Stored</x:v>
+        <x:v>Historical definition retired; see cleanup change log for rollback.</x:v>
       </x:c>
     </x:row>
     <x:row r="385" ht="15" customHeight="1">
@@ -14569,16 +14569,16 @@
         <x:v>Physical / Yes/No</x:v>
       </x:c>
       <x:c r="E385" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired — neither app</x:v>
       </x:c>
       <x:c r="F385" s="87" t="str">
-        <x:v>Editable</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="G385" s="87" t="str">
-        <x:v>Deactivate instead of deleting used accounts.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
       <x:c r="H385" s="87" t="str">
-        <x:v>Stored; initial value TRUE</x:v>
+        <x:v>Historical definition retired; see cleanup change log for rollback.</x:v>
       </x:c>
     </x:row>
     <x:row r="386" ht="15" customHeight="1">
@@ -14595,16 +14595,16 @@
         <x:v>Virtual / List (Ref)</x:v>
       </x:c>
       <x:c r="E386" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired — neither app</x:v>
       </x:c>
       <x:c r="F386" s="87" t="str">
-        <x:v>Read-only</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="G386" s="87" t="str">
-        <x:v>Default-setting reverse reference.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
       <x:c r="H386" s="87" t="str">
-        <x:v>REF_ROWS("Collection Settings", "Default Receiving Bank Account")</x:v>
+        <x:v>Historical definition retired; see cleanup change log for rollback.</x:v>
       </x:c>
     </x:row>
     <x:row r="387" ht="15" customHeight="1">
@@ -14621,16 +14621,16 @@
         <x:v>Virtual / List (Ref)</x:v>
       </x:c>
       <x:c r="E387" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired — neither app</x:v>
       </x:c>
       <x:c r="F387" s="87" t="str">
-        <x:v>Read-only</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="G387" s="87" t="str">
-        <x:v>Borrower override reverse reference.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
       <x:c r="H387" s="87" t="str">
-        <x:v>REF_ROWS("Borrowers", "Receiving Bank Account")</x:v>
+        <x:v>Historical definition retired; see cleanup change log for rollback.</x:v>
       </x:c>
     </x:row>
     <x:row r="388" ht="30" customHeight="1">
@@ -14647,16 +14647,16 @@
         <x:v>Virtual / List (Ref)</x:v>
       </x:c>
       <x:c r="E388" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired — neither app</x:v>
       </x:c>
       <x:c r="F388" s="87" t="str">
-        <x:v>Read-only</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="G388" s="87" t="str">
-        <x:v>Includes borrowers inheriting the shared default.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
       <x:c r="H388" s="87" t="str">
-        <x:v>REF_ROWS("Borrowers", "Effective Receiving Bank Account")</x:v>
+        <x:v>Historical definition retired; see cleanup change log for rollback.</x:v>
       </x:c>
     </x:row>
     <x:row r="389" ht="15" customHeight="1">
@@ -14673,16 +14673,16 @@
         <x:v>Physical / Number</x:v>
       </x:c>
       <x:c r="E389" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired — neither app</x:v>
       </x:c>
       <x:c r="F389" s="87" t="str">
-        <x:v>Hidden</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="G389" s="87" t="str">
-        <x:v>Source ordinal, never identity.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
       <x:c r="H389" s="87" t="str">
-        <x:v>Stored system column</x:v>
+        <x:v>Historical definition retired; see cleanup change log for rollback.</x:v>
       </x:c>
     </x:row>
     <x:row r="390" ht="15" customHeight="1">
@@ -14699,16 +14699,16 @@
         <x:v>Physical / Text</x:v>
       </x:c>
       <x:c r="E390" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired — neither app</x:v>
       </x:c>
       <x:c r="F390" s="87" t="str">
-        <x:v>Key, Required, Hidden</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="G390" s="87" t="str">
-        <x:v>Immutable native key.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
       <x:c r="H390" s="87" t="str">
-        <x:v>Stored; initial value UNIQUEID("PackedUUID")</x:v>
+        <x:v>Historical definition retired; see cleanup change log for rollback.</x:v>
       </x:c>
     </x:row>
     <x:row r="391" ht="15" customHeight="1">
@@ -14725,16 +14725,16 @@
         <x:v>Physical / Text</x:v>
       </x:c>
       <x:c r="E391" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired — neither app</x:v>
       </x:c>
       <x:c r="F391" s="87" t="str">
-        <x:v>Label, Not editable</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="G391" s="87" t="str">
-        <x:v>Singleton setting label; one shared row.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
       <x:c r="H391" s="87" t="str">
-        <x:v>Stored</x:v>
+        <x:v>Historical definition retired; see cleanup change log for rollback.</x:v>
       </x:c>
     </x:row>
     <x:row r="392" ht="15" customHeight="1">
@@ -14751,16 +14751,16 @@
         <x:v>Physical / Ref</x:v>
       </x:c>
       <x:c r="E392" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired — neither app</x:v>
       </x:c>
       <x:c r="F392" s="87" t="str">
-        <x:v>Required, Editable</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="G392" s="87" t="str">
-        <x:v>Shared default for borrowers without override.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
       <x:c r="H392" s="87" t="str">
-        <x:v>Stored native Reference and app Ref -&gt; Collection Bank Accounts; independent lifecycle</x:v>
+        <x:v>Historical definition retired; see cleanup change log for rollback.</x:v>
       </x:c>
     </x:row>
     <x:row r="393" ht="135" customHeight="1">
@@ -14884,13 +14884,13 @@
         <x:v>OLTP + OLAP</x:v>
       </x:c>
       <x:c r="F397" s="73" t="str">
-        <x:v>OLTP required; OLAP prior optional, table read-only. Pending final reconciliation.</x:v>
+        <x:v>Required; OLTP editable, OLAP table read-only</x:v>
       </x:c>
       <x:c r="G397" s="73" t="str">
-        <x:v>Borrower city from the owner location sheet. App position 15.</x:v>
+        <x:v>Borrower city from owner location sheet. Stored position 10 in both apps.</x:v>
       </x:c>
       <x:c r="H397" s="73" t="str">
-        <x:v>OLTP Require enabled; display เมือง / City and blank initial retained. OLAP reconciliation pending. Final readback/tests pending.</x:v>
+        <x:v>Required in both apps. Blank initial value; display เมือง / City. Existing values preserved.</x:v>
       </x:c>
     </x:row>
     <x:row r="398" ht="78" customHeight="1">
@@ -14913,10 +14913,36 @@
         <x:v>OLTP editable; OLAP table read-only; shown, optional, searchable</x:v>
       </x:c>
       <x:c r="G398" s="73" t="str">
-        <x:v>Workplace/locality from the owner location sheet. App position 16.</x:v>
+        <x:v>Workplace/locality from owner location sheet. Stored position 11 in both apps.</x:v>
       </x:c>
       <x:c r="H398" s="73" t="str">
         <x:v>Stored; blank initial value; display name: "สถานที่ทำงาน / Working Location". Uncertainty preserved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="399" ht="78" customHeight="1">
+      <x:c r="A399" s="73" t="str">
+        <x:v>Borrowers</x:v>
+      </x:c>
+      <x:c r="B399" s="73" t="n">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="C399" s="73" t="str">
+        <x:v>Address</x:v>
+      </x:c>
+      <x:c r="D399" s="73" t="str">
+        <x:v>Physical / Text</x:v>
+      </x:c>
+      <x:c r="E399" s="73" t="str">
+        <x:v>OLTP + OLAP</x:v>
+      </x:c>
+      <x:c r="F399" s="73" t="str">
+        <x:v>Optional; OLTP editable, OLAP table read-only</x:v>
+      </x:c>
+      <x:c r="G399" s="73" t="str">
+        <x:v>Borrower address from owner location sheet; seven exact-name matches imported.</x:v>
+      </x:c>
+      <x:c r="H399" s="73" t="str">
+        <x:v>Blank initial; no formula. Included in both apps borrower views and affected slices.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14930,7 +14956,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbefa88207b7e4147"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb09b089999644e46"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15303,7 +15329,7 @@
     </x:row>
     <x:row r="19" ht="15" customHeight="1">
       <x:c r="A19" s="87" t="str">
-        <x:v>Borrowers</x:v>
+        <x:v>Retired — Borrowers</x:v>
       </x:c>
       <x:c r="B19" s="87" t="str">
         <x:v>Receiving Bank Account</x:v>
@@ -15320,7 +15346,7 @@
     </x:row>
     <x:row r="20" ht="15" customHeight="1">
       <x:c r="A20" s="87" t="str">
-        <x:v>Borrowers</x:v>
+        <x:v>Retired — Borrowers</x:v>
       </x:c>
       <x:c r="B20" s="87" t="str">
         <x:v>Effective Receiving Bank Account</x:v>
@@ -15337,7 +15363,7 @@
     </x:row>
     <x:row r="21" ht="15" customHeight="1">
       <x:c r="A21" s="87" t="str">
-        <x:v>Collection Settings</x:v>
+        <x:v>Retired — Collection Settings</x:v>
       </x:c>
       <x:c r="B21" s="87" t="str">
         <x:v>Default Receiving Bank Account</x:v>
@@ -15359,7 +15385,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71c01aec0b6d4a7a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c64ae7a7f954995"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15455,13 +15481,13 @@
         <x:v>Read-only</x:v>
       </x:c>
       <x:c r="F5" s="83" t="n">
-        <x:v>21</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G5" s="83" t="str">
         <x:v>Existing daily collection population. Future agent additionally requires due/overdue and AI Collection Enabled; dashboard filter unchanged.</x:v>
       </x:c>
       <x:c r="H5" s="83" t="str">
-        <x:v>OLTP 3.000050; location columns included after regeneration. Existing row filter and update mode retained.</x:v>
+        <x:v>Cleanup reconciled. Address included; filters and permissions preserved.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="55" customHeight="1">
@@ -15481,13 +15507,13 @@
         <x:v>Adds, Updates, Deletes</x:v>
       </x:c>
       <x:c r="F6" s="83" t="n">
-        <x:v>45</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="G6" s="83" t="str">
         <x:v>Primary borrower list; City and Working Location exposed in existing form/detail views.</x:v>
       </x:c>
       <x:c r="H6" s="83" t="str">
-        <x:v>OLTP 3.000050; location columns included after regeneration. Existing row filter and update mode retained.</x:v>
+        <x:v>Cleanup reconciled. Address included; filters and permissions preserved.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="96" customHeight="1">
@@ -15513,7 +15539,7 @@
         <x:v>Read-only OLAP subset of borrowers whose outstanding principal is greater than zero.</x:v>
       </x:c>
       <x:c r="H7" s="59" t="str">
-        <x:v>OLAP 1.100031: exact membership reconciled; City and Working Location appended. Existing filter, actions and read-only mode retained. Earlier membership gaps corrected in inventory.</x:v>
+        <x:v>Cleanup reconciled. Address included; filters and permissions preserved.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="96" customHeight="1">
@@ -15539,7 +15565,7 @@
         <x:v>Read-only OLAP subset of borrowers contributing positive interest profit in the last 30 days.</x:v>
       </x:c>
       <x:c r="H8" s="59" t="str">
-        <x:v>OLAP 1.100031: exact membership reconciled; City and Working Location appended. Existing filter, actions and read-only mode retained. Earlier membership gaps corrected in inventory.</x:v>
+        <x:v>Cleanup reconciled. Address included; filters and permissions preserved.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="96" customHeight="1">
@@ -15559,13 +15585,13 @@
         <x:v>Read-only</x:v>
       </x:c>
       <x:c r="F9" s="57" t="n">
-        <x:v>56</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="G9" s="59" t="str">
         <x:v>Curated, read-only borrower feed for downstream reporting and dashboard reconciliation, including the borrower value/stability matrix fields.</x:v>
       </x:c>
       <x:c r="H9" s="59" t="str">
-        <x:v>OLAP 1.100031: exact membership reconciled; City and Working Location appended. Existing filter, actions and read-only mode retained. Earlier membership gaps corrected in inventory.</x:v>
+        <x:v>Cleanup reconciled. Address included; filters and permissions preserved.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" customHeight="1">
@@ -15777,18 +15803,18 @@
         <x:v>Read-only</x:v>
       </x:c>
       <x:c r="F18" s="72" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G18" s="72" t="str">
         <x:v>Read-only daily collection export and message-review slice using OLAP-native current-status, amount, charge-list, hidden-flag, and overdue fields.</x:v>
       </x:c>
       <x:c r="H18" s="72" t="str">
-        <x:v>OLAP 1.100031: exact membership reconciled; City and Working Location appended. Existing filter, actions and read-only mode retained. Earlier membership gaps corrected in inventory.</x:v>
+        <x:v>Cleanup reconciled. Address included; filters and permissions preserved.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" customHeight="1">
       <x:c r="A19" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B19" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -15797,19 +15823,19 @@
         <x:v>Borrowers</x:v>
       </x:c>
       <x:c r="D19" s="87" t="str">
-        <x:v>AND([AI Collection Enabled], ISNOTBLANK([Collection Setup Issues]))</x:v>
+        <x:v>Not active</x:v>
       </x:c>
       <x:c r="E19" s="87" t="str">
-        <x:v>Updates only</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="F19" s="87" t="n">
-        <x:v>45</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G19" s="87" t="str">
-        <x:v>Enabled borrowers needing name, Instagram or receiving-bank setup.</x:v>
+        <x:v>Historical setup-review slice</x:v>
       </x:c>
       <x:c r="H19" s="87" t="str">
-        <x:v>OLTP 3.000050; location columns included after regeneration. Existing row filter and update mode retained.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -15819,7 +15845,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R742f04d9bb684197"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ba644b5b14846d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15914,7 +15940,7 @@
     </x:row>
     <x:row r="8" ht="15" customHeight="1">
       <x:c r="A8" s="57" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B8" s="59" t="str">
         <x:v>Visible Borrowers</x:v>
@@ -15934,7 +15960,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C9" s="57" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D9" s="59" t="str">
         <x:v>Description</x:v>
@@ -15948,7 +15974,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C10" s="57" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D10" s="59" t="str">
         <x:v>Creation Date</x:v>
@@ -15962,7 +15988,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C11" s="57" t="n">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D11" s="59" t="str">
         <x:v>Hidden Flag</x:v>
@@ -15976,7 +16002,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C12" s="57" t="n">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D12" s="59" t="str">
         <x:v>Related Loans</x:v>
@@ -15990,7 +16016,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C13" s="57" t="n">
-        <x:v>9</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D13" s="59" t="str">
         <x:v>Total Interest Earned</x:v>
@@ -16004,7 +16030,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C14" s="57" t="n">
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D14" s="59" t="str">
         <x:v>Total Amount Loaned</x:v>
@@ -16018,7 +16044,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C15" s="57" t="n">
-        <x:v>11</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D15" s="59" t="str">
         <x:v>Total Number of Loans</x:v>
@@ -16032,7 +16058,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C16" s="57" t="n">
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D16" s="59" t="str">
         <x:v>Total Outstanding Principal</x:v>
@@ -16046,7 +16072,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C17" s="57" t="n">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D17" s="59" t="str">
         <x:v>Header - Active Loans</x:v>
@@ -16060,7 +16086,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C18" s="57" t="n">
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D18" s="59" t="str">
         <x:v>Borrower Name TE</x:v>
@@ -16074,7 +16100,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C19" s="57" t="n">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D19" s="59" t="str">
         <x:v>Return on Active Principal</x:v>
@@ -16088,7 +16114,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C20" s="57" t="n">
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D20" s="59" t="str">
         <x:v>Active Loan Interest Earned</x:v>
@@ -16102,7 +16128,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C21" s="57" t="n">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D21" s="59" t="str">
         <x:v>Active Daily Interest</x:v>
@@ -16116,7 +16142,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C22" s="57" t="n">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D22" s="59" t="str">
         <x:v>Projected Interest Coverage Date</x:v>
@@ -16130,7 +16156,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C23" s="57" t="n">
-        <x:v>19</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D23" s="59" t="str">
         <x:v>Closed Loan Interest Earned</x:v>
@@ -16144,7 +16170,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C24" s="57" t="n">
-        <x:v>20</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D24" s="59" t="str">
         <x:v>Closed Loan Principle</x:v>
@@ -16158,7 +16184,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C25" s="57" t="n">
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D25" s="59" t="str">
         <x:v>Has Closed Loan</x:v>
@@ -16172,7 +16198,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C26" s="57" t="n">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D26" s="59" t="str">
         <x:v>Return on Closed Loans</x:v>
@@ -16186,7 +16212,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C27" s="57" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D27" s="59" t="str">
         <x:v>Header - Closed Loans</x:v>
@@ -16200,7 +16226,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C28" s="57" t="n">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D28" s="59" t="str">
         <x:v>Has Active Loan</x:v>
@@ -16214,7 +16240,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C29" s="57" t="n">
-        <x:v>25</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D29" s="59" t="str">
         <x:v>Daily Collection Status</x:v>
@@ -16228,7 +16254,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C30" s="57" t="n">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D30" s="59" t="str">
         <x:v>Todays Collection Charges</x:v>
@@ -16242,7 +16268,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C31" s="57" t="n">
-        <x:v>27</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="D31" s="59" t="str">
         <x:v>Todays Amount Due</x:v>
@@ -16256,7 +16282,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C32" s="57" t="n">
-        <x:v>28</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D32" s="59" t="str">
         <x:v>Todays Amount Collected</x:v>
@@ -16270,7 +16296,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C33" s="57" t="n">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="D33" s="59" t="str">
         <x:v>Todays Amount Remaining</x:v>
@@ -16284,7 +16310,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C34" s="57" t="n">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="D34" s="59" t="str">
         <x:v>Daily Collection Status - Order</x:v>
@@ -16298,7 +16324,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C35" s="57" t="n">
-        <x:v>31</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D35" s="59" t="str">
         <x:v>Borrower Name - Collection</x:v>
@@ -16312,7 +16338,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C36" s="57" t="n">
-        <x:v>32</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D36" s="59" t="str">
         <x:v>Active Profit After Principal Coverage</x:v>
@@ -16326,7 +16352,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C37" s="57" t="n">
-        <x:v>33</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="D37" s="59" t="str">
         <x:v>Related Payments</x:v>
@@ -16544,7 +16570,7 @@
     </x:row>
     <x:row r="53" ht="15" customHeight="1">
       <x:c r="A53" s="57" t="str">
-        <x:v>OLAP</x:v>
+        <x:v>Retired OLAP</x:v>
       </x:c>
       <x:c r="B53" s="59" t="str">
         <x:v>Borrowers with Outstanding Loans</x:v>
@@ -16564,7 +16590,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C54" s="57" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D54" s="59" t="str">
         <x:v>Description</x:v>
@@ -16578,7 +16604,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C55" s="57" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D55" s="59" t="str">
         <x:v>Creation Date</x:v>
@@ -16592,7 +16618,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C56" s="57" t="n">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D56" s="59" t="str">
         <x:v>Related Loans</x:v>
@@ -16606,7 +16632,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C57" s="57" t="n">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D57" s="59" t="str">
         <x:v>Total Interest Earned</x:v>
@@ -16620,7 +16646,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C58" s="57" t="n">
-        <x:v>9</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D58" s="59" t="str">
         <x:v>Total Amount Loaned</x:v>
@@ -16634,7 +16660,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C59" s="57" t="n">
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D59" s="59" t="str">
         <x:v>Total Number of Loans</x:v>
@@ -16648,7 +16674,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C60" s="57" t="n">
-        <x:v>11</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D60" s="59" t="str">
         <x:v>Total Outstanding Principal</x:v>
@@ -16662,7 +16688,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C61" s="57" t="n">
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D61" s="59" t="str">
         <x:v>Header - Active Loans</x:v>
@@ -16676,7 +16702,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C62" s="57" t="n">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D62" s="59" t="str">
         <x:v>Borrower Name TE</x:v>
@@ -16690,7 +16716,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C63" s="57" t="n">
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D63" s="59" t="str">
         <x:v>Return on Active Principal</x:v>
@@ -16704,7 +16730,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C64" s="57" t="n">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D64" s="59" t="str">
         <x:v>Profit Last 30 Days</x:v>
@@ -16718,7 +16744,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C65" s="57" t="n">
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D65" s="59" t="str">
         <x:v>Projected Interest Coverage Date</x:v>
@@ -16732,7 +16758,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C66" s="57" t="n">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D66" s="59" t="str">
         <x:v>Active Loan Interest Earned</x:v>
@@ -16746,7 +16772,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C67" s="57" t="n">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D67" s="59" t="str">
         <x:v>Active Daily Interest</x:v>
@@ -16760,7 +16786,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C68" s="57" t="n">
-        <x:v>19</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D68" s="59" t="str">
         <x:v>Related Loan Assessments</x:v>
@@ -16774,7 +16800,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C69" s="57" t="n">
-        <x:v>20</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D69" s="59" t="str">
         <x:v>Related Calendars</x:v>
@@ -16788,7 +16814,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C70" s="57" t="n">
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D70" s="59" t="str">
         <x:v>Closed Loan Interest Earned</x:v>
@@ -16802,7 +16828,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C71" s="57" t="n">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D71" s="59" t="str">
         <x:v>Closed Loan Principle</x:v>
@@ -16816,7 +16842,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C72" s="57" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D72" s="59" t="str">
         <x:v>Has Closed Loan</x:v>
@@ -16830,7 +16856,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C73" s="57" t="n">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D73" s="59" t="str">
         <x:v>Return on Closed Loans</x:v>
@@ -16844,7 +16870,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C74" s="57" t="n">
-        <x:v>25</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D74" s="59" t="str">
         <x:v>Header - Closed Loans</x:v>
@@ -16858,7 +16884,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C75" s="57" t="n">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D75" s="59" t="str">
         <x:v>Has Active Loan</x:v>
@@ -16872,7 +16898,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C76" s="57" t="n">
-        <x:v>27</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="D76" s="59" t="str">
         <x:v>30D Gross Principal Days</x:v>
@@ -16886,7 +16912,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C77" s="57" t="n">
-        <x:v>28</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D77" s="59" t="str">
         <x:v>30D Principal Reduction Days</x:v>
@@ -16900,7 +16926,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C78" s="57" t="n">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="D78" s="59" t="str">
         <x:v>30D Average Outstanding Principal</x:v>
@@ -16914,7 +16940,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C79" s="57" t="n">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="D79" s="59" t="str">
         <x:v>30D Return on Average Principal</x:v>
@@ -16928,7 +16954,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C80" s="57" t="n">
-        <x:v>31</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D80" s="59" t="str">
         <x:v>Daily Collection Status</x:v>
@@ -16942,7 +16968,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C81" s="57" t="n">
-        <x:v>32</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D81" s="59" t="str">
         <x:v>Todays Collection Charges</x:v>
@@ -16956,7 +16982,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C82" s="57" t="n">
-        <x:v>33</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="D82" s="59" t="str">
         <x:v>Todays Amount Due</x:v>
@@ -16970,7 +16996,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C83" s="57" t="n">
-        <x:v>34</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="D83" s="59" t="str">
         <x:v>Todays Amount Collected</x:v>
@@ -16984,7 +17010,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C84" s="57" t="n">
-        <x:v>35</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="D84" s="59" t="str">
         <x:v>Todays Amount Remaining</x:v>
@@ -16998,7 +17024,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C85" s="57" t="n">
-        <x:v>36</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="D85" s="59" t="str">
         <x:v>Portfolio Exposure %</x:v>
@@ -17012,7 +17038,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C86" s="57" t="n">
-        <x:v>37</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="D86" s="59" t="str">
         <x:v>Active Loan Count</x:v>
@@ -17026,7 +17052,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C87" s="57" t="n">
-        <x:v>38</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="D87" s="59" t="str">
         <x:v>Oldest Active Loan Age</x:v>
@@ -17040,7 +17066,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C88" s="57" t="n">
-        <x:v>39</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="D88" s="59" t="str">
         <x:v>Overdue Amount</x:v>
@@ -17054,7 +17080,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C89" s="57" t="n">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D89" s="59" t="str">
         <x:v>Overdue Charge Count</x:v>
@@ -17068,7 +17094,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C90" s="57" t="n">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="D90" s="59" t="str">
         <x:v>Historical Charge Count</x:v>
@@ -17082,7 +17108,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C91" s="57" t="n">
-        <x:v>42</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="D91" s="59" t="str">
         <x:v>On Time Charge Count</x:v>
@@ -17096,7 +17122,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C92" s="57" t="n">
-        <x:v>43</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="D92" s="59" t="str">
         <x:v>Lifetime On Time Rate</x:v>
@@ -17110,7 +17136,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C93" s="57" t="n">
-        <x:v>44</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="D93" s="59" t="str">
         <x:v>Recent 30D Charge Count</x:v>
@@ -17124,7 +17150,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C94" s="57" t="n">
-        <x:v>45</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="D94" s="59" t="str">
         <x:v>Recent 30D On Time Count</x:v>
@@ -17138,7 +17164,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C95" s="57" t="n">
-        <x:v>46</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="D95" s="59" t="str">
         <x:v>Recent 30D On Time Rate</x:v>
@@ -17152,7 +17178,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C96" s="57" t="n">
-        <x:v>47</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="D96" s="59" t="str">
         <x:v>Lifetime Late Payment Count</x:v>
@@ -17166,7 +17192,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C97" s="57" t="n">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="D97" s="59" t="str">
         <x:v>Recent 30D Late Payment Count</x:v>
@@ -17180,7 +17206,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C98" s="57" t="n">
-        <x:v>49</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D98" s="59" t="str">
         <x:v>Maximum Days Late</x:v>
@@ -17194,7 +17220,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C99" s="57" t="n">
-        <x:v>50</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="D99" s="59" t="str">
         <x:v>Last Late Payment Date</x:v>
@@ -17208,7 +17234,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C100" s="57" t="n">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="D100" s="59" t="str">
         <x:v>Largest Successful Loan</x:v>
@@ -17222,7 +17248,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C101" s="57" t="n">
-        <x:v>52</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="D101" s="59" t="str">
         <x:v>Average Successful Loan Size</x:v>
@@ -17236,7 +17262,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C102" s="57" t="n">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="D102" s="59" t="str">
         <x:v>Default Count</x:v>
@@ -17250,7 +17276,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C103" s="57" t="n">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="D103" s="59" t="str">
         <x:v>Lifetime Default Loss</x:v>
@@ -17264,7 +17290,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C104" s="57" t="n">
-        <x:v>55</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="D104" s="59" t="str">
         <x:v>Portfolio Outstanding Principal</x:v>
@@ -17278,7 +17304,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C105" s="57" t="n">
-        <x:v>56</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="D105" s="59" t="str">
         <x:v>Portfolio Share Join Key</x:v>
@@ -17328,7 +17354,7 @@
     </x:row>
     <x:row r="109" ht="15" customHeight="1">
       <x:c r="A109" s="57" t="str">
-        <x:v>OLAP</x:v>
+        <x:v>Retired OLAP</x:v>
       </x:c>
       <x:c r="B109" s="59" t="str">
         <x:v>Profit Contribution 30D</x:v>
@@ -17348,7 +17374,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C110" s="57" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D110" s="59" t="str">
         <x:v>Description</x:v>
@@ -17362,7 +17388,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C111" s="57" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D111" s="59" t="str">
         <x:v>Creation Date</x:v>
@@ -17376,7 +17402,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C112" s="57" t="n">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D112" s="59" t="str">
         <x:v>Related Loans</x:v>
@@ -17390,7 +17416,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C113" s="57" t="n">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D113" s="59" t="str">
         <x:v>Total Interest Earned</x:v>
@@ -17404,7 +17430,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C114" s="57" t="n">
-        <x:v>9</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D114" s="59" t="str">
         <x:v>Total Amount Loaned</x:v>
@@ -17418,7 +17444,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C115" s="57" t="n">
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D115" s="59" t="str">
         <x:v>Total Number of Loans</x:v>
@@ -17432,7 +17458,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C116" s="57" t="n">
-        <x:v>11</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D116" s="59" t="str">
         <x:v>Total Outstanding Principal</x:v>
@@ -17446,7 +17472,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C117" s="57" t="n">
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D117" s="59" t="str">
         <x:v>Header - Active Loans</x:v>
@@ -17460,7 +17486,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C118" s="57" t="n">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D118" s="59" t="str">
         <x:v>Borrower Name TE</x:v>
@@ -17474,7 +17500,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C119" s="57" t="n">
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D119" s="59" t="str">
         <x:v>Return on Active Principal</x:v>
@@ -17488,7 +17514,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C120" s="57" t="n">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D120" s="59" t="str">
         <x:v>Profit Last 30 Days</x:v>
@@ -17502,7 +17528,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C121" s="57" t="n">
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D121" s="59" t="str">
         <x:v>Projected Interest Coverage Date</x:v>
@@ -17516,7 +17542,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C122" s="57" t="n">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D122" s="59" t="str">
         <x:v>Active Loan Interest Earned</x:v>
@@ -17530,7 +17556,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C123" s="57" t="n">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D123" s="59" t="str">
         <x:v>Active Daily Interest</x:v>
@@ -17544,7 +17570,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C124" s="57" t="n">
-        <x:v>19</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D124" s="59" t="str">
         <x:v>Related Loan Assessments</x:v>
@@ -17558,7 +17584,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C125" s="57" t="n">
-        <x:v>20</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D125" s="59" t="str">
         <x:v>Related Calendars</x:v>
@@ -17572,7 +17598,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C126" s="57" t="n">
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D126" s="59" t="str">
         <x:v>Closed Loan Interest Earned</x:v>
@@ -17586,7 +17612,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C127" s="57" t="n">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D127" s="59" t="str">
         <x:v>Closed Loan Principle</x:v>
@@ -17600,7 +17626,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C128" s="57" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D128" s="59" t="str">
         <x:v>Has Closed Loan</x:v>
@@ -17614,7 +17640,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C129" s="57" t="n">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D129" s="59" t="str">
         <x:v>Return on Closed Loans</x:v>
@@ -17628,7 +17654,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C130" s="57" t="n">
-        <x:v>25</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D130" s="59" t="str">
         <x:v>Header - Closed Loans</x:v>
@@ -17642,7 +17668,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C131" s="57" t="n">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D131" s="59" t="str">
         <x:v>Has Active Loan</x:v>
@@ -17656,7 +17682,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C132" s="57" t="n">
-        <x:v>27</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="D132" s="59" t="str">
         <x:v>30D Gross Principal Days</x:v>
@@ -17670,7 +17696,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C133" s="57" t="n">
-        <x:v>28</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D133" s="59" t="str">
         <x:v>30D Principal Reduction Days</x:v>
@@ -17684,7 +17710,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C134" s="57" t="n">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="D134" s="59" t="str">
         <x:v>30D Average Outstanding Principal</x:v>
@@ -17698,7 +17724,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C135" s="57" t="n">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="D135" s="59" t="str">
         <x:v>30D Return on Average Principal</x:v>
@@ -17712,7 +17738,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C136" s="57" t="n">
-        <x:v>31</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D136" s="59" t="str">
         <x:v>Daily Collection Status</x:v>
@@ -17726,7 +17752,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C137" s="57" t="n">
-        <x:v>32</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D137" s="59" t="str">
         <x:v>Todays Collection Charges</x:v>
@@ -17740,7 +17766,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C138" s="57" t="n">
-        <x:v>33</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="D138" s="59" t="str">
         <x:v>Todays Amount Due</x:v>
@@ -17754,7 +17780,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C139" s="57" t="n">
-        <x:v>34</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="D139" s="59" t="str">
         <x:v>Todays Amount Collected</x:v>
@@ -17768,7 +17794,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C140" s="57" t="n">
-        <x:v>35</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="D140" s="59" t="str">
         <x:v>Todays Amount Remaining</x:v>
@@ -17782,7 +17808,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C141" s="57" t="n">
-        <x:v>36</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="D141" s="59" t="str">
         <x:v>Portfolio Exposure %</x:v>
@@ -17796,7 +17822,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C142" s="57" t="n">
-        <x:v>37</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="D142" s="59" t="str">
         <x:v>Active Loan Count</x:v>
@@ -17810,7 +17836,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C143" s="57" t="n">
-        <x:v>38</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="D143" s="59" t="str">
         <x:v>Oldest Active Loan Age</x:v>
@@ -17824,7 +17850,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C144" s="57" t="n">
-        <x:v>39</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="D144" s="59" t="str">
         <x:v>Overdue Amount</x:v>
@@ -17838,7 +17864,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C145" s="57" t="n">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D145" s="59" t="str">
         <x:v>Overdue Charge Count</x:v>
@@ -17852,7 +17878,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C146" s="57" t="n">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="D146" s="59" t="str">
         <x:v>Historical Charge Count</x:v>
@@ -17866,7 +17892,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C147" s="57" t="n">
-        <x:v>42</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="D147" s="59" t="str">
         <x:v>On Time Charge Count</x:v>
@@ -17880,7 +17906,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C148" s="57" t="n">
-        <x:v>43</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="D148" s="59" t="str">
         <x:v>Lifetime On Time Rate</x:v>
@@ -17894,7 +17920,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C149" s="57" t="n">
-        <x:v>44</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="D149" s="59" t="str">
         <x:v>Recent 30D Charge Count</x:v>
@@ -17908,7 +17934,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C150" s="57" t="n">
-        <x:v>45</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="D150" s="59" t="str">
         <x:v>Recent 30D On Time Count</x:v>
@@ -17922,7 +17948,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C151" s="57" t="n">
-        <x:v>46</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="D151" s="59" t="str">
         <x:v>Recent 30D On Time Rate</x:v>
@@ -17936,7 +17962,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C152" s="57" t="n">
-        <x:v>47</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="D152" s="59" t="str">
         <x:v>Lifetime Late Payment Count</x:v>
@@ -17950,7 +17976,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C153" s="57" t="n">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="D153" s="59" t="str">
         <x:v>Recent 30D Late Payment Count</x:v>
@@ -17964,7 +17990,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C154" s="57" t="n">
-        <x:v>49</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D154" s="59" t="str">
         <x:v>Maximum Days Late</x:v>
@@ -17978,7 +18004,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C155" s="57" t="n">
-        <x:v>50</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="D155" s="59" t="str">
         <x:v>Last Late Payment Date</x:v>
@@ -17992,7 +18018,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C156" s="57" t="n">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="D156" s="59" t="str">
         <x:v>Largest Successful Loan</x:v>
@@ -18006,7 +18032,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C157" s="57" t="n">
-        <x:v>52</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="D157" s="59" t="str">
         <x:v>Average Successful Loan Size</x:v>
@@ -18020,7 +18046,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C158" s="57" t="n">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="D158" s="59" t="str">
         <x:v>Default Count</x:v>
@@ -18034,7 +18060,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C159" s="57" t="n">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="D159" s="59" t="str">
         <x:v>Lifetime Default Loss</x:v>
@@ -18048,7 +18074,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C160" s="57" t="n">
-        <x:v>55</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="D160" s="59" t="str">
         <x:v>Portfolio Outstanding Principal</x:v>
@@ -18062,7 +18088,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C161" s="57" t="n">
-        <x:v>56</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="D161" s="59" t="str">
         <x:v>Portfolio Share Join Key</x:v>
@@ -21170,7 +21196,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C383" s="87" t="n">
-        <x:v>34</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="D383" s="87" t="str">
         <x:v>Communication Name</x:v>
@@ -21184,7 +21210,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C384" s="87" t="n">
-        <x:v>35</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="D384" s="87" t="str">
         <x:v>Instagram Username</x:v>
@@ -21192,7 +21218,7 @@
     </x:row>
     <x:row r="385" ht="15" customHeight="1">
       <x:c r="A385" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B385" s="87" t="str">
         <x:v>Visible Borrowers</x:v>
@@ -21206,7 +21232,7 @@
     </x:row>
     <x:row r="386" ht="15" customHeight="1">
       <x:c r="A386" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B386" s="87" t="str">
         <x:v>Visible Borrowers</x:v>
@@ -21226,7 +21252,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C387" s="87" t="n">
-        <x:v>38</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="D387" s="87" t="str">
         <x:v>AI Collection Enabled</x:v>
@@ -21234,7 +21260,7 @@
     </x:row>
     <x:row r="388" ht="15" customHeight="1">
       <x:c r="A388" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B388" s="87" t="str">
         <x:v>Visible Borrowers</x:v>
@@ -21248,7 +21274,7 @@
     </x:row>
     <x:row r="389" ht="15" customHeight="1">
       <x:c r="A389" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B389" s="87" t="str">
         <x:v>Visible Borrowers</x:v>
@@ -21262,7 +21288,7 @@
     </x:row>
     <x:row r="390" ht="15" customHeight="1">
       <x:c r="A390" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B390" s="87" t="str">
         <x:v>Visible Borrowers</x:v>
@@ -21276,7 +21302,7 @@
     </x:row>
     <x:row r="391" ht="15" customHeight="1">
       <x:c r="A391" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B391" s="87" t="str">
         <x:v>Visible Borrowers</x:v>
@@ -21318,7 +21344,7 @@
     </x:row>
     <x:row r="394" ht="15" customHeight="1">
       <x:c r="A394" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B394" s="87" t="str">
         <x:v>Todays Collection Board</x:v>
@@ -21332,7 +21358,7 @@
     </x:row>
     <x:row r="395" ht="15" customHeight="1">
       <x:c r="A395" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B395" s="87" t="str">
         <x:v>Todays Collection Board</x:v>
@@ -21352,7 +21378,7 @@
         <x:v>Todays Collection Board</x:v>
       </x:c>
       <x:c r="C396" s="87" t="n">
-        <x:v>17</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D396" s="87" t="str">
         <x:v>AI Collection Enabled</x:v>
@@ -21360,7 +21386,7 @@
     </x:row>
     <x:row r="397" ht="15" customHeight="1">
       <x:c r="A397" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B397" s="87" t="str">
         <x:v>Todays Collection Board</x:v>
@@ -21374,7 +21400,7 @@
     </x:row>
     <x:row r="398" ht="15" customHeight="1">
       <x:c r="A398" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B398" s="87" t="str">
         <x:v>Todays Collection Board</x:v>
@@ -21388,7 +21414,7 @@
     </x:row>
     <x:row r="399" ht="15" customHeight="1">
       <x:c r="A399" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B399" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21402,7 +21428,7 @@
     </x:row>
     <x:row r="400" ht="15" customHeight="1">
       <x:c r="A400" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B400" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21416,7 +21442,7 @@
     </x:row>
     <x:row r="401" ht="15" customHeight="1">
       <x:c r="A401" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B401" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21430,7 +21456,7 @@
     </x:row>
     <x:row r="402" ht="15" customHeight="1">
       <x:c r="A402" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B402" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21444,7 +21470,7 @@
     </x:row>
     <x:row r="403" ht="15" customHeight="1">
       <x:c r="A403" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B403" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21458,7 +21484,7 @@
     </x:row>
     <x:row r="404" ht="15" customHeight="1">
       <x:c r="A404" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B404" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21472,7 +21498,7 @@
     </x:row>
     <x:row r="405" ht="15" customHeight="1">
       <x:c r="A405" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B405" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21486,7 +21512,7 @@
     </x:row>
     <x:row r="406" ht="15" customHeight="1">
       <x:c r="A406" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B406" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21500,7 +21526,7 @@
     </x:row>
     <x:row r="407" ht="15" customHeight="1">
       <x:c r="A407" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B407" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21514,7 +21540,7 @@
     </x:row>
     <x:row r="408" ht="15" customHeight="1">
       <x:c r="A408" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B408" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21528,7 +21554,7 @@
     </x:row>
     <x:row r="409" ht="15" customHeight="1">
       <x:c r="A409" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B409" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21542,7 +21568,7 @@
     </x:row>
     <x:row r="410" ht="15" customHeight="1">
       <x:c r="A410" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B410" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21556,7 +21582,7 @@
     </x:row>
     <x:row r="411" ht="15" customHeight="1">
       <x:c r="A411" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B411" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21570,7 +21596,7 @@
     </x:row>
     <x:row r="412" ht="15" customHeight="1">
       <x:c r="A412" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B412" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21584,7 +21610,7 @@
     </x:row>
     <x:row r="413" ht="15" customHeight="1">
       <x:c r="A413" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B413" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21598,7 +21624,7 @@
     </x:row>
     <x:row r="414" ht="15" customHeight="1">
       <x:c r="A414" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B414" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21612,7 +21638,7 @@
     </x:row>
     <x:row r="415" ht="15" customHeight="1">
       <x:c r="A415" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B415" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21626,7 +21652,7 @@
     </x:row>
     <x:row r="416" ht="15" customHeight="1">
       <x:c r="A416" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B416" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21640,7 +21666,7 @@
     </x:row>
     <x:row r="417" ht="15" customHeight="1">
       <x:c r="A417" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B417" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21654,7 +21680,7 @@
     </x:row>
     <x:row r="418" ht="15" customHeight="1">
       <x:c r="A418" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B418" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21668,7 +21694,7 @@
     </x:row>
     <x:row r="419" ht="15" customHeight="1">
       <x:c r="A419" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B419" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21682,7 +21708,7 @@
     </x:row>
     <x:row r="420" ht="15" customHeight="1">
       <x:c r="A420" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B420" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21696,7 +21722,7 @@
     </x:row>
     <x:row r="421" ht="15" customHeight="1">
       <x:c r="A421" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B421" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21710,7 +21736,7 @@
     </x:row>
     <x:row r="422" ht="15" customHeight="1">
       <x:c r="A422" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B422" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21724,7 +21750,7 @@
     </x:row>
     <x:row r="423" ht="15" customHeight="1">
       <x:c r="A423" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B423" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21738,7 +21764,7 @@
     </x:row>
     <x:row r="424" ht="15" customHeight="1">
       <x:c r="A424" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B424" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21752,7 +21778,7 @@
     </x:row>
     <x:row r="425" ht="15" customHeight="1">
       <x:c r="A425" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B425" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21766,7 +21792,7 @@
     </x:row>
     <x:row r="426" ht="15" customHeight="1">
       <x:c r="A426" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B426" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21780,7 +21806,7 @@
     </x:row>
     <x:row r="427" ht="15" customHeight="1">
       <x:c r="A427" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B427" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21794,7 +21820,7 @@
     </x:row>
     <x:row r="428" ht="15" customHeight="1">
       <x:c r="A428" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B428" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21808,7 +21834,7 @@
     </x:row>
     <x:row r="429" ht="15" customHeight="1">
       <x:c r="A429" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B429" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21822,7 +21848,7 @@
     </x:row>
     <x:row r="430" ht="15" customHeight="1">
       <x:c r="A430" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B430" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21836,7 +21862,7 @@
     </x:row>
     <x:row r="431" ht="15" customHeight="1">
       <x:c r="A431" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B431" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21850,7 +21876,7 @@
     </x:row>
     <x:row r="432" ht="15" customHeight="1">
       <x:c r="A432" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B432" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21864,7 +21890,7 @@
     </x:row>
     <x:row r="433" ht="15" customHeight="1">
       <x:c r="A433" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B433" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21878,7 +21904,7 @@
     </x:row>
     <x:row r="434" ht="15" customHeight="1">
       <x:c r="A434" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B434" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21892,7 +21918,7 @@
     </x:row>
     <x:row r="435" ht="15" customHeight="1">
       <x:c r="A435" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B435" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21906,7 +21932,7 @@
     </x:row>
     <x:row r="436" ht="15" customHeight="1">
       <x:c r="A436" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B436" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21920,7 +21946,7 @@
     </x:row>
     <x:row r="437" ht="15" customHeight="1">
       <x:c r="A437" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B437" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21934,7 +21960,7 @@
     </x:row>
     <x:row r="438" ht="15" customHeight="1">
       <x:c r="A438" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B438" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21948,7 +21974,7 @@
     </x:row>
     <x:row r="439" ht="15" customHeight="1">
       <x:c r="A439" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B439" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21962,7 +21988,7 @@
     </x:row>
     <x:row r="440" ht="15" customHeight="1">
       <x:c r="A440" s="87" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B440" s="87" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21976,7 +22002,7 @@
     </x:row>
     <x:row r="441">
       <x:c r="A441" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B441" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -21990,7 +22016,7 @@
     </x:row>
     <x:row r="442">
       <x:c r="A442" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B442" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -22004,7 +22030,7 @@
     </x:row>
     <x:row r="443">
       <x:c r="A443" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B443" t="str">
         <x:v>Collection Setup Review</x:v>
@@ -22024,7 +22050,7 @@
         <x:v>Todays Collection Board</x:v>
       </x:c>
       <x:c r="C444" t="n">
-        <x:v>20</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D444" t="str">
         <x:v>City</x:v>
@@ -22038,7 +22064,7 @@
         <x:v>Todays Collection Board</x:v>
       </x:c>
       <x:c r="C445" t="n">
-        <x:v>21</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D445" t="str">
         <x:v>Working Location</x:v>
@@ -22046,7 +22072,7 @@
     </x:row>
     <x:row r="446">
       <x:c r="A446" t="str">
-        <x:v>OLTP</x:v>
+        <x:v>Retired OLTP</x:v>
       </x:c>
       <x:c r="B446" t="str">
         <x:v>Visible Borrowers</x:v>
@@ -22066,7 +22092,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C447" t="n">
-        <x:v>44</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="D447" t="str">
         <x:v>City</x:v>
@@ -22080,7 +22106,7 @@
         <x:v>Visible Borrowers</x:v>
       </x:c>
       <x:c r="C448" t="n">
-        <x:v>45</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="D448" t="str">
         <x:v>Working Location</x:v>
@@ -22164,7 +22190,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C454" t="n">
-        <x:v>57</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="D454" t="str">
         <x:v>Hidden Flag</x:v>
@@ -22178,7 +22204,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C455" t="n">
-        <x:v>58</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="D455" t="str">
         <x:v>Projected Monthly Profit Contribution</x:v>
@@ -22192,7 +22218,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C456" t="n">
-        <x:v>59</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="D456" t="str">
         <x:v>Matrix Active Borrower Count</x:v>
@@ -22206,7 +22232,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C457" t="n">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="D457" t="str">
         <x:v>Matrix Equal Share Benchmark</x:v>
@@ -22220,7 +22246,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C458" t="n">
-        <x:v>61</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="D458" t="str">
         <x:v>Matrix Economic Contribution</x:v>
@@ -22234,7 +22260,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C459" t="n">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="D459" t="str">
         <x:v>Matrix Recent Reliability Score</x:v>
@@ -22248,7 +22274,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C460" t="n">
-        <x:v>63</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="D460" t="str">
         <x:v>Matrix Historical Reliability Score</x:v>
@@ -22262,7 +22288,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C461" t="n">
-        <x:v>64</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="D461" t="str">
         <x:v>Matrix Delay Severity Score</x:v>
@@ -22276,7 +22302,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C462" t="n">
-        <x:v>65</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="D462" t="str">
         <x:v>Matrix Current Condition Score</x:v>
@@ -22290,7 +22316,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C463" t="n">
-        <x:v>66</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="D463" t="str">
         <x:v>Matrix History Sufficient</x:v>
@@ -22304,7 +22330,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C464" t="n">
-        <x:v>67</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="D464" t="str">
         <x:v>Matrix Stability Score</x:v>
@@ -22318,7 +22344,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C465" t="n">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="D465" t="str">
         <x:v>Matrix Quadrant</x:v>
@@ -22332,7 +22358,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C466" t="n">
-        <x:v>69</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="D466" t="str">
         <x:v>Matrix Bubble Label</x:v>
@@ -22346,7 +22372,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C467" t="n">
-        <x:v>70</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D467" t="str">
         <x:v>Profit Last 10 Days</x:v>
@@ -22360,7 +22386,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C468" t="n">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="D468" t="str">
         <x:v>Matrix Scaled Economic Contribution</x:v>
@@ -22374,7 +22400,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C469" t="n">
-        <x:v>72</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="D469" t="str">
         <x:v>Related Payments</x:v>
@@ -22388,7 +22414,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C470" t="n">
-        <x:v>73</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="D470" t="str">
         <x:v>City</x:v>
@@ -22402,7 +22428,7 @@
         <x:v>Borrowers with Outstanding Loans</x:v>
       </x:c>
       <x:c r="C471" t="n">
-        <x:v>74</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="D471" t="str">
         <x:v>Working Location</x:v>
@@ -22416,7 +22442,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C472" t="n">
-        <x:v>57</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="D472" t="str">
         <x:v>Hidden Flag</x:v>
@@ -22430,7 +22456,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C473" t="n">
-        <x:v>58</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="D473" t="str">
         <x:v>Projected Monthly Profit Contribution</x:v>
@@ -22444,7 +22470,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C474" t="n">
-        <x:v>59</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="D474" t="str">
         <x:v>Matrix Active Borrower Count</x:v>
@@ -22458,7 +22484,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C475" t="n">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="D475" t="str">
         <x:v>Matrix Equal Share Benchmark</x:v>
@@ -22472,7 +22498,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C476" t="n">
-        <x:v>61</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="D476" t="str">
         <x:v>Matrix Economic Contribution</x:v>
@@ -22486,7 +22512,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C477" t="n">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="D477" t="str">
         <x:v>Matrix Recent Reliability Score</x:v>
@@ -22500,7 +22526,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C478" t="n">
-        <x:v>63</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="D478" t="str">
         <x:v>Matrix Historical Reliability Score</x:v>
@@ -22514,7 +22540,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C479" t="n">
-        <x:v>64</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="D479" t="str">
         <x:v>Matrix Delay Severity Score</x:v>
@@ -22528,7 +22554,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C480" t="n">
-        <x:v>65</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="D480" t="str">
         <x:v>Matrix Current Condition Score</x:v>
@@ -22542,7 +22568,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C481" t="n">
-        <x:v>66</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="D481" t="str">
         <x:v>Matrix History Sufficient</x:v>
@@ -22556,7 +22582,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C482" t="n">
-        <x:v>67</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="D482" t="str">
         <x:v>Matrix Stability Score</x:v>
@@ -22570,7 +22596,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C483" t="n">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="D483" t="str">
         <x:v>Matrix Quadrant</x:v>
@@ -22584,7 +22610,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C484" t="n">
-        <x:v>69</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="D484" t="str">
         <x:v>Matrix Bubble Label</x:v>
@@ -22598,7 +22624,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C485" t="n">
-        <x:v>70</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D485" t="str">
         <x:v>Profit Last 10 Days</x:v>
@@ -22612,7 +22638,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C486" t="n">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="D486" t="str">
         <x:v>Matrix Scaled Economic Contribution</x:v>
@@ -22626,7 +22652,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C487" t="n">
-        <x:v>72</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="D487" t="str">
         <x:v>Related Payments</x:v>
@@ -22640,7 +22666,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C488" t="n">
-        <x:v>73</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="D488" t="str">
         <x:v>City</x:v>
@@ -22654,7 +22680,7 @@
         <x:v>Profit Contribution 30D</x:v>
       </x:c>
       <x:c r="C489" t="n">
-        <x:v>74</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="D489" t="str">
         <x:v>Working Location</x:v>
@@ -22700,6 +22726,90 @@
       </x:c>
       <x:c r="D492" t="str">
         <x:v>Working Location</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="493">
+      <x:c r="A493" t="str">
+        <x:v>OLTP</x:v>
+      </x:c>
+      <x:c r="B493" t="str">
+        <x:v>Todays Collection Board</x:v>
+      </x:c>
+      <x:c r="C493" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D493" t="str">
+        <x:v>Address</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="494">
+      <x:c r="A494" t="str">
+        <x:v>OLTP</x:v>
+      </x:c>
+      <x:c r="B494" t="str">
+        <x:v>Visible Borrowers</x:v>
+      </x:c>
+      <x:c r="C494" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="D494" t="str">
+        <x:v>Address</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="495">
+      <x:c r="A495" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B495" t="str">
+        <x:v>Borrowers with Outstanding Loans</x:v>
+      </x:c>
+      <x:c r="C495" t="n">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="D495" t="str">
+        <x:v>Address</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="496">
+      <x:c r="A496" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B496" t="str">
+        <x:v>Profit Contribution 30D</x:v>
+      </x:c>
+      <x:c r="C496" t="n">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="D496" t="str">
+        <x:v>Address</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="497">
+      <x:c r="A497" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B497" t="str">
+        <x:v>Reporting Borrowers</x:v>
+      </x:c>
+      <x:c r="C497" t="n">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="D497" t="str">
+        <x:v>Address</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="498">
+      <x:c r="A498" t="str">
+        <x:v>OLAP</x:v>
+      </x:c>
+      <x:c r="B498" t="str">
+        <x:v>Todays Collection Board</x:v>
+      </x:c>
+      <x:c r="C498" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="D498" t="str">
+        <x:v>Address</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -22709,7 +22819,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb899178b9b345b0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb2f9462cb394bf4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26735,7 +26845,7 @@
         <x:v>Yes — 1.100031</x:v>
       </x:c>
       <x:c r="F204" s="87" t="str">
-        <x:v>Verified loaded in OLAP. Partner fields managed in OLAP; borrower table remains read-only. Existing financial formulas and row flags unchanged.</x:v>
+        <x:v>Required in both apps. OLTP editable; OLAP table remains read-only. Blank initial value.</x:v>
       </x:c>
     </x:row>
     <x:row r="205" ht="15" customHeight="1">
@@ -26769,13 +26879,13 @@
         <x:v>Instagram Conversation URL</x:v>
       </x:c>
       <x:c r="D206" s="87" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="E206" s="87" t="str">
-        <x:v>Yes — 1.100031</x:v>
+        <x:v>Removed / absent</x:v>
       </x:c>
       <x:c r="F206" s="87" t="str">
-        <x:v>OLTP Url; OLAP Text; native Text. Existing type variance preserved. Both initial values blank.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
     </x:row>
     <x:row r="207" ht="15" customHeight="1">
@@ -26789,13 +26899,13 @@
         <x:v>Instagram Verified At</x:v>
       </x:c>
       <x:c r="D207" s="87" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="E207" s="87" t="str">
-        <x:v>Yes — 1.100031</x:v>
+        <x:v>Removed / absent</x:v>
       </x:c>
       <x:c r="F207" s="87" t="str">
-        <x:v>Verified loaded in OLAP. Partner fields managed in OLAP; borrower table remains read-only. Existing financial formulas and row flags unchanged.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
     </x:row>
     <x:row r="208" ht="15" customHeight="1">
@@ -26815,7 +26925,7 @@
         <x:v>Yes — 1.100031</x:v>
       </x:c>
       <x:c r="F208" s="87" t="str">
-        <x:v>Verified loaded in OLAP. Partner fields managed in OLAP; borrower table remains read-only. Existing financial formulas and row flags unchanged.</x:v>
+        <x:v>Initial TRUE in both apps for new rows only. Existing row values not edited by cleanup.</x:v>
       </x:c>
     </x:row>
     <x:row r="209" ht="15" customHeight="1">
@@ -26829,13 +26939,13 @@
         <x:v>Late Penalty Enabled</x:v>
       </x:c>
       <x:c r="D209" s="87" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="E209" s="87" t="str">
-        <x:v>Yes — 1.100031</x:v>
+        <x:v>Removed / absent</x:v>
       </x:c>
       <x:c r="F209" s="87" t="str">
-        <x:v>Verified loaded in OLAP. Partner fields managed in OLAP; borrower table remains read-only. Existing financial formulas and row flags unchanged.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
     </x:row>
     <x:row r="210" ht="15" customHeight="1">
@@ -26849,13 +26959,13 @@
         <x:v>Receiving Bank Account</x:v>
       </x:c>
       <x:c r="D210" s="87" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="E210" s="87" t="str">
-        <x:v>Yes — 1.100031</x:v>
+        <x:v>Removed / absent</x:v>
       </x:c>
       <x:c r="F210" s="87" t="str">
-        <x:v>Verified loaded in OLAP. Partner fields managed in OLAP; borrower table remains read-only. Existing financial formulas and row flags unchanged.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
     </x:row>
     <x:row r="211" ht="15" customHeight="1">
@@ -26869,13 +26979,13 @@
         <x:v>Effective Receiving Bank Account</x:v>
       </x:c>
       <x:c r="D211" s="87" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="E211" s="87" t="str">
-        <x:v>Not configured by this build</x:v>
+        <x:v>Removed / absent</x:v>
       </x:c>
       <x:c r="F211" s="87" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); collection settings owned by OLTP.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
     </x:row>
     <x:row r="212" ht="15" customHeight="1">
@@ -26889,13 +26999,13 @@
         <x:v>Collection Setup Issues</x:v>
       </x:c>
       <x:c r="D212" s="87" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="E212" s="87" t="str">
-        <x:v>Not configured by this build</x:v>
+        <x:v>Removed / absent</x:v>
       </x:c>
       <x:c r="F212" s="87" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); collection settings owned by OLTP.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
     </x:row>
     <x:row r="213" ht="15" customHeight="1">
@@ -26909,13 +27019,13 @@
         <x:v>_RowNumber</x:v>
       </x:c>
       <x:c r="D213" s="87" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="E213" s="87" t="str">
-        <x:v>Not configured by this build</x:v>
+        <x:v>Removed / absent</x:v>
       </x:c>
       <x:c r="F213" s="87" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); collection settings owned by OLTP.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
     </x:row>
     <x:row r="214" ht="15" customHeight="1">
@@ -26929,13 +27039,13 @@
         <x:v>Row ID</x:v>
       </x:c>
       <x:c r="D214" s="87" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="E214" s="87" t="str">
-        <x:v>Not configured by this build</x:v>
+        <x:v>Removed / absent</x:v>
       </x:c>
       <x:c r="F214" s="87" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); collection settings owned by OLTP.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
     </x:row>
     <x:row r="215" ht="15" customHeight="1">
@@ -26949,13 +27059,13 @@
         <x:v>Account Label</x:v>
       </x:c>
       <x:c r="D215" s="87" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="E215" s="87" t="str">
-        <x:v>Not configured by this build</x:v>
+        <x:v>Removed / absent</x:v>
       </x:c>
       <x:c r="F215" s="87" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); collection settings owned by OLTP.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
     </x:row>
     <x:row r="216" ht="15" customHeight="1">
@@ -26969,13 +27079,13 @@
         <x:v>Bank Name</x:v>
       </x:c>
       <x:c r="D216" s="87" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="E216" s="87" t="str">
-        <x:v>Not configured by this build</x:v>
+        <x:v>Removed / absent</x:v>
       </x:c>
       <x:c r="F216" s="87" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); collection settings owned by OLTP.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
     </x:row>
     <x:row r="217" ht="15" customHeight="1">
@@ -26989,13 +27099,13 @@
         <x:v>Account Number</x:v>
       </x:c>
       <x:c r="D217" s="87" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="E217" s="87" t="str">
-        <x:v>Not configured by this build</x:v>
+        <x:v>Removed / absent</x:v>
       </x:c>
       <x:c r="F217" s="87" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); collection settings owned by OLTP.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
     </x:row>
     <x:row r="218" ht="15" customHeight="1">
@@ -27009,13 +27119,13 @@
         <x:v>Account Holder Name</x:v>
       </x:c>
       <x:c r="D218" s="87" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="E218" s="87" t="str">
-        <x:v>Not configured by this build</x:v>
+        <x:v>Removed / absent</x:v>
       </x:c>
       <x:c r="F218" s="87" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); collection settings owned by OLTP.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
     </x:row>
     <x:row r="219" ht="15" customHeight="1">
@@ -27029,13 +27139,13 @@
         <x:v>Active</x:v>
       </x:c>
       <x:c r="D219" s="87" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="E219" s="87" t="str">
-        <x:v>Not configured by this build</x:v>
+        <x:v>Removed / absent</x:v>
       </x:c>
       <x:c r="F219" s="87" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); collection settings owned by OLTP.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
     </x:row>
     <x:row r="220" ht="15" customHeight="1">
@@ -27049,13 +27159,13 @@
         <x:v>Related Collection Settings</x:v>
       </x:c>
       <x:c r="D220" s="87" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="E220" s="87" t="str">
-        <x:v>Not configured by this build</x:v>
+        <x:v>Removed / absent</x:v>
       </x:c>
       <x:c r="F220" s="87" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); collection settings owned by OLTP.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
     </x:row>
     <x:row r="221" ht="15" customHeight="1">
@@ -27069,13 +27179,13 @@
         <x:v>Related Borrowers</x:v>
       </x:c>
       <x:c r="D221" s="87" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="E221" s="87" t="str">
-        <x:v>Not configured by this build</x:v>
+        <x:v>Removed / absent</x:v>
       </x:c>
       <x:c r="F221" s="87" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); collection settings owned by OLTP.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
     </x:row>
     <x:row r="222" ht="15" customHeight="1">
@@ -27089,13 +27199,13 @@
         <x:v>Related Borrowers By Effective Receiving Bank Account</x:v>
       </x:c>
       <x:c r="D222" s="87" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="E222" s="87" t="str">
-        <x:v>Not configured by this build</x:v>
+        <x:v>Removed / absent</x:v>
       </x:c>
       <x:c r="F222" s="87" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); collection settings owned by OLTP.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
     </x:row>
     <x:row r="223" ht="15" customHeight="1">
@@ -27109,13 +27219,13 @@
         <x:v>_RowNumber</x:v>
       </x:c>
       <x:c r="D223" s="87" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="E223" s="87" t="str">
-        <x:v>Not configured by this build</x:v>
+        <x:v>Removed / absent</x:v>
       </x:c>
       <x:c r="F223" s="87" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); collection settings owned by OLTP.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
     </x:row>
     <x:row r="224" ht="15" customHeight="1">
@@ -27129,13 +27239,13 @@
         <x:v>Row ID</x:v>
       </x:c>
       <x:c r="D224" s="87" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="E224" s="87" t="str">
-        <x:v>Not configured by this build</x:v>
+        <x:v>Removed / absent</x:v>
       </x:c>
       <x:c r="F224" s="87" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); collection settings owned by OLTP.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
     </x:row>
     <x:row r="225" ht="15" customHeight="1">
@@ -27149,13 +27259,13 @@
         <x:v>Setting Name</x:v>
       </x:c>
       <x:c r="D225" s="87" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="E225" s="87" t="str">
-        <x:v>Not configured by this build</x:v>
+        <x:v>Removed / absent</x:v>
       </x:c>
       <x:c r="F225" s="87" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); collection settings owned by OLTP.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
     </x:row>
     <x:row r="226" ht="15" customHeight="1">
@@ -27169,13 +27279,13 @@
         <x:v>Default Receiving Bank Account</x:v>
       </x:c>
       <x:c r="D226" s="87" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="E226" s="87" t="str">
-        <x:v>Not configured by this build</x:v>
+        <x:v>Removed / absent</x:v>
       </x:c>
       <x:c r="F226" s="87" t="str">
-        <x:v>OLTP 3.000024; 8 September 2026 (Asia/Bangkok); collection settings owned by OLTP.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
     </x:row>
     <x:row r="227" ht="15" customHeight="1">
@@ -27189,13 +27299,13 @@
         <x:v>Collection Setup Review</x:v>
       </x:c>
       <x:c r="D227" s="87" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Removed</x:v>
       </x:c>
       <x:c r="E227" s="87" t="str">
-        <x:v>No</x:v>
+        <x:v>Removed / absent</x:v>
       </x:c>
       <x:c r="F227" s="87" t="str">
-        <x:v>Enabled borrowers with setup issues; 45 columns at OLTP 3.000050; update only.</x:v>
+        <x:v>Removed 13 September 2026; historical inventory only, not an active dependency.</x:v>
       </x:c>
     </x:row>
     <x:row r="228">
@@ -27275,7 +27385,7 @@
         <x:v>Yes — 1.100031</x:v>
       </x:c>
       <x:c r="F231" t="str">
-        <x:v>Verified loaded in OLAP. Partner fields managed in OLAP; borrower table remains read-only. Existing financial formulas and row flags unchanged.</x:v>
+        <x:v>Required in both apps. Blank initial value; display เมือง / City. Existing values preserved.</x:v>
       </x:c>
     </x:row>
     <x:row r="232">
@@ -27296,6 +27406,26 @@
       </x:c>
       <x:c r="F232" t="str">
         <x:v>Verified loaded in OLAP. Partner fields managed in OLAP; borrower table remains read-only. Existing financial formulas and row flags unchanged.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="233">
+      <x:c r="A233" t="str">
+        <x:v>Column</x:v>
+      </x:c>
+      <x:c r="B233" t="str">
+        <x:v>Borrowers</x:v>
+      </x:c>
+      <x:c r="C233" t="str">
+        <x:v>Address</x:v>
+      </x:c>
+      <x:c r="D233" t="str">
+        <x:v>Yes — 3.000064</x:v>
+      </x:c>
+      <x:c r="E233" t="str">
+        <x:v>Yes — 1.100041</x:v>
+      </x:c>
+      <x:c r="F233" t="str">
+        <x:v>Text, optional; blank initial. Seven source addresses imported and reloaded.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -27308,7 +27438,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bf1c2fe6a734552"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R196b4f6281b84e49"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27507,7 +27637,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbec54b2403354202"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc396ec1e9a8432c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29160,7 +29290,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a2caa9c6b2f4583"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref1d43f31d454711"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Verify AppSheet PostgreSQL sync and exact-case references
</commit_message>
<xml_diff>
--- a/Documents/AppSheet_Data_Dictionary.xlsx
+++ b/Documents/AppSheet_Data_Dictionary.xlsx
@@ -2,18 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rb9853f0907c541e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="Rc818e69beb2a4e35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R5e6079b1c2934bbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R4bebfdc085464e4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="Rfc856e925703480f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R7c83090d20924339"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="R114839d9779d4251"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R98ba3e208b9a45e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="R84a3dc1cfc4b409b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R54931ad81cbb4447"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="Rf9ef1b83482c4b54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="Rd158215a355f46b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R16ef4dce4a404f59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="R3a3c1dbe9cde4888"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R7d7c6d1b0b9b4855"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="Rf0274cd7b5cf4361"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="R795c4633819943b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R6a70cd4520b24fbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Rad8890efd2ad4c8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R4f71724f3ba14f40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="R99d46dde0e634099"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R3cb019cf2f464b6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="R37b3e1a8ef934be5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="Rc3e951c7837740e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Sync POC" sheetId="13" r:id="R1c3d80887d6444f6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -98,7 +99,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="24">
+  <x:fills count="25">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -133,6 +134,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -345,7 +351,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="111">
+  <x:cellXfs count="114">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -585,6 +591,11 @@
     <x:xf numFmtId="0" fontId="11" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="12" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="12" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2492,7 +2503,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79a4e735b1af4cdc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R392b43b532d44c18"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3878,6 +3889,1199 @@
       </x:c>
       <x:c r="H7" s="93" t="str">
         <x:v>Inline</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="38" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="55" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="100" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="113" t="str">
+        <x:v>Experiment</x:v>
+      </x:c>
+      <x:c r="B1" s="113" t="str">
+        <x:v>App version</x:v>
+      </x:c>
+      <x:c r="C1" s="113" t="str">
+        <x:v>Table</x:v>
+      </x:c>
+      <x:c r="D1" s="113" t="str">
+        <x:v>Column / setting</x:v>
+      </x:c>
+      <x:c r="E1" s="113" t="str">
+        <x:v>Type</x:v>
+      </x:c>
+      <x:c r="F1" s="113" t="str">
+        <x:v>Scope / status</x:v>
+      </x:c>
+      <x:c r="G1" s="113" t="str">
+        <x:v>Purpose / dependencies</x:v>
+      </x:c>
+      <x:c r="H1" s="113" t="str">
+        <x:v>Exact definition</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="150" customHeight="1">
+      <x:c r="A2" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B2" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C2" s="93" t="str">
+        <x:v>poc_source</x:v>
+      </x:c>
+      <x:c r="D2" s="93" t="str">
+        <x:v>Table access</x:v>
+      </x:c>
+      <x:c r="E2" s="93" t="str">
+        <x:v>Configuration</x:v>
+      </x:c>
+      <x:c r="F2" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G2" s="93" t="str">
+        <x:v>Source: database-1</x:v>
+      </x:c>
+      <x:c r="H2" s="93" t="str">
+        <x:v>UPDATES_ONLY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="150" customHeight="1">
+      <x:c r="A3" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B3" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C3" s="93" t="str">
+        <x:v>_Per User Settings</x:v>
+      </x:c>
+      <x:c r="D3" s="93" t="str">
+        <x:v>Table access</x:v>
+      </x:c>
+      <x:c r="E3" s="93" t="str">
+        <x:v>Configuration</x:v>
+      </x:c>
+      <x:c r="F3" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G3" s="93" t="str">
+        <x:v>Source: native</x:v>
+      </x:c>
+      <x:c r="H3" s="93" t="str">
+        <x:v>UPDATES_ONLY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="150" customHeight="1">
+      <x:c r="A4" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B4" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C4" s="93" t="str">
+        <x:v>poc_projection</x:v>
+      </x:c>
+      <x:c r="D4" s="93" t="str">
+        <x:v>Table access</x:v>
+      </x:c>
+      <x:c r="E4" s="93" t="str">
+        <x:v>Configuration</x:v>
+      </x:c>
+      <x:c r="F4" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G4" s="93" t="str">
+        <x:v>Source: database-1</x:v>
+      </x:c>
+      <x:c r="H4" s="93" t="str">
+        <x:v>READ_ONLY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="150" customHeight="1">
+      <x:c r="A5" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B5" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C5" s="93" t="str">
+        <x:v>poc_events</x:v>
+      </x:c>
+      <x:c r="D5" s="93" t="str">
+        <x:v>Table access</x:v>
+      </x:c>
+      <x:c r="E5" s="93" t="str">
+        <x:v>Configuration</x:v>
+      </x:c>
+      <x:c r="F5" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G5" s="93" t="str">
+        <x:v>Source: database-1</x:v>
+      </x:c>
+      <x:c r="H5" s="93" t="str">
+        <x:v>READ_ONLY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="150" customHeight="1">
+      <x:c r="A6" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B6" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C6" s="93" t="str">
+        <x:v>_Per User Settings</x:v>
+      </x:c>
+      <x:c r="D6" s="93" t="str">
+        <x:v>_RowNumber</x:v>
+      </x:c>
+      <x:c r="E6" s="93" t="str">
+        <x:v>Number</x:v>
+      </x:c>
+      <x:c r="F6" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G6" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H6" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: Yes
+Hidden: Yes
+Virtual?: No
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="150" customHeight="1">
+      <x:c r="A7" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B7" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C7" s="93" t="str">
+        <x:v>_Per User Settings</x:v>
+      </x:c>
+      <x:c r="D7" s="93" t="str">
+        <x:v>_EMAIL</x:v>
+      </x:c>
+      <x:c r="E7" s="93" t="str">
+        <x:v>Email</x:v>
+      </x:c>
+      <x:c r="F7" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G7" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H7" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: No
+Hidden: Yes
+Virtual?: No
+App formula: USEREMAIL()
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="150" customHeight="1">
+      <x:c r="A8" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B8" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C8" s="93" t="str">
+        <x:v>_Per User Settings</x:v>
+      </x:c>
+      <x:c r="D8" s="93" t="str">
+        <x:v>_NAME</x:v>
+      </x:c>
+      <x:c r="E8" s="93" t="str">
+        <x:v>Name</x:v>
+      </x:c>
+      <x:c r="F8" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G8" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H8" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: No
+Hidden: Yes
+Virtual?: No
+App formula: USERNAME()
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="150" customHeight="1">
+      <x:c r="A9" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B9" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C9" s="93" t="str">
+        <x:v>_Per User Settings</x:v>
+      </x:c>
+      <x:c r="D9" s="93" t="str">
+        <x:v>_LOCATION</x:v>
+      </x:c>
+      <x:c r="E9" s="93" t="str">
+        <x:v>LatLong</x:v>
+      </x:c>
+      <x:c r="F9" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G9" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H9" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: No
+Hidden: Yes
+Virtual?: No
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="150" customHeight="1">
+      <x:c r="A10" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B10" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C10" s="93" t="str">
+        <x:v>_Per User Settings</x:v>
+      </x:c>
+      <x:c r="D10" s="93" t="str">
+        <x:v>Options Heading</x:v>
+      </x:c>
+      <x:c r="E10" s="93" t="str">
+        <x:v>Show</x:v>
+      </x:c>
+      <x:c r="F10" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G10" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H10" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: Yes
+Hidden: Yes
+Virtual?: No
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="150" customHeight="1">
+      <x:c r="A11" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B11" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C11" s="93" t="str">
+        <x:v>_Per User Settings</x:v>
+      </x:c>
+      <x:c r="D11" s="93" t="str">
+        <x:v>Option 1</x:v>
+      </x:c>
+      <x:c r="E11" s="93" t="str">
+        <x:v>Text</x:v>
+      </x:c>
+      <x:c r="F11" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G11" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H11" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: No
+Hidden: Yes
+Virtual?: No
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="150" customHeight="1">
+      <x:c r="A12" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B12" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C12" s="93" t="str">
+        <x:v>_Per User Settings</x:v>
+      </x:c>
+      <x:c r="D12" s="93" t="str">
+        <x:v>Option 2</x:v>
+      </x:c>
+      <x:c r="E12" s="93" t="str">
+        <x:v>Number</x:v>
+      </x:c>
+      <x:c r="F12" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G12" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H12" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: No
+Hidden: Yes
+Virtual?: No
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="150" customHeight="1">
+      <x:c r="A13" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B13" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C13" s="93" t="str">
+        <x:v>_Per User Settings</x:v>
+      </x:c>
+      <x:c r="D13" s="93" t="str">
+        <x:v>Country Option</x:v>
+      </x:c>
+      <x:c r="E13" s="93" t="str">
+        <x:v>Enum</x:v>
+      </x:c>
+      <x:c r="F13" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G13" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H13" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: No
+Hidden: Yes
+Virtual?: No
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="150" customHeight="1">
+      <x:c r="A14" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B14" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C14" s="93" t="str">
+        <x:v>_Per User Settings</x:v>
+      </x:c>
+      <x:c r="D14" s="93" t="str">
+        <x:v>Language Option</x:v>
+      </x:c>
+      <x:c r="E14" s="93" t="str">
+        <x:v>Enum</x:v>
+      </x:c>
+      <x:c r="F14" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G14" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H14" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: No
+Hidden: Yes
+Virtual?: No
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="150" customHeight="1">
+      <x:c r="A15" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B15" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C15" s="93" t="str">
+        <x:v>_Per User Settings</x:v>
+      </x:c>
+      <x:c r="D15" s="93" t="str">
+        <x:v>Option 5</x:v>
+      </x:c>
+      <x:c r="E15" s="93" t="str">
+        <x:v>Text</x:v>
+      </x:c>
+      <x:c r="F15" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G15" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H15" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: No
+Hidden: Yes
+Virtual?: No
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="150" customHeight="1">
+      <x:c r="A16" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B16" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C16" s="93" t="str">
+        <x:v>_Per User Settings</x:v>
+      </x:c>
+      <x:c r="D16" s="93" t="str">
+        <x:v>Option 6</x:v>
+      </x:c>
+      <x:c r="E16" s="93" t="str">
+        <x:v>Number</x:v>
+      </x:c>
+      <x:c r="F16" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G16" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H16" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: No
+Hidden: Yes
+Virtual?: No
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="150" customHeight="1">
+      <x:c r="A17" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B17" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C17" s="93" t="str">
+        <x:v>_Per User Settings</x:v>
+      </x:c>
+      <x:c r="D17" s="93" t="str">
+        <x:v>Option 7</x:v>
+      </x:c>
+      <x:c r="E17" s="93" t="str">
+        <x:v>Text</x:v>
+      </x:c>
+      <x:c r="F17" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G17" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H17" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: No
+Hidden: Yes
+Virtual?: No
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="150" customHeight="1">
+      <x:c r="A18" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B18" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C18" s="93" t="str">
+        <x:v>_Per User Settings</x:v>
+      </x:c>
+      <x:c r="D18" s="93" t="str">
+        <x:v>Option 8</x:v>
+      </x:c>
+      <x:c r="E18" s="93" t="str">
+        <x:v>Text</x:v>
+      </x:c>
+      <x:c r="F18" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G18" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H18" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: No
+Hidden: Yes
+Virtual?: No
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="150" customHeight="1">
+      <x:c r="A19" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B19" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C19" s="93" t="str">
+        <x:v>_Per User Settings</x:v>
+      </x:c>
+      <x:c r="D19" s="93" t="str">
+        <x:v>Option 9</x:v>
+      </x:c>
+      <x:c r="E19" s="93" t="str">
+        <x:v>Text</x:v>
+      </x:c>
+      <x:c r="F19" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G19" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H19" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: No
+Hidden: Yes
+Virtual?: No
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="150" customHeight="1">
+      <x:c r="A20" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B20" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C20" s="93" t="str">
+        <x:v>_Per User Settings</x:v>
+      </x:c>
+      <x:c r="D20" s="93" t="str">
+        <x:v>_THISUSER</x:v>
+      </x:c>
+      <x:c r="E20" s="93" t="str">
+        <x:v>Text</x:v>
+      </x:c>
+      <x:c r="F20" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G20" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H20" s="93" t="str">
+        <x:v>Key: Yes
+Label: No
+Read-Only: No
+Hidden: Yes
+Virtual?: No
+Initial value: onlyvalue
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="150" customHeight="1">
+      <x:c r="A21" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B21" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C21" s="93" t="str">
+        <x:v>poc_source</x:v>
+      </x:c>
+      <x:c r="D21" s="93" t="str">
+        <x:v>_RowNumber</x:v>
+      </x:c>
+      <x:c r="E21" s="93" t="str">
+        <x:v>Number</x:v>
+      </x:c>
+      <x:c r="F21" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G21" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H21" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: Yes
+Hidden: Yes
+Virtual?: No
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="150" customHeight="1">
+      <x:c r="A22" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B22" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C22" s="93" t="str">
+        <x:v>poc_source</x:v>
+      </x:c>
+      <x:c r="D22" s="93" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="E22" s="93" t="str">
+        <x:v>Text</x:v>
+      </x:c>
+      <x:c r="F22" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G22" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H22" s="93" t="str">
+        <x:v>Key: Yes
+Label: Yes
+Read-Only: Yes
+Hidden: No
+Virtual?: No
+Initial value: UNIQUEID()
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="150" customHeight="1">
+      <x:c r="A23" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B23" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C23" s="93" t="str">
+        <x:v>poc_source</x:v>
+      </x:c>
+      <x:c r="D23" s="93" t="str">
+        <x:v>input_value</x:v>
+      </x:c>
+      <x:c r="E23" s="93" t="str">
+        <x:v>Number</x:v>
+      </x:c>
+      <x:c r="F23" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G23" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H23" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: No
+Hidden: No
+Virtual?: No
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="150" customHeight="1">
+      <x:c r="A24" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B24" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C24" s="93" t="str">
+        <x:v>poc_source</x:v>
+      </x:c>
+      <x:c r="D24" s="93" t="str">
+        <x:v>revision</x:v>
+      </x:c>
+      <x:c r="E24" s="93" t="str">
+        <x:v>Number</x:v>
+      </x:c>
+      <x:c r="F24" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G24" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H24" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: No
+Hidden: No
+Virtual?: No
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="150" customHeight="1">
+      <x:c r="A25" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B25" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C25" s="93" t="str">
+        <x:v>poc_source</x:v>
+      </x:c>
+      <x:c r="D25" s="93" t="str">
+        <x:v>Related poc_events</x:v>
+      </x:c>
+      <x:c r="E25" s="93" t="str">
+        <x:v>List</x:v>
+      </x:c>
+      <x:c r="F25" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G25" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H25" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: Yes
+Hidden: No
+Virtual?: Yes
+App formula: REF_ROWS("poc_events", "source_id")
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="150" customHeight="1">
+      <x:c r="A26" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B26" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C26" s="93" t="str">
+        <x:v>poc_projection</x:v>
+      </x:c>
+      <x:c r="D26" s="93" t="str">
+        <x:v>_RowNumber</x:v>
+      </x:c>
+      <x:c r="E26" s="93" t="str">
+        <x:v>Number</x:v>
+      </x:c>
+      <x:c r="F26" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G26" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H26" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: Yes
+Hidden: Yes
+Virtual?: No
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="150" customHeight="1">
+      <x:c r="A27" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B27" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C27" s="93" t="str">
+        <x:v>poc_projection</x:v>
+      </x:c>
+      <x:c r="D27" s="93" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="E27" s="93" t="str">
+        <x:v>Text</x:v>
+      </x:c>
+      <x:c r="F27" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G27" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H27" s="93" t="str">
+        <x:v>Key: Yes
+Label: Yes
+Read-Only: No
+Hidden: No
+Virtual?: No
+Initial value: UNIQUEID()
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="150" customHeight="1">
+      <x:c r="A28" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B28" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C28" s="93" t="str">
+        <x:v>poc_projection</x:v>
+      </x:c>
+      <x:c r="D28" s="93" t="str">
+        <x:v>applied_revision</x:v>
+      </x:c>
+      <x:c r="E28" s="93" t="str">
+        <x:v>Number</x:v>
+      </x:c>
+      <x:c r="F28" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G28" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H28" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: No
+Hidden: No
+Virtual?: No
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="150" customHeight="1">
+      <x:c r="A29" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B29" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C29" s="93" t="str">
+        <x:v>poc_projection</x:v>
+      </x:c>
+      <x:c r="D29" s="93" t="str">
+        <x:v>derived_value</x:v>
+      </x:c>
+      <x:c r="E29" s="93" t="str">
+        <x:v>Number</x:v>
+      </x:c>
+      <x:c r="F29" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G29" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H29" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: No
+Hidden: No
+Virtual?: No
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="150" customHeight="1">
+      <x:c r="A30" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B30" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C30" s="93" t="str">
+        <x:v>poc_events</x:v>
+      </x:c>
+      <x:c r="D30" s="93" t="str">
+        <x:v>_RowNumber</x:v>
+      </x:c>
+      <x:c r="E30" s="93" t="str">
+        <x:v>Number</x:v>
+      </x:c>
+      <x:c r="F30" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G30" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H30" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: Yes
+Hidden: Yes
+Virtual?: No
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="150" customHeight="1">
+      <x:c r="A31" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B31" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C31" s="93" t="str">
+        <x:v>poc_events</x:v>
+      </x:c>
+      <x:c r="D31" s="93" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="E31" s="93" t="str">
+        <x:v>Text</x:v>
+      </x:c>
+      <x:c r="F31" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G31" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H31" s="93" t="str">
+        <x:v>Key: Yes
+Label: Yes
+Read-Only: No
+Hidden: No
+Virtual?: No
+Initial value: UNIQUEID()
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="150" customHeight="1">
+      <x:c r="A32" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B32" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C32" s="93" t="str">
+        <x:v>poc_events</x:v>
+      </x:c>
+      <x:c r="D32" s="93" t="str">
+        <x:v>source_id</x:v>
+      </x:c>
+      <x:c r="E32" s="93" t="str">
+        <x:v>Ref</x:v>
+      </x:c>
+      <x:c r="F32" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G32" s="93" t="str">
+        <x:v>Ref -&gt; poc_source[id]; IsAPartOf=false</x:v>
+      </x:c>
+      <x:c r="H32" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: No
+Hidden: No
+Virtual?: No
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="150" customHeight="1">
+      <x:c r="A33" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B33" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C33" s="93" t="str">
+        <x:v>poc_events</x:v>
+      </x:c>
+      <x:c r="D33" s="93" t="str">
+        <x:v>revision</x:v>
+      </x:c>
+      <x:c r="E33" s="93" t="str">
+        <x:v>Number</x:v>
+      </x:c>
+      <x:c r="F33" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G33" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H33" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: No
+Hidden: No
+Virtual?: No
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="150" customHeight="1">
+      <x:c r="A34" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B34" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C34" s="93" t="str">
+        <x:v>poc_events</x:v>
+      </x:c>
+      <x:c r="D34" s="93" t="str">
+        <x:v>input_value</x:v>
+      </x:c>
+      <x:c r="E34" s="93" t="str">
+        <x:v>Number</x:v>
+      </x:c>
+      <x:c r="F34" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G34" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H34" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: No
+Hidden: No
+Virtual?: No
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="150" customHeight="1">
+      <x:c r="A35" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B35" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C35" s="93" t="str">
+        <x:v>poc_events</x:v>
+      </x:c>
+      <x:c r="D35" s="93" t="str">
+        <x:v>derived_value</x:v>
+      </x:c>
+      <x:c r="E35" s="93" t="str">
+        <x:v>Number</x:v>
+      </x:c>
+      <x:c r="F35" s="93" t="str">
+        <x:v>Test only; live appdoc reconciled</x:v>
+      </x:c>
+      <x:c r="G35" s="93" t="str">
+        <x:v>POC only; no OLTP/OLAP consumer</x:v>
+      </x:c>
+      <x:c r="H35" s="93" t="str">
+        <x:v>Key: No
+Label: No
+Read-Only: No
+Hidden: No
+Virtual?: No
+Reset on edit?: No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="150" customHeight="1">
+      <x:c r="A36" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B36" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C36" s="93" t="str">
+        <x:v>poc_source / poc_projection / poc_events</x:v>
+      </x:c>
+      <x:c r="D36" s="93" t="str">
+        <x:v>SQL key types</x:v>
+      </x:c>
+      <x:c r="E36" s="93" t="str">
+        <x:v>varchar</x:v>
+      </x:c>
+      <x:c r="F36" s="93" t="str">
+        <x:v>Test only; DDL and UI verified</x:v>
+      </x:c>
+      <x:c r="G36" s="93" t="str">
+        <x:v>Preserve exact key and Ref text; no uuid casts</x:v>
+      </x:c>
+      <x:c r="H36" s="93" t="str">
+        <x:v>source.id / projection.id / events.source_id: varchar(64)
+events.id: varchar(100)
+projection.id and events.source_id FK -&gt; source.id
+events UNIQUE(source_id, revision)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="150" customHeight="1">
+      <x:c r="A37" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B37" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C37" s="93" t="str">
+        <x:v>poc_source</x:v>
+      </x:c>
+      <x:c r="D37" s="93" t="str">
+        <x:v>AFTER UPDATE trigger</x:v>
+      </x:c>
+      <x:c r="E37" s="93" t="str">
+        <x:v>PL/pgSQL</x:v>
+      </x:c>
+      <x:c r="F37" s="93" t="str">
+        <x:v>Test only; engine + new GUI verified</x:v>
+      </x:c>
+      <x:c r="G37" s="93" t="str">
+        <x:v>One transaction changes source, projection and event</x:v>
+      </x:c>
+      <x:c r="H37" s="93" t="str">
+        <x:v>Unchanged input/revision -&gt; no-op. Otherwise revision=old+1. projection.derived_value=input_value::bigint*2; insert event id=source.id || single hyphen || revision. Negative input deliberately raises after downstream writes, rolling back the transaction. Exact SQL: scripts/cloud-sql-poc-schema.sql.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="150" customHeight="1">
+      <x:c r="A38" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B38" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C38" s="93" t="str">
+        <x:v>App</x:v>
+      </x:c>
+      <x:c r="D38" s="93" t="str">
+        <x:v>Sync settings</x:v>
+      </x:c>
+      <x:c r="E38" s="93" t="str">
+        <x:v>Configuration</x:v>
+      </x:c>
+      <x:c r="F38" s="93" t="str">
+        <x:v>Test only; UI verified before tests</x:v>
+      </x:c>
+      <x:c r="G38" s="93" t="str">
+        <x:v>Full sync required for this acceptance result</x:v>
+      </x:c>
+      <x:c r="H38" s="93" t="str">
+        <x:v>Server cache OFF; delta sync OFF; quick sync OFF; delayed sync OFF; automatic updates ON; sync on start OFF; new desktop design ON.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="150" customHeight="1">
+      <x:c r="A39" s="93" t="str">
+        <x:v>SQL POC</x:v>
+      </x:c>
+      <x:c r="B39" s="93" t="str">
+        <x:v>1.000008</x:v>
+      </x:c>
+      <x:c r="C39" s="93" t="str">
+        <x:v>App</x:v>
+      </x:c>
+      <x:c r="D39" s="93" t="str">
+        <x:v>Validation scope</x:v>
+      </x:c>
+      <x:c r="E39" s="93" t="str">
+        <x:v>Evidence</x:v>
+      </x:c>
+      <x:c r="F39" s="93" t="str">
+        <x:v>Owner acceptance pending</x:v>
+      </x:c>
+      <x:c r="G39" s="93" t="str">
+        <x:v>Results: POC_TEST_REPORT.md and ui-test-evidence.json</x:v>
+      </x:c>
+      <x:c r="H39" s="93" t="str">
+        <x:v>Uppercase and mixed-case updates, trigger propagation, parent Ref navigation and reverse related events passed. Full loan dataset key/Ref reconciliation, concurrency, offline and loan performance are pending.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4299,7 +5503,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40613c357604443c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44948d70ec54414d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14956,7 +16160,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb09b089999644e46"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R333cebd994c54469"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15385,7 +16589,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c64ae7a7f954995"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac3ce967758442ea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15845,7 +17049,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ba644b5b14846d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20a7c82882aa44a6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22819,7 +24023,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb2f9462cb394bf4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb26f1692330943fe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27438,7 +28642,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R196b4f6281b84e49"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R512ac91e94294119"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27637,7 +28841,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc396ec1e9a8432c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb76306cbb864d41"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29290,7 +30494,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref1d43f31d454711"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28fdf7c84b0641a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record failed migration cleanup and documented restart checkpoint
</commit_message>
<xml_diff>
--- a/Documents/AppSheet_Data_Dictionary.xlsx
+++ b/Documents/AppSheet_Data_Dictionary.xlsx
@@ -2,19 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R16ef4dce4a404f59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="R3a3c1dbe9cde4888"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R7d7c6d1b0b9b4855"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="Rf0274cd7b5cf4361"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="R795c4633819943b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R6a70cd4520b24fbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Rad8890efd2ad4c8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R4f71724f3ba14f40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="R99d46dde0e634099"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R3cb019cf2f464b6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="R37b3e1a8ef934be5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="Rc3e951c7837740e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Sync POC" sheetId="13" r:id="R1c3d80887d6444f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R2a51903f200049b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="R4b18e28353fd42f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="Rf4457ea5ad9e4679"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R0a6b44f9bd1c426a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="Ra94b83812d474397"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="Rec1a96e5461e41e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Racf454f55e914f95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R1e488bf945044610"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="R2866498f13144e6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R781c18d6bfd24003"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="Rd6834490d3b34c4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="R5daac30fb46d4b51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Sync POC" sheetId="13" r:id="R7f68816dae59450a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Migration Trial" sheetId="14" r:id="Rcb71592da0d84e82"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -99,7 +100,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="25">
+  <x:fills count="29">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -134,6 +135,26 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -351,7 +372,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="114">
+  <x:cellXfs count="120">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -596,6 +617,20 @@
     <x:xf numFmtId="0" fontId="11" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="12" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="12" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2503,7 +2538,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R392b43b532d44c18"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f8ff738ec7f4404"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5082,6 +5117,779 @@
       </x:c>
       <x:c r="H39" s="93" t="str">
         <x:v>Uppercase and mixed-case updates, trigger propagation, parent Ref navigation and reverse related events passed. Full loan dataset key/Ref reconciliation, concurrency, offline and loan performance are pending.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="38" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="55" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="100" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="119" t="str">
+        <x:v>Experiment</x:v>
+      </x:c>
+      <x:c r="B1" s="119" t="str">
+        <x:v>App version</x:v>
+      </x:c>
+      <x:c r="C1" s="119" t="str">
+        <x:v>Table</x:v>
+      </x:c>
+      <x:c r="D1" s="119" t="str">
+        <x:v>Column / setting</x:v>
+      </x:c>
+      <x:c r="E1" s="119" t="str">
+        <x:v>Type</x:v>
+      </x:c>
+      <x:c r="F1" s="119" t="str">
+        <x:v>Scope / status</x:v>
+      </x:c>
+      <x:c r="G1" s="119" t="str">
+        <x:v>Purpose / dependencies</x:v>
+      </x:c>
+      <x:c r="H1" s="119" t="str">
+        <x:v>Exact definition</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="55" customHeight="1">
+      <x:c r="A2" s="93" t="str">
+        <x:v>OLTP trial</x:v>
+      </x:c>
+      <x:c r="B2" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C2" s="93" t="str">
+        <x:v>Borrowers</x:v>
+      </x:c>
+      <x:c r="D2" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E2" s="93" t="str">
+        <x:v>AppSheet database</x:v>
+      </x:c>
+      <x:c r="F2" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G2" s="93" t="str">
+        <x:v>Shared native copy; source rollback 3.000064; clone rollback 1.000002</x:v>
+      </x:c>
+      <x:c r="H2" s="93" t="str">
+        <x:v>ID=base/GhFoIWUelX4UMyCCNLda80/tables/Iya7C1Iv_z4ZmO0tyMrMme</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="55" customHeight="1">
+      <x:c r="A3" s="93" t="str">
+        <x:v>OLTP trial</x:v>
+      </x:c>
+      <x:c r="B3" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C3" s="93" t="str">
+        <x:v>Loans</x:v>
+      </x:c>
+      <x:c r="D3" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E3" s="93" t="str">
+        <x:v>AppSheet database</x:v>
+      </x:c>
+      <x:c r="F3" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G3" s="93" t="str">
+        <x:v>Shared native copy; source rollback 3.000064; clone rollback 1.000002</x:v>
+      </x:c>
+      <x:c r="H3" s="93" t="str">
+        <x:v>ID=base/GhFoIWUelX4UMyCCNLda80/tables/uhIsbxFaUV4P2yCFRPUWoa</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="55" customHeight="1">
+      <x:c r="A4" s="93" t="str">
+        <x:v>OLTP trial</x:v>
+      </x:c>
+      <x:c r="B4" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C4" s="93" t="str">
+        <x:v>Repayments</x:v>
+      </x:c>
+      <x:c r="D4" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E4" s="93" t="str">
+        <x:v>AppSheet database</x:v>
+      </x:c>
+      <x:c r="F4" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G4" s="93" t="str">
+        <x:v>Shared native copy; source rollback 3.000064; clone rollback 1.000002</x:v>
+      </x:c>
+      <x:c r="H4" s="93" t="str">
+        <x:v>ID=base/GhFoIWUelX4UMyCCNLda80/tables/TA6YmxJirY4Y2DSpa7aR17</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="55" customHeight="1">
+      <x:c r="A5" s="93" t="str">
+        <x:v>OLTP trial</x:v>
+      </x:c>
+      <x:c r="B5" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C5" s="93" t="str">
+        <x:v>Statistics</x:v>
+      </x:c>
+      <x:c r="D5" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E5" s="93" t="str">
+        <x:v>AppSheet database</x:v>
+      </x:c>
+      <x:c r="F5" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G5" s="93" t="str">
+        <x:v>Shared native copy; source rollback 3.000064; clone rollback 1.000002</x:v>
+      </x:c>
+      <x:c r="H5" s="93" t="str">
+        <x:v>ID=base/GhFoIWUelX4UMyCCNLda80/tables/MoJ3e9N4iC4rE7kW9wLSt9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="55" customHeight="1">
+      <x:c r="A6" s="93" t="str">
+        <x:v>OLTP trial</x:v>
+      </x:c>
+      <x:c r="B6" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C6" s="93" t="str">
+        <x:v>Charges</x:v>
+      </x:c>
+      <x:c r="D6" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E6" s="93" t="str">
+        <x:v>AppSheet database</x:v>
+      </x:c>
+      <x:c r="F6" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G6" s="93" t="str">
+        <x:v>Shared native copy; source rollback 3.000064; clone rollback 1.000002</x:v>
+      </x:c>
+      <x:c r="H6" s="93" t="str">
+        <x:v>ID=base/GhFoIWUelX4UMyCCNLda80/tables/3EhKRaJBK64SAsNbtGBQU1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="55" customHeight="1">
+      <x:c r="A7" s="93" t="str">
+        <x:v>OLTP trial</x:v>
+      </x:c>
+      <x:c r="B7" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C7" s="93" t="str">
+        <x:v>Partners</x:v>
+      </x:c>
+      <x:c r="D7" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E7" s="93" t="str">
+        <x:v>AppSheet database</x:v>
+      </x:c>
+      <x:c r="F7" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G7" s="93" t="str">
+        <x:v>Shared native copy; source rollback 3.000064; clone rollback 1.000002</x:v>
+      </x:c>
+      <x:c r="H7" s="93" t="str">
+        <x:v>ID=base/GhFoIWUelX4UMyCCNLda80/tables/cxkDtKcsOZ4vm4kMSHOr66</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="55" customHeight="1">
+      <x:c r="A8" s="93" t="str">
+        <x:v>OLTP trial</x:v>
+      </x:c>
+      <x:c r="B8" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C8" s="93" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D8" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E8" s="93" t="str">
+        <x:v>AppSheet database</x:v>
+      </x:c>
+      <x:c r="F8" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G8" s="93" t="str">
+        <x:v>Shared native copy; source rollback 3.000064; clone rollback 1.000002</x:v>
+      </x:c>
+      <x:c r="H8" s="93" t="str">
+        <x:v>ID=base/GhFoIWUelX4UMyCCNLda80/tables/MFKNswyWeK4HYkVSIutpvb</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="55" customHeight="1">
+      <x:c r="A9" s="93" t="str">
+        <x:v>OLTP trial</x:v>
+      </x:c>
+      <x:c r="B9" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C9" s="93" t="str">
+        <x:v>Payments</x:v>
+      </x:c>
+      <x:c r="D9" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E9" s="93" t="str">
+        <x:v>AppSheet database</x:v>
+      </x:c>
+      <x:c r="F9" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G9" s="93" t="str">
+        <x:v>Shared native copy; source rollback 3.000064; clone rollback 1.000002</x:v>
+      </x:c>
+      <x:c r="H9" s="93" t="str">
+        <x:v>ID=base/GhFoIWUelX4UMyCCNLda80/tables/ULg9Cchxjz4oyzeQgeF-59</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="55" customHeight="1">
+      <x:c r="A10" s="93" t="str">
+        <x:v>OLAP trial</x:v>
+      </x:c>
+      <x:c r="B10" s="93" t="str">
+        <x:v>1.000004</x:v>
+      </x:c>
+      <x:c r="C10" s="93" t="str">
+        <x:v>Borrowers</x:v>
+      </x:c>
+      <x:c r="D10" s="93" t="str">
+        <x:v>Data source / permissions</x:v>
+      </x:c>
+      <x:c r="E10" s="93" t="str">
+        <x:v>AppSheet database</x:v>
+      </x:c>
+      <x:c r="F10" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G10" s="93" t="str">
+        <x:v>Shared native copy; source rollback 1.100041; clone rollback 1.000002</x:v>
+      </x:c>
+      <x:c r="H10" s="93" t="str">
+        <x:v>Database GhFoIWUelX4UMyCCNLda80; qualifier Borrowers; READ_ONLY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="55" customHeight="1">
+      <x:c r="A11" s="93" t="str">
+        <x:v>OLAP trial</x:v>
+      </x:c>
+      <x:c r="B11" s="93" t="str">
+        <x:v>1.000004</x:v>
+      </x:c>
+      <x:c r="C11" s="93" t="str">
+        <x:v>Loans</x:v>
+      </x:c>
+      <x:c r="D11" s="93" t="str">
+        <x:v>Data source / permissions</x:v>
+      </x:c>
+      <x:c r="E11" s="93" t="str">
+        <x:v>AppSheet database</x:v>
+      </x:c>
+      <x:c r="F11" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G11" s="93" t="str">
+        <x:v>Shared native copy; source rollback 1.100041; clone rollback 1.000002</x:v>
+      </x:c>
+      <x:c r="H11" s="93" t="str">
+        <x:v>Database GhFoIWUelX4UMyCCNLda80; qualifier Loans; READ_ONLY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="55" customHeight="1">
+      <x:c r="A12" s="93" t="str">
+        <x:v>OLAP trial</x:v>
+      </x:c>
+      <x:c r="B12" s="93" t="str">
+        <x:v>1.000004</x:v>
+      </x:c>
+      <x:c r="C12" s="93" t="str">
+        <x:v>Repayments</x:v>
+      </x:c>
+      <x:c r="D12" s="93" t="str">
+        <x:v>Data source / permissions</x:v>
+      </x:c>
+      <x:c r="E12" s="93" t="str">
+        <x:v>AppSheet database</x:v>
+      </x:c>
+      <x:c r="F12" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G12" s="93" t="str">
+        <x:v>Shared native copy; source rollback 1.100041; clone rollback 1.000002</x:v>
+      </x:c>
+      <x:c r="H12" s="93" t="str">
+        <x:v>Database GhFoIWUelX4UMyCCNLda80; qualifier Repayments; READ_ONLY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="55" customHeight="1">
+      <x:c r="A13" s="93" t="str">
+        <x:v>OLAP trial</x:v>
+      </x:c>
+      <x:c r="B13" s="93" t="str">
+        <x:v>1.000004</x:v>
+      </x:c>
+      <x:c r="C13" s="93" t="str">
+        <x:v>Statistics</x:v>
+      </x:c>
+      <x:c r="D13" s="93" t="str">
+        <x:v>Data source / permissions</x:v>
+      </x:c>
+      <x:c r="E13" s="93" t="str">
+        <x:v>AppSheet database</x:v>
+      </x:c>
+      <x:c r="F13" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G13" s="93" t="str">
+        <x:v>Shared native copy; source rollback 1.100041; clone rollback 1.000002</x:v>
+      </x:c>
+      <x:c r="H13" s="93" t="str">
+        <x:v>Database GhFoIWUelX4UMyCCNLda80; qualifier Statistics; ALL_CHANGES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="55" customHeight="1">
+      <x:c r="A14" s="93" t="str">
+        <x:v>OLAP trial</x:v>
+      </x:c>
+      <x:c r="B14" s="93" t="str">
+        <x:v>1.000004</x:v>
+      </x:c>
+      <x:c r="C14" s="93" t="str">
+        <x:v>Charges</x:v>
+      </x:c>
+      <x:c r="D14" s="93" t="str">
+        <x:v>Data source / permissions</x:v>
+      </x:c>
+      <x:c r="E14" s="93" t="str">
+        <x:v>AppSheet database</x:v>
+      </x:c>
+      <x:c r="F14" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G14" s="93" t="str">
+        <x:v>Shared native copy; source rollback 1.100041; clone rollback 1.000002</x:v>
+      </x:c>
+      <x:c r="H14" s="93" t="str">
+        <x:v>Database GhFoIWUelX4UMyCCNLda80; qualifier Charges; READ_ONLY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="55" customHeight="1">
+      <x:c r="A15" s="93" t="str">
+        <x:v>OLAP trial</x:v>
+      </x:c>
+      <x:c r="B15" s="93" t="str">
+        <x:v>1.000004</x:v>
+      </x:c>
+      <x:c r="C15" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D15" s="93" t="str">
+        <x:v>Data source / permissions</x:v>
+      </x:c>
+      <x:c r="E15" s="93" t="str">
+        <x:v>AppSheet database</x:v>
+      </x:c>
+      <x:c r="F15" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G15" s="93" t="str">
+        <x:v>Shared native copy; source rollback 1.100041; clone rollback 1.000002</x:v>
+      </x:c>
+      <x:c r="H15" s="93" t="str">
+        <x:v>Database GhFoIWUelX4UMyCCNLda80; qualifier Loan Assessment; ALL_CHANGES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="55" customHeight="1">
+      <x:c r="A16" s="93" t="str">
+        <x:v>OLAP trial</x:v>
+      </x:c>
+      <x:c r="B16" s="93" t="str">
+        <x:v>1.000004</x:v>
+      </x:c>
+      <x:c r="C16" s="93" t="str">
+        <x:v>Cash Pool Contributions</x:v>
+      </x:c>
+      <x:c r="D16" s="93" t="str">
+        <x:v>Data source / permissions</x:v>
+      </x:c>
+      <x:c r="E16" s="93" t="str">
+        <x:v>AppSheet database</x:v>
+      </x:c>
+      <x:c r="F16" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G16" s="93" t="str">
+        <x:v>Shared native copy; source rollback 1.100041; clone rollback 1.000002</x:v>
+      </x:c>
+      <x:c r="H16" s="93" t="str">
+        <x:v>Database GhFoIWUelX4UMyCCNLda80; qualifier Cash Pool Contributions; ADDS_AND_UPDATES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="55" customHeight="1">
+      <x:c r="A17" s="93" t="str">
+        <x:v>OLAP trial</x:v>
+      </x:c>
+      <x:c r="B17" s="93" t="str">
+        <x:v>1.000004</x:v>
+      </x:c>
+      <x:c r="C17" s="93" t="str">
+        <x:v>Partners</x:v>
+      </x:c>
+      <x:c r="D17" s="93" t="str">
+        <x:v>Data source / permissions</x:v>
+      </x:c>
+      <x:c r="E17" s="93" t="str">
+        <x:v>AppSheet database</x:v>
+      </x:c>
+      <x:c r="F17" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G17" s="93" t="str">
+        <x:v>Shared native copy; source rollback 1.100041; clone rollback 1.000002</x:v>
+      </x:c>
+      <x:c r="H17" s="93" t="str">
+        <x:v>Database GhFoIWUelX4UMyCCNLda80; qualifier Partners; ALL_CHANGES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="55" customHeight="1">
+      <x:c r="A18" s="93" t="str">
+        <x:v>OLAP trial</x:v>
+      </x:c>
+      <x:c r="B18" s="93" t="str">
+        <x:v>1.000004</x:v>
+      </x:c>
+      <x:c r="C18" s="93" t="str">
+        <x:v>Settlements</x:v>
+      </x:c>
+      <x:c r="D18" s="93" t="str">
+        <x:v>Data source / permissions</x:v>
+      </x:c>
+      <x:c r="E18" s="93" t="str">
+        <x:v>AppSheet database</x:v>
+      </x:c>
+      <x:c r="F18" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G18" s="93" t="str">
+        <x:v>Shared native copy; source rollback 1.100041; clone rollback 1.000002</x:v>
+      </x:c>
+      <x:c r="H18" s="93" t="str">
+        <x:v>Database GhFoIWUelX4UMyCCNLda80; qualifier Settlements; ALL_CHANGES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="55" customHeight="1">
+      <x:c r="A19" s="93" t="str">
+        <x:v>OLAP trial</x:v>
+      </x:c>
+      <x:c r="B19" s="93" t="str">
+        <x:v>1.000004</x:v>
+      </x:c>
+      <x:c r="C19" s="93" t="str">
+        <x:v>Daily Analytics</x:v>
+      </x:c>
+      <x:c r="D19" s="93" t="str">
+        <x:v>Data source / permissions</x:v>
+      </x:c>
+      <x:c r="E19" s="93" t="str">
+        <x:v>AppSheet database</x:v>
+      </x:c>
+      <x:c r="F19" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G19" s="93" t="str">
+        <x:v>Shared native copy; source rollback 1.100041; clone rollback 1.000002</x:v>
+      </x:c>
+      <x:c r="H19" s="93" t="str">
+        <x:v>Database GhFoIWUelX4UMyCCNLda80; qualifier Daily Analytics; ALL_CHANGES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="55" customHeight="1">
+      <x:c r="A20" s="93" t="str">
+        <x:v>OLAP trial</x:v>
+      </x:c>
+      <x:c r="B20" s="93" t="str">
+        <x:v>1.000004</x:v>
+      </x:c>
+      <x:c r="C20" s="93" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D20" s="93" t="str">
+        <x:v>Data source / permissions</x:v>
+      </x:c>
+      <x:c r="E20" s="93" t="str">
+        <x:v>AppSheet database</x:v>
+      </x:c>
+      <x:c r="F20" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G20" s="93" t="str">
+        <x:v>Shared native copy; source rollback 1.100041; clone rollback 1.000002</x:v>
+      </x:c>
+      <x:c r="H20" s="93" t="str">
+        <x:v>Database GhFoIWUelX4UMyCCNLda80; qualifier Payment Allocations; READ_ONLY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="55" customHeight="1">
+      <x:c r="A21" s="93" t="str">
+        <x:v>OLAP trial</x:v>
+      </x:c>
+      <x:c r="B21" s="93" t="str">
+        <x:v>1.000004</x:v>
+      </x:c>
+      <x:c r="C21" s="93" t="str">
+        <x:v>Payments</x:v>
+      </x:c>
+      <x:c r="D21" s="93" t="str">
+        <x:v>Data source / permissions</x:v>
+      </x:c>
+      <x:c r="E21" s="93" t="str">
+        <x:v>AppSheet database</x:v>
+      </x:c>
+      <x:c r="F21" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G21" s="93" t="str">
+        <x:v>Shared native copy; source rollback 1.100041; clone rollback 1.000002</x:v>
+      </x:c>
+      <x:c r="H21" s="93" t="str">
+        <x:v>Database GhFoIWUelX4UMyCCNLda80; qualifier Payments; READ_ONLY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="55" customHeight="1">
+      <x:c r="A22" s="93" t="str">
+        <x:v>OLAP trial</x:v>
+      </x:c>
+      <x:c r="B22" s="93" t="str">
+        <x:v>1.000004</x:v>
+      </x:c>
+      <x:c r="C22" s="93" t="str">
+        <x:v>Calendar</x:v>
+      </x:c>
+      <x:c r="D22" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E22" s="93" t="str">
+        <x:v>Google Sheets</x:v>
+      </x:c>
+      <x:c r="F22" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G22" s="93" t="str">
+        <x:v>Separate source outside shared native database</x:v>
+      </x:c>
+      <x:c r="H22" s="93" t="str">
+        <x:v>Calendar Help Table / Sheet1; READ_ONLY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="55" customHeight="1">
+      <x:c r="A23" s="93" t="str">
+        <x:v>OLTP trial</x:v>
+      </x:c>
+      <x:c r="B23" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C23" s="93" t="str">
+        <x:v>Automation</x:v>
+      </x:c>
+      <x:c r="D23" s="93" t="str">
+        <x:v>Notification - New Loan Created</x:v>
+      </x:c>
+      <x:c r="E23" s="93" t="str">
+        <x:v>Bot</x:v>
+      </x:c>
+      <x:c r="F23" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G23" s="93" t="str">
+        <x:v>Prevent notifications or scheduled mutations during migration</x:v>
+      </x:c>
+      <x:c r="H23" s="93" t="str">
+        <x:v>Disabled; production unchanged</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="55" customHeight="1">
+      <x:c r="A24" s="93" t="str">
+        <x:v>OLTP trial</x:v>
+      </x:c>
+      <x:c r="B24" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C24" s="93" t="str">
+        <x:v>Automation</x:v>
+      </x:c>
+      <x:c r="D24" s="93" t="str">
+        <x:v>Notification - Loan Closed</x:v>
+      </x:c>
+      <x:c r="E24" s="93" t="str">
+        <x:v>Bot</x:v>
+      </x:c>
+      <x:c r="F24" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G24" s="93" t="str">
+        <x:v>Prevent notifications or scheduled mutations during migration</x:v>
+      </x:c>
+      <x:c r="H24" s="93" t="str">
+        <x:v>Disabled; production unchanged</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="55" customHeight="1">
+      <x:c r="A25" s="93" t="str">
+        <x:v>OLTP trial</x:v>
+      </x:c>
+      <x:c r="B25" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C25" s="93" t="str">
+        <x:v>Automation</x:v>
+      </x:c>
+      <x:c r="D25" s="93" t="str">
+        <x:v>Notification - Charge Received</x:v>
+      </x:c>
+      <x:c r="E25" s="93" t="str">
+        <x:v>Bot</x:v>
+      </x:c>
+      <x:c r="F25" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G25" s="93" t="str">
+        <x:v>Prevent notifications or scheduled mutations during migration</x:v>
+      </x:c>
+      <x:c r="H25" s="93" t="str">
+        <x:v>Disabled; production unchanged</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="55" customHeight="1">
+      <x:c r="A26" s="93" t="str">
+        <x:v>OLTP trial</x:v>
+      </x:c>
+      <x:c r="B26" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C26" s="93" t="str">
+        <x:v>Automation</x:v>
+      </x:c>
+      <x:c r="D26" s="93" t="str">
+        <x:v>Generate Daily Charges</x:v>
+      </x:c>
+      <x:c r="E26" s="93" t="str">
+        <x:v>Bot</x:v>
+      </x:c>
+      <x:c r="F26" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G26" s="93" t="str">
+        <x:v>Prevent notifications or scheduled mutations during migration</x:v>
+      </x:c>
+      <x:c r="H26" s="93" t="str">
+        <x:v>Disabled; production unchanged</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="55" customHeight="1">
+      <x:c r="A27" s="93" t="str">
+        <x:v>OLAP trial</x:v>
+      </x:c>
+      <x:c r="B27" s="93" t="str">
+        <x:v>1.000004</x:v>
+      </x:c>
+      <x:c r="C27" s="93" t="str">
+        <x:v>Automation</x:v>
+      </x:c>
+      <x:c r="D27" s="93" t="str">
+        <x:v>Refresh Daily Analytics Daily 2</x:v>
+      </x:c>
+      <x:c r="E27" s="93" t="str">
+        <x:v>Bot</x:v>
+      </x:c>
+      <x:c r="F27" s="93" t="str">
+        <x:v>DELETED by owner request; historical configuration only</x:v>
+      </x:c>
+      <x:c r="G27" s="93" t="str">
+        <x:v>Other two bots already disabled</x:v>
+      </x:c>
+      <x:c r="H27" s="93" t="str">
+        <x:v>All three OLAP bots disabled; production unchanged</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="55" customHeight="1">
+      <x:c r="A28" s="93" t="str">
+        <x:v>SQL POC cleanup</x:v>
+      </x:c>
+      <x:c r="B28" s="93" t="str">
+        <x:v>Historical</x:v>
+      </x:c>
+      <x:c r="C28" s="93" t="str">
+        <x:v>All three synthetic POC tables</x:v>
+      </x:c>
+      <x:c r="D28" s="93" t="str">
+        <x:v>Backend deleted</x:v>
+      </x:c>
+      <x:c r="E28" s="93" t="str">
+        <x:v>PostgreSQL</x:v>
+      </x:c>
+      <x:c r="F28" s="93" t="str">
+        <x:v>DELETED by owner request</x:v>
+      </x:c>
+      <x:c r="G28" s="93" t="str">
+        <x:v>Existing SQL Sync POC app remains; backend unavailable</x:v>
+      </x:c>
+      <x:c r="H28" s="93" t="str">
+        <x:v>appsheet-pg-test-20260914 deletion confirmed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="55" customHeight="1">
+      <x:c r="A29" s="93" t="str">
+        <x:v>Fresh setup</x:v>
+      </x:c>
+      <x:c r="B29" s="93" t="str">
+        <x:v>Not created</x:v>
+      </x:c>
+      <x:c r="C29" s="93" t="str">
+        <x:v>No tables yet</x:v>
+      </x:c>
+      <x:c r="D29" s="93" t="str">
+        <x:v>Instance draft</x:v>
+      </x:c>
+      <x:c r="E29" s="93" t="str">
+        <x:v>PostgreSQL 18</x:v>
+      </x:c>
+      <x:c r="F29" s="93" t="str">
+        <x:v>UNSUBMITTED; password handoff pending</x:v>
+      </x:c>
+      <x:c r="G29" s="93" t="str">
+        <x:v>Copy original app using documented SQL copy workflow</x:v>
+      </x:c>
+      <x:c r="H29" s="93" t="str">
+        <x:v>appsheet-pg-prod-20260914; db-f1-micro; Singapore; single zone; 10 GB HDD; public IP; SSL-only</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5503,7 +6311,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44948d70ec54414d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raaccfb212f8b4af0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16160,7 +16968,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R333cebd994c54469"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R248039cf41224928"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16589,7 +17397,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac3ce967758442ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb21a841f4df4525"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17049,7 +17857,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20a7c82882aa44a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64c3ef939b93434c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24023,7 +24831,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb26f1692330943fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R453477b2163d4927"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28642,7 +29450,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R512ac91e94294119"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fd05bfb46214694"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28841,7 +29649,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb76306cbb864d41"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc9f6aa42dff461d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30494,7 +31302,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28fdf7c84b0641a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46d825d5fdc443fa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document clean SQL migration reproduction and PostgreSQL copy errors
</commit_message>
<xml_diff>
--- a/Documents/AppSheet_Data_Dictionary.xlsx
+++ b/Documents/AppSheet_Data_Dictionary.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R2a51903f200049b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="R4b18e28353fd42f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="Rf4457ea5ad9e4679"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R0a6b44f9bd1c426a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="Ra94b83812d474397"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="Rec1a96e5461e41e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Racf454f55e914f95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R1e488bf945044610"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="R2866498f13144e6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R781c18d6bfd24003"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="Rd6834490d3b34c4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="R5daac30fb46d4b51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Sync POC" sheetId="13" r:id="R7f68816dae59450a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Migration Trial" sheetId="14" r:id="Rcb71592da0d84e82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R56e4083ab8794a59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="R72ea041642594fba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R6019169fab574fc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R4de7abfc3f744cde"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="R52b4144bae784889"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R171dc5013b994a9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Rcb0e8bfa24fd491d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R0c253c55837b4300"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="Rdb3ada79839b4d29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R60d8610f8df043ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="R8e3c3f92534b414e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="R05e2c3a06e924062"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Sync POC" sheetId="13" r:id="R797cd80da9e44298"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Migration Trial" sheetId="14" r:id="Rcb8a72f1cfae4857"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -100,7 +100,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="29">
+  <x:fills count="30">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -135,6 +135,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -372,7 +377,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="120">
+  <x:cellXfs count="121">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -631,6 +636,9 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="12" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2538,7 +2546,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f8ff738ec7f4404"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R744e30cf91c94f45"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5139,28 +5147,28 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="119" t="str">
+      <x:c r="A1" s="120" t="str">
         <x:v>Experiment</x:v>
       </x:c>
-      <x:c r="B1" s="119" t="str">
+      <x:c r="B1" s="120" t="str">
         <x:v>App version</x:v>
       </x:c>
-      <x:c r="C1" s="119" t="str">
+      <x:c r="C1" s="120" t="str">
         <x:v>Table</x:v>
       </x:c>
-      <x:c r="D1" s="119" t="str">
+      <x:c r="D1" s="120" t="str">
         <x:v>Column / setting</x:v>
       </x:c>
-      <x:c r="E1" s="119" t="str">
+      <x:c r="E1" s="120" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="F1" s="119" t="str">
+      <x:c r="F1" s="120" t="str">
         <x:v>Scope / status</x:v>
       </x:c>
-      <x:c r="G1" s="119" t="str">
+      <x:c r="G1" s="120" t="str">
         <x:v>Purpose / dependencies</x:v>
       </x:c>
-      <x:c r="H1" s="119" t="str">
+      <x:c r="H1" s="120" t="str">
         <x:v>Exact definition</x:v>
       </x:c>
     </x:row>
@@ -5883,13 +5891,377 @@
         <x:v>PostgreSQL 18</x:v>
       </x:c>
       <x:c r="F29" s="93" t="str">
-        <x:v>UNSUBMITTED; password handoff pending</x:v>
+        <x:v>CREATED; official copy transfer blocked</x:v>
       </x:c>
       <x:c r="G29" s="93" t="str">
         <x:v>Copy original app using documented SQL copy workflow</x:v>
       </x:c>
       <x:c r="H29" s="93" t="str">
-        <x:v>appsheet-pg-prod-20260914; db-f1-micro; Singapore; single zone; 10 GB HDD; public IP; SSL-only</x:v>
+        <x:v>34.21.174.215; loan_manager_prod; 13 empty SQL tables; SSL database-2 verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="55" customHeight="1">
+      <x:c r="A30" s="93" t="str">
+        <x:v>Clean restart</x:v>
+      </x:c>
+      <x:c r="B30" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C30" s="93" t="str">
+        <x:v>Borrowers</x:v>
+      </x:c>
+      <x:c r="D30" s="93" t="str">
+        <x:v>SQL transfer status</x:v>
+      </x:c>
+      <x:c r="E30" s="93" t="str">
+        <x:v>PostgreSQL table</x:v>
+      </x:c>
+      <x:c r="F30" s="93" t="str">
+        <x:v>CREATED; 0 rows; not used by copied app</x:v>
+      </x:c>
+      <x:c r="G30" s="93" t="str">
+        <x:v>Schema types and data correctness not reconciled; preserve for diagnosis</x:v>
+      </x:c>
+      <x:c r="H30" s="93" t="str">
+        <x:v>public."Borrowers"; app 494cd013-0d9b-482f-9559-c9d83059de91 still uses original data sources</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="55" customHeight="1">
+      <x:c r="A31" s="93" t="str">
+        <x:v>Clean restart</x:v>
+      </x:c>
+      <x:c r="B31" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C31" s="93" t="str">
+        <x:v>Calendar</x:v>
+      </x:c>
+      <x:c r="D31" s="93" t="str">
+        <x:v>SQL transfer status</x:v>
+      </x:c>
+      <x:c r="E31" s="93" t="str">
+        <x:v>PostgreSQL table</x:v>
+      </x:c>
+      <x:c r="F31" s="93" t="str">
+        <x:v>CREATED; 0 rows; not used by copied app</x:v>
+      </x:c>
+      <x:c r="G31" s="93" t="str">
+        <x:v>Schema types and data correctness not reconciled; preserve for diagnosis</x:v>
+      </x:c>
+      <x:c r="H31" s="93" t="str">
+        <x:v>public."Calendar"; app 494cd013-0d9b-482f-9559-c9d83059de91 still uses original data sources</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="55" customHeight="1">
+      <x:c r="A32" s="93" t="str">
+        <x:v>Clean restart</x:v>
+      </x:c>
+      <x:c r="B32" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C32" s="93" t="str">
+        <x:v>Cash Pool Contributions</x:v>
+      </x:c>
+      <x:c r="D32" s="93" t="str">
+        <x:v>SQL transfer status</x:v>
+      </x:c>
+      <x:c r="E32" s="93" t="str">
+        <x:v>PostgreSQL table</x:v>
+      </x:c>
+      <x:c r="F32" s="93" t="str">
+        <x:v>CREATED; 0 rows; not used by copied app</x:v>
+      </x:c>
+      <x:c r="G32" s="93" t="str">
+        <x:v>Schema types and data correctness not reconciled; preserve for diagnosis</x:v>
+      </x:c>
+      <x:c r="H32" s="93" t="str">
+        <x:v>public."Cash Pool Contributions"; app 494cd013-0d9b-482f-9559-c9d83059de91 still uses original data sources</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="55" customHeight="1">
+      <x:c r="A33" s="93" t="str">
+        <x:v>Clean restart</x:v>
+      </x:c>
+      <x:c r="B33" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C33" s="93" t="str">
+        <x:v>Charges</x:v>
+      </x:c>
+      <x:c r="D33" s="93" t="str">
+        <x:v>SQL transfer status</x:v>
+      </x:c>
+      <x:c r="E33" s="93" t="str">
+        <x:v>PostgreSQL table</x:v>
+      </x:c>
+      <x:c r="F33" s="93" t="str">
+        <x:v>CREATED; 0 rows; not used by copied app</x:v>
+      </x:c>
+      <x:c r="G33" s="93" t="str">
+        <x:v>Schema types and data correctness not reconciled; preserve for diagnosis</x:v>
+      </x:c>
+      <x:c r="H33" s="93" t="str">
+        <x:v>public."Charges"; app 494cd013-0d9b-482f-9559-c9d83059de91 still uses original data sources</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="55" customHeight="1">
+      <x:c r="A34" s="93" t="str">
+        <x:v>Clean restart</x:v>
+      </x:c>
+      <x:c r="B34" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C34" s="93" t="str">
+        <x:v>Daily Analytics</x:v>
+      </x:c>
+      <x:c r="D34" s="93" t="str">
+        <x:v>SQL transfer status</x:v>
+      </x:c>
+      <x:c r="E34" s="93" t="str">
+        <x:v>PostgreSQL table</x:v>
+      </x:c>
+      <x:c r="F34" s="93" t="str">
+        <x:v>CREATED; 0 rows; not used by copied app</x:v>
+      </x:c>
+      <x:c r="G34" s="93" t="str">
+        <x:v>Schema types and data correctness not reconciled; preserve for diagnosis</x:v>
+      </x:c>
+      <x:c r="H34" s="93" t="str">
+        <x:v>public."Daily Analytics"; app 494cd013-0d9b-482f-9559-c9d83059de91 still uses original data sources</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="55" customHeight="1">
+      <x:c r="A35" s="93" t="str">
+        <x:v>Clean restart</x:v>
+      </x:c>
+      <x:c r="B35" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C35" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D35" s="93" t="str">
+        <x:v>SQL transfer status</x:v>
+      </x:c>
+      <x:c r="E35" s="93" t="str">
+        <x:v>PostgreSQL table</x:v>
+      </x:c>
+      <x:c r="F35" s="93" t="str">
+        <x:v>CREATED; 0 rows; not used by copied app</x:v>
+      </x:c>
+      <x:c r="G35" s="93" t="str">
+        <x:v>Schema types and data correctness not reconciled; preserve for diagnosis</x:v>
+      </x:c>
+      <x:c r="H35" s="93" t="str">
+        <x:v>public."Loan Assessment"; app 494cd013-0d9b-482f-9559-c9d83059de91 still uses original data sources</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="55" customHeight="1">
+      <x:c r="A36" s="93" t="str">
+        <x:v>Clean restart</x:v>
+      </x:c>
+      <x:c r="B36" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C36" s="93" t="str">
+        <x:v>Loans</x:v>
+      </x:c>
+      <x:c r="D36" s="93" t="str">
+        <x:v>SQL transfer status</x:v>
+      </x:c>
+      <x:c r="E36" s="93" t="str">
+        <x:v>PostgreSQL table</x:v>
+      </x:c>
+      <x:c r="F36" s="93" t="str">
+        <x:v>CREATED; 0 rows; not used by copied app</x:v>
+      </x:c>
+      <x:c r="G36" s="93" t="str">
+        <x:v>Schema types and data correctness not reconciled; preserve for diagnosis</x:v>
+      </x:c>
+      <x:c r="H36" s="93" t="str">
+        <x:v>public."Loans"; app 494cd013-0d9b-482f-9559-c9d83059de91 still uses original data sources</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="55" customHeight="1">
+      <x:c r="A37" s="93" t="str">
+        <x:v>Clean restart</x:v>
+      </x:c>
+      <x:c r="B37" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C37" s="93" t="str">
+        <x:v>Partners</x:v>
+      </x:c>
+      <x:c r="D37" s="93" t="str">
+        <x:v>SQL transfer status</x:v>
+      </x:c>
+      <x:c r="E37" s="93" t="str">
+        <x:v>PostgreSQL table</x:v>
+      </x:c>
+      <x:c r="F37" s="93" t="str">
+        <x:v>CREATED; 0 rows; not used by copied app</x:v>
+      </x:c>
+      <x:c r="G37" s="93" t="str">
+        <x:v>Schema types and data correctness not reconciled; preserve for diagnosis</x:v>
+      </x:c>
+      <x:c r="H37" s="93" t="str">
+        <x:v>public."Partners"; app 494cd013-0d9b-482f-9559-c9d83059de91 still uses original data sources</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="55" customHeight="1">
+      <x:c r="A38" s="93" t="str">
+        <x:v>Clean restart</x:v>
+      </x:c>
+      <x:c r="B38" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C38" s="93" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D38" s="93" t="str">
+        <x:v>SQL transfer status</x:v>
+      </x:c>
+      <x:c r="E38" s="93" t="str">
+        <x:v>PostgreSQL table</x:v>
+      </x:c>
+      <x:c r="F38" s="93" t="str">
+        <x:v>CREATED; 0 rows; not used by copied app</x:v>
+      </x:c>
+      <x:c r="G38" s="93" t="str">
+        <x:v>Schema types and data correctness not reconciled; preserve for diagnosis</x:v>
+      </x:c>
+      <x:c r="H38" s="93" t="str">
+        <x:v>public."Payment Allocations"; app 494cd013-0d9b-482f-9559-c9d83059de91 still uses original data sources</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="55" customHeight="1">
+      <x:c r="A39" s="93" t="str">
+        <x:v>Clean restart</x:v>
+      </x:c>
+      <x:c r="B39" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C39" s="93" t="str">
+        <x:v>Payments</x:v>
+      </x:c>
+      <x:c r="D39" s="93" t="str">
+        <x:v>SQL transfer status</x:v>
+      </x:c>
+      <x:c r="E39" s="93" t="str">
+        <x:v>PostgreSQL table</x:v>
+      </x:c>
+      <x:c r="F39" s="93" t="str">
+        <x:v>CREATED; 0 rows; not used by copied app</x:v>
+      </x:c>
+      <x:c r="G39" s="93" t="str">
+        <x:v>Schema types and data correctness not reconciled; preserve for diagnosis</x:v>
+      </x:c>
+      <x:c r="H39" s="93" t="str">
+        <x:v>public."Payments"; app 494cd013-0d9b-482f-9559-c9d83059de91 still uses original data sources</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="55" customHeight="1">
+      <x:c r="A40" s="93" t="str">
+        <x:v>Clean restart</x:v>
+      </x:c>
+      <x:c r="B40" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C40" s="93" t="str">
+        <x:v>Repayments</x:v>
+      </x:c>
+      <x:c r="D40" s="93" t="str">
+        <x:v>SQL transfer status</x:v>
+      </x:c>
+      <x:c r="E40" s="93" t="str">
+        <x:v>PostgreSQL table</x:v>
+      </x:c>
+      <x:c r="F40" s="93" t="str">
+        <x:v>CREATED; 0 rows; not used by copied app</x:v>
+      </x:c>
+      <x:c r="G40" s="93" t="str">
+        <x:v>Schema types and data correctness not reconciled; preserve for diagnosis</x:v>
+      </x:c>
+      <x:c r="H40" s="93" t="str">
+        <x:v>public."Repayments"; app 494cd013-0d9b-482f-9559-c9d83059de91 still uses original data sources</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="55" customHeight="1">
+      <x:c r="A41" s="93" t="str">
+        <x:v>Clean restart</x:v>
+      </x:c>
+      <x:c r="B41" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C41" s="93" t="str">
+        <x:v>Settlements</x:v>
+      </x:c>
+      <x:c r="D41" s="93" t="str">
+        <x:v>SQL transfer status</x:v>
+      </x:c>
+      <x:c r="E41" s="93" t="str">
+        <x:v>PostgreSQL table</x:v>
+      </x:c>
+      <x:c r="F41" s="93" t="str">
+        <x:v>CREATED; 0 rows; not used by copied app</x:v>
+      </x:c>
+      <x:c r="G41" s="93" t="str">
+        <x:v>Schema types and data correctness not reconciled; preserve for diagnosis</x:v>
+      </x:c>
+      <x:c r="H41" s="93" t="str">
+        <x:v>public."Settlements"; app 494cd013-0d9b-482f-9559-c9d83059de91 still uses original data sources</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="55" customHeight="1">
+      <x:c r="A42" s="93" t="str">
+        <x:v>Clean restart</x:v>
+      </x:c>
+      <x:c r="B42" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C42" s="93" t="str">
+        <x:v>Statistics</x:v>
+      </x:c>
+      <x:c r="D42" s="93" t="str">
+        <x:v>SQL transfer status</x:v>
+      </x:c>
+      <x:c r="E42" s="93" t="str">
+        <x:v>PostgreSQL table</x:v>
+      </x:c>
+      <x:c r="F42" s="93" t="str">
+        <x:v>CREATED; 0 rows; not used by copied app</x:v>
+      </x:c>
+      <x:c r="G42" s="93" t="str">
+        <x:v>Schema types and data correctness not reconciled; preserve for diagnosis</x:v>
+      </x:c>
+      <x:c r="H42" s="93" t="str">
+        <x:v>public."Statistics"; app 494cd013-0d9b-482f-9559-c9d83059de91 still uses original data sources</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="55" customHeight="1">
+      <x:c r="A43" s="93" t="str">
+        <x:v>Clean restart</x:v>
+      </x:c>
+      <x:c r="B43" s="93" t="str">
+        <x:v>1.000003</x:v>
+      </x:c>
+      <x:c r="C43" s="93" t="str">
+        <x:v>Automation</x:v>
+      </x:c>
+      <x:c r="D43" s="93" t="str">
+        <x:v>Refresh Daily Analytics Daily 2</x:v>
+      </x:c>
+      <x:c r="E43" s="93" t="str">
+        <x:v>Bot</x:v>
+      </x:c>
+      <x:c r="F43" s="93" t="str">
+        <x:v>DISABLED in copied app</x:v>
+      </x:c>
+      <x:c r="G43" s="93" t="str">
+        <x:v>Prevent scheduled writes to original sources; rollback 1.000002</x:v>
+      </x:c>
+      <x:c r="H43" s="93" t="str">
+        <x:v>Disabled; Refresh Daily Analytics Daily already disabled</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6311,7 +6683,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raaccfb212f8b4af0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5c9fe4033dd4b44"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16968,7 +17340,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R248039cf41224928"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15cf8c62969a4ebf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17397,7 +17769,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb21a841f4df4525"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67018b76133e4a93"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17857,7 +18229,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64c3ef939b93434c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ca5c585eae54427"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24831,7 +25203,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R453477b2163d4927"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5a6382b59f34226"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29450,7 +29822,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fd05bfb46214694"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16beae1c0aaa4d14"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29649,7 +30021,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc9f6aa42dff461d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9493056924574cf1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31302,7 +31674,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46d825d5fdc443fa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f64535a51d64121"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document verified Statistics manual PostgreSQL migration trial
</commit_message>
<xml_diff>
--- a/Documents/AppSheet_Data_Dictionary.xlsx
+++ b/Documents/AppSheet_Data_Dictionary.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R56e4083ab8794a59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="R72ea041642594fba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R6019169fab574fc4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R4de7abfc3f744cde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="R52b4144bae784889"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R171dc5013b994a9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Rcb0e8bfa24fd491d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R0c253c55837b4300"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="Rdb3ada79839b4d29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R60d8610f8df043ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="R8e3c3f92534b414e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="R05e2c3a06e924062"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Sync POC" sheetId="13" r:id="R797cd80da9e44298"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Migration Trial" sheetId="14" r:id="Rcb8a72f1cfae4857"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Re00d28e4307f4496"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="Rca873092791f4db3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="Rfd61cd50b99442cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R7f273980703b4f37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="R669fcf656b4e4bdb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R593bbe8299d64d7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="R461adc2bbb9f4c13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="Rcbf11a1877f44017"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="R56dfa8d28a4d4fb0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="Rc97794ccaaba4d3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="Rc7b7f5d5e04e4dc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="R63bb829c1f9f4c15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Sync POC" sheetId="13" r:id="R1398610c05a64cf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Migration Trial" sheetId="14" r:id="R473eea63780f4761"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -100,7 +100,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="30">
+  <x:fills count="31">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -135,6 +135,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -377,7 +382,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="121">
+  <x:cellXfs count="122">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -639,6 +644,9 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="12" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2546,7 +2554,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R744e30cf91c94f45"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2708053733d48c4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5147,28 +5155,28 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="120" t="str">
+      <x:c r="A1" s="121" t="str">
         <x:v>Experiment</x:v>
       </x:c>
-      <x:c r="B1" s="120" t="str">
+      <x:c r="B1" s="121" t="str">
         <x:v>App version</x:v>
       </x:c>
-      <x:c r="C1" s="120" t="str">
+      <x:c r="C1" s="121" t="str">
         <x:v>Table</x:v>
       </x:c>
-      <x:c r="D1" s="120" t="str">
+      <x:c r="D1" s="121" t="str">
         <x:v>Column / setting</x:v>
       </x:c>
-      <x:c r="E1" s="120" t="str">
+      <x:c r="E1" s="121" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="F1" s="120" t="str">
+      <x:c r="F1" s="121" t="str">
         <x:v>Scope / status</x:v>
       </x:c>
-      <x:c r="G1" s="120" t="str">
+      <x:c r="G1" s="121" t="str">
         <x:v>Purpose / dependencies</x:v>
       </x:c>
-      <x:c r="H1" s="120" t="str">
+      <x:c r="H1" s="121" t="str">
         <x:v>Exact definition</x:v>
       </x:c>
     </x:row>
@@ -6217,7 +6225,7 @@
         <x:v>Clean restart</x:v>
       </x:c>
       <x:c r="B42" s="93" t="str">
-        <x:v>1.000003</x:v>
+        <x:v>1.000004</x:v>
       </x:c>
       <x:c r="C42" s="93" t="str">
         <x:v>Statistics</x:v>
@@ -6229,13 +6237,13 @@
         <x:v>PostgreSQL table</x:v>
       </x:c>
       <x:c r="F42" s="93" t="str">
-        <x:v>CREATED; 0 rows; not used by copied app</x:v>
+        <x:v>MANUAL COPY PASSED; 1 exact row</x:v>
       </x:c>
       <x:c r="G42" s="93" t="str">
-        <x:v>Schema types and data correctness not reconciled; preserve for diagnosis</x:v>
+        <x:v>39 Statistics column configurations preserved; eight dashboard metrics match; other tables still original</x:v>
       </x:c>
       <x:c r="H42" s="93" t="str">
-        <x:v>public."Statistics"; app 494cd013-0d9b-482f-9559-c9d83059de91 still uses original data sources</x:v>
+        <x:v>database-2; Source Path Statistics; Table=public.Statistics__Statistics</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="55" customHeight="1">
@@ -6262,6 +6270,58 @@
       </x:c>
       <x:c r="H43" s="93" t="str">
         <x:v>Disabled; Refresh Daily Analytics Daily already disabled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="55" customHeight="1">
+      <x:c r="A44" s="93" t="str">
+        <x:v>Statistics manual</x:v>
+      </x:c>
+      <x:c r="B44" s="93" t="str">
+        <x:v>1.000004</x:v>
+      </x:c>
+      <x:c r="C44" s="93" t="str">
+        <x:v>Statistics</x:v>
+      </x:c>
+      <x:c r="D44" s="93" t="str">
+        <x:v>Row ID</x:v>
+      </x:c>
+      <x:c r="E44" s="93" t="str">
+        <x:v>Text / SQL text</x:v>
+      </x:c>
+      <x:c r="F44" s="93" t="str">
+        <x:v>Physical key; exact source key copied</x:v>
+      </x:c>
+      <x:c r="G44" s="93" t="str">
+        <x:v>Not nullable; no SQL default; unchanged app settings</x:v>
+      </x:c>
+      <x:c r="H44" s="93" t="str">
+        <x:v>Key Yes; Initial value UNIQUEID("PackedUUID"); Read-Only Yes; no normalization</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="55" customHeight="1">
+      <x:c r="A45" s="93" t="str">
+        <x:v>Statistics manual</x:v>
+      </x:c>
+      <x:c r="B45" s="93" t="str">
+        <x:v>1.000004</x:v>
+      </x:c>
+      <x:c r="C45" s="93" t="str">
+        <x:v>Statistics</x:v>
+      </x:c>
+      <x:c r="D45" s="93" t="str">
+        <x:v>Statistics ID</x:v>
+      </x:c>
+      <x:c r="E45" s="93" t="str">
+        <x:v>Text / SQL text</x:v>
+      </x:c>
+      <x:c r="F45" s="93" t="str">
+        <x:v>Physical label; MAIN copied</x:v>
+      </x:c>
+      <x:c r="G45" s="93" t="str">
+        <x:v>Nullable; no SQL default; unchanged app settings</x:v>
+      </x:c>
+      <x:c r="H45" s="93" t="str">
+        <x:v>Label Yes; Read-Only No; one row</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6683,7 +6743,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5c9fe4033dd4b44"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96c3d0ef9da743b4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17340,7 +17400,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15cf8c62969a4ebf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8d9f438897c453f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17769,7 +17829,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67018b76133e4a93"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R576798a7d0bf4450"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18229,7 +18289,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ca5c585eae54427"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbe18dbd49a74e09"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25203,7 +25263,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5a6382b59f34226"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2308807ce4d84f18"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29822,7 +29882,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16beae1c0aaa4d14"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R829a6bbc7b6b464e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30021,7 +30081,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9493056924574cf1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf459737b2ac45b5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31674,7 +31734,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f64535a51d64121"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R126a37544b1b4181"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Migrate all native tables in OLAP PostgreSQL trial and verify data
</commit_message>
<xml_diff>
--- a/Documents/AppSheet_Data_Dictionary.xlsx
+++ b/Documents/AppSheet_Data_Dictionary.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Re00d28e4307f4496"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="Rca873092791f4db3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="Rfd61cd50b99442cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R7f273980703b4f37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="R669fcf656b4e4bdb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R593bbe8299d64d7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="R461adc2bbb9f4c13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="Rcbf11a1877f44017"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="R56dfa8d28a4d4fb0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="Rc97794ccaaba4d3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="Rc7b7f5d5e04e4dc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="R63bb829c1f9f4c15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Sync POC" sheetId="13" r:id="R1398610c05a64cf4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Migration Trial" sheetId="14" r:id="R473eea63780f4761"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R0cf92f2c00ff4e1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="Rf66215da1caf44f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="Rfbf9b2e2e07243fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="Rf9557621dbef4d0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="R1a0b3883428b4bde"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="Rf13958d1aff0438f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="R3cd6c6a1ef3c4c26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R8fa53bf809984729"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="Ra3b9441c805d4311"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="Rf16b15d151074b5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="Rbe2c42ac0bc3428c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="R84861ec9994d41f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Sync POC" sheetId="13" r:id="Rf31c3c015d484f7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Migration Trial" sheetId="14" r:id="Rf8ba14654f974d83"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -100,7 +100,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="31">
+  <x:fills count="32">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -135,6 +135,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -382,7 +387,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="122">
+  <x:cellXfs count="123">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -647,6 +652,9 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="12" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2554,7 +2562,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2708053733d48c4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55aa89467b404526"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5155,28 +5163,28 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="121" t="str">
+      <x:c r="A1" s="122" t="str">
         <x:v>Experiment</x:v>
       </x:c>
-      <x:c r="B1" s="121" t="str">
+      <x:c r="B1" s="122" t="str">
         <x:v>App version</x:v>
       </x:c>
-      <x:c r="C1" s="121" t="str">
+      <x:c r="C1" s="122" t="str">
         <x:v>Table</x:v>
       </x:c>
-      <x:c r="D1" s="121" t="str">
+      <x:c r="D1" s="122" t="str">
         <x:v>Column / setting</x:v>
       </x:c>
-      <x:c r="E1" s="121" t="str">
+      <x:c r="E1" s="122" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="F1" s="121" t="str">
+      <x:c r="F1" s="122" t="str">
         <x:v>Scope / status</x:v>
       </x:c>
-      <x:c r="G1" s="121" t="str">
+      <x:c r="G1" s="122" t="str">
         <x:v>Purpose / dependencies</x:v>
       </x:c>
-      <x:c r="H1" s="121" t="str">
+      <x:c r="H1" s="122" t="str">
         <x:v>Exact definition</x:v>
       </x:c>
     </x:row>
@@ -5913,7 +5921,7 @@
         <x:v>Clean restart</x:v>
       </x:c>
       <x:c r="B30" s="93" t="str">
-        <x:v>1.000003</x:v>
+        <x:v>1.000007</x:v>
       </x:c>
       <x:c r="C30" s="93" t="str">
         <x:v>Borrowers</x:v>
@@ -5925,13 +5933,13 @@
         <x:v>PostgreSQL table</x:v>
       </x:c>
       <x:c r="F30" s="93" t="str">
-        <x:v>CREATED; 0 rows; not used by copied app</x:v>
+        <x:v>COPIED AND VERIFIED; 29 rows</x:v>
       </x:c>
       <x:c r="G30" s="93" t="str">
-        <x:v>Schema types and data correctness not reconciled; preserve for diagnosis</x:v>
+        <x:v>Trial now reads SQL; all stored fields and related membership verified</x:v>
       </x:c>
       <x:c r="H30" s="93" t="str">
-        <x:v>public."Borrowers"; app 494cd013-0d9b-482f-9559-c9d83059de91 still uses original data sources</x:v>
+        <x:v>public."Borrowers"; 11 physical columns; exact keys and all fields matched</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="55" customHeight="1">
@@ -5965,7 +5973,7 @@
         <x:v>Clean restart</x:v>
       </x:c>
       <x:c r="B32" s="93" t="str">
-        <x:v>1.000003</x:v>
+        <x:v>1.000007</x:v>
       </x:c>
       <x:c r="C32" s="93" t="str">
         <x:v>Cash Pool Contributions</x:v>
@@ -5977,13 +5985,13 @@
         <x:v>PostgreSQL table</x:v>
       </x:c>
       <x:c r="F32" s="93" t="str">
-        <x:v>CREATED; 0 rows; not used by copied app</x:v>
+        <x:v>COPIED AND VERIFIED; 5 rows</x:v>
       </x:c>
       <x:c r="G32" s="93" t="str">
-        <x:v>Schema types and data correctness not reconciled; preserve for diagnosis</x:v>
+        <x:v>Trial now reads SQL; all stored fields and related membership verified</x:v>
       </x:c>
       <x:c r="H32" s="93" t="str">
-        <x:v>public."Cash Pool Contributions"; app 494cd013-0d9b-482f-9559-c9d83059de91 still uses original data sources</x:v>
+        <x:v>public."Cash Pool Contributions"; 6 physical columns; exact keys and all fields matched</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="55" customHeight="1">
@@ -5991,7 +5999,7 @@
         <x:v>Clean restart</x:v>
       </x:c>
       <x:c r="B33" s="93" t="str">
-        <x:v>1.000003</x:v>
+        <x:v>1.000007</x:v>
       </x:c>
       <x:c r="C33" s="93" t="str">
         <x:v>Charges</x:v>
@@ -6003,13 +6011,13 @@
         <x:v>PostgreSQL table</x:v>
       </x:c>
       <x:c r="F33" s="93" t="str">
-        <x:v>CREATED; 0 rows; not used by copied app</x:v>
+        <x:v>COPIED AND VERIFIED; 745 rows</x:v>
       </x:c>
       <x:c r="G33" s="93" t="str">
-        <x:v>Schema types and data correctness not reconciled; preserve for diagnosis</x:v>
+        <x:v>Trial now reads SQL; all stored fields and related membership verified</x:v>
       </x:c>
       <x:c r="H33" s="93" t="str">
-        <x:v>public."Charges"; app 494cd013-0d9b-482f-9559-c9d83059de91 still uses original data sources</x:v>
+        <x:v>public."Charges"; 6 physical columns; exact keys and all fields matched</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="55" customHeight="1">
@@ -6017,7 +6025,7 @@
         <x:v>Clean restart</x:v>
       </x:c>
       <x:c r="B34" s="93" t="str">
-        <x:v>1.000003</x:v>
+        <x:v>1.000007</x:v>
       </x:c>
       <x:c r="C34" s="93" t="str">
         <x:v>Daily Analytics</x:v>
@@ -6029,13 +6037,13 @@
         <x:v>PostgreSQL table</x:v>
       </x:c>
       <x:c r="F34" s="93" t="str">
-        <x:v>CREATED; 0 rows; not used by copied app</x:v>
+        <x:v>COPIED AND VERIFIED; 41 rows</x:v>
       </x:c>
       <x:c r="G34" s="93" t="str">
-        <x:v>Schema types and data correctness not reconciled; preserve for diagnosis</x:v>
+        <x:v>Trial now reads SQL; all stored fields and related membership verified</x:v>
       </x:c>
       <x:c r="H34" s="93" t="str">
-        <x:v>public."Daily Analytics"; app 494cd013-0d9b-482f-9559-c9d83059de91 still uses original data sources</x:v>
+        <x:v>public."Daily Analytics"; 16 physical columns; exact keys and all fields matched</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="55" customHeight="1">
@@ -6043,7 +6051,7 @@
         <x:v>Clean restart</x:v>
       </x:c>
       <x:c r="B35" s="93" t="str">
-        <x:v>1.000003</x:v>
+        <x:v>1.000007</x:v>
       </x:c>
       <x:c r="C35" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -6055,13 +6063,13 @@
         <x:v>PostgreSQL table</x:v>
       </x:c>
       <x:c r="F35" s="93" t="str">
-        <x:v>CREATED; 0 rows; not used by copied app</x:v>
+        <x:v>COPIED AND VERIFIED; 1 rows</x:v>
       </x:c>
       <x:c r="G35" s="93" t="str">
-        <x:v>Schema types and data correctness not reconciled; preserve for diagnosis</x:v>
+        <x:v>Trial now reads SQL; all stored fields and related membership verified</x:v>
       </x:c>
       <x:c r="H35" s="93" t="str">
-        <x:v>public."Loan Assessment"; app 494cd013-0d9b-482f-9559-c9d83059de91 still uses original data sources</x:v>
+        <x:v>public."Loan Assessment"; 5 physical columns; exact keys and all fields matched</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="55" customHeight="1">
@@ -6069,7 +6077,7 @@
         <x:v>Clean restart</x:v>
       </x:c>
       <x:c r="B36" s="93" t="str">
-        <x:v>1.000003</x:v>
+        <x:v>1.000007</x:v>
       </x:c>
       <x:c r="C36" s="93" t="str">
         <x:v>Loans</x:v>
@@ -6081,13 +6089,13 @@
         <x:v>PostgreSQL table</x:v>
       </x:c>
       <x:c r="F36" s="93" t="str">
-        <x:v>CREATED; 0 rows; not used by copied app</x:v>
+        <x:v>COPIED AND VERIFIED; 62 rows</x:v>
       </x:c>
       <x:c r="G36" s="93" t="str">
-        <x:v>Schema types and data correctness not reconciled; preserve for diagnosis</x:v>
+        <x:v>Trial now reads SQL; all stored fields and related membership verified</x:v>
       </x:c>
       <x:c r="H36" s="93" t="str">
-        <x:v>public."Loans"; app 494cd013-0d9b-482f-9559-c9d83059de91 still uses original data sources</x:v>
+        <x:v>public."Loans"; 20 physical columns; exact keys and all fields matched</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="55" customHeight="1">
@@ -6095,7 +6103,7 @@
         <x:v>Clean restart</x:v>
       </x:c>
       <x:c r="B37" s="93" t="str">
-        <x:v>1.000003</x:v>
+        <x:v>1.000007</x:v>
       </x:c>
       <x:c r="C37" s="93" t="str">
         <x:v>Partners</x:v>
@@ -6107,13 +6115,13 @@
         <x:v>PostgreSQL table</x:v>
       </x:c>
       <x:c r="F37" s="93" t="str">
-        <x:v>CREATED; 0 rows; not used by copied app</x:v>
+        <x:v>COPIED AND VERIFIED; 2 rows</x:v>
       </x:c>
       <x:c r="G37" s="93" t="str">
-        <x:v>Schema types and data correctness not reconciled; preserve for diagnosis</x:v>
+        <x:v>Trial now reads SQL; all stored fields and related membership verified</x:v>
       </x:c>
       <x:c r="H37" s="93" t="str">
-        <x:v>public."Partners"; app 494cd013-0d9b-482f-9559-c9d83059de91 still uses original data sources</x:v>
+        <x:v>public."Partners"; 7 physical columns; exact keys and all fields matched</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="55" customHeight="1">
@@ -6121,7 +6129,7 @@
         <x:v>Clean restart</x:v>
       </x:c>
       <x:c r="B38" s="93" t="str">
-        <x:v>1.000003</x:v>
+        <x:v>1.000007</x:v>
       </x:c>
       <x:c r="C38" s="93" t="str">
         <x:v>Payment Allocations</x:v>
@@ -6133,13 +6141,13 @@
         <x:v>PostgreSQL table</x:v>
       </x:c>
       <x:c r="F38" s="93" t="str">
-        <x:v>CREATED; 0 rows; not used by copied app</x:v>
+        <x:v>COPIED AND VERIFIED; 263 rows</x:v>
       </x:c>
       <x:c r="G38" s="93" t="str">
-        <x:v>Schema types and data correctness not reconciled; preserve for diagnosis</x:v>
+        <x:v>Trial now reads SQL; all stored fields and related membership verified</x:v>
       </x:c>
       <x:c r="H38" s="93" t="str">
-        <x:v>public."Payment Allocations"; app 494cd013-0d9b-482f-9559-c9d83059de91 still uses original data sources</x:v>
+        <x:v>public."Payment Allocations"; 13 physical columns; exact keys and all fields matched</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="55" customHeight="1">
@@ -6147,7 +6155,7 @@
         <x:v>Clean restart</x:v>
       </x:c>
       <x:c r="B39" s="93" t="str">
-        <x:v>1.000003</x:v>
+        <x:v>1.000007</x:v>
       </x:c>
       <x:c r="C39" s="93" t="str">
         <x:v>Payments</x:v>
@@ -6159,13 +6167,13 @@
         <x:v>PostgreSQL table</x:v>
       </x:c>
       <x:c r="F39" s="93" t="str">
-        <x:v>CREATED; 0 rows; not used by copied app</x:v>
+        <x:v>COPIED AND VERIFIED; 140 rows</x:v>
       </x:c>
       <x:c r="G39" s="93" t="str">
-        <x:v>Schema types and data correctness not reconciled; preserve for diagnosis</x:v>
+        <x:v>Trial now reads SQL; all stored fields and related membership verified</x:v>
       </x:c>
       <x:c r="H39" s="93" t="str">
-        <x:v>public."Payments"; app 494cd013-0d9b-482f-9559-c9d83059de91 still uses original data sources</x:v>
+        <x:v>public."Payments"; 13 physical columns; exact keys and all fields matched</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="55" customHeight="1">
@@ -6173,7 +6181,7 @@
         <x:v>Clean restart</x:v>
       </x:c>
       <x:c r="B40" s="93" t="str">
-        <x:v>1.000003</x:v>
+        <x:v>1.000007</x:v>
       </x:c>
       <x:c r="C40" s="93" t="str">
         <x:v>Repayments</x:v>
@@ -6185,13 +6193,13 @@
         <x:v>PostgreSQL table</x:v>
       </x:c>
       <x:c r="F40" s="93" t="str">
-        <x:v>CREATED; 0 rows; not used by copied app</x:v>
+        <x:v>COPIED AND VERIFIED; 644 rows</x:v>
       </x:c>
       <x:c r="G40" s="93" t="str">
-        <x:v>Schema types and data correctness not reconciled; preserve for diagnosis</x:v>
+        <x:v>Trial now reads SQL; all stored fields and related membership verified</x:v>
       </x:c>
       <x:c r="H40" s="93" t="str">
-        <x:v>public."Repayments"; app 494cd013-0d9b-482f-9559-c9d83059de91 still uses original data sources</x:v>
+        <x:v>public."Repayments"; 10 physical columns; exact keys and all fields matched</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="55" customHeight="1">
@@ -6199,7 +6207,7 @@
         <x:v>Clean restart</x:v>
       </x:c>
       <x:c r="B41" s="93" t="str">
-        <x:v>1.000003</x:v>
+        <x:v>1.000007</x:v>
       </x:c>
       <x:c r="C41" s="93" t="str">
         <x:v>Settlements</x:v>
@@ -6211,13 +6219,13 @@
         <x:v>PostgreSQL table</x:v>
       </x:c>
       <x:c r="F41" s="93" t="str">
-        <x:v>CREATED; 0 rows; not used by copied app</x:v>
+        <x:v>COPIED AND VERIFIED; 2 rows</x:v>
       </x:c>
       <x:c r="G41" s="93" t="str">
-        <x:v>Schema types and data correctness not reconciled; preserve for diagnosis</x:v>
+        <x:v>Trial now reads SQL; all stored fields and related membership verified</x:v>
       </x:c>
       <x:c r="H41" s="93" t="str">
-        <x:v>public."Settlements"; app 494cd013-0d9b-482f-9559-c9d83059de91 still uses original data sources</x:v>
+        <x:v>public."Settlements"; 7 physical columns; exact keys and all fields matched</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="55" customHeight="1">
@@ -6322,6 +6330,344 @@
       </x:c>
       <x:c r="H45" s="93" t="str">
         <x:v>Label Yes; Read-Only No; one row</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="55" customHeight="1">
+      <x:c r="A46" s="93" t="str">
+        <x:v>Master switch</x:v>
+      </x:c>
+      <x:c r="B46" s="93" t="str">
+        <x:v>1.000006</x:v>
+      </x:c>
+      <x:c r="C46" s="93" t="str">
+        <x:v>Borrowers</x:v>
+      </x:c>
+      <x:c r="D46" s="93" t="str">
+        <x:v>Source binding</x:v>
+      </x:c>
+      <x:c r="E46" s="93" t="str">
+        <x:v>PostgreSQL table</x:v>
+      </x:c>
+      <x:c r="F46" s="93" t="str">
+        <x:v>READ_ONLY</x:v>
+      </x:c>
+      <x:c r="G46" s="93" t="str">
+        <x:v>Trial only; existing schema, Refs, slices and calculations preserved</x:v>
+      </x:c>
+      <x:c r="H46" s="93" t="str">
+        <x:v>database-2; Source Path Borrowers; Table=public.Borrowers__Borrowers</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="55" customHeight="1">
+      <x:c r="A47" s="93" t="str">
+        <x:v>Master switch</x:v>
+      </x:c>
+      <x:c r="B47" s="93" t="str">
+        <x:v>1.000006</x:v>
+      </x:c>
+      <x:c r="C47" s="93" t="str">
+        <x:v>Loans</x:v>
+      </x:c>
+      <x:c r="D47" s="93" t="str">
+        <x:v>Source binding</x:v>
+      </x:c>
+      <x:c r="E47" s="93" t="str">
+        <x:v>PostgreSQL table</x:v>
+      </x:c>
+      <x:c r="F47" s="93" t="str">
+        <x:v>READ_ONLY</x:v>
+      </x:c>
+      <x:c r="G47" s="93" t="str">
+        <x:v>Trial only; existing schema, Refs, slices and calculations preserved</x:v>
+      </x:c>
+      <x:c r="H47" s="93" t="str">
+        <x:v>database-2; Source Path Loans; Table=public.Loans__Loans</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="55" customHeight="1">
+      <x:c r="A48" s="93" t="str">
+        <x:v>Master switch</x:v>
+      </x:c>
+      <x:c r="B48" s="93" t="str">
+        <x:v>1.000006</x:v>
+      </x:c>
+      <x:c r="C48" s="93" t="str">
+        <x:v>Partners</x:v>
+      </x:c>
+      <x:c r="D48" s="93" t="str">
+        <x:v>Source binding</x:v>
+      </x:c>
+      <x:c r="E48" s="93" t="str">
+        <x:v>PostgreSQL table</x:v>
+      </x:c>
+      <x:c r="F48" s="93" t="str">
+        <x:v>ALL_CHANGES</x:v>
+      </x:c>
+      <x:c r="G48" s="93" t="str">
+        <x:v>Trial only; existing schema, Refs, slices and calculations preserved</x:v>
+      </x:c>
+      <x:c r="H48" s="93" t="str">
+        <x:v>database-2; Source Path Partners; Table=public.Partners__Partners</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="55" customHeight="1">
+      <x:c r="A49" s="93" t="str">
+        <x:v>Master switch</x:v>
+      </x:c>
+      <x:c r="B49" s="93" t="str">
+        <x:v>1.000005</x:v>
+      </x:c>
+      <x:c r="C49" s="93" t="str">
+        <x:v>Trial app</x:v>
+      </x:c>
+      <x:c r="D49" s="93" t="str">
+        <x:v>Cloud API</x:v>
+      </x:c>
+      <x:c r="E49" s="93" t="str">
+        <x:v>Integration</x:v>
+      </x:c>
+      <x:c r="F49" s="93" t="str">
+        <x:v>ENABLED with explicit owner confirmation</x:v>
+      </x:c>
+      <x:c r="G49" s="93" t="str">
+        <x:v>Extraction script uses Find only; access key itself is not read-only</x:v>
+      </x:c>
+      <x:c r="H49" s="93" t="str">
+        <x:v>Key and raw extracts stored outside Git; original app API settings unchanged</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="55" customHeight="1">
+      <x:c r="A50" s="93" t="str">
+        <x:v>Remaining switch</x:v>
+      </x:c>
+      <x:c r="B50" s="93" t="str">
+        <x:v>1.000007</x:v>
+      </x:c>
+      <x:c r="C50" s="93" t="str">
+        <x:v>Repayments</x:v>
+      </x:c>
+      <x:c r="D50" s="93" t="str">
+        <x:v>Source binding</x:v>
+      </x:c>
+      <x:c r="E50" s="93" t="str">
+        <x:v>PostgreSQL table</x:v>
+      </x:c>
+      <x:c r="F50" s="93" t="str">
+        <x:v>READ_ONLY</x:v>
+      </x:c>
+      <x:c r="G50" s="93" t="str">
+        <x:v>Trial only; schema and formulas unchanged</x:v>
+      </x:c>
+      <x:c r="H50" s="93" t="str">
+        <x:v>database-2; Source Path Repayments; Table=public.Repayments__Repayments</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="55" customHeight="1">
+      <x:c r="A51" s="93" t="str">
+        <x:v>Remaining switch</x:v>
+      </x:c>
+      <x:c r="B51" s="93" t="str">
+        <x:v>1.000007</x:v>
+      </x:c>
+      <x:c r="C51" s="93" t="str">
+        <x:v>Charges</x:v>
+      </x:c>
+      <x:c r="D51" s="93" t="str">
+        <x:v>Source binding</x:v>
+      </x:c>
+      <x:c r="E51" s="93" t="str">
+        <x:v>PostgreSQL table</x:v>
+      </x:c>
+      <x:c r="F51" s="93" t="str">
+        <x:v>READ_ONLY</x:v>
+      </x:c>
+      <x:c r="G51" s="93" t="str">
+        <x:v>Trial only; schema and formulas unchanged</x:v>
+      </x:c>
+      <x:c r="H51" s="93" t="str">
+        <x:v>database-2; Source Path Charges; Table=public.Charges__Charges</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="55" customHeight="1">
+      <x:c r="A52" s="93" t="str">
+        <x:v>Remaining switch</x:v>
+      </x:c>
+      <x:c r="B52" s="93" t="str">
+        <x:v>1.000007</x:v>
+      </x:c>
+      <x:c r="C52" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D52" s="93" t="str">
+        <x:v>Source binding</x:v>
+      </x:c>
+      <x:c r="E52" s="93" t="str">
+        <x:v>PostgreSQL table</x:v>
+      </x:c>
+      <x:c r="F52" s="93" t="str">
+        <x:v>ALL_CHANGES</x:v>
+      </x:c>
+      <x:c r="G52" s="93" t="str">
+        <x:v>Trial only; schema and formulas unchanged</x:v>
+      </x:c>
+      <x:c r="H52" s="93" t="str">
+        <x:v>database-2; Source Path Loan Assessment; Table=public.Loan Assessment__Loan Assessment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="55" customHeight="1">
+      <x:c r="A53" s="93" t="str">
+        <x:v>Remaining switch</x:v>
+      </x:c>
+      <x:c r="B53" s="93" t="str">
+        <x:v>1.000007</x:v>
+      </x:c>
+      <x:c r="C53" s="93" t="str">
+        <x:v>Cash Pool Contributions</x:v>
+      </x:c>
+      <x:c r="D53" s="93" t="str">
+        <x:v>Source binding</x:v>
+      </x:c>
+      <x:c r="E53" s="93" t="str">
+        <x:v>PostgreSQL table</x:v>
+      </x:c>
+      <x:c r="F53" s="93" t="str">
+        <x:v>ADDS_AND_UPDATES</x:v>
+      </x:c>
+      <x:c r="G53" s="93" t="str">
+        <x:v>Trial only; schema and formulas unchanged</x:v>
+      </x:c>
+      <x:c r="H53" s="93" t="str">
+        <x:v>database-2; Source Path Cash Pool Contributions; Table=public.Cash Pool Contributions__Cash Pool Contributions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="55" customHeight="1">
+      <x:c r="A54" s="93" t="str">
+        <x:v>Remaining switch</x:v>
+      </x:c>
+      <x:c r="B54" s="93" t="str">
+        <x:v>1.000007</x:v>
+      </x:c>
+      <x:c r="C54" s="93" t="str">
+        <x:v>Settlements</x:v>
+      </x:c>
+      <x:c r="D54" s="93" t="str">
+        <x:v>Source binding</x:v>
+      </x:c>
+      <x:c r="E54" s="93" t="str">
+        <x:v>PostgreSQL table</x:v>
+      </x:c>
+      <x:c r="F54" s="93" t="str">
+        <x:v>ALL_CHANGES</x:v>
+      </x:c>
+      <x:c r="G54" s="93" t="str">
+        <x:v>Trial only; schema and formulas unchanged</x:v>
+      </x:c>
+      <x:c r="H54" s="93" t="str">
+        <x:v>database-2; Source Path Settlements; Table=public.Settlements__Settlements</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="55" customHeight="1">
+      <x:c r="A55" s="93" t="str">
+        <x:v>Remaining switch</x:v>
+      </x:c>
+      <x:c r="B55" s="93" t="str">
+        <x:v>1.000007</x:v>
+      </x:c>
+      <x:c r="C55" s="93" t="str">
+        <x:v>Daily Analytics</x:v>
+      </x:c>
+      <x:c r="D55" s="93" t="str">
+        <x:v>Source binding</x:v>
+      </x:c>
+      <x:c r="E55" s="93" t="str">
+        <x:v>PostgreSQL table</x:v>
+      </x:c>
+      <x:c r="F55" s="93" t="str">
+        <x:v>ALL_CHANGES</x:v>
+      </x:c>
+      <x:c r="G55" s="93" t="str">
+        <x:v>Trial only; schema and formulas unchanged</x:v>
+      </x:c>
+      <x:c r="H55" s="93" t="str">
+        <x:v>database-2; Source Path Daily Analytics; Table=public.Daily Analytics__Daily Analytics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="55" customHeight="1">
+      <x:c r="A56" s="93" t="str">
+        <x:v>Remaining switch</x:v>
+      </x:c>
+      <x:c r="B56" s="93" t="str">
+        <x:v>1.000007</x:v>
+      </x:c>
+      <x:c r="C56" s="93" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D56" s="93" t="str">
+        <x:v>Source binding</x:v>
+      </x:c>
+      <x:c r="E56" s="93" t="str">
+        <x:v>PostgreSQL table</x:v>
+      </x:c>
+      <x:c r="F56" s="93" t="str">
+        <x:v>READ_ONLY</x:v>
+      </x:c>
+      <x:c r="G56" s="93" t="str">
+        <x:v>Trial only; schema and formulas unchanged</x:v>
+      </x:c>
+      <x:c r="H56" s="93" t="str">
+        <x:v>database-2; Source Path Payment Allocations; Table=public.Payment Allocations__Payment Allocations</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="55" customHeight="1">
+      <x:c r="A57" s="93" t="str">
+        <x:v>Remaining switch</x:v>
+      </x:c>
+      <x:c r="B57" s="93" t="str">
+        <x:v>1.000007</x:v>
+      </x:c>
+      <x:c r="C57" s="93" t="str">
+        <x:v>Payments</x:v>
+      </x:c>
+      <x:c r="D57" s="93" t="str">
+        <x:v>Source binding</x:v>
+      </x:c>
+      <x:c r="E57" s="93" t="str">
+        <x:v>PostgreSQL table</x:v>
+      </x:c>
+      <x:c r="F57" s="93" t="str">
+        <x:v>READ_ONLY</x:v>
+      </x:c>
+      <x:c r="G57" s="93" t="str">
+        <x:v>Trial only; schema and formulas unchanged</x:v>
+      </x:c>
+      <x:c r="H57" s="93" t="str">
+        <x:v>database-2; Source Path Payments; Table=public.Payments__Payments</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="55" customHeight="1">
+      <x:c r="A58" s="93" t="str">
+        <x:v>Remaining switch</x:v>
+      </x:c>
+      <x:c r="B58" s="93" t="str">
+        <x:v>1.000007</x:v>
+      </x:c>
+      <x:c r="C58" s="93" t="str">
+        <x:v>Charges / Repayments</x:v>
+      </x:c>
+      <x:c r="D58" s="93" t="str">
+        <x:v>Provider row order</x:v>
+      </x:c>
+      <x:c r="E58" s="93" t="str">
+        <x:v>System metadata</x:v>
+      </x:c>
+      <x:c r="F58" s="93" t="str">
+        <x:v>201 Charges and 144 Repayments row numbers changed</x:v>
+      </x:c>
+      <x:c r="G58" s="93" t="str">
+        <x:v>Business values unchanged; 4 related lists reordered with identical membership</x:v>
+      </x:c>
+      <x:c r="H58" s="93" t="str">
+        <x:v>Never treat _RowNumber or unsorted REF_ROWS order as stable; validate write workflows separately</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6743,7 +7089,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96c3d0ef9da743b4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06d63c999d584a27"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17400,7 +17746,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8d9f438897c453f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree75edcddda04939"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17829,7 +18175,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R576798a7d0bf4450"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re25b44cc55da45d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18289,7 +18635,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbe18dbd49a74e09"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30fe6472ce884c45"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25263,7 +25609,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2308807ce4d84f18"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rabef0a776c244b82"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29882,7 +30228,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R829a6bbc7b6b464e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18aa1fe2329a49a5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30081,7 +30427,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf459737b2ac45b5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf352d63251904d05"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31734,7 +32080,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R126a37544b1b4181"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7097c9961c0d45d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add and validate PostgreSQL Ref constraints with rollback evidence
</commit_message>
<xml_diff>
--- a/Documents/AppSheet_Data_Dictionary.xlsx
+++ b/Documents/AppSheet_Data_Dictionary.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R0cf92f2c00ff4e1a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="Rf66215da1caf44f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="Rfbf9b2e2e07243fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="Rf9557621dbef4d0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="R1a0b3883428b4bde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="Rf13958d1aff0438f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="R3cd6c6a1ef3c4c26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R8fa53bf809984729"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="Ra3b9441c805d4311"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="Rf16b15d151074b5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="Rbe2c42ac0bc3428c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="R84861ec9994d41f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Sync POC" sheetId="13" r:id="Rf31c3c015d484f7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Migration Trial" sheetId="14" r:id="Rf8ba14654f974d83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rc8a1b42326d94b1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="R330d00b3f1f04219"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="Ra2d90ba617ba4459"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="Rb62581c186ff4e87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="Rcafc24c049cd4ec5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="Rc3cebf60981b453b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="R1d6ca97856a84b97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R82cabff2644e4d64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="Rfd2096e1cabb4fef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="Rb53e77ec525b4f3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="Red02d9a3a6794ff9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="R4292b49d83b24e9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Sync POC" sheetId="13" r:id="R805f2d64b5214280"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Migration Trial" sheetId="14" r:id="Ra3efeb3eb4894156"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -100,7 +100,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="32">
+  <x:fills count="33">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -135,6 +135,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -387,7 +392,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="123">
+  <x:cellXfs count="124">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -655,6 +660,9 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="12" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2562,7 +2570,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55aa89467b404526"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d08b96d50c14684"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5163,28 +5171,28 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="122" t="str">
+      <x:c r="A1" s="123" t="str">
         <x:v>Experiment</x:v>
       </x:c>
-      <x:c r="B1" s="122" t="str">
+      <x:c r="B1" s="123" t="str">
         <x:v>App version</x:v>
       </x:c>
-      <x:c r="C1" s="122" t="str">
+      <x:c r="C1" s="123" t="str">
         <x:v>Table</x:v>
       </x:c>
-      <x:c r="D1" s="122" t="str">
+      <x:c r="D1" s="123" t="str">
         <x:v>Column / setting</x:v>
       </x:c>
-      <x:c r="E1" s="122" t="str">
+      <x:c r="E1" s="123" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="F1" s="122" t="str">
+      <x:c r="F1" s="123" t="str">
         <x:v>Scope / status</x:v>
       </x:c>
-      <x:c r="G1" s="122" t="str">
+      <x:c r="G1" s="123" t="str">
         <x:v>Purpose / dependencies</x:v>
       </x:c>
-      <x:c r="H1" s="122" t="str">
+      <x:c r="H1" s="123" t="str">
         <x:v>Exact definition</x:v>
       </x:c>
     </x:row>
@@ -6668,6 +6676,370 @@
       </x:c>
       <x:c r="H58" s="93" t="str">
         <x:v>Never treat _RowNumber or unsorted REF_ROWS order as stable; validate write workflows separately</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="55" customHeight="1">
+      <x:c r="A59" s="93" t="str">
+        <x:v>SQL foreign keys</x:v>
+      </x:c>
+      <x:c r="B59" s="93" t="str">
+        <x:v>1.000007</x:v>
+      </x:c>
+      <x:c r="C59" s="93" t="str">
+        <x:v>Loans</x:v>
+      </x:c>
+      <x:c r="D59" s="93" t="str">
+        <x:v>Ref Borrowers</x:v>
+      </x:c>
+      <x:c r="E59" s="93" t="str">
+        <x:v>Foreign key</x:v>
+      </x:c>
+      <x:c r="F59" s="93" t="str">
+        <x:v>Validated; future production DB</x:v>
+      </x:c>
+      <x:c r="G59" s="93" t="str">
+        <x:v>Parent Borrowers.Row ID; app Ref unchanged</x:v>
+      </x:c>
+      <x:c r="H59" s="93" t="str">
+        <x:v>appsheet_ref_01: REFERENCES public.Borrowers(Row ID); UPDATE/DELETE NO ACTION; NOT DEFERRABLE; blank Ref text normalized to NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="55" customHeight="1">
+      <x:c r="A60" s="93" t="str">
+        <x:v>SQL foreign keys</x:v>
+      </x:c>
+      <x:c r="B60" s="93" t="str">
+        <x:v>1.000007</x:v>
+      </x:c>
+      <x:c r="C60" s="93" t="str">
+        <x:v>Repayments</x:v>
+      </x:c>
+      <x:c r="D60" s="93" t="str">
+        <x:v>Ref Loans</x:v>
+      </x:c>
+      <x:c r="E60" s="93" t="str">
+        <x:v>Foreign key</x:v>
+      </x:c>
+      <x:c r="F60" s="93" t="str">
+        <x:v>Validated; future production DB</x:v>
+      </x:c>
+      <x:c r="G60" s="93" t="str">
+        <x:v>Parent Loans.Row ID; app Ref unchanged</x:v>
+      </x:c>
+      <x:c r="H60" s="93" t="str">
+        <x:v>appsheet_ref_02: REFERENCES public.Loans(Row ID); UPDATE/DELETE NO ACTION; NOT DEFERRABLE; blank Ref text normalized to NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="55" customHeight="1">
+      <x:c r="A61" s="93" t="str">
+        <x:v>SQL foreign keys</x:v>
+      </x:c>
+      <x:c r="B61" s="93" t="str">
+        <x:v>1.000007</x:v>
+      </x:c>
+      <x:c r="C61" s="93" t="str">
+        <x:v>Repayments</x:v>
+      </x:c>
+      <x:c r="D61" s="93" t="str">
+        <x:v>Ref Charges</x:v>
+      </x:c>
+      <x:c r="E61" s="93" t="str">
+        <x:v>Foreign key</x:v>
+      </x:c>
+      <x:c r="F61" s="93" t="str">
+        <x:v>Validated; future production DB</x:v>
+      </x:c>
+      <x:c r="G61" s="93" t="str">
+        <x:v>Parent Charges.Row ID; app Ref unchanged</x:v>
+      </x:c>
+      <x:c r="H61" s="93" t="str">
+        <x:v>appsheet_ref_03: REFERENCES public.Charges(Row ID); UPDATE/DELETE NO ACTION; NOT DEFERRABLE; blank Ref text normalized to NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="55" customHeight="1">
+      <x:c r="A62" s="93" t="str">
+        <x:v>SQL foreign keys</x:v>
+      </x:c>
+      <x:c r="B62" s="93" t="str">
+        <x:v>1.000007</x:v>
+      </x:c>
+      <x:c r="C62" s="93" t="str">
+        <x:v>Repayments</x:v>
+      </x:c>
+      <x:c r="D62" s="93" t="str">
+        <x:v>Ref Payment</x:v>
+      </x:c>
+      <x:c r="E62" s="93" t="str">
+        <x:v>Foreign key</x:v>
+      </x:c>
+      <x:c r="F62" s="93" t="str">
+        <x:v>Validated; future production DB</x:v>
+      </x:c>
+      <x:c r="G62" s="93" t="str">
+        <x:v>Parent Payments.Row ID; app Ref unchanged</x:v>
+      </x:c>
+      <x:c r="H62" s="93" t="str">
+        <x:v>appsheet_ref_04: REFERENCES public.Payments(Row ID); UPDATE/DELETE NO ACTION; NOT DEFERRABLE; blank Ref text normalized to NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="55" customHeight="1">
+      <x:c r="A63" s="93" t="str">
+        <x:v>SQL foreign keys</x:v>
+      </x:c>
+      <x:c r="B63" s="93" t="str">
+        <x:v>1.000007</x:v>
+      </x:c>
+      <x:c r="C63" s="93" t="str">
+        <x:v>Repayments</x:v>
+      </x:c>
+      <x:c r="D63" s="93" t="str">
+        <x:v>Ref Payment Allocation</x:v>
+      </x:c>
+      <x:c r="E63" s="93" t="str">
+        <x:v>Foreign key</x:v>
+      </x:c>
+      <x:c r="F63" s="93" t="str">
+        <x:v>Validated; future production DB</x:v>
+      </x:c>
+      <x:c r="G63" s="93" t="str">
+        <x:v>Parent Payment Allocations.Row ID; app Ref unchanged</x:v>
+      </x:c>
+      <x:c r="H63" s="93" t="str">
+        <x:v>appsheet_ref_05: REFERENCES public.Payment Allocations(Row ID); UPDATE/DELETE NO ACTION; NOT DEFERRABLE; blank Ref text normalized to NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="55" customHeight="1">
+      <x:c r="A64" s="93" t="str">
+        <x:v>SQL foreign keys</x:v>
+      </x:c>
+      <x:c r="B64" s="93" t="str">
+        <x:v>1.000007</x:v>
+      </x:c>
+      <x:c r="C64" s="93" t="str">
+        <x:v>Charges</x:v>
+      </x:c>
+      <x:c r="D64" s="93" t="str">
+        <x:v>Ref Loans</x:v>
+      </x:c>
+      <x:c r="E64" s="93" t="str">
+        <x:v>Foreign key</x:v>
+      </x:c>
+      <x:c r="F64" s="93" t="str">
+        <x:v>Validated; future production DB</x:v>
+      </x:c>
+      <x:c r="G64" s="93" t="str">
+        <x:v>Parent Loans.Row ID; app Ref unchanged</x:v>
+      </x:c>
+      <x:c r="H64" s="93" t="str">
+        <x:v>appsheet_ref_06: REFERENCES public.Loans(Row ID); UPDATE/DELETE NO ACTION; NOT DEFERRABLE; blank Ref text normalized to NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="55" customHeight="1">
+      <x:c r="A65" s="93" t="str">
+        <x:v>SQL foreign keys</x:v>
+      </x:c>
+      <x:c r="B65" s="93" t="str">
+        <x:v>1.000007</x:v>
+      </x:c>
+      <x:c r="C65" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D65" s="93" t="str">
+        <x:v>Ref Borrower</x:v>
+      </x:c>
+      <x:c r="E65" s="93" t="str">
+        <x:v>Foreign key</x:v>
+      </x:c>
+      <x:c r="F65" s="93" t="str">
+        <x:v>Validated; future production DB</x:v>
+      </x:c>
+      <x:c r="G65" s="93" t="str">
+        <x:v>Parent Borrowers.Row ID; app Ref unchanged</x:v>
+      </x:c>
+      <x:c r="H65" s="93" t="str">
+        <x:v>appsheet_ref_07: REFERENCES public.Borrowers(Row ID); UPDATE/DELETE NO ACTION; NOT DEFERRABLE; blank Ref text normalized to NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="55" customHeight="1">
+      <x:c r="A66" s="93" t="str">
+        <x:v>SQL foreign keys</x:v>
+      </x:c>
+      <x:c r="B66" s="93" t="str">
+        <x:v>1.000007</x:v>
+      </x:c>
+      <x:c r="C66" s="93" t="str">
+        <x:v>Cash Pool Contributions</x:v>
+      </x:c>
+      <x:c r="D66" s="93" t="str">
+        <x:v>Ref Partner</x:v>
+      </x:c>
+      <x:c r="E66" s="93" t="str">
+        <x:v>Foreign key</x:v>
+      </x:c>
+      <x:c r="F66" s="93" t="str">
+        <x:v>Validated; future production DB</x:v>
+      </x:c>
+      <x:c r="G66" s="93" t="str">
+        <x:v>Parent Partners.Row ID; app Ref unchanged</x:v>
+      </x:c>
+      <x:c r="H66" s="93" t="str">
+        <x:v>appsheet_ref_08: REFERENCES public.Partners(Row ID); UPDATE/DELETE NO ACTION; NOT DEFERRABLE; blank Ref text normalized to NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="55" customHeight="1">
+      <x:c r="A67" s="93" t="str">
+        <x:v>SQL foreign keys</x:v>
+      </x:c>
+      <x:c r="B67" s="93" t="str">
+        <x:v>1.000007</x:v>
+      </x:c>
+      <x:c r="C67" s="93" t="str">
+        <x:v>Settlements</x:v>
+      </x:c>
+      <x:c r="D67" s="93" t="str">
+        <x:v>Ref Partner</x:v>
+      </x:c>
+      <x:c r="E67" s="93" t="str">
+        <x:v>Foreign key</x:v>
+      </x:c>
+      <x:c r="F67" s="93" t="str">
+        <x:v>Validated; future production DB</x:v>
+      </x:c>
+      <x:c r="G67" s="93" t="str">
+        <x:v>Parent Partners.Row ID; app Ref unchanged</x:v>
+      </x:c>
+      <x:c r="H67" s="93" t="str">
+        <x:v>appsheet_ref_09: REFERENCES public.Partners(Row ID); UPDATE/DELETE NO ACTION; NOT DEFERRABLE; blank Ref text normalized to NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="55" customHeight="1">
+      <x:c r="A68" s="93" t="str">
+        <x:v>SQL foreign keys</x:v>
+      </x:c>
+      <x:c r="B68" s="93" t="str">
+        <x:v>1.000007</x:v>
+      </x:c>
+      <x:c r="C68" s="93" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D68" s="93" t="str">
+        <x:v>Ref Payment</x:v>
+      </x:c>
+      <x:c r="E68" s="93" t="str">
+        <x:v>Foreign key</x:v>
+      </x:c>
+      <x:c r="F68" s="93" t="str">
+        <x:v>Validated; future production DB</x:v>
+      </x:c>
+      <x:c r="G68" s="93" t="str">
+        <x:v>Parent Payments.Row ID; app Ref unchanged</x:v>
+      </x:c>
+      <x:c r="H68" s="93" t="str">
+        <x:v>appsheet_ref_10: REFERENCES public.Payments(Row ID); UPDATE/DELETE NO ACTION; NOT DEFERRABLE; blank Ref text normalized to NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="55" customHeight="1">
+      <x:c r="A69" s="93" t="str">
+        <x:v>SQL foreign keys</x:v>
+      </x:c>
+      <x:c r="B69" s="93" t="str">
+        <x:v>1.000007</x:v>
+      </x:c>
+      <x:c r="C69" s="93" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D69" s="93" t="str">
+        <x:v>Ref Charge</x:v>
+      </x:c>
+      <x:c r="E69" s="93" t="str">
+        <x:v>Foreign key</x:v>
+      </x:c>
+      <x:c r="F69" s="93" t="str">
+        <x:v>Validated; future production DB</x:v>
+      </x:c>
+      <x:c r="G69" s="93" t="str">
+        <x:v>Parent Charges.Row ID; app Ref unchanged</x:v>
+      </x:c>
+      <x:c r="H69" s="93" t="str">
+        <x:v>appsheet_ref_11: REFERENCES public.Charges(Row ID); UPDATE/DELETE NO ACTION; NOT DEFERRABLE; blank Ref text normalized to NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="55" customHeight="1">
+      <x:c r="A70" s="93" t="str">
+        <x:v>SQL foreign keys</x:v>
+      </x:c>
+      <x:c r="B70" s="93" t="str">
+        <x:v>1.000007</x:v>
+      </x:c>
+      <x:c r="C70" s="93" t="str">
+        <x:v>Payments</x:v>
+      </x:c>
+      <x:c r="D70" s="93" t="str">
+        <x:v>Ref Borrower</x:v>
+      </x:c>
+      <x:c r="E70" s="93" t="str">
+        <x:v>Foreign key</x:v>
+      </x:c>
+      <x:c r="F70" s="93" t="str">
+        <x:v>Validated; future production DB</x:v>
+      </x:c>
+      <x:c r="G70" s="93" t="str">
+        <x:v>Parent Borrowers.Row ID; app Ref unchanged</x:v>
+      </x:c>
+      <x:c r="H70" s="93" t="str">
+        <x:v>appsheet_ref_12: REFERENCES public.Borrowers(Row ID); UPDATE/DELETE NO ACTION; NOT DEFERRABLE; blank Ref text normalized to NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="55" customHeight="1">
+      <x:c r="A71" s="93" t="str">
+        <x:v>SQL foreign keys</x:v>
+      </x:c>
+      <x:c r="B71" s="93" t="str">
+        <x:v>1.000007</x:v>
+      </x:c>
+      <x:c r="C71" s="93" t="str">
+        <x:v>Payments</x:v>
+      </x:c>
+      <x:c r="D71" s="93" t="str">
+        <x:v>Ref Target Charge</x:v>
+      </x:c>
+      <x:c r="E71" s="93" t="str">
+        <x:v>Foreign key</x:v>
+      </x:c>
+      <x:c r="F71" s="93" t="str">
+        <x:v>Validated; future production DB</x:v>
+      </x:c>
+      <x:c r="G71" s="93" t="str">
+        <x:v>Parent Charges.Row ID; app Ref unchanged</x:v>
+      </x:c>
+      <x:c r="H71" s="93" t="str">
+        <x:v>appsheet_ref_13: REFERENCES public.Charges(Row ID); UPDATE/DELETE NO ACTION; NOT DEFERRABLE; blank Ref text normalized to NULL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="55" customHeight="1">
+      <x:c r="A72" s="93" t="str">
+        <x:v>SQL foreign keys</x:v>
+      </x:c>
+      <x:c r="B72" s="93" t="str">
+        <x:v>1.000007</x:v>
+      </x:c>
+      <x:c r="C72" s="93" t="str">
+        <x:v>8 child tables</x:v>
+      </x:c>
+      <x:c r="D72" s="93" t="str">
+        <x:v>appsheet_blank_refs</x:v>
+      </x:c>
+      <x:c r="E72" s="93" t="str">
+        <x:v>BEFORE trigger</x:v>
+      </x:c>
+      <x:c r="F72" s="93" t="str">
+        <x:v>Installed; 1,010 blanks normalized</x:v>
+      </x:c>
+      <x:c r="G72" s="93" t="str">
+        <x:v>Future empty Ref values -&gt; NULL; nonblank values untouched</x:v>
+      </x:c>
+      <x:c r="H72" s="93" t="str">
+        <x:v>public.appsheet_normalize_blank_refs(); BEFORE INSERT OR UPDATE; 13 Ref columns only; no schema columns added</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7089,7 +7461,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06d63c999d584a27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f2faaa92fbc4d3e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17746,7 +18118,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree75edcddda04939"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c6dbb03541e44d0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18175,7 +18547,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re25b44cc55da45d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R011e64bf89ff4fff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18635,7 +19007,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30fe6472ce884c45"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81fa15aad90f4248"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25609,7 +25981,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rabef0a776c244b82"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01212b8001b34e2d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30228,7 +30600,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18aa1fe2329a49a5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R792cdcf434a644f4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30427,7 +30799,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf352d63251904d05"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4ad5836a5b049cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32080,7 +32452,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7097c9961c0d45d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00b32aade3dd4b64"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Checkpoint PostgreSQL OLTP lifecycle validation and restore borrower lookup
</commit_message>
<xml_diff>
--- a/Documents/AppSheet_Data_Dictionary.xlsx
+++ b/Documents/AppSheet_Data_Dictionary.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rc8a1b42326d94b1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="R330d00b3f1f04219"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="Ra2d90ba617ba4459"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="Rb62581c186ff4e87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="Rcafc24c049cd4ec5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="Rc3cebf60981b453b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="R1d6ca97856a84b97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R82cabff2644e4d64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="Rfd2096e1cabb4fef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="Rb53e77ec525b4f3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="Red02d9a3a6794ff9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="R4292b49d83b24e9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Sync POC" sheetId="13" r:id="R805f2d64b5214280"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Migration Trial" sheetId="14" r:id="Ra3efeb3eb4894156"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R698351cb75664772"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="Rbc128ea22bc94c34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R136cddf6a8434ef5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R458b9bc5436b42f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="R784292437e5f421e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="Raedeec4a5b13438e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Rb911b941130d40ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="Rdb0522a3484249d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="Rf4edd2e0cd7c476d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R6b7b32dda5e64a89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="R270b65d5f48b465e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="R5f3c539ea38047db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Sync POC" sheetId="13" r:id="Rcf0798dd5a9449ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Migration Trial" sheetId="14" r:id="R687d05a2fcc94212"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -100,7 +100,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="33">
+  <x:fills count="34">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -135,6 +135,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -392,7 +397,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="124">
+  <x:cellXfs count="125">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -663,6 +668,9 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="12" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2570,7 +2578,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d08b96d50c14684"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb617b213d034731"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5171,28 +5179,28 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="123" t="str">
+      <x:c r="A1" s="124" t="str">
         <x:v>Experiment</x:v>
       </x:c>
-      <x:c r="B1" s="123" t="str">
+      <x:c r="B1" s="124" t="str">
         <x:v>App version</x:v>
       </x:c>
-      <x:c r="C1" s="123" t="str">
+      <x:c r="C1" s="124" t="str">
         <x:v>Table</x:v>
       </x:c>
-      <x:c r="D1" s="123" t="str">
+      <x:c r="D1" s="124" t="str">
         <x:v>Column / setting</x:v>
       </x:c>
-      <x:c r="E1" s="123" t="str">
+      <x:c r="E1" s="124" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="F1" s="123" t="str">
+      <x:c r="F1" s="124" t="str">
         <x:v>Scope / status</x:v>
       </x:c>
-      <x:c r="G1" s="123" t="str">
+      <x:c r="G1" s="124" t="str">
         <x:v>Purpose / dependencies</x:v>
       </x:c>
-      <x:c r="H1" s="123" t="str">
+      <x:c r="H1" s="124" t="str">
         <x:v>Exact definition</x:v>
       </x:c>
     </x:row>
@@ -7040,6 +7048,266 @@
       </x:c>
       <x:c r="H72" s="93" t="str">
         <x:v>public.appsheet_normalize_blank_refs(); BEFORE INSERT OR UPDATE; 13 Ref columns only; no schema columns added</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="55" customHeight="1">
+      <x:c r="A73" s="93" t="str">
+        <x:v>OLTP SQL validation</x:v>
+      </x:c>
+      <x:c r="B73" s="93" t="str">
+        <x:v>1.000004</x:v>
+      </x:c>
+      <x:c r="C73" s="93" t="str">
+        <x:v>Borrowers</x:v>
+      </x:c>
+      <x:c r="D73" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E73" s="93" t="str">
+        <x:v>SQL binding</x:v>
+      </x:c>
+      <x:c r="F73" s="93" t="str">
+        <x:v>Copied OLTP; testing in progress</x:v>
+      </x:c>
+      <x:c r="G73" s="93" t="str">
+        <x:v>Original OLTP 3.000064 remains on Money</x:v>
+      </x:c>
+      <x:c r="H73" s="93" t="str">
+        <x:v>database-2; Borrowers</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="55" customHeight="1">
+      <x:c r="A74" s="93" t="str">
+        <x:v>OLTP SQL validation</x:v>
+      </x:c>
+      <x:c r="B74" s="93" t="str">
+        <x:v>1.000004</x:v>
+      </x:c>
+      <x:c r="C74" s="93" t="str">
+        <x:v>Loans</x:v>
+      </x:c>
+      <x:c r="D74" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E74" s="93" t="str">
+        <x:v>SQL binding</x:v>
+      </x:c>
+      <x:c r="F74" s="93" t="str">
+        <x:v>Copied OLTP; testing in progress</x:v>
+      </x:c>
+      <x:c r="G74" s="93" t="str">
+        <x:v>Original OLTP 3.000064 remains on Money</x:v>
+      </x:c>
+      <x:c r="H74" s="93" t="str">
+        <x:v>database-2; Loans</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="55" customHeight="1">
+      <x:c r="A75" s="93" t="str">
+        <x:v>OLTP SQL validation</x:v>
+      </x:c>
+      <x:c r="B75" s="93" t="str">
+        <x:v>1.000004</x:v>
+      </x:c>
+      <x:c r="C75" s="93" t="str">
+        <x:v>Repayments</x:v>
+      </x:c>
+      <x:c r="D75" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E75" s="93" t="str">
+        <x:v>SQL binding</x:v>
+      </x:c>
+      <x:c r="F75" s="93" t="str">
+        <x:v>Copied OLTP; testing in progress</x:v>
+      </x:c>
+      <x:c r="G75" s="93" t="str">
+        <x:v>Original OLTP 3.000064 remains on Money</x:v>
+      </x:c>
+      <x:c r="H75" s="93" t="str">
+        <x:v>database-2; Repayments</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="55" customHeight="1">
+      <x:c r="A76" s="93" t="str">
+        <x:v>OLTP SQL validation</x:v>
+      </x:c>
+      <x:c r="B76" s="93" t="str">
+        <x:v>1.000004</x:v>
+      </x:c>
+      <x:c r="C76" s="93" t="str">
+        <x:v>Statistics</x:v>
+      </x:c>
+      <x:c r="D76" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E76" s="93" t="str">
+        <x:v>SQL binding</x:v>
+      </x:c>
+      <x:c r="F76" s="93" t="str">
+        <x:v>Copied OLTP; testing in progress</x:v>
+      </x:c>
+      <x:c r="G76" s="93" t="str">
+        <x:v>Original OLTP 3.000064 remains on Money</x:v>
+      </x:c>
+      <x:c r="H76" s="93" t="str">
+        <x:v>database-2; Statistics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="55" customHeight="1">
+      <x:c r="A77" s="93" t="str">
+        <x:v>OLTP SQL validation</x:v>
+      </x:c>
+      <x:c r="B77" s="93" t="str">
+        <x:v>1.000004</x:v>
+      </x:c>
+      <x:c r="C77" s="93" t="str">
+        <x:v>Charges</x:v>
+      </x:c>
+      <x:c r="D77" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E77" s="93" t="str">
+        <x:v>SQL binding</x:v>
+      </x:c>
+      <x:c r="F77" s="93" t="str">
+        <x:v>Copied OLTP; testing in progress</x:v>
+      </x:c>
+      <x:c r="G77" s="93" t="str">
+        <x:v>Original OLTP 3.000064 remains on Money</x:v>
+      </x:c>
+      <x:c r="H77" s="93" t="str">
+        <x:v>database-2; Charges</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="55" customHeight="1">
+      <x:c r="A78" s="93" t="str">
+        <x:v>OLTP SQL validation</x:v>
+      </x:c>
+      <x:c r="B78" s="93" t="str">
+        <x:v>1.000004</x:v>
+      </x:c>
+      <x:c r="C78" s="93" t="str">
+        <x:v>Partners</x:v>
+      </x:c>
+      <x:c r="D78" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E78" s="93" t="str">
+        <x:v>SQL binding</x:v>
+      </x:c>
+      <x:c r="F78" s="93" t="str">
+        <x:v>Copied OLTP; testing in progress</x:v>
+      </x:c>
+      <x:c r="G78" s="93" t="str">
+        <x:v>Original OLTP 3.000064 remains on Money</x:v>
+      </x:c>
+      <x:c r="H78" s="93" t="str">
+        <x:v>database-2; Partners</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="55" customHeight="1">
+      <x:c r="A79" s="93" t="str">
+        <x:v>OLTP SQL validation</x:v>
+      </x:c>
+      <x:c r="B79" s="93" t="str">
+        <x:v>1.000004</x:v>
+      </x:c>
+      <x:c r="C79" s="93" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D79" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E79" s="93" t="str">
+        <x:v>SQL binding</x:v>
+      </x:c>
+      <x:c r="F79" s="93" t="str">
+        <x:v>Copied OLTP; testing in progress</x:v>
+      </x:c>
+      <x:c r="G79" s="93" t="str">
+        <x:v>Original OLTP 3.000064 remains on Money</x:v>
+      </x:c>
+      <x:c r="H79" s="93" t="str">
+        <x:v>database-2; Payment Allocations</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="55" customHeight="1">
+      <x:c r="A80" s="93" t="str">
+        <x:v>OLTP SQL validation</x:v>
+      </x:c>
+      <x:c r="B80" s="93" t="str">
+        <x:v>1.000004</x:v>
+      </x:c>
+      <x:c r="C80" s="93" t="str">
+        <x:v>Payments</x:v>
+      </x:c>
+      <x:c r="D80" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E80" s="93" t="str">
+        <x:v>SQL binding</x:v>
+      </x:c>
+      <x:c r="F80" s="93" t="str">
+        <x:v>Copied OLTP; testing in progress</x:v>
+      </x:c>
+      <x:c r="G80" s="93" t="str">
+        <x:v>Original OLTP 3.000064 remains on Money</x:v>
+      </x:c>
+      <x:c r="H80" s="93" t="str">
+        <x:v>database-2; Payments</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="55" customHeight="1">
+      <x:c r="A81" s="93" t="str">
+        <x:v>OLTP SQL validation</x:v>
+      </x:c>
+      <x:c r="B81" s="93" t="str">
+        <x:v>OLTP 1.000005; OLAP 1.000007</x:v>
+      </x:c>
+      <x:c r="C81" s="93" t="str">
+        <x:v>Loans</x:v>
+      </x:c>
+      <x:c r="D81" s="93" t="str">
+        <x:v>Borrower Name</x:v>
+      </x:c>
+      <x:c r="E81" s="93" t="str">
+        <x:v>SQL lookup triggers</x:v>
+      </x:c>
+      <x:c r="F81" s="93" t="str">
+        <x:v>Installed; insert and rename verified</x:v>
+      </x:c>
+      <x:c r="G81" s="93" t="str">
+        <x:v>Restores native Lookup on Borrowers.Borrower Name for both app consumers</x:v>
+      </x:c>
+      <x:c r="H81" s="93" t="str">
+        <x:v>BEFORE INSERT OR UPDATE Loans: resolve Borrower Name through Ref Borrowers; AFTER Borrower Name update: propagate to Loans. No added columns.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="55" customHeight="1">
+      <x:c r="A82" s="93" t="str">
+        <x:v>OLTP SQL validation</x:v>
+      </x:c>
+      <x:c r="B82" s="93" t="str">
+        <x:v>1.000005</x:v>
+      </x:c>
+      <x:c r="C82" s="93" t="str">
+        <x:v>Loans</x:v>
+      </x:c>
+      <x:c r="D82" s="93" t="str">
+        <x:v>Two charge actions</x:v>
+      </x:c>
+      <x:c r="E82" s="93" t="str">
+        <x:v>Display only</x:v>
+      </x:c>
+      <x:c r="F82" s="93" t="str">
+        <x:v>Temporary; restoration pending</x:v>
+      </x:c>
+      <x:c r="G82" s="93" t="str">
+        <x:v>New GUI lifecycle testing</x:v>
+      </x:c>
+      <x:c r="H82" s="93" t="str">
+        <x:v>Generate Today's Charge and New Loan Payment - Create First-Day Charge: Prominent instead of Hide.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7461,7 +7729,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f2faaa92fbc4d3e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8fcb02f90f3c4150"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18118,7 +18386,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c6dbb03541e44d0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f16b6fd4e6649b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18547,7 +18815,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R011e64bf89ff4fff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reea3f36dccbb40a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19007,7 +19275,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81fa15aad90f4248"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0116590085e14856"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25981,7 +26249,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01212b8001b34e2d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda2eb747a819434c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30600,7 +30868,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R792cdcf434a644f4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3966a8871ace4590"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30799,7 +31067,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4ad5836a5b049cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f1d691b7ad84891"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32452,7 +32720,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00b32aade3dd4b64"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R327d8e782f8d4470"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Verify all receipt methods and clean PostgreSQL migration test data
</commit_message>
<xml_diff>
--- a/Documents/AppSheet_Data_Dictionary.xlsx
+++ b/Documents/AppSheet_Data_Dictionary.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R698351cb75664772"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="Rbc128ea22bc94c34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R136cddf6a8434ef5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R458b9bc5436b42f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="R784292437e5f421e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="Raedeec4a5b13438e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Rb911b941130d40ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="Rdb0522a3484249d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="Rf4edd2e0cd7c476d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R6b7b32dda5e64a89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="R270b65d5f48b465e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="R5f3c539ea38047db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Sync POC" sheetId="13" r:id="Rcf0798dd5a9449ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Migration Trial" sheetId="14" r:id="R687d05a2fcc94212"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rf35ba5ba504c422b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="Radc5048076764115"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R093ea272035e4350"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R4d4e51304689413f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="Ra6e2b92f779c401f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R8a747f6090bd4b33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Rae693b7305794b90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R602678f15f8c47fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="Rf38d153789174d3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R721e6bb7024b4a4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="R8efe94af0a104724"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="Rcdf3ffcf3281427a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Sync POC" sheetId="13" r:id="Rea856778c17542c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Migration Trial" sheetId="14" r:id="Rf2a8ac9f44ee433e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -100,7 +100,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="34">
+  <x:fills count="35">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -135,6 +135,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -397,7 +402,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="125">
+  <x:cellXfs count="126">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -671,6 +676,9 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="12" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2578,7 +2586,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb617b213d034731"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52e2a617cd844bed"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5179,28 +5187,28 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="124" t="str">
+      <x:c r="A1" s="125" t="str">
         <x:v>Experiment</x:v>
       </x:c>
-      <x:c r="B1" s="124" t="str">
+      <x:c r="B1" s="125" t="str">
         <x:v>App version</x:v>
       </x:c>
-      <x:c r="C1" s="124" t="str">
+      <x:c r="C1" s="125" t="str">
         <x:v>Table</x:v>
       </x:c>
-      <x:c r="D1" s="124" t="str">
+      <x:c r="D1" s="125" t="str">
         <x:v>Column / setting</x:v>
       </x:c>
-      <x:c r="E1" s="124" t="str">
+      <x:c r="E1" s="125" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="F1" s="124" t="str">
+      <x:c r="F1" s="125" t="str">
         <x:v>Scope / status</x:v>
       </x:c>
-      <x:c r="G1" s="124" t="str">
+      <x:c r="G1" s="125" t="str">
         <x:v>Purpose / dependencies</x:v>
       </x:c>
-      <x:c r="H1" s="124" t="str">
+      <x:c r="H1" s="125" t="str">
         <x:v>Exact definition</x:v>
       </x:c>
     </x:row>
@@ -7289,7 +7297,7 @@
         <x:v>OLTP SQL validation</x:v>
       </x:c>
       <x:c r="B82" s="93" t="str">
-        <x:v>1.000005</x:v>
+        <x:v>1.000006</x:v>
       </x:c>
       <x:c r="C82" s="93" t="str">
         <x:v>Loans</x:v>
@@ -7301,13 +7309,13 @@
         <x:v>Display only</x:v>
       </x:c>
       <x:c r="F82" s="93" t="str">
-        <x:v>Temporary; restoration pending</x:v>
+        <x:v>Restored to baseline Hide</x:v>
       </x:c>
       <x:c r="G82" s="93" t="str">
-        <x:v>New GUI lifecycle testing</x:v>
+        <x:v>New GUI lifecycle testing complete</x:v>
       </x:c>
       <x:c r="H82" s="93" t="str">
-        <x:v>Generate Today's Charge and New Loan Payment - Create First-Day Charge: Prominent instead of Hide.</x:v>
+        <x:v>Generate Today's Charge and New Loan Payment - Create First-Day Charge: Hide. All 72 actions match copied baseline.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7729,7 +7737,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8fcb02f90f3c4150"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac8cbbe7055042a5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18386,7 +18394,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f16b6fd4e6649b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R860e73688a58498e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18815,7 +18823,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reea3f36dccbb40a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a94ab0d5d6a4bf3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19275,7 +19283,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0116590085e14856"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6022775a3534717"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26249,7 +26257,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda2eb747a819434c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1a339f52e654366"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30868,7 +30876,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3966a8871ace4590"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf62fd073135f4b50"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31067,7 +31075,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f1d691b7ad84891"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf0f3bc89adf4309"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32720,7 +32728,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R327d8e782f8d4470"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf305118bdaf54241"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Complete OLAP and OLTP PostgreSQL production cutover
</commit_message>
<xml_diff>
--- a/Documents/AppSheet_Data_Dictionary.xlsx
+++ b/Documents/AppSheet_Data_Dictionary.xlsx
@@ -2,20 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rf35ba5ba504c422b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="Radc5048076764115"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R093ea272035e4350"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R4d4e51304689413f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="Ra6e2b92f779c401f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R8a747f6090bd4b33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Rae693b7305794b90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R602678f15f8c47fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="Rf38d153789174d3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R721e6bb7024b4a4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="R8efe94af0a104724"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="Rcdf3ffcf3281427a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Sync POC" sheetId="13" r:id="Rea856778c17542c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Migration Trial" sheetId="14" r:id="Rf2a8ac9f44ee433e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R87f961343a4c4162"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="Raf890574b7404e37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R214a37e456924257"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="Rf1ef2366d0454831"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="R334a6ec9ba484853"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R0d60b2220f0c455b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="R0b86f1bd436f43d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R930fa9e07dea4184"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="Raf32ef7469bc4a46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R78da8a37e92b44cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="R1e49f9caa4c74c4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="R88dd66015c684121"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Sync POC" sheetId="13" r:id="R8f777c62be1f41b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Migration Trial" sheetId="14" r:id="R5848d795d9294f80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Production" sheetId="15" r:id="R65be325a420a4ad3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -100,7 +101,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="35">
+  <x:fills count="36">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -135,6 +136,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -402,7 +408,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="126">
+  <x:cellXfs count="129">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -679,6 +685,11 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="12" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2586,7 +2597,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52e2a617cd844bed"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f0b4debb7964235"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7316,6 +7327,779 @@
       </x:c>
       <x:c r="H82" s="93" t="str">
         <x:v>Generate Today's Charge and New Loan Payment - Create First-Day Charge: Hide. All 72 actions match copied baseline.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="38" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="55" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="100" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="128" t="str">
+        <x:v>Experiment</x:v>
+      </x:c>
+      <x:c r="B1" s="128" t="str">
+        <x:v>App version</x:v>
+      </x:c>
+      <x:c r="C1" s="128" t="str">
+        <x:v>Table</x:v>
+      </x:c>
+      <x:c r="D1" s="128" t="str">
+        <x:v>Column / setting</x:v>
+      </x:c>
+      <x:c r="E1" s="128" t="str">
+        <x:v>Type</x:v>
+      </x:c>
+      <x:c r="F1" s="128" t="str">
+        <x:v>Scope / status</x:v>
+      </x:c>
+      <x:c r="G1" s="128" t="str">
+        <x:v>Purpose / dependencies</x:v>
+      </x:c>
+      <x:c r="H1" s="128" t="str">
+        <x:v>Exact definition</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="70" customHeight="1">
+      <x:c r="A2" s="93" t="str">
+        <x:v>OLAP production</x:v>
+      </x:c>
+      <x:c r="B2" s="93" t="str">
+        <x:v>1.100044</x:v>
+      </x:c>
+      <x:c r="C2" s="93" t="str">
+        <x:v>Borrowers</x:v>
+      </x:c>
+      <x:c r="D2" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E2" s="93" t="str">
+        <x:v>PostgreSQL</x:v>
+      </x:c>
+      <x:c r="F2" s="93" t="str">
+        <x:v>Live; verified 15 September 2026</x:v>
+      </x:c>
+      <x:c r="G2" s="93" t="str">
+        <x:v>Reporting and partner management</x:v>
+      </x:c>
+      <x:c r="H2" s="93" t="str">
+        <x:v>database-2; public.Borrowers; loan_manager_prod</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="70" customHeight="1">
+      <x:c r="A3" s="93" t="str">
+        <x:v>OLAP production</x:v>
+      </x:c>
+      <x:c r="B3" s="93" t="str">
+        <x:v>1.100044</x:v>
+      </x:c>
+      <x:c r="C3" s="93" t="str">
+        <x:v>Loans</x:v>
+      </x:c>
+      <x:c r="D3" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E3" s="93" t="str">
+        <x:v>PostgreSQL</x:v>
+      </x:c>
+      <x:c r="F3" s="93" t="str">
+        <x:v>Live; verified 15 September 2026</x:v>
+      </x:c>
+      <x:c r="G3" s="93" t="str">
+        <x:v>Reporting and partner management</x:v>
+      </x:c>
+      <x:c r="H3" s="93" t="str">
+        <x:v>database-2; public.Loans; loan_manager_prod</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="70" customHeight="1">
+      <x:c r="A4" s="93" t="str">
+        <x:v>OLAP production</x:v>
+      </x:c>
+      <x:c r="B4" s="93" t="str">
+        <x:v>1.100044</x:v>
+      </x:c>
+      <x:c r="C4" s="93" t="str">
+        <x:v>Repayments</x:v>
+      </x:c>
+      <x:c r="D4" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E4" s="93" t="str">
+        <x:v>PostgreSQL</x:v>
+      </x:c>
+      <x:c r="F4" s="93" t="str">
+        <x:v>Live; verified 15 September 2026</x:v>
+      </x:c>
+      <x:c r="G4" s="93" t="str">
+        <x:v>Reporting and partner management</x:v>
+      </x:c>
+      <x:c r="H4" s="93" t="str">
+        <x:v>database-2; public.Repayments; loan_manager_prod</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="70" customHeight="1">
+      <x:c r="A5" s="93" t="str">
+        <x:v>OLAP production</x:v>
+      </x:c>
+      <x:c r="B5" s="93" t="str">
+        <x:v>1.100044</x:v>
+      </x:c>
+      <x:c r="C5" s="93" t="str">
+        <x:v>Statistics</x:v>
+      </x:c>
+      <x:c r="D5" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E5" s="93" t="str">
+        <x:v>PostgreSQL</x:v>
+      </x:c>
+      <x:c r="F5" s="93" t="str">
+        <x:v>Live; verified 15 September 2026</x:v>
+      </x:c>
+      <x:c r="G5" s="93" t="str">
+        <x:v>Reporting and partner management</x:v>
+      </x:c>
+      <x:c r="H5" s="93" t="str">
+        <x:v>database-2; public.Statistics; loan_manager_prod</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="70" customHeight="1">
+      <x:c r="A6" s="93" t="str">
+        <x:v>OLAP production</x:v>
+      </x:c>
+      <x:c r="B6" s="93" t="str">
+        <x:v>1.100044</x:v>
+      </x:c>
+      <x:c r="C6" s="93" t="str">
+        <x:v>Charges</x:v>
+      </x:c>
+      <x:c r="D6" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E6" s="93" t="str">
+        <x:v>PostgreSQL</x:v>
+      </x:c>
+      <x:c r="F6" s="93" t="str">
+        <x:v>Live; verified 15 September 2026</x:v>
+      </x:c>
+      <x:c r="G6" s="93" t="str">
+        <x:v>Reporting and partner management</x:v>
+      </x:c>
+      <x:c r="H6" s="93" t="str">
+        <x:v>database-2; public.Charges; loan_manager_prod</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="70" customHeight="1">
+      <x:c r="A7" s="93" t="str">
+        <x:v>OLAP production</x:v>
+      </x:c>
+      <x:c r="B7" s="93" t="str">
+        <x:v>1.100044</x:v>
+      </x:c>
+      <x:c r="C7" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D7" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E7" s="93" t="str">
+        <x:v>PostgreSQL</x:v>
+      </x:c>
+      <x:c r="F7" s="93" t="str">
+        <x:v>Live; verified 15 September 2026</x:v>
+      </x:c>
+      <x:c r="G7" s="93" t="str">
+        <x:v>Reporting and partner management</x:v>
+      </x:c>
+      <x:c r="H7" s="93" t="str">
+        <x:v>database-2; public.Loan Assessment; loan_manager_prod</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="70" customHeight="1">
+      <x:c r="A8" s="93" t="str">
+        <x:v>OLAP production</x:v>
+      </x:c>
+      <x:c r="B8" s="93" t="str">
+        <x:v>1.100044</x:v>
+      </x:c>
+      <x:c r="C8" s="93" t="str">
+        <x:v>Cash Pool Contributions</x:v>
+      </x:c>
+      <x:c r="D8" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E8" s="93" t="str">
+        <x:v>PostgreSQL</x:v>
+      </x:c>
+      <x:c r="F8" s="93" t="str">
+        <x:v>Live; verified 15 September 2026</x:v>
+      </x:c>
+      <x:c r="G8" s="93" t="str">
+        <x:v>Reporting and partner management</x:v>
+      </x:c>
+      <x:c r="H8" s="93" t="str">
+        <x:v>database-2; public.Cash Pool Contributions; loan_manager_prod</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="70" customHeight="1">
+      <x:c r="A9" s="93" t="str">
+        <x:v>OLAP production</x:v>
+      </x:c>
+      <x:c r="B9" s="93" t="str">
+        <x:v>1.100044</x:v>
+      </x:c>
+      <x:c r="C9" s="93" t="str">
+        <x:v>Partners</x:v>
+      </x:c>
+      <x:c r="D9" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E9" s="93" t="str">
+        <x:v>PostgreSQL</x:v>
+      </x:c>
+      <x:c r="F9" s="93" t="str">
+        <x:v>Live; verified 15 September 2026</x:v>
+      </x:c>
+      <x:c r="G9" s="93" t="str">
+        <x:v>Reporting and partner management</x:v>
+      </x:c>
+      <x:c r="H9" s="93" t="str">
+        <x:v>database-2; public.Partners; loan_manager_prod</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="70" customHeight="1">
+      <x:c r="A10" s="93" t="str">
+        <x:v>OLAP production</x:v>
+      </x:c>
+      <x:c r="B10" s="93" t="str">
+        <x:v>1.100044</x:v>
+      </x:c>
+      <x:c r="C10" s="93" t="str">
+        <x:v>Settlements</x:v>
+      </x:c>
+      <x:c r="D10" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E10" s="93" t="str">
+        <x:v>PostgreSQL</x:v>
+      </x:c>
+      <x:c r="F10" s="93" t="str">
+        <x:v>Live; verified 15 September 2026</x:v>
+      </x:c>
+      <x:c r="G10" s="93" t="str">
+        <x:v>Reporting and partner management</x:v>
+      </x:c>
+      <x:c r="H10" s="93" t="str">
+        <x:v>database-2; public.Settlements; loan_manager_prod</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="70" customHeight="1">
+      <x:c r="A11" s="93" t="str">
+        <x:v>OLAP production</x:v>
+      </x:c>
+      <x:c r="B11" s="93" t="str">
+        <x:v>1.100044</x:v>
+      </x:c>
+      <x:c r="C11" s="93" t="str">
+        <x:v>Daily Analytics</x:v>
+      </x:c>
+      <x:c r="D11" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E11" s="93" t="str">
+        <x:v>PostgreSQL</x:v>
+      </x:c>
+      <x:c r="F11" s="93" t="str">
+        <x:v>Live; verified 15 September 2026</x:v>
+      </x:c>
+      <x:c r="G11" s="93" t="str">
+        <x:v>Reporting and partner management</x:v>
+      </x:c>
+      <x:c r="H11" s="93" t="str">
+        <x:v>database-2; public.Daily Analytics; loan_manager_prod</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="70" customHeight="1">
+      <x:c r="A12" s="93" t="str">
+        <x:v>OLAP production</x:v>
+      </x:c>
+      <x:c r="B12" s="93" t="str">
+        <x:v>1.100044</x:v>
+      </x:c>
+      <x:c r="C12" s="93" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D12" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E12" s="93" t="str">
+        <x:v>PostgreSQL</x:v>
+      </x:c>
+      <x:c r="F12" s="93" t="str">
+        <x:v>Live; verified 15 September 2026</x:v>
+      </x:c>
+      <x:c r="G12" s="93" t="str">
+        <x:v>Reporting and partner management</x:v>
+      </x:c>
+      <x:c r="H12" s="93" t="str">
+        <x:v>database-2; public.Payment Allocations; loan_manager_prod</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="70" customHeight="1">
+      <x:c r="A13" s="93" t="str">
+        <x:v>OLAP production</x:v>
+      </x:c>
+      <x:c r="B13" s="93" t="str">
+        <x:v>1.100044</x:v>
+      </x:c>
+      <x:c r="C13" s="93" t="str">
+        <x:v>Payments</x:v>
+      </x:c>
+      <x:c r="D13" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E13" s="93" t="str">
+        <x:v>PostgreSQL</x:v>
+      </x:c>
+      <x:c r="F13" s="93" t="str">
+        <x:v>Live; verified 15 September 2026</x:v>
+      </x:c>
+      <x:c r="G13" s="93" t="str">
+        <x:v>Reporting and partner management</x:v>
+      </x:c>
+      <x:c r="H13" s="93" t="str">
+        <x:v>database-2; public.Payments; loan_manager_prod</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="70" customHeight="1">
+      <x:c r="A14" s="93" t="str">
+        <x:v>OLTP production</x:v>
+      </x:c>
+      <x:c r="B14" s="93" t="str">
+        <x:v>3.000067</x:v>
+      </x:c>
+      <x:c r="C14" s="93" t="str">
+        <x:v>Borrowers</x:v>
+      </x:c>
+      <x:c r="D14" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E14" s="93" t="str">
+        <x:v>PostgreSQL</x:v>
+      </x:c>
+      <x:c r="F14" s="93" t="str">
+        <x:v>Live; verified 15 September 2026</x:v>
+      </x:c>
+      <x:c r="G14" s="93" t="str">
+        <x:v>Operational workflow owner</x:v>
+      </x:c>
+      <x:c r="H14" s="93" t="str">
+        <x:v>database-2; public.Borrowers; loan_manager_prod</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="70" customHeight="1">
+      <x:c r="A15" s="93" t="str">
+        <x:v>OLTP production</x:v>
+      </x:c>
+      <x:c r="B15" s="93" t="str">
+        <x:v>3.000067</x:v>
+      </x:c>
+      <x:c r="C15" s="93" t="str">
+        <x:v>Loans</x:v>
+      </x:c>
+      <x:c r="D15" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E15" s="93" t="str">
+        <x:v>PostgreSQL</x:v>
+      </x:c>
+      <x:c r="F15" s="93" t="str">
+        <x:v>Live; verified 15 September 2026</x:v>
+      </x:c>
+      <x:c r="G15" s="93" t="str">
+        <x:v>Operational workflow owner</x:v>
+      </x:c>
+      <x:c r="H15" s="93" t="str">
+        <x:v>database-2; public.Loans; loan_manager_prod</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="70" customHeight="1">
+      <x:c r="A16" s="93" t="str">
+        <x:v>OLTP production</x:v>
+      </x:c>
+      <x:c r="B16" s="93" t="str">
+        <x:v>3.000067</x:v>
+      </x:c>
+      <x:c r="C16" s="93" t="str">
+        <x:v>Repayments</x:v>
+      </x:c>
+      <x:c r="D16" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E16" s="93" t="str">
+        <x:v>PostgreSQL</x:v>
+      </x:c>
+      <x:c r="F16" s="93" t="str">
+        <x:v>Live; verified 15 September 2026</x:v>
+      </x:c>
+      <x:c r="G16" s="93" t="str">
+        <x:v>Operational workflow owner</x:v>
+      </x:c>
+      <x:c r="H16" s="93" t="str">
+        <x:v>database-2; public.Repayments; loan_manager_prod</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="70" customHeight="1">
+      <x:c r="A17" s="93" t="str">
+        <x:v>OLTP production</x:v>
+      </x:c>
+      <x:c r="B17" s="93" t="str">
+        <x:v>3.000067</x:v>
+      </x:c>
+      <x:c r="C17" s="93" t="str">
+        <x:v>Statistics</x:v>
+      </x:c>
+      <x:c r="D17" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E17" s="93" t="str">
+        <x:v>PostgreSQL</x:v>
+      </x:c>
+      <x:c r="F17" s="93" t="str">
+        <x:v>Live; verified 15 September 2026</x:v>
+      </x:c>
+      <x:c r="G17" s="93" t="str">
+        <x:v>Operational workflow owner</x:v>
+      </x:c>
+      <x:c r="H17" s="93" t="str">
+        <x:v>database-2; public.Statistics; loan_manager_prod</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="70" customHeight="1">
+      <x:c r="A18" s="93" t="str">
+        <x:v>OLTP production</x:v>
+      </x:c>
+      <x:c r="B18" s="93" t="str">
+        <x:v>3.000067</x:v>
+      </x:c>
+      <x:c r="C18" s="93" t="str">
+        <x:v>Charges</x:v>
+      </x:c>
+      <x:c r="D18" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E18" s="93" t="str">
+        <x:v>PostgreSQL</x:v>
+      </x:c>
+      <x:c r="F18" s="93" t="str">
+        <x:v>Live; verified 15 September 2026</x:v>
+      </x:c>
+      <x:c r="G18" s="93" t="str">
+        <x:v>Operational workflow owner</x:v>
+      </x:c>
+      <x:c r="H18" s="93" t="str">
+        <x:v>database-2; public.Charges; loan_manager_prod</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="70" customHeight="1">
+      <x:c r="A19" s="93" t="str">
+        <x:v>OLTP production</x:v>
+      </x:c>
+      <x:c r="B19" s="93" t="str">
+        <x:v>3.000067</x:v>
+      </x:c>
+      <x:c r="C19" s="93" t="str">
+        <x:v>Partners</x:v>
+      </x:c>
+      <x:c r="D19" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E19" s="93" t="str">
+        <x:v>PostgreSQL</x:v>
+      </x:c>
+      <x:c r="F19" s="93" t="str">
+        <x:v>Live; verified 15 September 2026</x:v>
+      </x:c>
+      <x:c r="G19" s="93" t="str">
+        <x:v>Operational workflow owner</x:v>
+      </x:c>
+      <x:c r="H19" s="93" t="str">
+        <x:v>database-2; public.Partners; loan_manager_prod</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="70" customHeight="1">
+      <x:c r="A20" s="93" t="str">
+        <x:v>OLTP production</x:v>
+      </x:c>
+      <x:c r="B20" s="93" t="str">
+        <x:v>3.000067</x:v>
+      </x:c>
+      <x:c r="C20" s="93" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D20" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E20" s="93" t="str">
+        <x:v>PostgreSQL</x:v>
+      </x:c>
+      <x:c r="F20" s="93" t="str">
+        <x:v>Live; verified 15 September 2026</x:v>
+      </x:c>
+      <x:c r="G20" s="93" t="str">
+        <x:v>Operational workflow owner</x:v>
+      </x:c>
+      <x:c r="H20" s="93" t="str">
+        <x:v>database-2; public.Payment Allocations; loan_manager_prod</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="70" customHeight="1">
+      <x:c r="A21" s="93" t="str">
+        <x:v>OLTP production</x:v>
+      </x:c>
+      <x:c r="B21" s="93" t="str">
+        <x:v>3.000067</x:v>
+      </x:c>
+      <x:c r="C21" s="93" t="str">
+        <x:v>Payments</x:v>
+      </x:c>
+      <x:c r="D21" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E21" s="93" t="str">
+        <x:v>PostgreSQL</x:v>
+      </x:c>
+      <x:c r="F21" s="93" t="str">
+        <x:v>Live; verified 15 September 2026</x:v>
+      </x:c>
+      <x:c r="G21" s="93" t="str">
+        <x:v>Operational workflow owner</x:v>
+      </x:c>
+      <x:c r="H21" s="93" t="str">
+        <x:v>database-2; public.Payments; loan_manager_prod</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="70" customHeight="1">
+      <x:c r="A22" s="93" t="str">
+        <x:v>Shared production</x:v>
+      </x:c>
+      <x:c r="B22" s="93" t="str">
+        <x:v>OLAP 1.100044; OLTP 3.000067</x:v>
+      </x:c>
+      <x:c r="C22" s="93" t="str">
+        <x:v>All SQL tables</x:v>
+      </x:c>
+      <x:c r="D22" s="93" t="str">
+        <x:v>Row ID</x:v>
+      </x:c>
+      <x:c r="E22" s="93" t="str">
+        <x:v>Text key</x:v>
+      </x:c>
+      <x:c r="F22" s="93" t="str">
+        <x:v>Exact case and values preserved</x:v>
+      </x:c>
+      <x:c r="G22" s="93" t="str">
+        <x:v>Ref joins and offline identity</x:v>
+      </x:c>
+      <x:c r="H22" s="93" t="str">
+        <x:v>PostgreSQL text primary keys; AppSheet UNIQUEID("PackedUUID") initial preserved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="70" customHeight="1">
+      <x:c r="A23" s="93" t="str">
+        <x:v>Shared production</x:v>
+      </x:c>
+      <x:c r="B23" s="93" t="str">
+        <x:v>OLAP 1.100044; OLTP 3.000067</x:v>
+      </x:c>
+      <x:c r="C23" s="93" t="str">
+        <x:v>Loans</x:v>
+      </x:c>
+      <x:c r="D23" s="93" t="str">
+        <x:v>Borrower Name</x:v>
+      </x:c>
+      <x:c r="E23" s="93" t="str">
+        <x:v>SQL lookup</x:v>
+      </x:c>
+      <x:c r="F23" s="93" t="str">
+        <x:v>Insert and rename verified in copy</x:v>
+      </x:c>
+      <x:c r="G23" s="93" t="str">
+        <x:v>Both apps consume stored lookup</x:v>
+      </x:c>
+      <x:c r="H23" s="93" t="str">
+        <x:v>Existing SQL lookup and propagation triggers retained. No AppSheet formula change.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="70" customHeight="1">
+      <x:c r="A24" s="93" t="str">
+        <x:v>Shared production</x:v>
+      </x:c>
+      <x:c r="B24" s="93" t="str">
+        <x:v>OLAP 1.100044; OLTP 3.000067</x:v>
+      </x:c>
+      <x:c r="C24" s="93" t="str">
+        <x:v>Shared references</x:v>
+      </x:c>
+      <x:c r="D24" s="93" t="str">
+        <x:v>Foreign keys</x:v>
+      </x:c>
+      <x:c r="E24" s="93" t="str">
+        <x:v>13 constraints</x:v>
+      </x:c>
+      <x:c r="F24" s="93" t="str">
+        <x:v>Retained</x:v>
+      </x:c>
+      <x:c r="G24" s="93" t="str">
+        <x:v>Protect existing references</x:v>
+      </x:c>
+      <x:c r="H24" s="93" t="str">
+        <x:v>NO ACTION; validated; eight blank-Ref normalization triggers retained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="70" customHeight="1">
+      <x:c r="A25" s="93" t="str">
+        <x:v>OLAP production</x:v>
+      </x:c>
+      <x:c r="B25" s="93" t="str">
+        <x:v>1.100044</x:v>
+      </x:c>
+      <x:c r="C25" s="93" t="str">
+        <x:v>Calendar</x:v>
+      </x:c>
+      <x:c r="D25" s="93" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="E25" s="93" t="str">
+        <x:v>Google Sheets</x:v>
+      </x:c>
+      <x:c r="F25" s="93" t="str">
+        <x:v>Unchanged</x:v>
+      </x:c>
+      <x:c r="G25" s="93" t="str">
+        <x:v>Daily analytics and projections</x:v>
+      </x:c>
+      <x:c r="H25" s="93" t="str">
+        <x:v>Calendar Help Table / Sheet1; source google.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="70" customHeight="1">
+      <x:c r="A26" s="93" t="str">
+        <x:v>OLAP production</x:v>
+      </x:c>
+      <x:c r="B26" s="93" t="str">
+        <x:v>1.100044</x:v>
+      </x:c>
+      <x:c r="C26" s="93" t="str">
+        <x:v>Automation</x:v>
+      </x:c>
+      <x:c r="D26" s="93" t="str">
+        <x:v>Daily analytics schedules</x:v>
+      </x:c>
+      <x:c r="E26" s="93" t="str">
+        <x:v>Bot enablement</x:v>
+      </x:c>
+      <x:c r="F26" s="93" t="str">
+        <x:v>Original state restored</x:v>
+      </x:c>
+      <x:c r="G26" s="93" t="str">
+        <x:v>Reporting snapshots</x:v>
+      </x:c>
+      <x:c r="H26" s="93" t="str">
+        <x:v>Refresh Daily Analytics Daily 2 enabled; Refresh Daily Analytics Daily remains disabled.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="70" customHeight="1">
+      <x:c r="A27" s="93" t="str">
+        <x:v>OLTP production</x:v>
+      </x:c>
+      <x:c r="B27" s="93" t="str">
+        <x:v>3.000067</x:v>
+      </x:c>
+      <x:c r="C27" s="93" t="str">
+        <x:v>Automation</x:v>
+      </x:c>
+      <x:c r="D27" s="93" t="str">
+        <x:v>Generate Daily Charges</x:v>
+      </x:c>
+      <x:c r="E27" s="93" t="str">
+        <x:v>Bot enablement</x:v>
+      </x:c>
+      <x:c r="F27" s="93" t="str">
+        <x:v>Enabled; catch-up verified</x:v>
+      </x:c>
+      <x:c r="G27" s="93" t="str">
+        <x:v>Daily charge workflow</x:v>
+      </x:c>
+      <x:c r="H27" s="93" t="str">
+        <x:v>15 September: 28 eligible daily-interest loans; 28 charges; interest 8040; principal 0; no duplicates.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="70" customHeight="1">
+      <x:c r="A28" s="93" t="str">
+        <x:v>Shared production</x:v>
+      </x:c>
+      <x:c r="B28" s="93" t="str">
+        <x:v>OLAP 1.100044; OLTP 3.000067</x:v>
+      </x:c>
+      <x:c r="C28" s="93" t="str">
+        <x:v>All business tables</x:v>
+      </x:c>
+      <x:c r="D28" s="93" t="str">
+        <x:v>Reconciliation</x:v>
+      </x:c>
+      <x:c r="E28" s="93" t="str">
+        <x:v>Readback</x:v>
+      </x:c>
+      <x:c r="F28" s="93" t="str">
+        <x:v>1936 rows before catch-up</x:v>
+      </x:c>
+      <x:c r="G28" s="93" t="str">
+        <x:v>Frozen source versus SQL</x:v>
+      </x:c>
+      <x:c r="H28" s="93" t="str">
+        <x:v>Zero scalar or relationship membership differences. 42 relationship lists had ordering-only changes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="70" customHeight="1">
+      <x:c r="A29" s="93" t="str">
+        <x:v>Rollback</x:v>
+      </x:c>
+      <x:c r="B29" s="93" t="str">
+        <x:v>OLAP 1.100041; OLTP 3.000064</x:v>
+      </x:c>
+      <x:c r="C29" s="93" t="str">
+        <x:v>Money database</x:v>
+      </x:c>
+      <x:c r="D29" s="93" t="str">
+        <x:v>Retained source</x:v>
+      </x:c>
+      <x:c r="E29" s="93" t="str">
+        <x:v>Recovery</x:v>
+      </x:c>
+      <x:c r="F29" s="93" t="str">
+        <x:v>Not receiving production app writes</x:v>
+      </x:c>
+      <x:c r="G29" s="93" t="str">
+        <x:v>Preserve SQL writes before reverting</x:v>
+      </x:c>
+      <x:c r="H29" s="93" t="str">
+        <x:v>Pause writers, reconcile post-cutover SQL rows back to Money, then restore app versions. Version rollback alone is insufficient.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7737,7 +8521,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac8cbbe7055042a5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0994f172d94485e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18394,7 +19178,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R860e73688a58498e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3d5328b5ee9454e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18823,7 +19607,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a94ab0d5d6a4bf3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c3ba416a7af4209"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19283,7 +20067,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6022775a3534717"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re15634c62f4b4495"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26257,7 +27041,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1a339f52e654366"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58d5afb30c994d66"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30876,7 +31660,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf62fd073135f4b50"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re206edd6336e442e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31075,7 +31859,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf0f3bc89adf4309"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra978d656032e42da"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32728,7 +33512,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf305118bdaf54241"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32f018daf73d4ca8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Replace stored loan borrower name with virtual reference
</commit_message>
<xml_diff>
--- a/Documents/AppSheet_Data_Dictionary.xlsx
+++ b/Documents/AppSheet_Data_Dictionary.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R87f961343a4c4162"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="Raf890574b7404e37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R214a37e456924257"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="Rf1ef2366d0454831"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="R334a6ec9ba484853"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R0d60b2220f0c455b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="R0b86f1bd436f43d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R930fa9e07dea4184"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="Raf32ef7469bc4a46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R78da8a37e92b44cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="R1e49f9caa4c74c4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="R88dd66015c684121"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Sync POC" sheetId="13" r:id="R8f777c62be1f41b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Migration Trial" sheetId="14" r:id="R5848d795d9294f80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Production" sheetId="15" r:id="R65be325a420a4ad3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rf0ed312a3e6f4b9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="Rde46409949f642bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="Rab803b2955cf401b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="Rc075e7fd93ef4ca1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="R683d94cf57a14fcb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R447093ce53e54b82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="R3a4039ccda1a4913"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="Ree86cf3ec0b34ebc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="R7fec76bdb03147be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R53c4f39aea734918"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="Rbc03cfb8c9a54d90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="R2e1a80d6ed164700"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Sync POC" sheetId="13" r:id="R2db5f11bbc5247bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Migration Trial" sheetId="14" r:id="R6c46f41c58e04088"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Production" sheetId="15" r:id="Reef12395164f47f3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2597,7 +2597,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f0b4debb7964235"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ca0b1d095934b11"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7379,7 +7379,7 @@
         <x:v>OLAP production</x:v>
       </x:c>
       <x:c r="B2" s="93" t="str">
-        <x:v>1.100044</x:v>
+        <x:v>1.100046</x:v>
       </x:c>
       <x:c r="C2" s="93" t="str">
         <x:v>Borrowers</x:v>
@@ -7405,7 +7405,7 @@
         <x:v>OLAP production</x:v>
       </x:c>
       <x:c r="B3" s="93" t="str">
-        <x:v>1.100044</x:v>
+        <x:v>1.100046</x:v>
       </x:c>
       <x:c r="C3" s="93" t="str">
         <x:v>Loans</x:v>
@@ -7431,7 +7431,7 @@
         <x:v>OLAP production</x:v>
       </x:c>
       <x:c r="B4" s="93" t="str">
-        <x:v>1.100044</x:v>
+        <x:v>1.100046</x:v>
       </x:c>
       <x:c r="C4" s="93" t="str">
         <x:v>Repayments</x:v>
@@ -7457,7 +7457,7 @@
         <x:v>OLAP production</x:v>
       </x:c>
       <x:c r="B5" s="93" t="str">
-        <x:v>1.100044</x:v>
+        <x:v>1.100046</x:v>
       </x:c>
       <x:c r="C5" s="93" t="str">
         <x:v>Statistics</x:v>
@@ -7483,7 +7483,7 @@
         <x:v>OLAP production</x:v>
       </x:c>
       <x:c r="B6" s="93" t="str">
-        <x:v>1.100044</x:v>
+        <x:v>1.100046</x:v>
       </x:c>
       <x:c r="C6" s="93" t="str">
         <x:v>Charges</x:v>
@@ -7509,7 +7509,7 @@
         <x:v>OLAP production</x:v>
       </x:c>
       <x:c r="B7" s="93" t="str">
-        <x:v>1.100044</x:v>
+        <x:v>1.100046</x:v>
       </x:c>
       <x:c r="C7" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -7535,7 +7535,7 @@
         <x:v>OLAP production</x:v>
       </x:c>
       <x:c r="B8" s="93" t="str">
-        <x:v>1.100044</x:v>
+        <x:v>1.100046</x:v>
       </x:c>
       <x:c r="C8" s="93" t="str">
         <x:v>Cash Pool Contributions</x:v>
@@ -7561,7 +7561,7 @@
         <x:v>OLAP production</x:v>
       </x:c>
       <x:c r="B9" s="93" t="str">
-        <x:v>1.100044</x:v>
+        <x:v>1.100046</x:v>
       </x:c>
       <x:c r="C9" s="93" t="str">
         <x:v>Partners</x:v>
@@ -7587,7 +7587,7 @@
         <x:v>OLAP production</x:v>
       </x:c>
       <x:c r="B10" s="93" t="str">
-        <x:v>1.100044</x:v>
+        <x:v>1.100046</x:v>
       </x:c>
       <x:c r="C10" s="93" t="str">
         <x:v>Settlements</x:v>
@@ -7613,7 +7613,7 @@
         <x:v>OLAP production</x:v>
       </x:c>
       <x:c r="B11" s="93" t="str">
-        <x:v>1.100044</x:v>
+        <x:v>1.100046</x:v>
       </x:c>
       <x:c r="C11" s="93" t="str">
         <x:v>Daily Analytics</x:v>
@@ -7639,7 +7639,7 @@
         <x:v>OLAP production</x:v>
       </x:c>
       <x:c r="B12" s="93" t="str">
-        <x:v>1.100044</x:v>
+        <x:v>1.100046</x:v>
       </x:c>
       <x:c r="C12" s="93" t="str">
         <x:v>Payment Allocations</x:v>
@@ -7665,7 +7665,7 @@
         <x:v>OLAP production</x:v>
       </x:c>
       <x:c r="B13" s="93" t="str">
-        <x:v>1.100044</x:v>
+        <x:v>1.100046</x:v>
       </x:c>
       <x:c r="C13" s="93" t="str">
         <x:v>Payments</x:v>
@@ -7691,7 +7691,7 @@
         <x:v>OLTP production</x:v>
       </x:c>
       <x:c r="B14" s="93" t="str">
-        <x:v>3.000067</x:v>
+        <x:v>3.000069</x:v>
       </x:c>
       <x:c r="C14" s="93" t="str">
         <x:v>Borrowers</x:v>
@@ -7717,7 +7717,7 @@
         <x:v>OLTP production</x:v>
       </x:c>
       <x:c r="B15" s="93" t="str">
-        <x:v>3.000067</x:v>
+        <x:v>3.000069</x:v>
       </x:c>
       <x:c r="C15" s="93" t="str">
         <x:v>Loans</x:v>
@@ -7743,7 +7743,7 @@
         <x:v>OLTP production</x:v>
       </x:c>
       <x:c r="B16" s="93" t="str">
-        <x:v>3.000067</x:v>
+        <x:v>3.000069</x:v>
       </x:c>
       <x:c r="C16" s="93" t="str">
         <x:v>Repayments</x:v>
@@ -7769,7 +7769,7 @@
         <x:v>OLTP production</x:v>
       </x:c>
       <x:c r="B17" s="93" t="str">
-        <x:v>3.000067</x:v>
+        <x:v>3.000069</x:v>
       </x:c>
       <x:c r="C17" s="93" t="str">
         <x:v>Statistics</x:v>
@@ -7795,7 +7795,7 @@
         <x:v>OLTP production</x:v>
       </x:c>
       <x:c r="B18" s="93" t="str">
-        <x:v>3.000067</x:v>
+        <x:v>3.000069</x:v>
       </x:c>
       <x:c r="C18" s="93" t="str">
         <x:v>Charges</x:v>
@@ -7821,7 +7821,7 @@
         <x:v>OLTP production</x:v>
       </x:c>
       <x:c r="B19" s="93" t="str">
-        <x:v>3.000067</x:v>
+        <x:v>3.000069</x:v>
       </x:c>
       <x:c r="C19" s="93" t="str">
         <x:v>Partners</x:v>
@@ -7847,7 +7847,7 @@
         <x:v>OLTP production</x:v>
       </x:c>
       <x:c r="B20" s="93" t="str">
-        <x:v>3.000067</x:v>
+        <x:v>3.000069</x:v>
       </x:c>
       <x:c r="C20" s="93" t="str">
         <x:v>Payment Allocations</x:v>
@@ -7873,7 +7873,7 @@
         <x:v>OLTP production</x:v>
       </x:c>
       <x:c r="B21" s="93" t="str">
-        <x:v>3.000067</x:v>
+        <x:v>3.000069</x:v>
       </x:c>
       <x:c r="C21" s="93" t="str">
         <x:v>Payments</x:v>
@@ -7899,7 +7899,7 @@
         <x:v>Shared production</x:v>
       </x:c>
       <x:c r="B22" s="93" t="str">
-        <x:v>OLAP 1.100044; OLTP 3.000067</x:v>
+        <x:v>OLAP 1.100046; OLTP 3.000069</x:v>
       </x:c>
       <x:c r="C22" s="93" t="str">
         <x:v>All SQL tables</x:v>
@@ -7925,7 +7925,7 @@
         <x:v>Shared production</x:v>
       </x:c>
       <x:c r="B23" s="93" t="str">
-        <x:v>OLAP 1.100044; OLTP 3.000067</x:v>
+        <x:v>OLAP 1.100046; OLTP 3.000069</x:v>
       </x:c>
       <x:c r="C23" s="93" t="str">
         <x:v>Loans</x:v>
@@ -7934,16 +7934,16 @@
         <x:v>Borrower Name</x:v>
       </x:c>
       <x:c r="E23" s="93" t="str">
-        <x:v>SQL lookup</x:v>
+        <x:v>VC / Name</x:v>
       </x:c>
       <x:c r="F23" s="93" t="str">
-        <x:v>Insert and rename verified in copy</x:v>
+        <x:v>62/62 names verified</x:v>
       </x:c>
       <x:c r="G23" s="93" t="str">
-        <x:v>Both apps consume stored lookup</x:v>
+        <x:v>Both production apps and both SQL test copies</x:v>
       </x:c>
       <x:c r="H23" s="93" t="str">
-        <x:v>Existing SQL lookup and propagation triggers retained. No AppSheet formula change.</x:v>
+        <x:v>[Ref Borrowers].[Borrower Name]. Stored SQL column and two name triggers/functions removed.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="70" customHeight="1">
@@ -7951,7 +7951,7 @@
         <x:v>Shared production</x:v>
       </x:c>
       <x:c r="B24" s="93" t="str">
-        <x:v>OLAP 1.100044; OLTP 3.000067</x:v>
+        <x:v>OLAP 1.100046; OLTP 3.000069</x:v>
       </x:c>
       <x:c r="C24" s="93" t="str">
         <x:v>Shared references</x:v>
@@ -7977,7 +7977,7 @@
         <x:v>OLAP production</x:v>
       </x:c>
       <x:c r="B25" s="93" t="str">
-        <x:v>1.100044</x:v>
+        <x:v>1.100046</x:v>
       </x:c>
       <x:c r="C25" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8003,7 +8003,7 @@
         <x:v>OLAP production</x:v>
       </x:c>
       <x:c r="B26" s="93" t="str">
-        <x:v>1.100044</x:v>
+        <x:v>1.100046</x:v>
       </x:c>
       <x:c r="C26" s="93" t="str">
         <x:v>Automation</x:v>
@@ -8029,7 +8029,7 @@
         <x:v>OLTP production</x:v>
       </x:c>
       <x:c r="B27" s="93" t="str">
-        <x:v>3.000067</x:v>
+        <x:v>3.000069</x:v>
       </x:c>
       <x:c r="C27" s="93" t="str">
         <x:v>Automation</x:v>
@@ -8055,7 +8055,7 @@
         <x:v>Shared production</x:v>
       </x:c>
       <x:c r="B28" s="93" t="str">
-        <x:v>OLAP 1.100044; OLTP 3.000067</x:v>
+        <x:v>OLAP 1.100046; OLTP 3.000069</x:v>
       </x:c>
       <x:c r="C28" s="93" t="str">
         <x:v>All business tables</x:v>
@@ -8312,19 +8312,19 @@
         <x:v>Loans</x:v>
       </x:c>
       <x:c r="B11" s="59" t="str">
-        <x:v>Money database</x:v>
+        <x:v>PostgreSQL loan_manager_prod</x:v>
       </x:c>
       <x:c r="C11" s="57" t="str">
         <x:v>OLTP + OLAP</x:v>
       </x:c>
       <x:c r="D11" s="57" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E11" s="57" t="n">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="E11" s="57" t="n">
-        <x:v>20</x:v>
-      </x:c>
       <x:c r="F11" s="57" t="n">
-        <x:v>30</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="G11" s="59" t="str">
         <x:v>Loan contracts, commercial terms, lifecycle state, balances, daily-installment reporting, and loan-level risk metrics.</x:v>
@@ -8521,7 +8521,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0994f172d94485e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3bea91a1e86d4b56"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13480,30 +13480,30 @@
         <x:v>Stored source column; initial value: "ยังไม่ปิดยอด"</x:v>
       </x:c>
     </x:row>
-    <x:row r="185" ht="15" customHeight="1">
-      <x:c r="A185" s="57" t="str">
+    <x:row r="185" ht="85" customHeight="1">
+      <x:c r="A185" s="82" t="str">
         <x:v>Loans</x:v>
       </x:c>
-      <x:c r="B185" s="57" t="n">
+      <x:c r="B185" s="82" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C185" s="59" t="str">
+      <x:c r="C185" s="82" t="str">
         <x:v>Borrower Name</x:v>
       </x:c>
-      <x:c r="D185" s="59" t="str">
-        <x:v>Physical / Name</x:v>
-      </x:c>
-      <x:c r="E185" s="57" t="str">
+      <x:c r="D185" s="82" t="str">
+        <x:v>VC / Name</x:v>
+      </x:c>
+      <x:c r="E185" s="82" t="str">
         <x:v>OLTP + OLAP</x:v>
       </x:c>
-      <x:c r="F185" s="57" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G185" s="59" t="str">
-        <x:v>Stores the authoritative source value for Borrower Name.</x:v>
-      </x:c>
-      <x:c r="H185" s="59" t="str">
-        <x:v>Stored source column</x:v>
+      <x:c r="F185" s="82" t="str">
+        <x:v>Read-only; visible; searchable; display: ชื่อผู้กู้ / Borrower</x:v>
+      </x:c>
+      <x:c r="G185" s="82" t="str">
+        <x:v>Current name from referenced borrower; SQL stored copy and maintenance triggers removed. Verified OLTP 3.000069 / OLAP 1.100046.</x:v>
+      </x:c>
+      <x:c r="H185" s="82" t="str">
+        <x:v>[Ref Borrowers].[Borrower Name]</x:v>
       </x:c>
     </x:row>
     <x:row r="186" ht="15" customHeight="1">
@@ -19178,7 +19178,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3d5328b5ee9454e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref9309fac28842d7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19607,7 +19607,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c3ba416a7af4209"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra424ecf4053142ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20067,7 +20067,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re15634c62f4b4495"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47b05cd0d51b479b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27041,7 +27041,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58d5afb30c994d66"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f4cef7ad5234c95"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31660,7 +31660,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re206edd6336e442e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68a4b3d789b5468f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31859,7 +31859,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra978d656032e42da"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R121cfdcf720d426f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33512,7 +33512,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32f018daf73d4ca8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re27eaf22dae84519"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Prototype PostgreSQL OLAP assessment and verify performance
</commit_message>
<xml_diff>
--- a/Documents/AppSheet_Data_Dictionary.xlsx
+++ b/Documents/AppSheet_Data_Dictionary.xlsx
@@ -2,21 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rf0ed312a3e6f4b9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="Rde46409949f642bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="Rab803b2955cf401b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="Rc075e7fd93ef4ca1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="R683d94cf57a14fcb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R447093ce53e54b82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="R3a4039ccda1a4913"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="Ree86cf3ec0b34ebc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="R7fec76bdb03147be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R53c4f39aea734918"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="Rbc03cfb8c9a54d90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="R2e1a80d6ed164700"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Sync POC" sheetId="13" r:id="R2db5f11bbc5247bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Migration Trial" sheetId="14" r:id="R6c46f41c58e04088"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Production" sheetId="15" r:id="Reef12395164f47f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rc75993a5ae9741b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="R8e1e9dad4c3c4fc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R811906d220094419"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="Rb33b55c9f30e43c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="Re59298d9cf21435f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="Re38426ef954f449c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Re659dca2847d4cbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R110eb759a3d54f14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="Rcb9cca1bacd54321"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R7e36101782984bea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="R983ac1f63b5b4e99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="R76201da1b8b34104"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Sync POC" sheetId="13" r:id="R51a155331f904249"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Migration Trial" sheetId="14" r:id="R5ef0f4c5e673403b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Production" sheetId="15" r:id="Rb18515b98bd14dcb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLAP Assessment SQL" sheetId="16" r:id="Rca4c901941ff47c5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -101,7 +102,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="36">
+  <x:fills count="37">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -136,6 +137,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -408,7 +414,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="129">
+  <x:cellXfs count="132">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -690,6 +696,11 @@
     <x:xf numFmtId="0" fontId="11" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="12" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="12" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2597,7 +2608,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ca0b1d095934b11"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf252e8990e2d478d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8100,6 +8111,1585 @@
       </x:c>
       <x:c r="H29" s="93" t="str">
         <x:v>Pause writers, reconcile post-cutover SQL rows back to Money, then restore app versions. Version rollback alone is insufficient.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="17" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="35" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="30" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="55" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="100" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="131" t="str">
+        <x:v>Experiment</x:v>
+      </x:c>
+      <x:c r="B1" s="131" t="str">
+        <x:v>App version</x:v>
+      </x:c>
+      <x:c r="C1" s="131" t="str">
+        <x:v>Table</x:v>
+      </x:c>
+      <x:c r="D1" s="131" t="str">
+        <x:v>Column / setting</x:v>
+      </x:c>
+      <x:c r="E1" s="131" t="str">
+        <x:v>Type</x:v>
+      </x:c>
+      <x:c r="F1" s="131" t="str">
+        <x:v>Scope / status</x:v>
+      </x:c>
+      <x:c r="G1" s="131" t="str">
+        <x:v>Purpose / dependencies</x:v>
+      </x:c>
+      <x:c r="H1" s="131" t="str">
+        <x:v>Exact definition</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="65" customHeight="1">
+      <x:c r="A2" s="93" t="str">
+        <x:v>Scope</x:v>
+      </x:c>
+      <x:c r="B2" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C2" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D2" s="93" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="E2" s="93" t="str">
+        <x:v>PostgreSQL view</x:v>
+      </x:c>
+      <x:c r="F2" s="93" t="str">
+        <x:v>Test copy only; review pending</x:v>
+      </x:c>
+      <x:c r="G2" s="93" t="str">
+        <x:v>Own input/result table; reads shared financial data</x:v>
+      </x:c>
+      <x:c r="H2" s="93" t="str">
+        <x:v>public.Loan Assessment SQL Lab View → public.Loan Assessment SQL Lab</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="65" customHeight="1">
+      <x:c r="A3" s="93" t="str">
+        <x:v>Scope</x:v>
+      </x:c>
+      <x:c r="B3" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C3" s="93" t="str">
+        <x:v>Calendar</x:v>
+      </x:c>
+      <x:c r="D3" s="93" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="E3" s="93" t="str">
+        <x:v>Generated SQL view</x:v>
+      </x:c>
+      <x:c r="F3" s="93" t="str">
+        <x:v>Test copy only; read-only</x:v>
+      </x:c>
+      <x:c r="G3" s="93" t="str">
+        <x:v>153 dates retained for Daily Analytics; 16 assessment VCs removed</x:v>
+      </x:c>
+      <x:c r="H3" s="93" t="str">
+        <x:v>public.OLAP Calendar SQL Lab; 2026-08-01 through 2026-12-31</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="65" customHeight="1">
+      <x:c r="A4" s="93" t="str">
+        <x:v>Rollback</x:v>
+      </x:c>
+      <x:c r="B4" s="93" t="str">
+        <x:v>1.000013</x:v>
+      </x:c>
+      <x:c r="C4" s="93" t="str">
+        <x:v>OLAP test copy</x:v>
+      </x:c>
+      <x:c r="D4" s="93" t="str">
+        <x:v>Restore app version</x:v>
+      </x:c>
+      <x:c r="E4" s="93" t="str">
+        <x:v>AppSheet version</x:v>
+      </x:c>
+      <x:c r="F4" s="93" t="str">
+        <x:v>Production versions unchanged</x:v>
+      </x:c>
+      <x:c r="G4" s="93" t="str">
+        <x:v>Production OLAP 1.100046; OLTP 3.000069</x:v>
+      </x:c>
+      <x:c r="H4" s="93" t="str">
+        <x:v>Restores original Loan Assessment source and Calendar Help Table / Sheet1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="65" customHeight="1">
+      <x:c r="A5" s="93" t="str">
+        <x:v>Workflow</x:v>
+      </x:c>
+      <x:c r="B5" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C5" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D5" s="93" t="str">
+        <x:v>Refresh Assessment</x:v>
+      </x:c>
+      <x:c r="E5" s="93" t="str">
+        <x:v>Data action</x:v>
+      </x:c>
+      <x:c r="F5" s="93" t="str">
+        <x:v>Test copy only</x:v>
+      </x:c>
+      <x:c r="G5" s="93" t="str">
+        <x:v>Trigger recalculates current row; result timestamp shown</x:v>
+      </x:c>
+      <x:c r="H5" s="93" t="str">
+        <x:v>SQL Refresh Token = UNIQUEID()</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="65" customHeight="1">
+      <x:c r="A6" s="93" t="str">
+        <x:v>Freshness</x:v>
+      </x:c>
+      <x:c r="B6" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C6" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D6" s="93" t="str">
+        <x:v>SQL Source Current</x:v>
+      </x:c>
+      <x:c r="E6" s="93" t="str">
+        <x:v>View calculation</x:v>
+      </x:c>
+      <x:c r="F6" s="93" t="str">
+        <x:v>Checked on sync</x:v>
+      </x:c>
+      <x:c r="G6" s="93" t="str">
+        <x:v>Source fingerprint/date mismatch hides stale outputs; offline changes require sync</x:v>
+      </x:c>
+      <x:c r="H6" s="93" t="str">
+        <x:v>assessment_lab.fingerprint(assessment_lab.inputs(Ref Borrower)); Bangkok as-of date</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="65" customHeight="1">
+      <x:c r="A7" s="93" t="str">
+        <x:v>Window</x:v>
+      </x:c>
+      <x:c r="B7" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C7" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D7" s="93" t="str">
+        <x:v>Forecast boundaries</x:v>
+      </x:c>
+      <x:c r="E7" s="93" t="str">
+        <x:v>Explicit dates</x:v>
+      </x:c>
+      <x:c r="F7" s="93" t="str">
+        <x:v>Like-for-like test window</x:v>
+      </x:c>
+      <x:c r="G7" s="93" t="str">
+        <x:v>Rolling horizon and shared/per-user input workflow require review before cutover</x:v>
+      </x:c>
+      <x:c r="H7" s="93" t="str">
+        <x:v>SQL Forecast Start 2026-08-01; SQL Forecast End 2026-12-31</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="65" customHeight="1">
+      <x:c r="A8" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B8" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C8" s="93" t="str">
+        <x:v>Calendar</x:v>
+      </x:c>
+      <x:c r="D8" s="93" t="str">
+        <x:v>_RowNumber</x:v>
+      </x:c>
+      <x:c r="E8" s="93" t="str">
+        <x:v>Physical / Number</x:v>
+      </x:c>
+      <x:c r="F8" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G8" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden Yes</x:v>
+      </x:c>
+      <x:c r="H8" s="93" t="str">
+        <x:v>Stored SQL value / generated date</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="65" customHeight="1">
+      <x:c r="A9" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B9" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C9" s="93" t="str">
+        <x:v>Calendar</x:v>
+      </x:c>
+      <x:c r="D9" s="93" t="str">
+        <x:v>Date</x:v>
+      </x:c>
+      <x:c r="E9" s="93" t="str">
+        <x:v>Physical / Date</x:v>
+      </x:c>
+      <x:c r="F9" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G9" s="93" t="str">
+        <x:v>Key Yes; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H9" s="93" t="str">
+        <x:v>Stored SQL value / generated date</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="65" customHeight="1">
+      <x:c r="A10" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B10" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C10" s="93" t="str">
+        <x:v>Calendar</x:v>
+      </x:c>
+      <x:c r="D10" s="93" t="str">
+        <x:v>Year</x:v>
+      </x:c>
+      <x:c r="E10" s="93" t="str">
+        <x:v>VC / Number</x:v>
+      </x:c>
+      <x:c r="F10" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G10" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H10" s="93" t="str">
+        <x:v>YEAR([Date])</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="65" customHeight="1">
+      <x:c r="A11" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B11" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C11" s="93" t="str">
+        <x:v>Calendar</x:v>
+      </x:c>
+      <x:c r="D11" s="93" t="str">
+        <x:v>Month</x:v>
+      </x:c>
+      <x:c r="E11" s="93" t="str">
+        <x:v>VC / Number</x:v>
+      </x:c>
+      <x:c r="F11" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G11" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H11" s="93" t="str">
+        <x:v>MONTH([Date])</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="65" customHeight="1">
+      <x:c r="A12" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B12" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C12" s="93" t="str">
+        <x:v>Calendar</x:v>
+      </x:c>
+      <x:c r="D12" s="93" t="str">
+        <x:v>Month Name</x:v>
+      </x:c>
+      <x:c r="E12" s="93" t="str">
+        <x:v>VC / Text</x:v>
+      </x:c>
+      <x:c r="F12" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G12" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H12" s="93" t="str">
+        <x:v>TEXT([Date], "MMMM")</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="65" customHeight="1">
+      <x:c r="A13" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B13" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C13" s="93" t="str">
+        <x:v>Calendar</x:v>
+      </x:c>
+      <x:c r="D13" s="93" t="str">
+        <x:v>Year Month</x:v>
+      </x:c>
+      <x:c r="E13" s="93" t="str">
+        <x:v>VC / Text</x:v>
+      </x:c>
+      <x:c r="F13" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G13" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H13" s="93" t="str">
+        <x:v>TEXT([Date], "YYYY-MM")</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="65" customHeight="1">
+      <x:c r="A14" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B14" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C14" s="93" t="str">
+        <x:v>Calendar</x:v>
+      </x:c>
+      <x:c r="D14" s="93" t="str">
+        <x:v>Week</x:v>
+      </x:c>
+      <x:c r="E14" s="93" t="str">
+        <x:v>VC / Number</x:v>
+      </x:c>
+      <x:c r="F14" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G14" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H14" s="93" t="str">
+        <x:v>WEEKNUM([Date])</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="65" customHeight="1">
+      <x:c r="A15" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B15" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C15" s="93" t="str">
+        <x:v>Calendar</x:v>
+      </x:c>
+      <x:c r="D15" s="93" t="str">
+        <x:v>Year Week</x:v>
+      </x:c>
+      <x:c r="E15" s="93" t="str">
+        <x:v>VC / Text</x:v>
+      </x:c>
+      <x:c r="F15" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G15" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H15" s="93" t="str">
+        <x:v>CONCATENATE(YEAR([Date]), "-W", RIGHT("0" &amp; WEEKNUM([Date]), 2))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="65" customHeight="1">
+      <x:c r="A16" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B16" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C16" s="93" t="str">
+        <x:v>Calendar</x:v>
+      </x:c>
+      <x:c r="D16" s="93" t="str">
+        <x:v>Week Start</x:v>
+      </x:c>
+      <x:c r="E16" s="93" t="str">
+        <x:v>VC / Date</x:v>
+      </x:c>
+      <x:c r="F16" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G16" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H16" s="93" t="str">
+        <x:v>[Date] - MOD(WEEKDAY([Date]) + 5, 7)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="65" customHeight="1">
+      <x:c r="A17" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B17" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C17" s="93" t="str">
+        <x:v>Calendar</x:v>
+      </x:c>
+      <x:c r="D17" s="93" t="str">
+        <x:v>Quarter</x:v>
+      </x:c>
+      <x:c r="E17" s="93" t="str">
+        <x:v>VC / Text</x:v>
+      </x:c>
+      <x:c r="F17" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G17" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H17" s="93" t="str">
+        <x:v>CONCATENATE( "Q", CEILING(MONTH([Date]) / 3) )</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="65" customHeight="1">
+      <x:c r="A18" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B18" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C18" s="93" t="str">
+        <x:v>Calendar</x:v>
+      </x:c>
+      <x:c r="D18" s="93" t="str">
+        <x:v>Day of Week</x:v>
+      </x:c>
+      <x:c r="E18" s="93" t="str">
+        <x:v>VC / Text</x:v>
+      </x:c>
+      <x:c r="F18" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G18" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H18" s="93" t="str">
+        <x:v>TEXT([Date], "dddd")</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="65" customHeight="1">
+      <x:c r="A19" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B19" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C19" s="93" t="str">
+        <x:v>Calendar</x:v>
+      </x:c>
+      <x:c r="D19" s="93" t="str">
+        <x:v>Day of Month</x:v>
+      </x:c>
+      <x:c r="E19" s="93" t="str">
+        <x:v>VC / Number</x:v>
+      </x:c>
+      <x:c r="F19" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G19" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H19" s="93" t="str">
+        <x:v>DAY([Date])</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="65" customHeight="1">
+      <x:c r="A20" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B20" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C20" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D20" s="93" t="str">
+        <x:v>_RowNumber</x:v>
+      </x:c>
+      <x:c r="E20" s="93" t="str">
+        <x:v>Physical / Number</x:v>
+      </x:c>
+      <x:c r="F20" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G20" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden Yes</x:v>
+      </x:c>
+      <x:c r="H20" s="93" t="str">
+        <x:v>Stored SQL value / generated date</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="65" customHeight="1">
+      <x:c r="A21" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B21" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C21" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D21" s="93" t="str">
+        <x:v>Row ID</x:v>
+      </x:c>
+      <x:c r="E21" s="93" t="str">
+        <x:v>Physical / Text</x:v>
+      </x:c>
+      <x:c r="F21" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G21" s="93" t="str">
+        <x:v>Key Yes; read-only Yes; hidden Yes</x:v>
+      </x:c>
+      <x:c r="H21" s="93" t="str">
+        <x:v>UNIQUEID("PackedUUID")</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="65" customHeight="1">
+      <x:c r="A22" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B22" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C22" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D22" s="93" t="str">
+        <x:v>Assessment ID</x:v>
+      </x:c>
+      <x:c r="E22" s="93" t="str">
+        <x:v>Physical / Text</x:v>
+      </x:c>
+      <x:c r="F22" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G22" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H22" s="93" t="str">
+        <x:v>Stored SQL value / generated date</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="65" customHeight="1">
+      <x:c r="A23" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B23" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C23" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D23" s="93" t="str">
+        <x:v>Ref Borrower</x:v>
+      </x:c>
+      <x:c r="E23" s="93" t="str">
+        <x:v>Physical / Ref</x:v>
+      </x:c>
+      <x:c r="F23" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G23" s="93" t="str">
+        <x:v>Key No; read-only No; hidden No</x:v>
+      </x:c>
+      <x:c r="H23" s="93" t="str">
+        <x:v>Stored SQL value / generated date</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="65" customHeight="1">
+      <x:c r="A24" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B24" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C24" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D24" s="93" t="str">
+        <x:v>Proposed Loan Amount</x:v>
+      </x:c>
+      <x:c r="E24" s="93" t="str">
+        <x:v>Physical / Price</x:v>
+      </x:c>
+      <x:c r="F24" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G24" s="93" t="str">
+        <x:v>Key No; read-only No; hidden No</x:v>
+      </x:c>
+      <x:c r="H24" s="93" t="str">
+        <x:v>Stored SQL value / generated date</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="65" customHeight="1">
+      <x:c r="A25" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B25" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C25" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D25" s="93" t="str">
+        <x:v>Minimum Daily Profit Rate</x:v>
+      </x:c>
+      <x:c r="E25" s="93" t="str">
+        <x:v>Physical / Percent</x:v>
+      </x:c>
+      <x:c r="F25" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G25" s="93" t="str">
+        <x:v>Key No; read-only No; hidden No</x:v>
+      </x:c>
+      <x:c r="H25" s="93" t="str">
+        <x:v>Stored SQL value / generated date</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="65" customHeight="1">
+      <x:c r="A26" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B26" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C26" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D26" s="93" t="str">
+        <x:v>SQL Current Principal</x:v>
+      </x:c>
+      <x:c r="E26" s="93" t="str">
+        <x:v>Physical / Decimal</x:v>
+      </x:c>
+      <x:c r="F26" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G26" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden Yes</x:v>
+      </x:c>
+      <x:c r="H26" s="93" t="str">
+        <x:v>Stored SQL value / generated date</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="65" customHeight="1">
+      <x:c r="A27" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B27" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C27" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D27" s="93" t="str">
+        <x:v>SQL Interest Received</x:v>
+      </x:c>
+      <x:c r="E27" s="93" t="str">
+        <x:v>Physical / Decimal</x:v>
+      </x:c>
+      <x:c r="F27" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G27" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden Yes</x:v>
+      </x:c>
+      <x:c r="H27" s="93" t="str">
+        <x:v>Stored SQL value / generated date</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="65" customHeight="1">
+      <x:c r="A28" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B28" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C28" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D28" s="93" t="str">
+        <x:v>SQL Eligible Date</x:v>
+      </x:c>
+      <x:c r="E28" s="93" t="str">
+        <x:v>Physical / Date</x:v>
+      </x:c>
+      <x:c r="F28" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G28" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden Yes</x:v>
+      </x:c>
+      <x:c r="H28" s="93" t="str">
+        <x:v>TODAY()</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="65" customHeight="1">
+      <x:c r="A29" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B29" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C29" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D29" s="93" t="str">
+        <x:v>SQL Eligible Interest</x:v>
+      </x:c>
+      <x:c r="E29" s="93" t="str">
+        <x:v>Physical / Decimal</x:v>
+      </x:c>
+      <x:c r="F29" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G29" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden Yes</x:v>
+      </x:c>
+      <x:c r="H29" s="93" t="str">
+        <x:v>Stored SQL value / generated date</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="65" customHeight="1">
+      <x:c r="A30" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B30" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C30" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D30" s="93" t="str">
+        <x:v>SQL Eligible Principal</x:v>
+      </x:c>
+      <x:c r="E30" s="93" t="str">
+        <x:v>Physical / Decimal</x:v>
+      </x:c>
+      <x:c r="F30" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G30" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden Yes</x:v>
+      </x:c>
+      <x:c r="H30" s="93" t="str">
+        <x:v>Stored SQL value / generated date</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="65" customHeight="1">
+      <x:c r="A31" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B31" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C31" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D31" s="93" t="str">
+        <x:v>SQL Eligible Profit</x:v>
+      </x:c>
+      <x:c r="E31" s="93" t="str">
+        <x:v>Physical / Decimal</x:v>
+      </x:c>
+      <x:c r="F31" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G31" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden Yes</x:v>
+      </x:c>
+      <x:c r="H31" s="93" t="str">
+        <x:v>Stored SQL value / generated date</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="65" customHeight="1">
+      <x:c r="A32" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B32" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C32" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D32" s="93" t="str">
+        <x:v>SQL Eligible Coverage</x:v>
+      </x:c>
+      <x:c r="E32" s="93" t="str">
+        <x:v>Physical / Decimal</x:v>
+      </x:c>
+      <x:c r="F32" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G32" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden Yes</x:v>
+      </x:c>
+      <x:c r="H32" s="93" t="str">
+        <x:v>Stored SQL value / generated date</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="65" customHeight="1">
+      <x:c r="A33" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B33" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C33" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D33" s="93" t="str">
+        <x:v>SQL Eligible Margin</x:v>
+      </x:c>
+      <x:c r="E33" s="93" t="str">
+        <x:v>Physical / Decimal</x:v>
+      </x:c>
+      <x:c r="F33" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G33" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden Yes</x:v>
+      </x:c>
+      <x:c r="H33" s="93" t="str">
+        <x:v>Stored SQL value / generated date</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="65" customHeight="1">
+      <x:c r="A34" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B34" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C34" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D34" s="93" t="str">
+        <x:v>SQL Current Margin</x:v>
+      </x:c>
+      <x:c r="E34" s="93" t="str">
+        <x:v>Physical / Decimal</x:v>
+      </x:c>
+      <x:c r="F34" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G34" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden Yes</x:v>
+      </x:c>
+      <x:c r="H34" s="93" t="str">
+        <x:v>Stored SQL value / generated date</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="65" customHeight="1">
+      <x:c r="A35" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B35" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C35" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D35" s="93" t="str">
+        <x:v>SQL Calculated At</x:v>
+      </x:c>
+      <x:c r="E35" s="93" t="str">
+        <x:v>Physical / DateTime</x:v>
+      </x:c>
+      <x:c r="F35" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G35" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H35" s="93" t="str">
+        <x:v>NOW()</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="65" customHeight="1">
+      <x:c r="A36" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B36" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C36" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D36" s="93" t="str">
+        <x:v>SQL As Of</x:v>
+      </x:c>
+      <x:c r="E36" s="93" t="str">
+        <x:v>Physical / Date</x:v>
+      </x:c>
+      <x:c r="F36" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G36" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden Yes</x:v>
+      </x:c>
+      <x:c r="H36" s="93" t="str">
+        <x:v>TODAY()</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="65" customHeight="1">
+      <x:c r="A37" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B37" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C37" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D37" s="93" t="str">
+        <x:v>SQL Forecast Start</x:v>
+      </x:c>
+      <x:c r="E37" s="93" t="str">
+        <x:v>Physical / Date</x:v>
+      </x:c>
+      <x:c r="F37" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G37" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden Yes</x:v>
+      </x:c>
+      <x:c r="H37" s="93" t="str">
+        <x:v>TODAY()</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="65" customHeight="1">
+      <x:c r="A38" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B38" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C38" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D38" s="93" t="str">
+        <x:v>SQL Forecast End</x:v>
+      </x:c>
+      <x:c r="E38" s="93" t="str">
+        <x:v>Physical / Date</x:v>
+      </x:c>
+      <x:c r="F38" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G38" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden Yes</x:v>
+      </x:c>
+      <x:c r="H38" s="93" t="str">
+        <x:v>TODAY()</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="65" customHeight="1">
+      <x:c r="A39" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B39" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C39" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D39" s="93" t="str">
+        <x:v>SQL Refresh Token</x:v>
+      </x:c>
+      <x:c r="E39" s="93" t="str">
+        <x:v>Physical / LongText</x:v>
+      </x:c>
+      <x:c r="F39" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G39" s="93" t="str">
+        <x:v>Key No; read-only No; hidden Yes</x:v>
+      </x:c>
+      <x:c r="H39" s="93" t="str">
+        <x:v>Stored SQL value / generated date</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="65" customHeight="1">
+      <x:c r="A40" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B40" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C40" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D40" s="93" t="str">
+        <x:v>SQL Source Fingerprint</x:v>
+      </x:c>
+      <x:c r="E40" s="93" t="str">
+        <x:v>Physical / LongText</x:v>
+      </x:c>
+      <x:c r="F40" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G40" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden Yes</x:v>
+      </x:c>
+      <x:c r="H40" s="93" t="str">
+        <x:v>Stored SQL value / generated date</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="65" customHeight="1">
+      <x:c r="A41" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B41" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C41" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D41" s="93" t="str">
+        <x:v>SQL Input Borrower</x:v>
+      </x:c>
+      <x:c r="E41" s="93" t="str">
+        <x:v>Physical / LongText</x:v>
+      </x:c>
+      <x:c r="F41" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G41" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden Yes</x:v>
+      </x:c>
+      <x:c r="H41" s="93" t="str">
+        <x:v>Stored SQL value / generated date</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="65" customHeight="1">
+      <x:c r="A42" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B42" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C42" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D42" s="93" t="str">
+        <x:v>SQL Input Amount</x:v>
+      </x:c>
+      <x:c r="E42" s="93" t="str">
+        <x:v>Physical / Decimal</x:v>
+      </x:c>
+      <x:c r="F42" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G42" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden Yes</x:v>
+      </x:c>
+      <x:c r="H42" s="93" t="str">
+        <x:v>Stored SQL value / generated date</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="65" customHeight="1">
+      <x:c r="A43" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B43" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C43" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D43" s="93" t="str">
+        <x:v>SQL Input Rate</x:v>
+      </x:c>
+      <x:c r="E43" s="93" t="str">
+        <x:v>Physical / Decimal</x:v>
+      </x:c>
+      <x:c r="F43" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G43" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden Yes</x:v>
+      </x:c>
+      <x:c r="H43" s="93" t="str">
+        <x:v>Stored SQL value / generated date</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="65" customHeight="1">
+      <x:c r="A44" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B44" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C44" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D44" s="93" t="str">
+        <x:v>SQL Source Current</x:v>
+      </x:c>
+      <x:c r="E44" s="93" t="str">
+        <x:v>Physical / Yes/No</x:v>
+      </x:c>
+      <x:c r="F44" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G44" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden Yes</x:v>
+      </x:c>
+      <x:c r="H44" s="93" t="str">
+        <x:v>Stored SQL value / generated date</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="100" customHeight="1">
+      <x:c r="A45" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B45" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C45" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D45" s="93" t="str">
+        <x:v>Current Outstanding Principal</x:v>
+      </x:c>
+      <x:c r="E45" s="93" t="str">
+        <x:v>VC / Price</x:v>
+      </x:c>
+      <x:c r="F45" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G45" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H45" s="93" t="str">
+        <x:v>IF(AND([SQL Source Current], [SQL As Of] = TODAY(), [Ref Borrower] = [SQL Input Borrower], [Proposed Loan Amount] = [SQL Input Amount], ABS([Minimum Daily Profit Rate] - [SQL Input Rate]) &lt; (1.0 / 10000000)), [SQL Current Principal], "")</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="100" customHeight="1">
+      <x:c r="A46" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B46" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C46" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D46" s="93" t="str">
+        <x:v>Interest Earned from Active Loans</x:v>
+      </x:c>
+      <x:c r="E46" s="93" t="str">
+        <x:v>VC / Price</x:v>
+      </x:c>
+      <x:c r="F46" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G46" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H46" s="93" t="str">
+        <x:v>IF(AND([SQL Source Current], [SQL As Of] = TODAY(), [Ref Borrower] = [SQL Input Borrower], [Proposed Loan Amount] = [SQL Input Amount], ABS([Minimum Daily Profit Rate] - [SQL Input Rate]) &lt; (1.0 / 10000000)), [SQL Interest Received], "")</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="100" customHeight="1">
+      <x:c r="A47" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B47" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C47" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D47" s="93" t="str">
+        <x:v>Earliest Eligible Date</x:v>
+      </x:c>
+      <x:c r="E47" s="93" t="str">
+        <x:v>VC / Date</x:v>
+      </x:c>
+      <x:c r="F47" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G47" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H47" s="93" t="str">
+        <x:v>IF(AND([SQL Source Current], [SQL As Of] = TODAY(), [Ref Borrower] = [SQL Input Borrower], [Proposed Loan Amount] = [SQL Input Amount], ABS([Minimum Daily Profit Rate] - [SQL Input Rate]) &lt; (1.0 / 10000000)), [SQL Eligible Date], "")</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="65" customHeight="1">
+      <x:c r="A48" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B48" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C48" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D48" s="93" t="str">
+        <x:v>Days Until Eligible</x:v>
+      </x:c>
+      <x:c r="E48" s="93" t="str">
+        <x:v>VC / Number</x:v>
+      </x:c>
+      <x:c r="F48" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G48" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H48" s="93" t="str">
+        <x:v>IF( ISBLANK([Earliest Eligible Date]), "", TOTALHOURS([Earliest Eligible Date] - TODAY()) / 24 )</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="100" customHeight="1">
+      <x:c r="A49" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B49" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C49" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D49" s="93" t="str">
+        <x:v>Projected Interest at Eligible Date</x:v>
+      </x:c>
+      <x:c r="E49" s="93" t="str">
+        <x:v>VC / Price</x:v>
+      </x:c>
+      <x:c r="F49" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G49" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H49" s="93" t="str">
+        <x:v>IF(AND([SQL Source Current], [SQL As Of] = TODAY(), [Ref Borrower] = [SQL Input Borrower], [Proposed Loan Amount] = [SQL Input Amount], ABS([Minimum Daily Profit Rate] - [SQL Input Rate]) &lt; (1.0 / 10000000)), [SQL Eligible Interest], "")</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="100" customHeight="1">
+      <x:c r="A50" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B50" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C50" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D50" s="93" t="str">
+        <x:v>Outstanding Principal at Eligible Date</x:v>
+      </x:c>
+      <x:c r="E50" s="93" t="str">
+        <x:v>VC / Price</x:v>
+      </x:c>
+      <x:c r="F50" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G50" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H50" s="93" t="str">
+        <x:v>IF(AND([SQL Source Current], [SQL As Of] = TODAY(), [Ref Borrower] = [SQL Input Borrower], [Proposed Loan Amount] = [SQL Input Amount], ABS([Minimum Daily Profit Rate] - [SQL Input Rate]) &lt; (1.0 / 10000000)), [SQL Eligible Principal], "")</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="100" customHeight="1">
+      <x:c r="A51" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B51" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C51" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D51" s="93" t="str">
+        <x:v>Minimum Profit at Eligible Date</x:v>
+      </x:c>
+      <x:c r="E51" s="93" t="str">
+        <x:v>VC / Price</x:v>
+      </x:c>
+      <x:c r="F51" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G51" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H51" s="93" t="str">
+        <x:v>IF(AND([SQL Source Current], [SQL As Of] = TODAY(), [Ref Borrower] = [SQL Input Borrower], [Proposed Loan Amount] = [SQL Input Amount], ABS([Minimum Daily Profit Rate] - [SQL Input Rate]) &lt; (1.0 / 10000000)), [SQL Eligible Profit], "")</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="100" customHeight="1">
+      <x:c r="A52" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B52" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C52" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D52" s="93" t="str">
+        <x:v>Required Coverage at Eligible Date</x:v>
+      </x:c>
+      <x:c r="E52" s="93" t="str">
+        <x:v>VC / Price</x:v>
+      </x:c>
+      <x:c r="F52" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G52" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H52" s="93" t="str">
+        <x:v>IF(AND([SQL Source Current], [SQL As Of] = TODAY(), [Ref Borrower] = [SQL Input Borrower], [Proposed Loan Amount] = [SQL Input Amount], ABS([Minimum Daily Profit Rate] - [SQL Input Rate]) &lt; (1.0 / 10000000)), [SQL Eligible Coverage], "")</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="100" customHeight="1">
+      <x:c r="A53" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B53" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C53" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D53" s="93" t="str">
+        <x:v>Safety Margin</x:v>
+      </x:c>
+      <x:c r="E53" s="93" t="str">
+        <x:v>VC / Price</x:v>
+      </x:c>
+      <x:c r="F53" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G53" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H53" s="93" t="str">
+        <x:v>IF(AND([SQL Source Current], [SQL As Of] = TODAY(), [Ref Borrower] = [SQL Input Borrower], [Proposed Loan Amount] = [SQL Input Amount], ABS([Minimum Daily Profit Rate] - [SQL Input Rate]) &lt; (1.0 / 10000000)), [SQL Eligible Margin], "")</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="100" customHeight="1">
+      <x:c r="A54" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B54" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C54" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D54" s="93" t="str">
+        <x:v>Current Coverage Margin</x:v>
+      </x:c>
+      <x:c r="E54" s="93" t="str">
+        <x:v>VC / Price</x:v>
+      </x:c>
+      <x:c r="F54" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G54" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H54" s="93" t="str">
+        <x:v>IF(AND([SQL Source Current], [SQL As Of] = TODAY(), [Ref Borrower] = [SQL Input Borrower], [Proposed Loan Amount] = [SQL Input Amount], ABS([Minimum Daily Profit Rate] - [SQL Input Rate]) &lt; (1.0 / 10000000)), [SQL Current Margin], "")</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="65" customHeight="1">
+      <x:c r="A55" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B55" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C55" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D55" s="93" t="str">
+        <x:v>Coverage Ratio at Eligible Date</x:v>
+      </x:c>
+      <x:c r="E55" s="93" t="str">
+        <x:v>VC / Percent</x:v>
+      </x:c>
+      <x:c r="F55" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G55" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H55" s="93" t="str">
+        <x:v>IF( [Required Coverage at Eligible Date] &gt; 0, [Projected Interest at Eligible Date] / [Required Coverage at Eligible Date], 0 )</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="100" customHeight="1">
+      <x:c r="A56" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B56" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C56" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D56" s="93" t="str">
+        <x:v>Recommendation Status</x:v>
+      </x:c>
+      <x:c r="E56" s="93" t="str">
+        <x:v>VC / Text</x:v>
+      </x:c>
+      <x:c r="F56" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G56" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H56" s="93" t="str">
+        <x:v>IF(NOT(AND([SQL Source Current], [SQL As Of] = TODAY(), [Ref Borrower] = [SQL Input Borrower], [Proposed Loan Amount] = [SQL Input Amount], ABS([Minimum Daily Profit Rate] - [SQL Input Rate]) &lt; (1.0 / 10000000))), "ต้องคำนวณใหม่ / Refresh required", IFS( ISBLANK([Earliest Eligible Date]), "ยังไม่ผ่านเกณฑ์ - Not Eligible", [Earliest Eligible Date] &lt;= TODAY(), "ปล่อยกู้ได้ตอนนี้ - Eligible Now", TRUE, "ควรรอก่อน - Wait" ))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="180" customHeight="1">
+      <x:c r="A57" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B57" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C57" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D57" s="93" t="str">
+        <x:v>Recommendation</x:v>
+      </x:c>
+      <x:c r="E57" s="93" t="str">
+        <x:v>VC / Text</x:v>
+      </x:c>
+      <x:c r="F57" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G57" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H57" s="93" t="str">
+        <x:v>IF(NOT(AND([SQL Source Current], [SQL As Of] = TODAY(), [Ref Borrower] = [SQL Input Borrower], [Proposed Loan Amount] = [SQL Input Amount], ABS([Minimum Daily Profit Rate] - [SQL Input Rate]) &lt; (1.0 / 10000000))), "กรุณาคำนวณใหม่และซิงค์ / Refresh assessment and sync before using this result", CONCATENATE(IFS( ISBLANK([Ref Borrower]), "กรุณาเลือกผู้กู้ / Select a borrower", OR(ISBLANK([Proposed Loan Amount]), [Proposed Loan Amount] &lt;= 0), "กรุณากรอกวงเงินกู้ที่เสนอ / Enter the proposed loan amount", OR(ISBLANK([Minimum Daily Profit Rate]), [Minimum Daily Profit Rate] &lt;= 0), "กรุณากรอกอัตรากำไรขั้นต่ำ / Enter the minimum profit rate", ISBLANK([Earliest Eligible Date]), "ไม่พบวันที่ผ่านเกณฑ์ภายในช่วงเวลาที่ประเมิน / No eligible date found within the forecast period", [Earliest Eligible Date] = TODAY(), "สามารถปล่อยกู้ได้วันนี้ / Eligible to issue the loan today", TRUE, CONCATENATE( "วันที่แนะนำให้ปล่อยกู้ได้เร็วที่สุด / Earliest recommended issue date: ", TEXT([Earliest Eligible Date], "DD/MM/YYYY") ) ), " | คำนวณเมื่อ / Calculated: ", TEXT([SQL Calculated At], "DD/MM/YYYY HH:MM:SS")))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="65" customHeight="1">
+      <x:c r="A58" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B58" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C58" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D58" s="93" t="str">
+        <x:v>Header - Current Position</x:v>
+      </x:c>
+      <x:c r="E58" s="93" t="str">
+        <x:v>VC / Text</x:v>
+      </x:c>
+      <x:c r="F58" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G58" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H58" s="93" t="str">
+        <x:v>"──── สถานะปัจจุบัน / Current Position ────"</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="65" customHeight="1">
+      <x:c r="A59" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B59" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C59" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D59" s="93" t="str">
+        <x:v>Header - Recommendation</x:v>
+      </x:c>
+      <x:c r="E59" s="93" t="str">
+        <x:v>VC / Text</x:v>
+      </x:c>
+      <x:c r="F59" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G59" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H59" s="93" t="str">
+        <x:v>"──── คำแนะนำ / Recommendation ────"</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="65" customHeight="1">
+      <x:c r="A60" s="93" t="str">
+        <x:v>SQL assessment</x:v>
+      </x:c>
+      <x:c r="B60" s="93" t="str">
+        <x:v>1.000022</x:v>
+      </x:c>
+      <x:c r="C60" s="93" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D60" s="93" t="str">
+        <x:v>Header - Calculation</x:v>
+      </x:c>
+      <x:c r="E60" s="93" t="str">
+        <x:v>VC / Text</x:v>
+      </x:c>
+      <x:c r="F60" s="93" t="str">
+        <x:v>Test copy only; production unchanged</x:v>
+      </x:c>
+      <x:c r="G60" s="93" t="str">
+        <x:v>Key No; read-only Yes; hidden No</x:v>
+      </x:c>
+      <x:c r="H60" s="93" t="str">
+        <x:v>"──── รายละเอียดการคำนวณ / Calculation ────"</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8521,7 +10111,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3bea91a1e86d4b56"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07429ad8f8104e98"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19178,7 +20768,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref9309fac28842d7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d3dff0a11164357"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19607,7 +21197,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra424ecf4053142ff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R669e4d0221e5439f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20067,7 +21657,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47b05cd0d51b479b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6d88fa538394de0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27041,7 +28631,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f4cef7ad5234c95"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9c980a0a0954b6e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31660,7 +33250,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68a4b3d789b5468f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbaf3505c63164994"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31859,7 +33449,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R121cfdcf720d426f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1af788574afb429b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33512,7 +35102,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re27eaf22dae84519"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd0432557b1542a5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Remove assessment refresh action and clarify pending results
</commit_message>
<xml_diff>
--- a/Documents/AppSheet_Data_Dictionary.xlsx
+++ b/Documents/AppSheet_Data_Dictionary.xlsx
@@ -2,22 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rc75993a5ae9741b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="R8e1e9dad4c3c4fc7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R811906d220094419"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="Rb33b55c9f30e43c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="Re59298d9cf21435f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="Re38426ef954f449c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Re659dca2847d4cbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R110eb759a3d54f14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="Rcb9cca1bacd54321"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R7e36101782984bea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="R983ac1f63b5b4e99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="R76201da1b8b34104"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Sync POC" sheetId="13" r:id="R51a155331f904249"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Migration Trial" sheetId="14" r:id="R5ef0f4c5e673403b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Production" sheetId="15" r:id="Rb18515b98bd14dcb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLAP Assessment SQL" sheetId="16" r:id="Rca4c901941ff47c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R65c5c2b4935747f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="Rbde9266364574c37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="Rf298e23b877f4dac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="Rd56e44aed9fe450d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="Recd9fd0e796e40f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="Rccd61c6a98944262"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Rd01ac0ffe8b24a15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R8e2f6f2d8cb0447b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="R5822318f31644305"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R76c1f0296e444599"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="R2451753417b14c4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="R8a9930d95e3f4412"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Sync POC" sheetId="13" r:id="Rb3240f1e473642c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Migration Trial" sheetId="14" r:id="R50e17d3d49234d10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Production" sheetId="15" r:id="Rdfacc9061291421f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLAP Assessment SQL" sheetId="16" r:id="R8642b05e82c94094"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2608,7 +2608,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf252e8990e2d478d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3b96f9a4cc84023"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8163,7 +8163,7 @@
         <x:v>Scope</x:v>
       </x:c>
       <x:c r="B2" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C2" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8189,7 +8189,7 @@
         <x:v>Scope</x:v>
       </x:c>
       <x:c r="B3" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C3" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8241,25 +8241,25 @@
         <x:v>Workflow</x:v>
       </x:c>
       <x:c r="B5" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C5" s="93" t="str">
         <x:v>Loan Assessment</x:v>
       </x:c>
       <x:c r="D5" s="93" t="str">
-        <x:v>Refresh Assessment</x:v>
+        <x:v>Save inputs</x:v>
       </x:c>
       <x:c r="E5" s="93" t="str">
-        <x:v>Data action</x:v>
+        <x:v>Normal app update</x:v>
       </x:c>
       <x:c r="F5" s="93" t="str">
         <x:v>Test copy only</x:v>
       </x:c>
       <x:c r="G5" s="93" t="str">
-        <x:v>Trigger recalculates current row; result timestamp shown</x:v>
+        <x:v>No separate refresh action. Input save invokes existing database triggers.</x:v>
       </x:c>
       <x:c r="H5" s="93" t="str">
-        <x:v>SQL Refresh Token = UNIQUEID()</x:v>
+        <x:v>Input update → database calculation → automatic sync returns stored results.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="65" customHeight="1">
@@ -8267,7 +8267,7 @@
         <x:v>Freshness</x:v>
       </x:c>
       <x:c r="B6" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C6" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8293,7 +8293,7 @@
         <x:v>Window</x:v>
       </x:c>
       <x:c r="B7" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C7" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8319,7 +8319,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B8" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C8" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8345,7 +8345,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B9" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C9" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8371,7 +8371,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B10" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C10" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8397,7 +8397,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B11" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C11" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8423,7 +8423,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B12" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C12" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8449,7 +8449,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B13" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C13" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8475,7 +8475,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B14" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C14" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8501,7 +8501,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B15" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C15" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8527,7 +8527,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B16" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C16" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8553,7 +8553,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B17" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C17" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8579,7 +8579,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B18" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C18" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8605,7 +8605,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B19" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C19" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8631,7 +8631,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B20" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C20" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8657,7 +8657,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B21" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C21" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8683,7 +8683,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B22" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C22" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8709,7 +8709,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B23" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C23" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8735,7 +8735,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B24" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C24" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8761,7 +8761,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B25" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C25" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8787,7 +8787,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B26" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C26" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8813,7 +8813,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B27" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C27" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8839,7 +8839,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B28" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C28" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8865,7 +8865,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B29" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C29" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8891,7 +8891,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B30" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C30" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8917,7 +8917,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B31" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C31" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8943,7 +8943,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B32" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C32" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8969,7 +8969,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B33" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C33" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8995,7 +8995,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B34" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C34" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9021,7 +9021,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B35" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C35" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9047,7 +9047,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B36" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C36" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9073,7 +9073,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B37" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C37" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9099,7 +9099,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B38" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C38" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9125,7 +9125,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B39" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C39" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9151,7 +9151,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B40" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C40" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9177,7 +9177,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B41" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C41" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9203,7 +9203,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B42" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C42" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9229,7 +9229,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B43" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C43" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9255,7 +9255,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B44" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C44" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9281,7 +9281,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B45" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C45" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9307,7 +9307,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B46" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C46" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9333,7 +9333,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B47" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C47" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9359,7 +9359,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B48" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C48" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9385,7 +9385,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B49" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C49" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9411,7 +9411,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B50" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C50" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9437,7 +9437,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B51" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C51" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9463,7 +9463,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B52" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C52" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9489,7 +9489,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B53" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C53" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9515,7 +9515,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B54" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C54" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9541,7 +9541,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B55" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C55" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9567,7 +9567,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B56" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C56" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9585,15 +9585,15 @@
         <x:v>Key No; read-only Yes; hidden No</x:v>
       </x:c>
       <x:c r="H56" s="93" t="str">
-        <x:v>IF(NOT(AND([SQL Source Current], [SQL As Of] = TODAY(), [Ref Borrower] = [SQL Input Borrower], [Proposed Loan Amount] = [SQL Input Amount], ABS([Minimum Daily Profit Rate] - [SQL Input Rate]) &lt; (1.0 / 10000000))), "ต้องคำนวณใหม่ / Refresh required", IFS( ISBLANK([Earliest Eligible Date]), "ยังไม่ผ่านเกณฑ์ - Not Eligible", [Earliest Eligible Date] &lt;= TODAY(), "ปล่อยกู้ได้ตอนนี้ - Eligible Now", TRUE, "ควรรอก่อน - Wait" ))</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="57" ht="180" customHeight="1">
+        <x:v>IF(NOT(AND([SQL Source Current], [SQL As Of] = TODAY(), [Ref Borrower] = [SQL Input Borrower], [Proposed Loan Amount] = [SQL Input Amount], ABS([Minimum Daily Profit Rate] - [SQL Input Rate]) &lt; (1.0 / 10000000))), IF(NOT(AND([Ref Borrower] = [SQL Input Borrower], [Proposed Loan Amount] = [SQL Input Amount], ABS([Minimum Daily Profit Rate] - [SQL Input Rate]) &lt; (1.0 / 10000000))), "กำลังรอผล / Awaiting results", "ผลไม่เป็นปัจจุบัน / Out of date"), IFS( ISBLANK([Earliest Eligible Date]), "ยังไม่ผ่านเกณฑ์ - Not Eligible", [Earliest Eligible Date] &lt;= TODAY(), "ปล่อยกู้ได้ตอนนี้ - Eligible Now", TRUE, "ควรรอก่อน - Wait" ))</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="260" customHeight="1">
       <x:c r="A57" s="93" t="str">
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B57" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C57" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9611,7 +9611,7 @@
         <x:v>Key No; read-only Yes; hidden No</x:v>
       </x:c>
       <x:c r="H57" s="93" t="str">
-        <x:v>IF(NOT(AND([SQL Source Current], [SQL As Of] = TODAY(), [Ref Borrower] = [SQL Input Borrower], [Proposed Loan Amount] = [SQL Input Amount], ABS([Minimum Daily Profit Rate] - [SQL Input Rate]) &lt; (1.0 / 10000000))), "กรุณาคำนวณใหม่และซิงค์ / Refresh assessment and sync before using this result", CONCATENATE(IFS( ISBLANK([Ref Borrower]), "กรุณาเลือกผู้กู้ / Select a borrower", OR(ISBLANK([Proposed Loan Amount]), [Proposed Loan Amount] &lt;= 0), "กรุณากรอกวงเงินกู้ที่เสนอ / Enter the proposed loan amount", OR(ISBLANK([Minimum Daily Profit Rate]), [Minimum Daily Profit Rate] &lt;= 0), "กรุณากรอกอัตรากำไรขั้นต่ำ / Enter the minimum profit rate", ISBLANK([Earliest Eligible Date]), "ไม่พบวันที่ผ่านเกณฑ์ภายในช่วงเวลาที่ประเมิน / No eligible date found within the forecast period", [Earliest Eligible Date] = TODAY(), "สามารถปล่อยกู้ได้วันนี้ / Eligible to issue the loan today", TRUE, CONCATENATE( "วันที่แนะนำให้ปล่อยกู้ได้เร็วที่สุด / Earliest recommended issue date: ", TEXT([Earliest Eligible Date], "DD/MM/YYYY") ) ), " | คำนวณเมื่อ / Calculated: ", TEXT([SQL Calculated At], "DD/MM/YYYY HH:MM:SS")))</x:v>
+        <x:v>IF(NOT(AND([SQL Source Current], [SQL As Of] = TODAY(), [Ref Borrower] = [SQL Input Borrower], [Proposed Loan Amount] = [SQL Input Amount], ABS([Minimum Daily Profit Rate] - [SQL Input Rate]) &lt; (1.0 / 10000000))), IF(NOT(AND([Ref Borrower] = [SQL Input Borrower], [Proposed Loan Amount] = [SQL Input Amount], ABS([Minimum Daily Profit Rate] - [SQL Input Rate]) &lt; (1.0 / 10000000))), "กำลังรอผลการคำนวณ ผลจะแสดงหลังบันทึกและซิงค์ / Waiting for calculation results. Results appear after saving and syncing.", "ผลการประเมินไม่เป็นปัจจุบัน กรุณาแก้ไขและบันทึกข้อมูลการประเมิน / Assessment is out of date. Update and save the assessment inputs."), CONCATENATE(IFS( ISBLANK([Ref Borrower]), "กรุณาเลือกผู้กู้ / Select a borrower", OR(ISBLANK([Proposed Loan Amount]), [Proposed Loan Amount] &lt;= 0), "กรุณากรอกวงเงินกู้ที่เสนอ / Enter the proposed loan amount", OR(ISBLANK([Minimum Daily Profit Rate]), [Minimum Daily Profit Rate] &lt;= 0), "กรุณากรอกอัตรากำไรขั้นต่ำ / Enter the minimum profit rate", ISBLANK([Earliest Eligible Date]), "ไม่พบวันที่ผ่านเกณฑ์ภายในช่วงเวลาที่ประเมิน / No eligible date found within the forecast period", [Earliest Eligible Date] = TODAY(), "สามารถปล่อยกู้ได้วันนี้ / Eligible to issue the loan today", TRUE, CONCATENATE( "วันที่แนะนำให้ปล่อยกู้ได้เร็วที่สุด / Earliest recommended issue date: ", TEXT([Earliest Eligible Date], "DD/MM/YYYY") ) ), " | คำนวณเมื่อ / Calculated: ", TEXT([SQL Calculated At], "DD/MM/YYYY HH:MM:SS")))</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="65" customHeight="1">
@@ -9619,7 +9619,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B58" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C58" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9645,7 +9645,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B59" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C59" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9671,7 +9671,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B60" s="93" t="str">
-        <x:v>1.000022</x:v>
+        <x:v>1.000023</x:v>
       </x:c>
       <x:c r="C60" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -10111,7 +10111,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07429ad8f8104e98"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc4586c9697c4e1d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20768,7 +20768,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d3dff0a11164357"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9aa59a5acf934a39"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21197,7 +21197,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R669e4d0221e5439f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf71ee72aa27343ce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21657,7 +21657,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6d88fa538394de0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R87f521d7c4d14c3f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28631,7 +28631,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9c980a0a0954b6e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R333d4218c5024daf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33250,7 +33250,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbaf3505c63164994"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4062a1612cd4af7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33449,7 +33449,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1af788574afb429b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3ef8edbc23c4505"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35102,7 +35102,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd0432557b1542a5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9eb67ce2c5334b17"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Verify development SQL clone and isolate both test apps
</commit_message>
<xml_diff>
--- a/Documents/AppSheet_Data_Dictionary.xlsx
+++ b/Documents/AppSheet_Data_Dictionary.xlsx
@@ -2,22 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R65c5c2b4935747f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="Rbde9266364574c37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="Rf298e23b877f4dac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="Rd56e44aed9fe450d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="Recd9fd0e796e40f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="Rccd61c6a98944262"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Rd01ac0ffe8b24a15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R8e2f6f2d8cb0447b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="R5822318f31644305"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R76c1f0296e444599"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="R2451753417b14c4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="R8a9930d95e3f4412"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Sync POC" sheetId="13" r:id="Rb3240f1e473642c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Migration Trial" sheetId="14" r:id="R50e17d3d49234d10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Production" sheetId="15" r:id="Rdfacc9061291421f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLAP Assessment SQL" sheetId="16" r:id="R8642b05e82c94094"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rd0aa167cac724a17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" r:id="R4eec06431cd84f0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="3" r:id="R8836cc2d5dd14bd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" r:id="R001ba3c11cfe48b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slices" sheetId="5" r:id="R901714bdf58c47ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice Columns" sheetId="6" r:id="R3ad83d1f279148cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Variances" sheetId="7" r:id="Rff6f67367f1b4fbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="8" r:id="R432740b4fb7f4b2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone" sheetId="9" r:id="Rc5609fcfd97149a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments Clone Slices" sheetId="10" r:id="R1d2d802798b846c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Performance Lab" sheetId="11" r:id="R2e6c5caceac84c9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLTP Combined Test" sheetId="12" r:id="Rf3845f1e480a4ecb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Sync POC" sheetId="13" r:id="R61977f26d118433f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Migration Trial" sheetId="14" r:id="R4036b39eaaaa4440"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Production" sheetId="15" r:id="R4129f0347a9e4d95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLAP Assessment SQL" sheetId="16" r:id="Recb23578d60c4130"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL Development" sheetId="17" r:id="R43199f78449c45ad"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -31,7 +32,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="13">
+  <x:fonts count="14">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -101,8 +102,13 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="37">
+  <x:fills count="39">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -137,6 +143,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -414,7 +430,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="132">
+  <x:cellXfs count="137">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -701,6 +717,21 @@
     <x:xf numFmtId="0" fontId="11" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="12" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="12" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2608,7 +2639,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3b96f9a4cc84023"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04853c1de13a408d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8163,7 +8194,7 @@
         <x:v>Scope</x:v>
       </x:c>
       <x:c r="B2" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C2" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8178,7 +8209,7 @@
         <x:v>Test copy only; review pending</x:v>
       </x:c>
       <x:c r="G2" s="93" t="str">
-        <x:v>Own input/result table; reads shared financial data</x:v>
+        <x:v>Own input/result table; development financial data on appsheet-pg-dev-20260915</x:v>
       </x:c>
       <x:c r="H2" s="93" t="str">
         <x:v>public.Loan Assessment SQL Lab View → public.Loan Assessment SQL Lab</x:v>
@@ -8189,7 +8220,7 @@
         <x:v>Scope</x:v>
       </x:c>
       <x:c r="B3" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C3" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8204,7 +8235,7 @@
         <x:v>Test copy only; read-only</x:v>
       </x:c>
       <x:c r="G3" s="93" t="str">
-        <x:v>153 dates retained for Daily Analytics; 16 assessment VCs removed</x:v>
+        <x:v>Generated date view on appsheet-pg-dev-20260915</x:v>
       </x:c>
       <x:c r="H3" s="93" t="str">
         <x:v>public.OLAP Calendar SQL Lab; 2026-08-01 through 2026-12-31</x:v>
@@ -8241,7 +8272,7 @@
         <x:v>Workflow</x:v>
       </x:c>
       <x:c r="B5" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C5" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8267,7 +8298,7 @@
         <x:v>Freshness</x:v>
       </x:c>
       <x:c r="B6" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C6" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8293,7 +8324,7 @@
         <x:v>Window</x:v>
       </x:c>
       <x:c r="B7" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C7" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8319,7 +8350,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B8" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C8" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8345,7 +8376,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B9" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C9" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8371,7 +8402,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B10" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C10" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8397,7 +8428,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B11" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C11" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8423,7 +8454,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B12" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C12" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8449,7 +8480,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B13" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C13" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8475,7 +8506,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B14" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C14" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8501,7 +8532,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B15" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C15" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8527,7 +8558,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B16" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C16" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8553,7 +8584,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B17" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C17" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8579,7 +8610,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B18" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C18" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8605,7 +8636,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B19" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C19" s="93" t="str">
         <x:v>Calendar</x:v>
@@ -8631,7 +8662,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B20" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C20" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8657,7 +8688,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B21" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C21" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8683,7 +8714,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B22" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C22" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8709,7 +8740,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B23" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C23" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8735,7 +8766,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B24" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C24" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8761,7 +8792,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B25" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C25" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8787,7 +8818,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B26" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C26" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8813,7 +8844,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B27" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C27" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8839,7 +8870,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B28" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C28" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8865,7 +8896,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B29" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C29" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8891,7 +8922,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B30" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C30" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8917,7 +8948,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B31" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C31" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8943,7 +8974,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B32" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C32" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8969,7 +9000,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B33" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C33" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -8995,7 +9026,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B34" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C34" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9021,7 +9052,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B35" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C35" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9047,7 +9078,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B36" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C36" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9073,7 +9104,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B37" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C37" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9099,7 +9130,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B38" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C38" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9125,7 +9156,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B39" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C39" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9151,7 +9182,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B40" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C40" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9177,7 +9208,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B41" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C41" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9203,7 +9234,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B42" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C42" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9229,7 +9260,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B43" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C43" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9255,7 +9286,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B44" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C44" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9281,7 +9312,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B45" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C45" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9307,7 +9338,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B46" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C46" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9333,7 +9364,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B47" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C47" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9359,7 +9390,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B48" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C48" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9385,7 +9416,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B49" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C49" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9411,7 +9442,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B50" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C50" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9437,7 +9468,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B51" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C51" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9463,7 +9494,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B52" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C52" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9489,7 +9520,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B53" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C53" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9515,7 +9546,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B54" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C54" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9541,7 +9572,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B55" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C55" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9567,7 +9598,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B56" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C56" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9593,7 +9624,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B57" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C57" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9619,7 +9650,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B58" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C58" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9645,7 +9676,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B59" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C59" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9671,7 +9702,7 @@
         <x:v>SQL assessment</x:v>
       </x:c>
       <x:c r="B60" s="93" t="str">
-        <x:v>1.000023</x:v>
+        <x:v>1.000025</x:v>
       </x:c>
       <x:c r="C60" s="93" t="str">
         <x:v>Loan Assessment</x:v>
@@ -9690,6 +9721,597 @@
       </x:c>
       <x:c r="H60" s="93" t="str">
         <x:v>"──── รายละเอียดการคำนวณ / Calculation ────"</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="32" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="34" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="34" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="60" customHeight="1">
+      <x:c r="A1" s="136" t="str">
+        <x:v>App</x:v>
+      </x:c>
+      <x:c r="B1" s="136" t="str">
+        <x:v>Version</x:v>
+      </x:c>
+      <x:c r="C1" s="136" t="str">
+        <x:v>Logical table</x:v>
+      </x:c>
+      <x:c r="D1" s="136" t="str">
+        <x:v>Source path</x:v>
+      </x:c>
+      <x:c r="E1" s="136" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="F1" s="136" t="str">
+        <x:v>Instance</x:v>
+      </x:c>
+      <x:c r="G1" s="136" t="str">
+        <x:v>Database</x:v>
+      </x:c>
+      <x:c r="H1" s="136" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="60" customHeight="1">
+      <x:c r="A2" s="73" t="str">
+        <x:v>LoanInsights PG Trial 20260914</x:v>
+      </x:c>
+      <x:c r="B2" s="73" t="str">
+        <x:v>1.000025</x:v>
+      </x:c>
+      <x:c r="C2" s="73" t="str">
+        <x:v>Borrowers</x:v>
+      </x:c>
+      <x:c r="D2" s="73" t="str">
+        <x:v>Borrowers</x:v>
+      </x:c>
+      <x:c r="E2" s="73" t="str">
+        <x:v>database-3</x:v>
+      </x:c>
+      <x:c r="F2" s="73" t="str">
+        <x:v>appsheet-pg-dev-20260915</x:v>
+      </x:c>
+      <x:c r="G2" s="73" t="str">
+        <x:v>loan_manager_prod</x:v>
+      </x:c>
+      <x:c r="H2" s="73" t="str">
+        <x:v>Development only; source binding verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="60" customHeight="1">
+      <x:c r="A3" s="73" t="str">
+        <x:v>LoanInsights PG Trial 20260914</x:v>
+      </x:c>
+      <x:c r="B3" s="73" t="str">
+        <x:v>1.000025</x:v>
+      </x:c>
+      <x:c r="C3" s="73" t="str">
+        <x:v>Loans</x:v>
+      </x:c>
+      <x:c r="D3" s="73" t="str">
+        <x:v>Loans</x:v>
+      </x:c>
+      <x:c r="E3" s="73" t="str">
+        <x:v>database-3</x:v>
+      </x:c>
+      <x:c r="F3" s="73" t="str">
+        <x:v>appsheet-pg-dev-20260915</x:v>
+      </x:c>
+      <x:c r="G3" s="73" t="str">
+        <x:v>loan_manager_prod</x:v>
+      </x:c>
+      <x:c r="H3" s="73" t="str">
+        <x:v>Development only; source binding verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="60" customHeight="1">
+      <x:c r="A4" s="73" t="str">
+        <x:v>LoanInsights PG Trial 20260914</x:v>
+      </x:c>
+      <x:c r="B4" s="73" t="str">
+        <x:v>1.000025</x:v>
+      </x:c>
+      <x:c r="C4" s="73" t="str">
+        <x:v>Repayments</x:v>
+      </x:c>
+      <x:c r="D4" s="73" t="str">
+        <x:v>Repayments</x:v>
+      </x:c>
+      <x:c r="E4" s="73" t="str">
+        <x:v>database-3</x:v>
+      </x:c>
+      <x:c r="F4" s="73" t="str">
+        <x:v>appsheet-pg-dev-20260915</x:v>
+      </x:c>
+      <x:c r="G4" s="73" t="str">
+        <x:v>loan_manager_prod</x:v>
+      </x:c>
+      <x:c r="H4" s="73" t="str">
+        <x:v>Development only; source binding verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="60" customHeight="1">
+      <x:c r="A5" s="73" t="str">
+        <x:v>LoanInsights PG Trial 20260914</x:v>
+      </x:c>
+      <x:c r="B5" s="73" t="str">
+        <x:v>1.000025</x:v>
+      </x:c>
+      <x:c r="C5" s="73" t="str">
+        <x:v>Statistics</x:v>
+      </x:c>
+      <x:c r="D5" s="73" t="str">
+        <x:v>Statistics</x:v>
+      </x:c>
+      <x:c r="E5" s="73" t="str">
+        <x:v>database-3</x:v>
+      </x:c>
+      <x:c r="F5" s="73" t="str">
+        <x:v>appsheet-pg-dev-20260915</x:v>
+      </x:c>
+      <x:c r="G5" s="73" t="str">
+        <x:v>loan_manager_prod</x:v>
+      </x:c>
+      <x:c r="H5" s="73" t="str">
+        <x:v>Development only; source binding verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="60" customHeight="1">
+      <x:c r="A6" s="73" t="str">
+        <x:v>LoanInsights PG Trial 20260914</x:v>
+      </x:c>
+      <x:c r="B6" s="73" t="str">
+        <x:v>1.000025</x:v>
+      </x:c>
+      <x:c r="C6" s="73" t="str">
+        <x:v>Charges</x:v>
+      </x:c>
+      <x:c r="D6" s="73" t="str">
+        <x:v>Charges</x:v>
+      </x:c>
+      <x:c r="E6" s="73" t="str">
+        <x:v>database-3</x:v>
+      </x:c>
+      <x:c r="F6" s="73" t="str">
+        <x:v>appsheet-pg-dev-20260915</x:v>
+      </x:c>
+      <x:c r="G6" s="73" t="str">
+        <x:v>loan_manager_prod</x:v>
+      </x:c>
+      <x:c r="H6" s="73" t="str">
+        <x:v>Development only; source binding verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="60" customHeight="1">
+      <x:c r="A7" s="73" t="str">
+        <x:v>LoanInsights PG Trial 20260914</x:v>
+      </x:c>
+      <x:c r="B7" s="73" t="str">
+        <x:v>1.000025</x:v>
+      </x:c>
+      <x:c r="C7" s="73" t="str">
+        <x:v>Calendar</x:v>
+      </x:c>
+      <x:c r="D7" s="73" t="str">
+        <x:v>OLAP Calendar SQL Lab</x:v>
+      </x:c>
+      <x:c r="E7" s="73" t="str">
+        <x:v>database-3</x:v>
+      </x:c>
+      <x:c r="F7" s="73" t="str">
+        <x:v>appsheet-pg-dev-20260915</x:v>
+      </x:c>
+      <x:c r="G7" s="73" t="str">
+        <x:v>loan_manager_prod</x:v>
+      </x:c>
+      <x:c r="H7" s="73" t="str">
+        <x:v>Development only; source binding verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="60" customHeight="1">
+      <x:c r="A8" s="73" t="str">
+        <x:v>LoanInsights PG Trial 20260914</x:v>
+      </x:c>
+      <x:c r="B8" s="73" t="str">
+        <x:v>1.000025</x:v>
+      </x:c>
+      <x:c r="C8" s="73" t="str">
+        <x:v>Loan Assessment</x:v>
+      </x:c>
+      <x:c r="D8" s="73" t="str">
+        <x:v>Loan Assessment SQL Lab View</x:v>
+      </x:c>
+      <x:c r="E8" s="73" t="str">
+        <x:v>database-3</x:v>
+      </x:c>
+      <x:c r="F8" s="73" t="str">
+        <x:v>appsheet-pg-dev-20260915</x:v>
+      </x:c>
+      <x:c r="G8" s="73" t="str">
+        <x:v>loan_manager_prod</x:v>
+      </x:c>
+      <x:c r="H8" s="73" t="str">
+        <x:v>Development only; source binding verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="60" customHeight="1">
+      <x:c r="A9" s="73" t="str">
+        <x:v>LoanInsights PG Trial 20260914</x:v>
+      </x:c>
+      <x:c r="B9" s="73" t="str">
+        <x:v>1.000025</x:v>
+      </x:c>
+      <x:c r="C9" s="73" t="str">
+        <x:v>Cash Pool Contributions</x:v>
+      </x:c>
+      <x:c r="D9" s="73" t="str">
+        <x:v>Cash Pool Contributions</x:v>
+      </x:c>
+      <x:c r="E9" s="73" t="str">
+        <x:v>database-3</x:v>
+      </x:c>
+      <x:c r="F9" s="73" t="str">
+        <x:v>appsheet-pg-dev-20260915</x:v>
+      </x:c>
+      <x:c r="G9" s="73" t="str">
+        <x:v>loan_manager_prod</x:v>
+      </x:c>
+      <x:c r="H9" s="73" t="str">
+        <x:v>Development only; source binding verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="60" customHeight="1">
+      <x:c r="A10" s="73" t="str">
+        <x:v>LoanInsights PG Trial 20260914</x:v>
+      </x:c>
+      <x:c r="B10" s="73" t="str">
+        <x:v>1.000025</x:v>
+      </x:c>
+      <x:c r="C10" s="73" t="str">
+        <x:v>Partners</x:v>
+      </x:c>
+      <x:c r="D10" s="73" t="str">
+        <x:v>Partners</x:v>
+      </x:c>
+      <x:c r="E10" s="73" t="str">
+        <x:v>database-3</x:v>
+      </x:c>
+      <x:c r="F10" s="73" t="str">
+        <x:v>appsheet-pg-dev-20260915</x:v>
+      </x:c>
+      <x:c r="G10" s="73" t="str">
+        <x:v>loan_manager_prod</x:v>
+      </x:c>
+      <x:c r="H10" s="73" t="str">
+        <x:v>Development only; source binding verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="60" customHeight="1">
+      <x:c r="A11" s="73" t="str">
+        <x:v>LoanInsights PG Trial 20260914</x:v>
+      </x:c>
+      <x:c r="B11" s="73" t="str">
+        <x:v>1.000025</x:v>
+      </x:c>
+      <x:c r="C11" s="73" t="str">
+        <x:v>Settlements</x:v>
+      </x:c>
+      <x:c r="D11" s="73" t="str">
+        <x:v>Settlements</x:v>
+      </x:c>
+      <x:c r="E11" s="73" t="str">
+        <x:v>database-3</x:v>
+      </x:c>
+      <x:c r="F11" s="73" t="str">
+        <x:v>appsheet-pg-dev-20260915</x:v>
+      </x:c>
+      <x:c r="G11" s="73" t="str">
+        <x:v>loan_manager_prod</x:v>
+      </x:c>
+      <x:c r="H11" s="73" t="str">
+        <x:v>Development only; source binding verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="60" customHeight="1">
+      <x:c r="A12" s="73" t="str">
+        <x:v>LoanInsights PG Trial 20260914</x:v>
+      </x:c>
+      <x:c r="B12" s="73" t="str">
+        <x:v>1.000025</x:v>
+      </x:c>
+      <x:c r="C12" s="73" t="str">
+        <x:v>Daily Analytics</x:v>
+      </x:c>
+      <x:c r="D12" s="73" t="str">
+        <x:v>Daily Analytics</x:v>
+      </x:c>
+      <x:c r="E12" s="73" t="str">
+        <x:v>database-3</x:v>
+      </x:c>
+      <x:c r="F12" s="73" t="str">
+        <x:v>appsheet-pg-dev-20260915</x:v>
+      </x:c>
+      <x:c r="G12" s="73" t="str">
+        <x:v>loan_manager_prod</x:v>
+      </x:c>
+      <x:c r="H12" s="73" t="str">
+        <x:v>Development only; source binding verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="60" customHeight="1">
+      <x:c r="A13" s="73" t="str">
+        <x:v>LoanInsights PG Trial 20260914</x:v>
+      </x:c>
+      <x:c r="B13" s="73" t="str">
+        <x:v>1.000025</x:v>
+      </x:c>
+      <x:c r="C13" s="73" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D13" s="73" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="E13" s="73" t="str">
+        <x:v>database-3</x:v>
+      </x:c>
+      <x:c r="F13" s="73" t="str">
+        <x:v>appsheet-pg-dev-20260915</x:v>
+      </x:c>
+      <x:c r="G13" s="73" t="str">
+        <x:v>loan_manager_prod</x:v>
+      </x:c>
+      <x:c r="H13" s="73" t="str">
+        <x:v>Development only; source binding verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="60" customHeight="1">
+      <x:c r="A14" s="73" t="str">
+        <x:v>LoanInsights PG Trial 20260914</x:v>
+      </x:c>
+      <x:c r="B14" s="73" t="str">
+        <x:v>1.000025</x:v>
+      </x:c>
+      <x:c r="C14" s="73" t="str">
+        <x:v>Payments</x:v>
+      </x:c>
+      <x:c r="D14" s="73" t="str">
+        <x:v>Payments</x:v>
+      </x:c>
+      <x:c r="E14" s="73" t="str">
+        <x:v>database-3</x:v>
+      </x:c>
+      <x:c r="F14" s="73" t="str">
+        <x:v>appsheet-pg-dev-20260915</x:v>
+      </x:c>
+      <x:c r="G14" s="73" t="str">
+        <x:v>loan_manager_prod</x:v>
+      </x:c>
+      <x:c r="H14" s="73" t="str">
+        <x:v>Development only; source binding verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="60" customHeight="1">
+      <x:c r="A15" s="73" t="str">
+        <x:v>LoanMgr PG Test 20260914</x:v>
+      </x:c>
+      <x:c r="B15" s="73" t="str">
+        <x:v>1.000011</x:v>
+      </x:c>
+      <x:c r="C15" s="73" t="str">
+        <x:v>Borrowers</x:v>
+      </x:c>
+      <x:c r="D15" s="73" t="str">
+        <x:v>Borrowers</x:v>
+      </x:c>
+      <x:c r="E15" s="73" t="str">
+        <x:v>database-3</x:v>
+      </x:c>
+      <x:c r="F15" s="73" t="str">
+        <x:v>appsheet-pg-dev-20260915</x:v>
+      </x:c>
+      <x:c r="G15" s="73" t="str">
+        <x:v>loan_manager_prod</x:v>
+      </x:c>
+      <x:c r="H15" s="73" t="str">
+        <x:v>Development only; source binding verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="60" customHeight="1">
+      <x:c r="A16" s="73" t="str">
+        <x:v>LoanMgr PG Test 20260914</x:v>
+      </x:c>
+      <x:c r="B16" s="73" t="str">
+        <x:v>1.000011</x:v>
+      </x:c>
+      <x:c r="C16" s="73" t="str">
+        <x:v>Loans</x:v>
+      </x:c>
+      <x:c r="D16" s="73" t="str">
+        <x:v>Loans</x:v>
+      </x:c>
+      <x:c r="E16" s="73" t="str">
+        <x:v>database-3</x:v>
+      </x:c>
+      <x:c r="F16" s="73" t="str">
+        <x:v>appsheet-pg-dev-20260915</x:v>
+      </x:c>
+      <x:c r="G16" s="73" t="str">
+        <x:v>loan_manager_prod</x:v>
+      </x:c>
+      <x:c r="H16" s="73" t="str">
+        <x:v>Development only; source binding verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="60" customHeight="1">
+      <x:c r="A17" s="73" t="str">
+        <x:v>LoanMgr PG Test 20260914</x:v>
+      </x:c>
+      <x:c r="B17" s="73" t="str">
+        <x:v>1.000011</x:v>
+      </x:c>
+      <x:c r="C17" s="73" t="str">
+        <x:v>Repayments</x:v>
+      </x:c>
+      <x:c r="D17" s="73" t="str">
+        <x:v>Repayments</x:v>
+      </x:c>
+      <x:c r="E17" s="73" t="str">
+        <x:v>database-3</x:v>
+      </x:c>
+      <x:c r="F17" s="73" t="str">
+        <x:v>appsheet-pg-dev-20260915</x:v>
+      </x:c>
+      <x:c r="G17" s="73" t="str">
+        <x:v>loan_manager_prod</x:v>
+      </x:c>
+      <x:c r="H17" s="73" t="str">
+        <x:v>Development only; source binding verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="60" customHeight="1">
+      <x:c r="A18" s="73" t="str">
+        <x:v>LoanMgr PG Test 20260914</x:v>
+      </x:c>
+      <x:c r="B18" s="73" t="str">
+        <x:v>1.000011</x:v>
+      </x:c>
+      <x:c r="C18" s="73" t="str">
+        <x:v>Statistics</x:v>
+      </x:c>
+      <x:c r="D18" s="73" t="str">
+        <x:v>Statistics</x:v>
+      </x:c>
+      <x:c r="E18" s="73" t="str">
+        <x:v>database-3</x:v>
+      </x:c>
+      <x:c r="F18" s="73" t="str">
+        <x:v>appsheet-pg-dev-20260915</x:v>
+      </x:c>
+      <x:c r="G18" s="73" t="str">
+        <x:v>loan_manager_prod</x:v>
+      </x:c>
+      <x:c r="H18" s="73" t="str">
+        <x:v>Development only; source binding verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="60" customHeight="1">
+      <x:c r="A19" s="73" t="str">
+        <x:v>LoanMgr PG Test 20260914</x:v>
+      </x:c>
+      <x:c r="B19" s="73" t="str">
+        <x:v>1.000011</x:v>
+      </x:c>
+      <x:c r="C19" s="73" t="str">
+        <x:v>Charges</x:v>
+      </x:c>
+      <x:c r="D19" s="73" t="str">
+        <x:v>Charges</x:v>
+      </x:c>
+      <x:c r="E19" s="73" t="str">
+        <x:v>database-3</x:v>
+      </x:c>
+      <x:c r="F19" s="73" t="str">
+        <x:v>appsheet-pg-dev-20260915</x:v>
+      </x:c>
+      <x:c r="G19" s="73" t="str">
+        <x:v>loan_manager_prod</x:v>
+      </x:c>
+      <x:c r="H19" s="73" t="str">
+        <x:v>Development only; source binding verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="60" customHeight="1">
+      <x:c r="A20" s="73" t="str">
+        <x:v>LoanMgr PG Test 20260914</x:v>
+      </x:c>
+      <x:c r="B20" s="73" t="str">
+        <x:v>1.000011</x:v>
+      </x:c>
+      <x:c r="C20" s="73" t="str">
+        <x:v>Partners</x:v>
+      </x:c>
+      <x:c r="D20" s="73" t="str">
+        <x:v>Partners</x:v>
+      </x:c>
+      <x:c r="E20" s="73" t="str">
+        <x:v>database-3</x:v>
+      </x:c>
+      <x:c r="F20" s="73" t="str">
+        <x:v>appsheet-pg-dev-20260915</x:v>
+      </x:c>
+      <x:c r="G20" s="73" t="str">
+        <x:v>loan_manager_prod</x:v>
+      </x:c>
+      <x:c r="H20" s="73" t="str">
+        <x:v>Development only; source binding verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="60" customHeight="1">
+      <x:c r="A21" s="73" t="str">
+        <x:v>LoanMgr PG Test 20260914</x:v>
+      </x:c>
+      <x:c r="B21" s="73" t="str">
+        <x:v>1.000011</x:v>
+      </x:c>
+      <x:c r="C21" s="73" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="D21" s="73" t="str">
+        <x:v>Payment Allocations</x:v>
+      </x:c>
+      <x:c r="E21" s="73" t="str">
+        <x:v>database-3</x:v>
+      </x:c>
+      <x:c r="F21" s="73" t="str">
+        <x:v>appsheet-pg-dev-20260915</x:v>
+      </x:c>
+      <x:c r="G21" s="73" t="str">
+        <x:v>loan_manager_prod</x:v>
+      </x:c>
+      <x:c r="H21" s="73" t="str">
+        <x:v>Development only; source binding verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="60" customHeight="1">
+      <x:c r="A22" s="73" t="str">
+        <x:v>LoanMgr PG Test 20260914</x:v>
+      </x:c>
+      <x:c r="B22" s="73" t="str">
+        <x:v>1.000011</x:v>
+      </x:c>
+      <x:c r="C22" s="73" t="str">
+        <x:v>Payments</x:v>
+      </x:c>
+      <x:c r="D22" s="73" t="str">
+        <x:v>Payments</x:v>
+      </x:c>
+      <x:c r="E22" s="73" t="str">
+        <x:v>database-3</x:v>
+      </x:c>
+      <x:c r="F22" s="73" t="str">
+        <x:v>appsheet-pg-dev-20260915</x:v>
+      </x:c>
+      <x:c r="G22" s="73" t="str">
+        <x:v>loan_manager_prod</x:v>
+      </x:c>
+      <x:c r="H22" s="73" t="str">
+        <x:v>Development only; source binding verified</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -10111,7 +10733,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc4586c9697c4e1d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d5a760a9c9f4300"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20768,7 +21390,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9aa59a5acf934a39"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e6138cd4fac48bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21197,7 +21819,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf71ee72aa27343ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0029ef6058d24aeb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21657,7 +22279,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R87f521d7c4d14c3f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5199fd1f26984dba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28631,7 +29253,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R333d4218c5024daf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9acf103a4164e71"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33250,7 +33872,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4062a1612cd4af7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a86648460894460"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33449,7 +34071,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3ef8edbc23c4505"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe91c8096f154c9f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35102,7 +35724,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9eb67ce2c5334b17"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83d2ac6408584b89"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>